<commit_message>
Forecast update 2026-07-26 (100 days out)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Data as of 2026-07-25 · evaluated at 0 days to election (actual: 101 days out)</t>
+          <t>Data as of 2026-07-26 · evaluated at 0 days to election (actual: 100 days out)</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>50.9</v>
+        <v>50</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,10 +566,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.1</v>
+        <v>231.9</v>
       </c>
       <c r="C9" t="n">
-        <v>202.9</v>
+        <v>203.1</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.3</v>
+        <v>24.5</v>
       </c>
       <c r="C10" t="n">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
       <c r="D10" t="n">
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>39.5</v>
+        <v>41.6</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.6</v>
+        <v>-2.86</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>39.1</v>
+        <v>41</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>60.9</v>
+        <v>59</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="AB2" s="4" t="n">
-        <v>44.4</v>
+        <v>44.38</v>
       </c>
       <c r="AC2" s="4" t="n">
-        <v>47.6</v>
+        <v>47.62</v>
       </c>
       <c r="AD2" s="4" t="n">
         <v>8</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>26.78</v>
+        <v>26.81</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>100</v>
@@ -1394,10 +1394,10 @@
         <v>0</v>
       </c>
       <c r="AB6" s="4" t="n">
-        <v>63.39</v>
+        <v>63.4</v>
       </c>
       <c r="AC6" s="4" t="n">
-        <v>36.61</v>
+        <v>36.6</v>
       </c>
       <c r="AD6" s="4" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>17.56</v>
+        <v>17.6</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>99.59999999999999</v>
@@ -1610,10 +1610,10 @@
         <v>0</v>
       </c>
       <c r="AB8" s="4" t="n">
-        <v>58.78</v>
+        <v>58.8</v>
       </c>
       <c r="AC8" s="4" t="n">
-        <v>41.22</v>
+        <v>41.2</v>
       </c>
       <c r="AD8" s="4" t="n">
         <v>0</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>-6.05</v>
+        <v>-6.06</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>15.5</v>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2.88</v>
+        <v>2.86</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>73</v>
@@ -1818,10 +1818,10 @@
         <v>0</v>
       </c>
       <c r="AB10" s="4" t="n">
-        <v>51.44</v>
+        <v>51.43</v>
       </c>
       <c r="AC10" s="4" t="n">
-        <v>48.56</v>
+        <v>48.57</v>
       </c>
       <c r="AD10" s="4" t="n">
         <v>0</v>
@@ -2024,10 +2024,10 @@
         <v>0</v>
       </c>
       <c r="AB12" s="4" t="n">
-        <v>52.82</v>
+        <v>52.83</v>
       </c>
       <c r="AC12" s="4" t="n">
-        <v>47.18</v>
+        <v>47.17</v>
       </c>
       <c r="AD12" s="4" t="n">
         <v>0</v>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>29.24</v>
+        <v>29.26</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>100</v>
@@ -2440,10 +2440,10 @@
         <v>0</v>
       </c>
       <c r="AB16" s="4" t="n">
-        <v>64.62</v>
+        <v>64.63</v>
       </c>
       <c r="AC16" s="4" t="n">
-        <v>35.38</v>
+        <v>35.37</v>
       </c>
       <c r="AD16" s="4" t="n">
         <v>0</v>
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>12.58</v>
+        <v>12.56</v>
       </c>
       <c r="J18" s="4" t="n">
         <v>99</v>
@@ -2656,10 +2656,10 @@
         <v>0</v>
       </c>
       <c r="AB18" s="4" t="n">
-        <v>55.65</v>
+        <v>55.64</v>
       </c>
       <c r="AC18" s="4" t="n">
-        <v>43.21</v>
+        <v>43.22</v>
       </c>
       <c r="AD18" s="4" t="n">
         <v>0</v>
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="I19" s="4" t="n">
-        <v>12.39</v>
+        <v>12.4</v>
       </c>
       <c r="J19" s="4" t="n">
         <v>98.90000000000001</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>12.48</v>
+        <v>12.47</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>98.90000000000001</v>
@@ -2864,10 +2864,10 @@
         <v>0</v>
       </c>
       <c r="AB20" s="4" t="n">
-        <v>56.24</v>
+        <v>56.23</v>
       </c>
       <c r="AC20" s="4" t="n">
-        <v>43.76</v>
+        <v>43.77</v>
       </c>
       <c r="AD20" s="4" t="n">
         <v>0</v>
@@ -3027,13 +3027,13 @@
         </is>
       </c>
       <c r="I22" s="4" t="n">
-        <v>-10.6</v>
+        <v>-10.61</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>97.2</v>
+        <v>97.3</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -3084,10 +3084,10 @@
         <v>0</v>
       </c>
       <c r="AB22" s="4" t="n">
-        <v>44.7</v>
+        <v>44.69</v>
       </c>
       <c r="AC22" s="4" t="n">
-        <v>55.3</v>
+        <v>55.31</v>
       </c>
       <c r="AD22" s="4" t="n">
         <v>0</v>
@@ -3131,13 +3131,13 @@
         </is>
       </c>
       <c r="I23" s="4" t="n">
-        <v>6.63</v>
+        <v>6.68</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>86.3</v>
+        <v>86.5</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -3188,10 +3188,10 @@
         <v>0</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>53.31</v>
+        <v>53.34</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>46.69</v>
+        <v>46.66</v>
       </c>
       <c r="AD23" s="4" t="n">
         <v>0</v>
@@ -3239,7 +3239,7 @@
         </is>
       </c>
       <c r="I24" s="4" t="n">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
       <c r="J24" s="4" t="n">
         <v>67.8</v>
@@ -3296,10 +3296,10 @@
         <v>0</v>
       </c>
       <c r="AB24" s="4" t="n">
-        <v>50.76</v>
+        <v>50.77</v>
       </c>
       <c r="AC24" s="4" t="n">
-        <v>49.24</v>
+        <v>49.23</v>
       </c>
       <c r="AD24" s="4" t="n">
         <v>0</v>
@@ -3347,7 +3347,7 @@
         </is>
       </c>
       <c r="I25" s="4" t="n">
-        <v>15.13</v>
+        <v>15.12</v>
       </c>
       <c r="J25" s="4" t="n">
         <v>99.3</v>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="I26" s="4" t="n">
-        <v>-3.37</v>
+        <v>-3.38</v>
       </c>
       <c r="J26" s="4" t="n">
         <v>25.1</v>
@@ -3508,10 +3508,10 @@
         <v>0</v>
       </c>
       <c r="AB26" s="4" t="n">
-        <v>48.32</v>
+        <v>48.31</v>
       </c>
       <c r="AC26" s="4" t="n">
-        <v>51.68</v>
+        <v>51.69</v>
       </c>
       <c r="AD26" s="4" t="n">
         <v>0</v>
@@ -3657,13 +3657,13 @@
         </is>
       </c>
       <c r="I28" s="4" t="n">
-        <v>4.37</v>
+        <v>4.39</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>78.59999999999999</v>
+        <v>78.7</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="I29" s="4" t="n">
-        <v>16.45</v>
+        <v>16.46</v>
       </c>
       <c r="J29" s="4" t="n">
         <v>99.5</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>19.57</v>
+        <v>19.59</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.7</v>
@@ -4226,10 +4226,10 @@
         <v>0</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>39.42</v>
+        <v>39.43</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>60.58</v>
+        <v>60.57</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>0</v>
@@ -4277,7 +4277,7 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>-8.6</v>
+        <v>-8.609999999999999</v>
       </c>
       <c r="J34" s="4" t="n">
         <v>7.8</v>
@@ -4385,7 +4385,7 @@
         </is>
       </c>
       <c r="I35" s="4" t="n">
-        <v>-18.56</v>
+        <v>-18.66</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>0.3</v>
@@ -4442,10 +4442,10 @@
         <v>0</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>40.72</v>
+        <v>40.67</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>59.28</v>
+        <v>59.33</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>0</v>
@@ -4489,13 +4489,13 @@
         </is>
       </c>
       <c r="I36" s="4" t="n">
-        <v>1.9</v>
+        <v>1.92</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>69.2</v>
+        <v>69.3</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -4546,10 +4546,10 @@
         <v>0</v>
       </c>
       <c r="AB36" s="4" t="n">
-        <v>50.95</v>
+        <v>50.96</v>
       </c>
       <c r="AC36" s="4" t="n">
-        <v>49.05</v>
+        <v>49.04</v>
       </c>
       <c r="AD36" s="4" t="n">
         <v>0</v>
@@ -4695,27 +4695,27 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.19</v>
+        <v>-2.96</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>38.9</v>
+        <v>41.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>61.1</v>
+        <v>58.9</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.71</v>
+        <v>-2.51</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.41</v>
+        <v>-1.21</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.1</v>
@@ -4750,16 +4750,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.41</v>
+        <v>48.52</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>38.9</v>
+        <v>41.1</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.59</v>
+        <v>51.48</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -4962,10 +4962,10 @@
         <v>0</v>
       </c>
       <c r="AB40" s="4" t="n">
-        <v>48.4</v>
+        <v>48.41</v>
       </c>
       <c r="AC40" s="4" t="n">
-        <v>51.6</v>
+        <v>51.59</v>
       </c>
       <c r="AD40" s="4" t="n">
         <v>0</v>
@@ -6035,13 +6035,13 @@
         </is>
       </c>
       <c r="I51" s="4" t="n">
-        <v>-0.76</v>
+        <v>-0.72</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>64.7</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -6092,10 +6092,10 @@
         <v>0</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>49.62</v>
+        <v>49.64</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>50.38</v>
+        <v>50.36</v>
       </c>
       <c r="AD51" s="4" t="n">
         <v>0</v>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="I55" s="4" t="n">
-        <v>4.79</v>
+        <v>4.8</v>
       </c>
       <c r="J55" s="4" t="n">
         <v>80.09999999999999</v>
@@ -6502,10 +6502,10 @@
         <v>0</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>51.28</v>
+        <v>51.29</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>46.6</v>
+        <v>46.59</v>
       </c>
       <c r="AD55" s="4" t="n">
         <v>2.12</v>
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="M59" s="4" t="n">
-        <v>15.45</v>
+        <v>15.46</v>
       </c>
       <c r="N59" s="4" t="n">
         <v>5.13</v>
@@ -6961,7 +6961,7 @@
         </is>
       </c>
       <c r="I60" s="4" t="n">
-        <v>33.31</v>
+        <v>33.32</v>
       </c>
       <c r="J60" s="4" t="n">
         <v>100</v>
@@ -6975,13 +6975,13 @@
         </is>
       </c>
       <c r="M60" s="4" t="n">
-        <v>27.83</v>
+        <v>27.84</v>
       </c>
       <c r="N60" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O60" s="4" t="n">
-        <v>33.31</v>
+        <v>33.32</v>
       </c>
       <c r="P60" s="4" t="n">
         <v>0</v>
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="I61" s="4" t="n">
-        <v>21.12</v>
+        <v>21.13</v>
       </c>
       <c r="J61" s="4" t="n">
         <v>99.8</v>
@@ -7083,7 +7083,7 @@
         <v>5.13</v>
       </c>
       <c r="O61" s="4" t="n">
-        <v>21.12</v>
+        <v>21.13</v>
       </c>
       <c r="P61" s="4" t="n">
         <v>1.08</v>
@@ -7179,13 +7179,13 @@
         </is>
       </c>
       <c r="M62" s="4" t="n">
-        <v>18.28</v>
+        <v>18.29</v>
       </c>
       <c r="N62" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O62" s="4" t="n">
-        <v>26.54</v>
+        <v>26.55</v>
       </c>
       <c r="P62" s="4" t="n">
         <v>0</v>
@@ -7267,7 +7267,7 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>-18.24</v>
+        <v>-18.23</v>
       </c>
       <c r="J63" s="4" t="n">
         <v>0.3</v>
@@ -7287,7 +7287,7 @@
         <v>5.13</v>
       </c>
       <c r="O63" s="4" t="n">
-        <v>-18.24</v>
+        <v>-18.23</v>
       </c>
       <c r="P63" s="4" t="n">
         <v>-0.65</v>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="I64" s="4" t="n">
-        <v>12.39</v>
+        <v>12.4</v>
       </c>
       <c r="J64" s="4" t="n">
         <v>98.90000000000001</v>
@@ -7383,13 +7383,13 @@
         </is>
       </c>
       <c r="M64" s="4" t="n">
-        <v>11.25</v>
+        <v>11.26</v>
       </c>
       <c r="N64" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>12.39</v>
+        <v>12.4</v>
       </c>
       <c r="P64" s="4" t="n">
         <v>-0.35</v>
@@ -7491,7 +7491,7 @@
         <v>5.13</v>
       </c>
       <c r="O65" s="4" t="n">
-        <v>25.41</v>
+        <v>25.42</v>
       </c>
       <c r="P65" s="4" t="n">
         <v>0</v>
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="M66" s="4" t="n">
-        <v>39.18</v>
+        <v>39.19</v>
       </c>
       <c r="N66" s="4" t="n">
         <v>5.13</v>
@@ -7624,10 +7624,10 @@
         <v>0</v>
       </c>
       <c r="AB66" s="4" t="n">
-        <v>74.48</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="AC66" s="4" t="n">
-        <v>25.52</v>
+        <v>25.51</v>
       </c>
       <c r="AD66" s="4" t="n">
         <v>0</v>
@@ -7675,7 +7675,7 @@
         </is>
       </c>
       <c r="I67" s="4" t="n">
-        <v>30.7</v>
+        <v>30.71</v>
       </c>
       <c r="J67" s="4" t="n">
         <v>100</v>
@@ -7695,7 +7695,7 @@
         <v>5.13</v>
       </c>
       <c r="O67" s="4" t="n">
-        <v>30.7</v>
+        <v>30.71</v>
       </c>
       <c r="P67" s="4" t="n">
         <v>2.78</v>
@@ -7777,7 +7777,7 @@
         </is>
       </c>
       <c r="I68" s="4" t="n">
-        <v>42.87</v>
+        <v>42.88</v>
       </c>
       <c r="J68" s="4" t="n">
         <v>100</v>
@@ -7797,7 +7797,7 @@
         <v>5.13</v>
       </c>
       <c r="O68" s="4" t="n">
-        <v>42.87</v>
+        <v>42.88</v>
       </c>
       <c r="P68" s="4" t="n">
         <v>0</v>
@@ -7889,13 +7889,13 @@
         </is>
       </c>
       <c r="M69" s="4" t="n">
-        <v>74.04000000000001</v>
+        <v>74.05</v>
       </c>
       <c r="N69" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O69" s="4" t="n">
-        <v>78.86</v>
+        <v>78.87</v>
       </c>
       <c r="P69" s="4" t="n">
         <v>0</v>
@@ -8079,7 +8079,7 @@
         </is>
       </c>
       <c r="I71" s="4" t="n">
-        <v>21.59</v>
+        <v>21.6</v>
       </c>
       <c r="J71" s="4" t="n">
         <v>99.8</v>
@@ -8099,7 +8099,7 @@
         <v>5.13</v>
       </c>
       <c r="O71" s="4" t="n">
-        <v>21.59</v>
+        <v>21.6</v>
       </c>
       <c r="P71" s="4" t="n">
         <v>0.46</v>
@@ -8191,13 +8191,13 @@
         </is>
       </c>
       <c r="M72" s="4" t="n">
-        <v>40.71</v>
+        <v>40.72</v>
       </c>
       <c r="N72" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>45.96</v>
+        <v>45.97</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
@@ -8330,10 +8330,10 @@
         <v>0</v>
       </c>
       <c r="AB73" s="4" t="n">
-        <v>79.09999999999999</v>
+        <v>79.11</v>
       </c>
       <c r="AC73" s="4" t="n">
-        <v>20.9</v>
+        <v>20.89</v>
       </c>
       <c r="AD73" s="4" t="n">
         <v>0</v>
@@ -8395,7 +8395,7 @@
         </is>
       </c>
       <c r="M74" s="4" t="n">
-        <v>52.92</v>
+        <v>52.93</v>
       </c>
       <c r="N74" s="4" t="n">
         <v>5.13</v>
@@ -8483,7 +8483,7 @@
         </is>
       </c>
       <c r="I75" s="4" t="n">
-        <v>48.97</v>
+        <v>48.98</v>
       </c>
       <c r="J75" s="4" t="n">
         <v>100</v>
@@ -8503,7 +8503,7 @@
         <v>5.13</v>
       </c>
       <c r="O75" s="4" t="n">
-        <v>48.97</v>
+        <v>48.98</v>
       </c>
       <c r="P75" s="4" t="n">
         <v>3.69</v>
@@ -8585,7 +8585,7 @@
         </is>
       </c>
       <c r="I76" s="4" t="n">
-        <v>43.91</v>
+        <v>43.92</v>
       </c>
       <c r="J76" s="4" t="n">
         <v>100</v>
@@ -8605,7 +8605,7 @@
         <v>5.13</v>
       </c>
       <c r="O76" s="4" t="n">
-        <v>43.91</v>
+        <v>43.92</v>
       </c>
       <c r="P76" s="4" t="n">
         <v>2.1</v>
@@ -8701,13 +8701,13 @@
         </is>
       </c>
       <c r="M77" s="4" t="n">
-        <v>38.65</v>
+        <v>38.66</v>
       </c>
       <c r="N77" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O77" s="4" t="n">
-        <v>50.18</v>
+        <v>50.19</v>
       </c>
       <c r="P77" s="4" t="n">
         <v>2.46</v>
@@ -8789,7 +8789,7 @@
         </is>
       </c>
       <c r="I78" s="4" t="n">
-        <v>-28.63</v>
+        <v>-28.62</v>
       </c>
       <c r="J78" s="4" t="n">
         <v>0</v>
@@ -8803,13 +8803,13 @@
         </is>
       </c>
       <c r="M78" s="4" t="n">
-        <v>-30.32</v>
+        <v>-30.31</v>
       </c>
       <c r="N78" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O78" s="4" t="n">
-        <v>-28.63</v>
+        <v>-28.62</v>
       </c>
       <c r="P78" s="4" t="n">
         <v>-2.51</v>
@@ -8905,7 +8905,7 @@
         </is>
       </c>
       <c r="M79" s="4" t="n">
-        <v>11.79</v>
+        <v>11.8</v>
       </c>
       <c r="N79" s="4" t="n">
         <v>5.13</v>
@@ -8993,13 +8993,13 @@
         </is>
       </c>
       <c r="I80" s="4" t="n">
-        <v>5.43</v>
+        <v>5.45</v>
       </c>
       <c r="J80" s="4" t="n">
-        <v>82.3</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -9007,7 +9007,7 @@
         </is>
       </c>
       <c r="M80" s="4" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="N80" s="4" t="n">
         <v>5.13</v>
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="AB80" s="4" t="n">
-        <v>52.71</v>
+        <v>52.72</v>
       </c>
       <c r="AC80" s="4" t="n">
-        <v>47.29</v>
+        <v>47.28</v>
       </c>
       <c r="AD80" s="4" t="n">
         <v>0</v>
@@ -9217,7 +9217,7 @@
         </is>
       </c>
       <c r="M82" s="4" t="n">
-        <v>28.2</v>
+        <v>28.21</v>
       </c>
       <c r="N82" s="4" t="n">
         <v>5.13</v>
@@ -9254,10 +9254,10 @@
         <v>0</v>
       </c>
       <c r="AB82" s="4" t="n">
-        <v>68.31</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="AC82" s="4" t="n">
-        <v>31.69</v>
+        <v>31.68</v>
       </c>
       <c r="AD82" s="4" t="n">
         <v>0</v>
@@ -9356,10 +9356,10 @@
         <v>0</v>
       </c>
       <c r="AB83" s="4" t="n">
-        <v>59.86</v>
+        <v>59.87</v>
       </c>
       <c r="AC83" s="4" t="n">
-        <v>40.14</v>
+        <v>40.13</v>
       </c>
       <c r="AD83" s="4" t="n">
         <v>0</v>
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="I84" s="4" t="n">
-        <v>25.79</v>
+        <v>25.8</v>
       </c>
       <c r="J84" s="4" t="n">
         <v>100</v>
@@ -9423,7 +9423,7 @@
         <v>5.13</v>
       </c>
       <c r="O84" s="4" t="n">
-        <v>25.79</v>
+        <v>25.8</v>
       </c>
       <c r="P84" s="4" t="n">
         <v>0.63</v>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
       <c r="I86" s="4" t="n">
-        <v>39.75</v>
+        <v>39.76</v>
       </c>
       <c r="J86" s="4" t="n">
         <v>100</v>
@@ -9621,13 +9621,13 @@
         </is>
       </c>
       <c r="M86" s="4" t="n">
-        <v>29.79</v>
+        <v>29.8</v>
       </c>
       <c r="N86" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O86" s="4" t="n">
-        <v>39.75</v>
+        <v>39.76</v>
       </c>
       <c r="P86" s="4" t="n">
         <v>2.23</v>
@@ -9723,7 +9723,7 @@
         </is>
       </c>
       <c r="M87" s="4" t="n">
-        <v>41.35</v>
+        <v>41.36</v>
       </c>
       <c r="N87" s="4" t="n">
         <v>5.13</v>
@@ -9811,7 +9811,7 @@
         </is>
       </c>
       <c r="I88" s="4" t="n">
-        <v>51.65</v>
+        <v>51.66</v>
       </c>
       <c r="J88" s="4" t="n">
         <v>100</v>
@@ -9825,13 +9825,13 @@
         </is>
       </c>
       <c r="M88" s="4" t="n">
-        <v>44.8</v>
+        <v>44.81</v>
       </c>
       <c r="N88" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O88" s="4" t="n">
-        <v>51.65</v>
+        <v>51.66</v>
       </c>
       <c r="P88" s="4" t="n">
         <v>1.57</v>
@@ -9964,10 +9964,10 @@
         <v>0</v>
       </c>
       <c r="AB89" s="4" t="n">
-        <v>58.01</v>
+        <v>58.02</v>
       </c>
       <c r="AC89" s="4" t="n">
-        <v>41.99</v>
+        <v>41.98</v>
       </c>
       <c r="AD89" s="4" t="n">
         <v>0</v>
@@ -10029,7 +10029,7 @@
         </is>
       </c>
       <c r="M90" s="4" t="n">
-        <v>29.91</v>
+        <v>29.92</v>
       </c>
       <c r="N90" s="4" t="n">
         <v>5.13</v>
@@ -10066,10 +10066,10 @@
         <v>0</v>
       </c>
       <c r="AB90" s="4" t="n">
-        <v>69.75</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="AC90" s="4" t="n">
-        <v>30.25</v>
+        <v>30.24</v>
       </c>
       <c r="AD90" s="4" t="n">
         <v>0</v>
@@ -10117,7 +10117,7 @@
         </is>
       </c>
       <c r="I91" s="4" t="n">
-        <v>28.34</v>
+        <v>28.35</v>
       </c>
       <c r="J91" s="4" t="n">
         <v>100</v>
@@ -10131,13 +10131,13 @@
         </is>
       </c>
       <c r="M91" s="4" t="n">
-        <v>16.26</v>
+        <v>16.27</v>
       </c>
       <c r="N91" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O91" s="4" t="n">
-        <v>28.34</v>
+        <v>28.35</v>
       </c>
       <c r="P91" s="4" t="n">
         <v>0</v>
@@ -10233,7 +10233,7 @@
         </is>
       </c>
       <c r="M92" s="4" t="n">
-        <v>58.82</v>
+        <v>58.83</v>
       </c>
       <c r="N92" s="4" t="n">
         <v>5.13</v>
@@ -10321,7 +10321,7 @@
         </is>
       </c>
       <c r="I93" s="4" t="n">
-        <v>26.25</v>
+        <v>26.26</v>
       </c>
       <c r="J93" s="4" t="n">
         <v>100</v>
@@ -10341,7 +10341,7 @@
         <v>5.13</v>
       </c>
       <c r="O93" s="4" t="n">
-        <v>26.25</v>
+        <v>26.26</v>
       </c>
       <c r="P93" s="4" t="n">
         <v>2.03</v>
@@ -10423,7 +10423,7 @@
         </is>
       </c>
       <c r="I94" s="4" t="n">
-        <v>51.03</v>
+        <v>51.04</v>
       </c>
       <c r="J94" s="4" t="n">
         <v>100</v>
@@ -10437,13 +10437,13 @@
         </is>
       </c>
       <c r="M94" s="4" t="n">
-        <v>43.41</v>
+        <v>43.42</v>
       </c>
       <c r="N94" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O94" s="4" t="n">
-        <v>51.03</v>
+        <v>51.04</v>
       </c>
       <c r="P94" s="4" t="n">
         <v>2.66</v>
@@ -10545,7 +10545,7 @@
         <v>5.13</v>
       </c>
       <c r="O95" s="4" t="n">
-        <v>76.52</v>
+        <v>76.53</v>
       </c>
       <c r="P95" s="4" t="n">
         <v>0</v>
@@ -10674,10 +10674,10 @@
         <v>0</v>
       </c>
       <c r="AB96" s="4" t="n">
-        <v>62.98</v>
+        <v>62.99</v>
       </c>
       <c r="AC96" s="4" t="n">
-        <v>37.02</v>
+        <v>37.01</v>
       </c>
       <c r="AD96" s="4" t="n">
         <v>0</v>
@@ -10929,7 +10929,7 @@
         </is>
       </c>
       <c r="I99" s="4" t="n">
-        <v>31.1</v>
+        <v>31.11</v>
       </c>
       <c r="J99" s="4" t="n">
         <v>100</v>
@@ -10949,7 +10949,7 @@
         <v>5.13</v>
       </c>
       <c r="O99" s="4" t="n">
-        <v>31.1</v>
+        <v>31.11</v>
       </c>
       <c r="P99" s="4" t="n">
         <v>2.64</v>
@@ -11031,7 +11031,7 @@
         </is>
       </c>
       <c r="I100" s="4" t="n">
-        <v>26.2</v>
+        <v>26.21</v>
       </c>
       <c r="J100" s="4" t="n">
         <v>100</v>
@@ -11051,7 +11051,7 @@
         <v>5.13</v>
       </c>
       <c r="O100" s="4" t="n">
-        <v>26.2</v>
+        <v>26.21</v>
       </c>
       <c r="P100" s="4" t="n">
         <v>1.69</v>
@@ -11235,7 +11235,7 @@
         </is>
       </c>
       <c r="I102" s="4" t="n">
-        <v>58.85</v>
+        <v>58.86</v>
       </c>
       <c r="J102" s="4" t="n">
         <v>100</v>
@@ -11249,13 +11249,13 @@
         </is>
       </c>
       <c r="M102" s="4" t="n">
-        <v>43.5</v>
+        <v>43.51</v>
       </c>
       <c r="N102" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O102" s="4" t="n">
-        <v>58.85</v>
+        <v>58.86</v>
       </c>
       <c r="P102" s="4" t="n">
         <v>1.93</v>
@@ -11337,7 +11337,7 @@
         </is>
       </c>
       <c r="I103" s="4" t="n">
-        <v>20.23</v>
+        <v>20.24</v>
       </c>
       <c r="J103" s="4" t="n">
         <v>99.8</v>
@@ -11357,7 +11357,7 @@
         <v>5.13</v>
       </c>
       <c r="O103" s="4" t="n">
-        <v>20.23</v>
+        <v>20.24</v>
       </c>
       <c r="P103" s="4" t="n">
         <v>1.39</v>
@@ -11439,7 +11439,7 @@
         </is>
       </c>
       <c r="I104" s="4" t="n">
-        <v>39.35</v>
+        <v>39.36</v>
       </c>
       <c r="J104" s="4" t="n">
         <v>100</v>
@@ -11453,13 +11453,13 @@
         </is>
       </c>
       <c r="M104" s="4" t="n">
-        <v>21.96</v>
+        <v>21.97</v>
       </c>
       <c r="N104" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O104" s="4" t="n">
-        <v>39.35</v>
+        <v>39.36</v>
       </c>
       <c r="P104" s="4" t="n">
         <v>1.73</v>
@@ -11561,7 +11561,7 @@
         <v>5.13</v>
       </c>
       <c r="O105" s="4" t="n">
-        <v>22.44</v>
+        <v>22.45</v>
       </c>
       <c r="P105" s="4" t="n">
         <v>1.61</v>
@@ -11639,7 +11639,7 @@
         </is>
       </c>
       <c r="I106" s="4" t="n">
-        <v>11.7</v>
+        <v>11.71</v>
       </c>
       <c r="J106" s="4" t="n">
         <v>98.8</v>
@@ -11653,13 +11653,13 @@
         </is>
       </c>
       <c r="M106" s="4" t="n">
-        <v>5.58</v>
+        <v>5.59</v>
       </c>
       <c r="N106" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O106" s="4" t="n">
-        <v>11.7</v>
+        <v>11.71</v>
       </c>
       <c r="P106" s="4" t="n">
         <v>0.13</v>
@@ -11843,7 +11843,7 @@
         </is>
       </c>
       <c r="I108" s="4" t="n">
-        <v>26.17</v>
+        <v>26.18</v>
       </c>
       <c r="J108" s="4" t="n">
         <v>100</v>
@@ -11857,13 +11857,13 @@
         </is>
       </c>
       <c r="M108" s="4" t="n">
-        <v>20.74</v>
+        <v>20.75</v>
       </c>
       <c r="N108" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O108" s="4" t="n">
-        <v>26.17</v>
+        <v>26.18</v>
       </c>
       <c r="P108" s="4" t="n">
         <v>0</v>
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="I109" s="4" t="n">
-        <v>27.4</v>
+        <v>27.41</v>
       </c>
       <c r="J109" s="4" t="n">
         <v>100</v>
@@ -11959,13 +11959,13 @@
         </is>
       </c>
       <c r="M109" s="4" t="n">
-        <v>21.39</v>
+        <v>21.4</v>
       </c>
       <c r="N109" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O109" s="4" t="n">
-        <v>27.4</v>
+        <v>27.41</v>
       </c>
       <c r="P109" s="4" t="n">
         <v>0</v>
@@ -12047,7 +12047,7 @@
         </is>
       </c>
       <c r="I110" s="4" t="n">
-        <v>39.65</v>
+        <v>39.66</v>
       </c>
       <c r="J110" s="4" t="n">
         <v>100</v>
@@ -12067,7 +12067,7 @@
         <v>5.13</v>
       </c>
       <c r="O110" s="4" t="n">
-        <v>39.65</v>
+        <v>39.66</v>
       </c>
       <c r="P110" s="4" t="n">
         <v>1.58</v>
@@ -12973,7 +12973,7 @@
         </is>
       </c>
       <c r="I119" s="4" t="n">
-        <v>36.68</v>
+        <v>36.69</v>
       </c>
       <c r="J119" s="4" t="n">
         <v>100</v>
@@ -12987,13 +12987,13 @@
         </is>
       </c>
       <c r="M119" s="4" t="n">
-        <v>25.14</v>
+        <v>25.15</v>
       </c>
       <c r="N119" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O119" s="4" t="n">
-        <v>36.68</v>
+        <v>36.69</v>
       </c>
       <c r="P119" s="4" t="n">
         <v>2.93</v>
@@ -13075,7 +13075,7 @@
         </is>
       </c>
       <c r="I120" s="4" t="n">
-        <v>27.15</v>
+        <v>27.16</v>
       </c>
       <c r="J120" s="4" t="n">
         <v>100</v>
@@ -13089,13 +13089,13 @@
         </is>
       </c>
       <c r="M120" s="4" t="n">
-        <v>9.08</v>
+        <v>9.09</v>
       </c>
       <c r="N120" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O120" s="4" t="n">
-        <v>27.15</v>
+        <v>27.16</v>
       </c>
       <c r="P120" s="4" t="n">
         <v>1.43</v>
@@ -13177,7 +13177,7 @@
         </is>
       </c>
       <c r="I121" s="4" t="n">
-        <v>28.19</v>
+        <v>28.2</v>
       </c>
       <c r="J121" s="4" t="n">
         <v>100</v>
@@ -13191,13 +13191,13 @@
         </is>
       </c>
       <c r="M121" s="4" t="n">
-        <v>16.21</v>
+        <v>16.22</v>
       </c>
       <c r="N121" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O121" s="4" t="n">
-        <v>28.19</v>
+        <v>28.2</v>
       </c>
       <c r="P121" s="4" t="n">
         <v>2.19</v>
@@ -13279,7 +13279,7 @@
         </is>
       </c>
       <c r="I122" s="4" t="n">
-        <v>34.69</v>
+        <v>34.7</v>
       </c>
       <c r="J122" s="4" t="n">
         <v>100</v>
@@ -13293,13 +13293,13 @@
         </is>
       </c>
       <c r="M122" s="4" t="n">
-        <v>26.12</v>
+        <v>26.13</v>
       </c>
       <c r="N122" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O122" s="4" t="n">
-        <v>34.69</v>
+        <v>34.7</v>
       </c>
       <c r="P122" s="4" t="n">
         <v>2.06</v>
@@ -13381,7 +13381,7 @@
         </is>
       </c>
       <c r="I123" s="4" t="n">
-        <v>15.11</v>
+        <v>15.12</v>
       </c>
       <c r="J123" s="4" t="n">
         <v>99.3</v>
@@ -13395,13 +13395,13 @@
         </is>
       </c>
       <c r="M123" s="4" t="n">
-        <v>7.37</v>
+        <v>7.38</v>
       </c>
       <c r="N123" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O123" s="4" t="n">
-        <v>15.11</v>
+        <v>15.12</v>
       </c>
       <c r="P123" s="4" t="n">
         <v>1.9</v>
@@ -13432,10 +13432,10 @@
         <v>0</v>
       </c>
       <c r="AB123" s="4" t="n">
-        <v>57.55</v>
+        <v>57.56</v>
       </c>
       <c r="AC123" s="4" t="n">
-        <v>42.45</v>
+        <v>42.44</v>
       </c>
       <c r="AD123" s="4" t="n">
         <v>0</v>
@@ -14193,7 +14193,7 @@
         </is>
       </c>
       <c r="I131" s="4" t="n">
-        <v>-4.28</v>
+        <v>-4.29</v>
       </c>
       <c r="J131" s="4" t="n">
         <v>21.7</v>
@@ -16541,7 +16541,7 @@
         </is>
       </c>
       <c r="I154" s="4" t="n">
-        <v>24.24</v>
+        <v>24.23</v>
       </c>
       <c r="J154" s="4" t="n">
         <v>99.90000000000001</v>
@@ -16561,7 +16561,7 @@
         <v>5.13</v>
       </c>
       <c r="O154" s="4" t="n">
-        <v>24.24</v>
+        <v>24.23</v>
       </c>
       <c r="P154" s="4" t="n">
         <v>1.36</v>
@@ -16643,7 +16643,7 @@
         </is>
       </c>
       <c r="I155" s="4" t="n">
-        <v>-29.17</v>
+        <v>-29.18</v>
       </c>
       <c r="J155" s="4" t="n">
         <v>0</v>
@@ -16663,7 +16663,7 @@
         <v>5.13</v>
       </c>
       <c r="O155" s="4" t="n">
-        <v>-29.17</v>
+        <v>-29.18</v>
       </c>
       <c r="P155" s="4" t="n">
         <v>-1.75</v>
@@ -16847,7 +16847,7 @@
         </is>
       </c>
       <c r="I157" s="4" t="n">
-        <v>83.79000000000001</v>
+        <v>83.78</v>
       </c>
       <c r="J157" s="4" t="n">
         <v>100</v>
@@ -16867,7 +16867,7 @@
         <v>5.13</v>
       </c>
       <c r="O157" s="4" t="n">
-        <v>83.79000000000001</v>
+        <v>83.78</v>
       </c>
       <c r="P157" s="4" t="n">
         <v>0</v>
@@ -16949,7 +16949,7 @@
         </is>
       </c>
       <c r="I158" s="4" t="n">
-        <v>63.09</v>
+        <v>63.08</v>
       </c>
       <c r="J158" s="4" t="n">
         <v>100</v>
@@ -16969,7 +16969,7 @@
         <v>5.13</v>
       </c>
       <c r="O158" s="4" t="n">
-        <v>63.09</v>
+        <v>63.08</v>
       </c>
       <c r="P158" s="4" t="n">
         <v>2.07</v>
@@ -17553,7 +17553,7 @@
         </is>
       </c>
       <c r="I164" s="4" t="n">
-        <v>-11.69</v>
+        <v>-11.7</v>
       </c>
       <c r="J164" s="4" t="n">
         <v>1.2</v>
@@ -17573,7 +17573,7 @@
         <v>5.13</v>
       </c>
       <c r="O164" s="4" t="n">
-        <v>-11.69</v>
+        <v>-11.7</v>
       </c>
       <c r="P164" s="4" t="n">
         <v>-1.96</v>
@@ -17651,7 +17651,7 @@
         </is>
       </c>
       <c r="I165" s="4" t="n">
-        <v>50.88</v>
+        <v>50.87</v>
       </c>
       <c r="J165" s="4" t="n">
         <v>100</v>
@@ -17665,13 +17665,13 @@
         </is>
       </c>
       <c r="M165" s="4" t="n">
-        <v>45.48</v>
+        <v>45.47</v>
       </c>
       <c r="N165" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O165" s="4" t="n">
-        <v>50.88</v>
+        <v>50.87</v>
       </c>
       <c r="P165" s="4" t="n">
         <v>0</v>
@@ -18477,7 +18477,7 @@
         </is>
       </c>
       <c r="I173" s="4" t="n">
-        <v>-27.53</v>
+        <v>-27.84</v>
       </c>
       <c r="J173" s="4" t="n">
         <v>0</v>
@@ -18534,10 +18534,10 @@
         <v>0</v>
       </c>
       <c r="AB173" s="4" t="n">
-        <v>36.23</v>
+        <v>36.08</v>
       </c>
       <c r="AC173" s="4" t="n">
-        <v>63.77</v>
+        <v>63.92</v>
       </c>
       <c r="AD173" s="4" t="n">
         <v>0</v>
@@ -22229,7 +22229,7 @@
         </is>
       </c>
       <c r="I210" s="4" t="n">
-        <v>-7.57</v>
+        <v>-7.6</v>
       </c>
       <c r="J210" s="4" t="n">
         <v>10.7</v>
@@ -22286,10 +22286,10 @@
         <v>0</v>
       </c>
       <c r="AB210" s="4" t="n">
-        <v>46.21</v>
+        <v>46.2</v>
       </c>
       <c r="AC210" s="4" t="n">
-        <v>53.79</v>
+        <v>53.8</v>
       </c>
       <c r="AD210" s="4" t="n">
         <v>0</v>
@@ -22945,7 +22945,7 @@
         </is>
       </c>
       <c r="I217" s="4" t="n">
-        <v>24.01</v>
+        <v>24.03</v>
       </c>
       <c r="J217" s="4" t="n">
         <v>99.90000000000001</v>
@@ -22959,13 +22959,13 @@
         </is>
       </c>
       <c r="M217" s="4" t="n">
-        <v>17.34</v>
+        <v>17.35</v>
       </c>
       <c r="N217" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O217" s="4" t="n">
-        <v>24.01</v>
+        <v>24.03</v>
       </c>
       <c r="P217" s="4" t="n">
         <v>0</v>
@@ -23047,7 +23047,7 @@
         </is>
       </c>
       <c r="I218" s="4" t="n">
-        <v>33.63</v>
+        <v>33.64</v>
       </c>
       <c r="J218" s="4" t="n">
         <v>100</v>
@@ -23061,13 +23061,13 @@
         </is>
       </c>
       <c r="M218" s="4" t="n">
-        <v>27.29</v>
+        <v>27.3</v>
       </c>
       <c r="N218" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O218" s="4" t="n">
-        <v>33.63</v>
+        <v>33.64</v>
       </c>
       <c r="P218" s="4" t="n">
         <v>0</v>
@@ -23149,7 +23149,7 @@
         </is>
       </c>
       <c r="I219" s="4" t="n">
-        <v>32.19</v>
+        <v>32.2</v>
       </c>
       <c r="J219" s="4" t="n">
         <v>100</v>
@@ -23163,13 +23163,13 @@
         </is>
       </c>
       <c r="M219" s="4" t="n">
-        <v>22.79</v>
+        <v>22.8</v>
       </c>
       <c r="N219" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O219" s="4" t="n">
-        <v>32.19</v>
+        <v>32.2</v>
       </c>
       <c r="P219" s="4" t="n">
         <v>2.52</v>
@@ -23200,10 +23200,10 @@
         <v>0</v>
       </c>
       <c r="AB219" s="4" t="n">
-        <v>66.09</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AC219" s="4" t="n">
-        <v>33.91</v>
+        <v>33.9</v>
       </c>
       <c r="AD219" s="4" t="n">
         <v>0</v>
@@ -23251,7 +23251,7 @@
         </is>
       </c>
       <c r="I220" s="4" t="n">
-        <v>29.69</v>
+        <v>29.7</v>
       </c>
       <c r="J220" s="4" t="n">
         <v>100</v>
@@ -23265,13 +23265,13 @@
         </is>
       </c>
       <c r="M220" s="4" t="n">
-        <v>23.61</v>
+        <v>23.62</v>
       </c>
       <c r="N220" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O220" s="4" t="n">
-        <v>29.69</v>
+        <v>29.7</v>
       </c>
       <c r="P220" s="4" t="n">
         <v>0</v>
@@ -23302,10 +23302,10 @@
         <v>0</v>
       </c>
       <c r="AB220" s="4" t="n">
-        <v>64.84</v>
+        <v>64.84999999999999</v>
       </c>
       <c r="AC220" s="4" t="n">
-        <v>35.16</v>
+        <v>35.15</v>
       </c>
       <c r="AD220" s="4" t="n">
         <v>0</v>
@@ -23353,7 +23353,7 @@
         </is>
       </c>
       <c r="I221" s="4" t="n">
-        <v>55.31</v>
+        <v>55.32</v>
       </c>
       <c r="J221" s="4" t="n">
         <v>100</v>
@@ -23367,13 +23367,13 @@
         </is>
       </c>
       <c r="M221" s="4" t="n">
-        <v>48.97</v>
+        <v>48.98</v>
       </c>
       <c r="N221" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O221" s="4" t="n">
-        <v>55.31</v>
+        <v>55.32</v>
       </c>
       <c r="P221" s="4" t="n">
         <v>0</v>
@@ -23404,10 +23404,10 @@
         <v>0</v>
       </c>
       <c r="AB221" s="4" t="n">
-        <v>77.65000000000001</v>
+        <v>77.66</v>
       </c>
       <c r="AC221" s="4" t="n">
-        <v>22.35</v>
+        <v>22.34</v>
       </c>
       <c r="AD221" s="4" t="n">
         <v>0</v>
@@ -23451,7 +23451,7 @@
         </is>
       </c>
       <c r="I222" s="4" t="n">
-        <v>28.45</v>
+        <v>28.46</v>
       </c>
       <c r="J222" s="4" t="n">
         <v>100</v>
@@ -23465,13 +23465,13 @@
         </is>
       </c>
       <c r="M222" s="4" t="n">
-        <v>23.82</v>
+        <v>23.83</v>
       </c>
       <c r="N222" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O222" s="4" t="n">
-        <v>28.45</v>
+        <v>28.46</v>
       </c>
       <c r="P222" s="4" t="n">
         <v>0</v>
@@ -23502,10 +23502,10 @@
         <v>0</v>
       </c>
       <c r="AB222" s="4" t="n">
-        <v>64.22</v>
+        <v>64.23</v>
       </c>
       <c r="AC222" s="4" t="n">
-        <v>35.78</v>
+        <v>35.77</v>
       </c>
       <c r="AD222" s="4" t="n">
         <v>0</v>
@@ -23553,7 +23553,7 @@
         </is>
       </c>
       <c r="I223" s="4" t="n">
-        <v>76.09999999999999</v>
+        <v>76.11</v>
       </c>
       <c r="J223" s="4" t="n">
         <v>100</v>
@@ -23567,13 +23567,13 @@
         </is>
       </c>
       <c r="M223" s="4" t="n">
-        <v>68.98</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="N223" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O223" s="4" t="n">
-        <v>76.09999999999999</v>
+        <v>76.11</v>
       </c>
       <c r="P223" s="4" t="n">
         <v>0</v>
@@ -23604,10 +23604,10 @@
         <v>0</v>
       </c>
       <c r="AB223" s="4" t="n">
-        <v>88.05</v>
+        <v>88.06</v>
       </c>
       <c r="AC223" s="4" t="n">
-        <v>11.95</v>
+        <v>11.94</v>
       </c>
       <c r="AD223" s="4" t="n">
         <v>0</v>
@@ -23655,7 +23655,7 @@
         </is>
       </c>
       <c r="I224" s="4" t="n">
-        <v>45.42</v>
+        <v>45.43</v>
       </c>
       <c r="J224" s="4" t="n">
         <v>100</v>
@@ -23669,13 +23669,13 @@
         </is>
       </c>
       <c r="M224" s="4" t="n">
-        <v>30.38</v>
+        <v>30.4</v>
       </c>
       <c r="N224" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O224" s="4" t="n">
-        <v>45.42</v>
+        <v>45.43</v>
       </c>
       <c r="P224" s="4" t="n">
         <v>0</v>
@@ -23757,7 +23757,7 @@
         </is>
       </c>
       <c r="I225" s="4" t="n">
-        <v>22.43</v>
+        <v>22.45</v>
       </c>
       <c r="J225" s="4" t="n">
         <v>99.90000000000001</v>
@@ -23771,13 +23771,13 @@
         </is>
       </c>
       <c r="M225" s="4" t="n">
-        <v>13.86</v>
+        <v>13.87</v>
       </c>
       <c r="N225" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O225" s="4" t="n">
-        <v>22.43</v>
+        <v>22.45</v>
       </c>
       <c r="P225" s="4" t="n">
         <v>0.51</v>
@@ -24667,7 +24667,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.96</v>
+        <v>30.9</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24681,13 +24681,13 @@
         </is>
       </c>
       <c r="M234" s="4" t="n">
-        <v>22.29</v>
+        <v>22.28</v>
       </c>
       <c r="N234" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O234" s="4" t="n">
-        <v>31.25</v>
+        <v>31.24</v>
       </c>
       <c r="P234" s="4" t="n">
         <v>1</v>
@@ -24765,13 +24765,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-3.44</v>
+        <v>-3.84</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>39.6</v>
+        <v>39.7</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>60.4</v>
+        <v>60.3</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -24779,13 +24779,13 @@
         </is>
       </c>
       <c r="M235" s="4" t="n">
-        <v>-8.85</v>
+        <v>-8.859999999999999</v>
       </c>
       <c r="N235" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O235" s="4" t="n">
-        <v>-5.2</v>
+        <v>-5.21</v>
       </c>
       <c r="P235" s="4" t="n">
         <v>-0.48</v>
@@ -24822,10 +24822,10 @@
         <v>0</v>
       </c>
       <c r="AB235" s="4" t="n">
-        <v>45.47</v>
+        <v>45.46</v>
       </c>
       <c r="AC235" s="4" t="n">
-        <v>49.53</v>
+        <v>49.54</v>
       </c>
       <c r="AD235" s="4" t="n">
         <v>5</v>
@@ -24873,7 +24873,7 @@
         </is>
       </c>
       <c r="I236" s="4" t="n">
-        <v>-12.78</v>
+        <v>-12.77</v>
       </c>
       <c r="J236" s="4" t="n">
         <v>1</v>
@@ -24887,13 +24887,13 @@
         </is>
       </c>
       <c r="M236" s="4" t="n">
-        <v>-17.27</v>
+        <v>-17.26</v>
       </c>
       <c r="N236" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O236" s="4" t="n">
-        <v>-12.78</v>
+        <v>-12.77</v>
       </c>
       <c r="P236" s="4" t="n">
         <v>-0.61</v>
@@ -25199,7 +25199,7 @@
         <v>5.13</v>
       </c>
       <c r="O239" s="4" t="n">
-        <v>-2.07</v>
+        <v>-2.06</v>
       </c>
       <c r="P239" s="4" t="n">
         <v>-0.31</v>
@@ -25301,7 +25301,7 @@
         </is>
       </c>
       <c r="M240" s="4" t="n">
-        <v>-22.64</v>
+        <v>-22.63</v>
       </c>
       <c r="N240" s="4" t="n">
         <v>5.13</v>
@@ -25491,13 +25491,13 @@
         </is>
       </c>
       <c r="I242" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="J242" s="4" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="K242" s="4" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -25511,7 +25511,7 @@
         <v>5.13</v>
       </c>
       <c r="O242" s="4" t="n">
-        <v>3.09</v>
+        <v>3.1</v>
       </c>
       <c r="P242" s="4" t="n">
         <v>-0.62</v>
@@ -25548,10 +25548,10 @@
         <v>0</v>
       </c>
       <c r="AB242" s="4" t="n">
-        <v>50.43</v>
+        <v>50.44</v>
       </c>
       <c r="AC242" s="4" t="n">
-        <v>49.57</v>
+        <v>49.56</v>
       </c>
       <c r="AD242" s="4" t="n">
         <v>0</v>
@@ -25715,7 +25715,7 @@
         </is>
       </c>
       <c r="M244" s="4" t="n">
-        <v>-28.17</v>
+        <v>-28.16</v>
       </c>
       <c r="N244" s="4" t="n">
         <v>5.13</v>
@@ -25799,7 +25799,7 @@
         </is>
       </c>
       <c r="I245" s="4" t="n">
-        <v>2.31</v>
+        <v>2.32</v>
       </c>
       <c r="J245" s="4" t="n">
         <v>70.90000000000001</v>
@@ -25903,7 +25903,7 @@
         </is>
       </c>
       <c r="I246" s="4" t="n">
-        <v>27.77</v>
+        <v>27.78</v>
       </c>
       <c r="J246" s="4" t="n">
         <v>100</v>
@@ -25923,7 +25923,7 @@
         <v>5.13</v>
       </c>
       <c r="O246" s="4" t="n">
-        <v>27.77</v>
+        <v>27.78</v>
       </c>
       <c r="P246" s="4" t="n">
         <v>2.12</v>
@@ -26005,7 +26005,7 @@
         </is>
       </c>
       <c r="I247" s="4" t="n">
-        <v>56.32</v>
+        <v>56.33</v>
       </c>
       <c r="J247" s="4" t="n">
         <v>100</v>
@@ -26019,13 +26019,13 @@
         </is>
       </c>
       <c r="M247" s="4" t="n">
-        <v>46.21</v>
+        <v>46.22</v>
       </c>
       <c r="N247" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O247" s="4" t="n">
-        <v>56.32</v>
+        <v>56.33</v>
       </c>
       <c r="P247" s="4" t="n">
         <v>0</v>
@@ -26209,7 +26209,7 @@
         </is>
       </c>
       <c r="I249" s="4" t="n">
-        <v>-6.12</v>
+        <v>-6.13</v>
       </c>
       <c r="J249" s="4" t="n">
         <v>15.3</v>
@@ -26229,7 +26229,7 @@
         <v>5.13</v>
       </c>
       <c r="O249" s="4" t="n">
-        <v>-6.37</v>
+        <v>-6.38</v>
       </c>
       <c r="P249" s="4" t="n">
         <v>-0.02</v>
@@ -26313,7 +26313,7 @@
         </is>
       </c>
       <c r="I250" s="4" t="n">
-        <v>11.68</v>
+        <v>11.7</v>
       </c>
       <c r="J250" s="4" t="n">
         <v>98.8</v>
@@ -26333,7 +26333,7 @@
         <v>5.13</v>
       </c>
       <c r="O250" s="4" t="n">
-        <v>13.47</v>
+        <v>13.46</v>
       </c>
       <c r="P250" s="4" t="n">
         <v>0.47</v>
@@ -26370,10 +26370,10 @@
         <v>0</v>
       </c>
       <c r="AB250" s="4" t="n">
-        <v>55.84</v>
+        <v>55.85</v>
       </c>
       <c r="AC250" s="4" t="n">
-        <v>44.16</v>
+        <v>44.15</v>
       </c>
       <c r="AD250" s="4" t="n">
         <v>0</v>
@@ -26676,10 +26676,10 @@
         <v>0</v>
       </c>
       <c r="AB253" s="4" t="n">
-        <v>82.90000000000001</v>
+        <v>82.89</v>
       </c>
       <c r="AC253" s="4" t="n">
-        <v>17.1</v>
+        <v>17.11</v>
       </c>
       <c r="AD253" s="4" t="n">
         <v>0</v>
@@ -26727,7 +26727,7 @@
         </is>
       </c>
       <c r="I254" s="4" t="n">
-        <v>-14.68</v>
+        <v>-14.69</v>
       </c>
       <c r="J254" s="4" t="n">
         <v>0.7</v>
@@ -26747,7 +26747,7 @@
         <v>5.13</v>
       </c>
       <c r="O254" s="4" t="n">
-        <v>-14.68</v>
+        <v>-14.69</v>
       </c>
       <c r="P254" s="4" t="n">
         <v>0</v>
@@ -26829,7 +26829,7 @@
         </is>
       </c>
       <c r="I255" s="4" t="n">
-        <v>-31.02</v>
+        <v>-31.03</v>
       </c>
       <c r="J255" s="4" t="n">
         <v>0</v>
@@ -26843,13 +26843,13 @@
         </is>
       </c>
       <c r="M255" s="4" t="n">
-        <v>-33.64</v>
+        <v>-33.65</v>
       </c>
       <c r="N255" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O255" s="4" t="n">
-        <v>-31.02</v>
+        <v>-31.03</v>
       </c>
       <c r="P255" s="4" t="n">
         <v>0</v>
@@ -26931,7 +26931,7 @@
         </is>
       </c>
       <c r="I256" s="4" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="J256" s="4" t="n">
         <v>7.5</v>
@@ -26951,7 +26951,7 @@
         <v>5.13</v>
       </c>
       <c r="O256" s="4" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="P256" s="4" t="n">
         <v>0</v>
@@ -27135,7 +27135,7 @@
         </is>
       </c>
       <c r="I258" s="4" t="n">
-        <v>-10.61</v>
+        <v>-10.63</v>
       </c>
       <c r="J258" s="4" t="n">
         <v>2.7</v>
@@ -27192,10 +27192,10 @@
         <v>0</v>
       </c>
       <c r="AB258" s="4" t="n">
-        <v>44.69</v>
+        <v>44.68</v>
       </c>
       <c r="AC258" s="4" t="n">
-        <v>55.31</v>
+        <v>55.32</v>
       </c>
       <c r="AD258" s="4" t="n">
         <v>0</v>
@@ -28255,13 +28255,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-5.9</v>
+        <v>-5.94</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>16.1</v>
+        <v>15.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>83.90000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28269,13 +28269,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-11.02</v>
+        <v>-11.07</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-7.02</v>
+        <v>-7.06</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28312,10 +28312,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>47.05</v>
+        <v>47.03</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>52.95</v>
+        <v>52.97</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28363,7 +28363,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-32.75</v>
+        <v>-32.8</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28377,13 +28377,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-29.98</v>
+        <v>-30.03</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-32.75</v>
+        <v>-32.8</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28414,10 +28414,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.62</v>
+        <v>33.6</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.38</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -28675,7 +28675,7 @@
         </is>
       </c>
       <c r="I273" s="4" t="n">
-        <v>-8.1</v>
+        <v>-8.109999999999999</v>
       </c>
       <c r="J273" s="4" t="n">
         <v>9.199999999999999</v>
@@ -28689,13 +28689,13 @@
         </is>
       </c>
       <c r="M273" s="4" t="n">
-        <v>-9.91</v>
+        <v>-9.92</v>
       </c>
       <c r="N273" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O273" s="4" t="n">
-        <v>-8.1</v>
+        <v>-8.109999999999999</v>
       </c>
       <c r="P273" s="4" t="n">
         <v>-1.57</v>
@@ -28791,7 +28791,7 @@
         </is>
       </c>
       <c r="M274" s="4" t="n">
-        <v>48.6</v>
+        <v>48.59</v>
       </c>
       <c r="N274" s="4" t="n">
         <v>5.13</v>
@@ -29199,7 +29199,7 @@
         </is>
       </c>
       <c r="M278" s="4" t="n">
-        <v>-16.99</v>
+        <v>-17</v>
       </c>
       <c r="N278" s="4" t="n">
         <v>5.13</v>
@@ -29338,10 +29338,10 @@
         <v>0</v>
       </c>
       <c r="AB279" s="4" t="n">
-        <v>44.18</v>
+        <v>44.17</v>
       </c>
       <c r="AC279" s="4" t="n">
-        <v>55.82</v>
+        <v>55.83</v>
       </c>
       <c r="AD279" s="4" t="n">
         <v>0</v>
@@ -29511,7 +29511,7 @@
         </is>
       </c>
       <c r="M281" s="4" t="n">
-        <v>-7.93</v>
+        <v>-7.94</v>
       </c>
       <c r="N281" s="4" t="n">
         <v>5.13</v>
@@ -29727,7 +29727,7 @@
         <v>5.13</v>
       </c>
       <c r="O283" s="4" t="n">
-        <v>-13.17</v>
+        <v>-13.18</v>
       </c>
       <c r="P283" s="4" t="n">
         <v>-0.19</v>
@@ -29809,7 +29809,7 @@
         </is>
       </c>
       <c r="I284" s="4" t="n">
-        <v>-13.12</v>
+        <v>-13.13</v>
       </c>
       <c r="J284" s="4" t="n">
         <v>0.9</v>
@@ -30019,13 +30019,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.68</v>
+        <v>-9.76</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>95.09999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -30033,13 +30033,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.94</v>
+        <v>-9.029999999999999</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.3</v>
+        <v>-10.39</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30076,10 +30076,10 @@
         <v>0</v>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>45.16</v>
+        <v>45.12</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>54.84</v>
+        <v>54.88</v>
       </c>
       <c r="AD286" s="4" t="n">
         <v>0</v>
@@ -30123,7 +30123,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>12.45</v>
+        <v>12.38</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>98.90000000000001</v>
@@ -30137,13 +30137,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.92</v>
+        <v>8.83</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.12</v>
+        <v>14.03</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30180,10 +30180,10 @@
         <v>0</v>
       </c>
       <c r="AB287" s="4" t="n">
-        <v>56.22</v>
+        <v>56.19</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>43.78</v>
+        <v>43.81</v>
       </c>
       <c r="AD287" s="4" t="n">
         <v>0</v>
@@ -30231,7 +30231,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.85</v>
+        <v>-52.94</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30245,13 +30245,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.89</v>
+        <v>-49.98</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.85</v>
+        <v>-52.94</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30282,10 +30282,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.57</v>
+        <v>23.53</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.43000000000001</v>
+        <v>76.47</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -31157,7 +31157,7 @@
         </is>
       </c>
       <c r="I297" s="4" t="n">
-        <v>4.48</v>
+        <v>4.49</v>
       </c>
       <c r="J297" s="4" t="n">
         <v>79</v>
@@ -31771,7 +31771,7 @@
         </is>
       </c>
       <c r="I303" s="4" t="n">
-        <v>25.8</v>
+        <v>25.81</v>
       </c>
       <c r="J303" s="4" t="n">
         <v>100</v>
@@ -31785,13 +31785,13 @@
         </is>
       </c>
       <c r="M303" s="4" t="n">
-        <v>15.79</v>
+        <v>15.8</v>
       </c>
       <c r="N303" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O303" s="4" t="n">
-        <v>25.8</v>
+        <v>25.81</v>
       </c>
       <c r="P303" s="4" t="n">
         <v>1.68</v>
@@ -31822,10 +31822,10 @@
         <v>0</v>
       </c>
       <c r="AB303" s="4" t="n">
-        <v>62.9</v>
+        <v>62.91</v>
       </c>
       <c r="AC303" s="4" t="n">
-        <v>37.1</v>
+        <v>37.09</v>
       </c>
       <c r="AD303" s="4" t="n">
         <v>0</v>
@@ -31873,7 +31873,7 @@
         </is>
       </c>
       <c r="I304" s="4" t="n">
-        <v>14.2</v>
+        <v>14.22</v>
       </c>
       <c r="J304" s="4" t="n">
         <v>99.2</v>
@@ -31887,13 +31887,13 @@
         </is>
       </c>
       <c r="M304" s="4" t="n">
-        <v>2.94</v>
+        <v>2.95</v>
       </c>
       <c r="N304" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O304" s="4" t="n">
-        <v>16.22</v>
+        <v>16.23</v>
       </c>
       <c r="P304" s="4" t="n">
         <v>0.67</v>
@@ -31930,10 +31930,10 @@
         <v>0</v>
       </c>
       <c r="AB304" s="4" t="n">
-        <v>57.1</v>
+        <v>57.11</v>
       </c>
       <c r="AC304" s="4" t="n">
-        <v>42.9</v>
+        <v>42.89</v>
       </c>
       <c r="AD304" s="4" t="n">
         <v>0</v>
@@ -31981,7 +31981,7 @@
         </is>
       </c>
       <c r="I305" s="4" t="n">
-        <v>22.82</v>
+        <v>22.83</v>
       </c>
       <c r="J305" s="4" t="n">
         <v>99.90000000000001</v>
@@ -31995,13 +31995,13 @@
         </is>
       </c>
       <c r="M305" s="4" t="n">
-        <v>9.550000000000001</v>
+        <v>9.56</v>
       </c>
       <c r="N305" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O305" s="4" t="n">
-        <v>22.82</v>
+        <v>22.83</v>
       </c>
       <c r="P305" s="4" t="n">
         <v>0.73</v>
@@ -32083,7 +32083,7 @@
         </is>
       </c>
       <c r="I306" s="4" t="n">
-        <v>16.18</v>
+        <v>16.19</v>
       </c>
       <c r="J306" s="4" t="n">
         <v>99.5</v>
@@ -32103,7 +32103,7 @@
         <v>5.13</v>
       </c>
       <c r="O306" s="4" t="n">
-        <v>16.18</v>
+        <v>16.19</v>
       </c>
       <c r="P306" s="4" t="n">
         <v>-0.16</v>
@@ -32181,13 +32181,13 @@
         </is>
       </c>
       <c r="I307" s="4" t="n">
-        <v>-3.63</v>
+        <v>-3.72</v>
       </c>
       <c r="J307" s="4" t="n">
-        <v>24.1</v>
+        <v>23.8</v>
       </c>
       <c r="K307" s="4" t="n">
-        <v>75.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -32195,13 +32195,13 @@
         </is>
       </c>
       <c r="M307" s="4" t="n">
-        <v>-12.43</v>
+        <v>-12.42</v>
       </c>
       <c r="N307" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O307" s="4" t="n">
-        <v>-8.630000000000001</v>
+        <v>-8.619999999999999</v>
       </c>
       <c r="P307" s="4" t="n">
         <v>-1.32</v>
@@ -32238,10 +32238,10 @@
         <v>0</v>
       </c>
       <c r="AB307" s="4" t="n">
-        <v>48.18</v>
+        <v>48.14</v>
       </c>
       <c r="AC307" s="4" t="n">
-        <v>51.82</v>
+        <v>51.86</v>
       </c>
       <c r="AD307" s="4" t="n">
         <v>0</v>
@@ -32289,7 +32289,7 @@
         </is>
       </c>
       <c r="I308" s="4" t="n">
-        <v>11.65</v>
+        <v>11.66</v>
       </c>
       <c r="J308" s="4" t="n">
         <v>98.8</v>
@@ -32303,13 +32303,13 @@
         </is>
       </c>
       <c r="M308" s="4" t="n">
-        <v>2.5</v>
+        <v>2.51</v>
       </c>
       <c r="N308" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O308" s="4" t="n">
-        <v>11.65</v>
+        <v>11.66</v>
       </c>
       <c r="P308" s="4" t="n">
         <v>0.06</v>
@@ -32391,7 +32391,7 @@
         </is>
       </c>
       <c r="I309" s="4" t="n">
-        <v>17.44</v>
+        <v>17.45</v>
       </c>
       <c r="J309" s="4" t="n">
         <v>99.59999999999999</v>
@@ -32405,13 +32405,13 @@
         </is>
       </c>
       <c r="M309" s="4" t="n">
-        <v>5.43</v>
+        <v>5.44</v>
       </c>
       <c r="N309" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O309" s="4" t="n">
-        <v>17.44</v>
+        <v>17.45</v>
       </c>
       <c r="P309" s="4" t="n">
         <v>0.97</v>
@@ -34121,13 +34121,13 @@
         </is>
       </c>
       <c r="I326" s="4" t="n">
-        <v>2.3</v>
+        <v>2.32</v>
       </c>
       <c r="J326" s="4" t="n">
-        <v>70.8</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K326" s="4" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -34178,10 +34178,10 @@
         <v>0</v>
       </c>
       <c r="AB326" s="4" t="n">
-        <v>51.15</v>
+        <v>51.16</v>
       </c>
       <c r="AC326" s="4" t="n">
-        <v>48.85</v>
+        <v>48.84</v>
       </c>
       <c r="AD326" s="4" t="n">
         <v>0</v>
@@ -34537,7 +34537,7 @@
         </is>
       </c>
       <c r="I330" s="4" t="n">
-        <v>-12.53</v>
+        <v>-12.57</v>
       </c>
       <c r="J330" s="4" t="n">
         <v>1</v>
@@ -34594,10 +34594,10 @@
         <v>0</v>
       </c>
       <c r="AB330" s="4" t="n">
-        <v>43.73</v>
+        <v>43.72</v>
       </c>
       <c r="AC330" s="4" t="n">
-        <v>56.27</v>
+        <v>56.28</v>
       </c>
       <c r="AD330" s="4" t="n">
         <v>0</v>
@@ -35155,7 +35155,7 @@
         </is>
       </c>
       <c r="I336" s="4" t="n">
-        <v>11.64</v>
+        <v>11.63</v>
       </c>
       <c r="J336" s="4" t="n">
         <v>98.8</v>
@@ -35169,13 +35169,13 @@
         </is>
       </c>
       <c r="M336" s="4" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="N336" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O336" s="4" t="n">
-        <v>11.64</v>
+        <v>11.63</v>
       </c>
       <c r="P336" s="4" t="n">
         <v>0.77</v>
@@ -35308,10 +35308,10 @@
         <v>0</v>
       </c>
       <c r="AB337" s="4" t="n">
-        <v>31.85</v>
+        <v>31.84</v>
       </c>
       <c r="AC337" s="4" t="n">
-        <v>68.15000000000001</v>
+        <v>68.16</v>
       </c>
       <c r="AD337" s="4" t="n">
         <v>0</v>
@@ -35359,7 +35359,7 @@
         </is>
       </c>
       <c r="I338" s="4" t="n">
-        <v>52.59</v>
+        <v>52.58</v>
       </c>
       <c r="J338" s="4" t="n">
         <v>100</v>
@@ -35379,7 +35379,7 @@
         <v>5.13</v>
       </c>
       <c r="O338" s="4" t="n">
-        <v>52.59</v>
+        <v>52.58</v>
       </c>
       <c r="P338" s="4" t="n">
         <v>0</v>
@@ -35461,7 +35461,7 @@
         </is>
       </c>
       <c r="I339" s="4" t="n">
-        <v>-38.7</v>
+        <v>-38.71</v>
       </c>
       <c r="J339" s="4" t="n">
         <v>0</v>
@@ -35481,7 +35481,7 @@
         <v>5.13</v>
       </c>
       <c r="O339" s="4" t="n">
-        <v>-38.7</v>
+        <v>-38.71</v>
       </c>
       <c r="P339" s="4" t="n">
         <v>-3.15</v>
@@ -35577,7 +35577,7 @@
         </is>
       </c>
       <c r="M340" s="4" t="n">
-        <v>-19.28</v>
+        <v>-19.29</v>
       </c>
       <c r="N340" s="4" t="n">
         <v>5.13</v>
@@ -35767,13 +35767,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>-6.61</v>
+        <v>-6.63</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>13.7</v>
+        <v>13.6</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>86.3</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35824,10 +35824,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>46.69</v>
+        <v>46.68</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>53.31</v>
+        <v>53.32</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -35926,10 +35926,10 @@
         <v>0</v>
       </c>
       <c r="AB343" s="4" t="n">
-        <v>45.6</v>
+        <v>45.59</v>
       </c>
       <c r="AC343" s="4" t="n">
-        <v>54.4</v>
+        <v>54.41</v>
       </c>
       <c r="AD343" s="4" t="n">
         <v>0</v>
@@ -35977,7 +35977,7 @@
         </is>
       </c>
       <c r="I344" s="4" t="n">
-        <v>9.18</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J344" s="4" t="n">
         <v>93.8</v>
@@ -35991,7 +35991,7 @@
         </is>
       </c>
       <c r="M344" s="4" t="n">
-        <v>-5.63</v>
+        <v>-5.64</v>
       </c>
       <c r="N344" s="4" t="n">
         <v>5.13</v>
@@ -36034,10 +36034,10 @@
         <v>0</v>
       </c>
       <c r="AB344" s="4" t="n">
-        <v>54.59</v>
+        <v>54.6</v>
       </c>
       <c r="AC344" s="4" t="n">
-        <v>45.41</v>
+        <v>45.4</v>
       </c>
       <c r="AD344" s="4" t="n">
         <v>0</v>
@@ -36085,13 +36085,13 @@
         </is>
       </c>
       <c r="I345" s="4" t="n">
-        <v>-8</v>
+        <v>-8.029999999999999</v>
       </c>
       <c r="J345" s="4" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="K345" s="4" t="n">
-        <v>90.5</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="L345" t="inlineStr">
         <is>
@@ -36142,10 +36142,10 @@
         <v>0</v>
       </c>
       <c r="AB345" s="4" t="n">
-        <v>46</v>
+        <v>45.98</v>
       </c>
       <c r="AC345" s="4" t="n">
-        <v>54</v>
+        <v>54.02</v>
       </c>
       <c r="AD345" s="4" t="n">
         <v>0</v>
@@ -36193,7 +36193,7 @@
         </is>
       </c>
       <c r="I346" s="4" t="n">
-        <v>70.48999999999999</v>
+        <v>70.48</v>
       </c>
       <c r="J346" s="4" t="n">
         <v>100</v>
@@ -36207,13 +36207,13 @@
         </is>
       </c>
       <c r="M346" s="4" t="n">
-        <v>60.42</v>
+        <v>60.41</v>
       </c>
       <c r="N346" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O346" s="4" t="n">
-        <v>70.48999999999999</v>
+        <v>70.48</v>
       </c>
       <c r="P346" s="4" t="n">
         <v>0</v>
@@ -36295,7 +36295,7 @@
         </is>
       </c>
       <c r="I347" s="4" t="n">
-        <v>-25.88</v>
+        <v>-25.89</v>
       </c>
       <c r="J347" s="4" t="n">
         <v>0</v>
@@ -36309,13 +36309,13 @@
         </is>
       </c>
       <c r="M347" s="4" t="n">
-        <v>-26.34</v>
+        <v>-26.35</v>
       </c>
       <c r="N347" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O347" s="4" t="n">
-        <v>-25.88</v>
+        <v>-25.89</v>
       </c>
       <c r="P347" s="4" t="n">
         <v>-1.94</v>
@@ -36411,7 +36411,7 @@
         </is>
       </c>
       <c r="M348" s="4" t="n">
-        <v>7.92</v>
+        <v>7.91</v>
       </c>
       <c r="N348" s="4" t="n">
         <v>5.13</v>
@@ -36513,7 +36513,7 @@
         </is>
       </c>
       <c r="M349" s="4" t="n">
-        <v>-15.7</v>
+        <v>-15.71</v>
       </c>
       <c r="N349" s="4" t="n">
         <v>5.13</v>
@@ -36652,10 +36652,10 @@
         <v>0</v>
       </c>
       <c r="AB350" s="4" t="n">
-        <v>47.08</v>
+        <v>47.07</v>
       </c>
       <c r="AC350" s="4" t="n">
-        <v>52.92</v>
+        <v>52.93</v>
       </c>
       <c r="AD350" s="4" t="n">
         <v>0</v>
@@ -37209,7 +37209,7 @@
         </is>
       </c>
       <c r="I356" s="4" t="n">
-        <v>49.25</v>
+        <v>49.26</v>
       </c>
       <c r="J356" s="4" t="n">
         <v>100</v>
@@ -37223,13 +37223,13 @@
         </is>
       </c>
       <c r="M356" s="4" t="n">
-        <v>38.57</v>
+        <v>38.58</v>
       </c>
       <c r="N356" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O356" s="4" t="n">
-        <v>49.25</v>
+        <v>49.26</v>
       </c>
       <c r="P356" s="4" t="n">
         <v>2.08</v>
@@ -37325,7 +37325,7 @@
         </is>
       </c>
       <c r="M357" s="4" t="n">
-        <v>-28.25</v>
+        <v>-28.24</v>
       </c>
       <c r="N357" s="4" t="n">
         <v>5.13</v>
@@ -37413,7 +37413,7 @@
         </is>
       </c>
       <c r="I358" s="4" t="n">
-        <v>54.96</v>
+        <v>54.97</v>
       </c>
       <c r="J358" s="4" t="n">
         <v>100</v>
@@ -37433,7 +37433,7 @@
         <v>5.13</v>
       </c>
       <c r="O358" s="4" t="n">
-        <v>54.96</v>
+        <v>54.97</v>
       </c>
       <c r="P358" s="4" t="n">
         <v>0</v>
@@ -37515,7 +37515,7 @@
         </is>
       </c>
       <c r="I359" s="4" t="n">
-        <v>16.8</v>
+        <v>16.81</v>
       </c>
       <c r="J359" s="4" t="n">
         <v>99.5</v>
@@ -37529,13 +37529,13 @@
         </is>
       </c>
       <c r="M359" s="4" t="n">
-        <v>11.65</v>
+        <v>11.66</v>
       </c>
       <c r="N359" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O359" s="4" t="n">
-        <v>16.8</v>
+        <v>16.81</v>
       </c>
       <c r="P359" s="4" t="n">
         <v>0.47</v>
@@ -37733,7 +37733,7 @@
         </is>
       </c>
       <c r="M361" s="4" t="n">
-        <v>11.1</v>
+        <v>11.11</v>
       </c>
       <c r="N361" s="4" t="n">
         <v>5.13</v>
@@ -37770,10 +37770,10 @@
         <v>0</v>
       </c>
       <c r="AB361" s="4" t="n">
-        <v>58.89</v>
+        <v>58.9</v>
       </c>
       <c r="AC361" s="4" t="n">
-        <v>41.11</v>
+        <v>41.1</v>
       </c>
       <c r="AD361" s="4" t="n">
         <v>0</v>
@@ -37821,7 +37821,7 @@
         </is>
       </c>
       <c r="I362" s="4" t="n">
-        <v>-2.16</v>
+        <v>-2.15</v>
       </c>
       <c r="J362" s="4" t="n">
         <v>29.8</v>
@@ -38435,7 +38435,7 @@
         </is>
       </c>
       <c r="I368" s="4" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
       <c r="J368" s="4" t="n">
         <v>70.7</v>
@@ -38492,10 +38492,10 @@
         <v>0</v>
       </c>
       <c r="AB368" s="4" t="n">
-        <v>51.13</v>
+        <v>51.14</v>
       </c>
       <c r="AC368" s="4" t="n">
-        <v>48.87</v>
+        <v>48.86</v>
       </c>
       <c r="AD368" s="4" t="n">
         <v>0</v>
@@ -38747,7 +38747,7 @@
         </is>
       </c>
       <c r="I371" s="4" t="n">
-        <v>8.67</v>
+        <v>8.68</v>
       </c>
       <c r="J371" s="4" t="n">
         <v>92.40000000000001</v>
@@ -39569,7 +39569,7 @@
         </is>
       </c>
       <c r="I379" s="4" t="n">
-        <v>40.38</v>
+        <v>40.39</v>
       </c>
       <c r="J379" s="4" t="n">
         <v>100</v>
@@ -39583,13 +39583,13 @@
         </is>
       </c>
       <c r="M379" s="4" t="n">
-        <v>27.1</v>
+        <v>27.11</v>
       </c>
       <c r="N379" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O379" s="4" t="n">
-        <v>40.38</v>
+        <v>40.39</v>
       </c>
       <c r="P379" s="4" t="n">
         <v>0</v>
@@ -39620,10 +39620,10 @@
         <v>0</v>
       </c>
       <c r="AB379" s="4" t="n">
-        <v>70.19</v>
+        <v>70.2</v>
       </c>
       <c r="AC379" s="4" t="n">
-        <v>29.81</v>
+        <v>29.8</v>
       </c>
       <c r="AD379" s="4" t="n">
         <v>0</v>
@@ -39671,7 +39671,7 @@
         </is>
       </c>
       <c r="I380" s="4" t="n">
-        <v>17.09</v>
+        <v>17.1</v>
       </c>
       <c r="J380" s="4" t="n">
         <v>99.59999999999999</v>
@@ -39685,13 +39685,13 @@
         </is>
       </c>
       <c r="M380" s="4" t="n">
-        <v>11.24</v>
+        <v>11.25</v>
       </c>
       <c r="N380" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O380" s="4" t="n">
-        <v>17.09</v>
+        <v>17.1</v>
       </c>
       <c r="P380" s="4" t="n">
         <v>-0.61</v>
@@ -40985,7 +40985,7 @@
         </is>
       </c>
       <c r="I393" s="4" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="J393" s="4" t="n">
         <v>0.8</v>
@@ -41507,7 +41507,7 @@
         </is>
       </c>
       <c r="M398" s="4" t="n">
-        <v>-44.68</v>
+        <v>-44.69</v>
       </c>
       <c r="N398" s="4" t="n">
         <v>5.13</v>
@@ -41693,7 +41693,7 @@
         </is>
       </c>
       <c r="I400" s="4" t="n">
-        <v>-16.08</v>
+        <v>-16.09</v>
       </c>
       <c r="J400" s="4" t="n">
         <v>0.5</v>
@@ -41707,13 +41707,13 @@
         </is>
       </c>
       <c r="M400" s="4" t="n">
-        <v>-19.28</v>
+        <v>-19.29</v>
       </c>
       <c r="N400" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O400" s="4" t="n">
-        <v>-16.08</v>
+        <v>-16.09</v>
       </c>
       <c r="P400" s="4" t="n">
         <v>-0.25</v>
@@ -41897,7 +41897,7 @@
         </is>
       </c>
       <c r="I402" s="4" t="n">
-        <v>-14.04</v>
+        <v>-14.05</v>
       </c>
       <c r="J402" s="4" t="n">
         <v>0.8</v>
@@ -41917,7 +41917,7 @@
         <v>5.13</v>
       </c>
       <c r="O402" s="4" t="n">
-        <v>-14.04</v>
+        <v>-14.05</v>
       </c>
       <c r="P402" s="4" t="n">
         <v>-2.23</v>
@@ -41999,7 +41999,7 @@
         </is>
       </c>
       <c r="I403" s="4" t="n">
-        <v>-19.42</v>
+        <v>-19.43</v>
       </c>
       <c r="J403" s="4" t="n">
         <v>0.3</v>
@@ -42019,7 +42019,7 @@
         <v>5.13</v>
       </c>
       <c r="O403" s="4" t="n">
-        <v>-19.42</v>
+        <v>-19.43</v>
       </c>
       <c r="P403" s="4" t="n">
         <v>-2.94</v>
@@ -42101,7 +42101,7 @@
         </is>
       </c>
       <c r="I404" s="4" t="n">
-        <v>40.34</v>
+        <v>40.33</v>
       </c>
       <c r="J404" s="4" t="n">
         <v>100</v>
@@ -42121,7 +42121,7 @@
         <v>5.13</v>
       </c>
       <c r="O404" s="4" t="n">
-        <v>40.34</v>
+        <v>40.33</v>
       </c>
       <c r="P404" s="4" t="n">
         <v>1.84</v>
@@ -42297,7 +42297,7 @@
         </is>
       </c>
       <c r="I406" s="4" t="n">
-        <v>-7.34</v>
+        <v>-7.35</v>
       </c>
       <c r="J406" s="4" t="n">
         <v>11.4</v>
@@ -42317,7 +42317,7 @@
         <v>5.13</v>
       </c>
       <c r="O406" s="4" t="n">
-        <v>-7.34</v>
+        <v>-7.35</v>
       </c>
       <c r="P406" s="4" t="n">
         <v>-1.92</v>
@@ -42395,7 +42395,7 @@
         </is>
       </c>
       <c r="I407" s="4" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="J407" s="4" t="n">
         <v>0.8</v>
@@ -42409,13 +42409,13 @@
         </is>
       </c>
       <c r="M407" s="4" t="n">
-        <v>-17.41</v>
+        <v>-17.42</v>
       </c>
       <c r="N407" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O407" s="4" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="P407" s="4" t="n">
         <v>-1.52</v>
@@ -42497,7 +42497,7 @@
         </is>
       </c>
       <c r="I408" s="4" t="n">
-        <v>-28.09</v>
+        <v>-28.1</v>
       </c>
       <c r="J408" s="4" t="n">
         <v>0</v>
@@ -42511,13 +42511,13 @@
         </is>
       </c>
       <c r="M408" s="4" t="n">
-        <v>-30.1</v>
+        <v>-30.11</v>
       </c>
       <c r="N408" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O408" s="4" t="n">
-        <v>-28.09</v>
+        <v>-28.1</v>
       </c>
       <c r="P408" s="4" t="n">
         <v>-2.36</v>
@@ -42613,7 +42613,7 @@
         </is>
       </c>
       <c r="M409" s="4" t="n">
-        <v>-19.05</v>
+        <v>-19.06</v>
       </c>
       <c r="N409" s="4" t="n">
         <v>5.13</v>
@@ -42650,10 +42650,10 @@
         <v>0</v>
       </c>
       <c r="AB409" s="4" t="n">
-        <v>40.28</v>
+        <v>40.27</v>
       </c>
       <c r="AC409" s="4" t="n">
-        <v>59.72</v>
+        <v>59.73</v>
       </c>
       <c r="AD409" s="4" t="n">
         <v>0</v>
@@ -42701,7 +42701,7 @@
         </is>
       </c>
       <c r="I410" s="4" t="n">
-        <v>-41.39</v>
+        <v>-41.4</v>
       </c>
       <c r="J410" s="4" t="n">
         <v>0</v>
@@ -42721,7 +42721,7 @@
         <v>5.13</v>
       </c>
       <c r="O410" s="4" t="n">
-        <v>-41.39</v>
+        <v>-41.4</v>
       </c>
       <c r="P410" s="4" t="n">
         <v>-2.49</v>
@@ -42803,7 +42803,7 @@
         </is>
       </c>
       <c r="I411" s="4" t="n">
-        <v>-20.32</v>
+        <v>-20.33</v>
       </c>
       <c r="J411" s="4" t="n">
         <v>0.2</v>
@@ -42823,7 +42823,7 @@
         <v>5.13</v>
       </c>
       <c r="O411" s="4" t="n">
-        <v>-20.32</v>
+        <v>-20.33</v>
       </c>
       <c r="P411" s="4" t="n">
         <v>-1.89</v>
@@ -42905,7 +42905,7 @@
         </is>
       </c>
       <c r="I412" s="4" t="n">
-        <v>-2.56</v>
+        <v>-2.57</v>
       </c>
       <c r="J412" s="4" t="n">
         <v>28.2</v>
@@ -42925,7 +42925,7 @@
         <v>5.13</v>
       </c>
       <c r="O412" s="4" t="n">
-        <v>-2.25</v>
+        <v>-2.26</v>
       </c>
       <c r="P412" s="4" t="n">
         <v>-0.33</v>
@@ -43027,7 +43027,7 @@
         </is>
       </c>
       <c r="M413" s="4" t="n">
-        <v>26.25</v>
+        <v>26.24</v>
       </c>
       <c r="N413" s="4" t="n">
         <v>5.13</v>
@@ -43115,7 +43115,7 @@
         </is>
       </c>
       <c r="I414" s="4" t="n">
-        <v>-15.51</v>
+        <v>-15.52</v>
       </c>
       <c r="J414" s="4" t="n">
         <v>0.6</v>
@@ -43129,13 +43129,13 @@
         </is>
       </c>
       <c r="M414" s="4" t="n">
-        <v>-16.88</v>
+        <v>-16.89</v>
       </c>
       <c r="N414" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O414" s="4" t="n">
-        <v>-15.51</v>
+        <v>-15.52</v>
       </c>
       <c r="P414" s="4" t="n">
         <v>0</v>
@@ -43329,7 +43329,7 @@
         </is>
       </c>
       <c r="M416" s="4" t="n">
-        <v>-47.06</v>
+        <v>-47.07</v>
       </c>
       <c r="N416" s="4" t="n">
         <v>5.13</v>
@@ -43417,7 +43417,7 @@
         </is>
       </c>
       <c r="I417" s="4" t="n">
-        <v>48.56</v>
+        <v>48.55</v>
       </c>
       <c r="J417" s="4" t="n">
         <v>100</v>
@@ -43431,13 +43431,13 @@
         </is>
       </c>
       <c r="M417" s="4" t="n">
-        <v>36.09</v>
+        <v>36.08</v>
       </c>
       <c r="N417" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O417" s="4" t="n">
-        <v>48.56</v>
+        <v>48.55</v>
       </c>
       <c r="P417" s="4" t="n">
         <v>1.31</v>
@@ -43613,7 +43613,7 @@
         </is>
       </c>
       <c r="I419" s="4" t="n">
-        <v>-13.71</v>
+        <v>-13.72</v>
       </c>
       <c r="J419" s="4" t="n">
         <v>0.8</v>
@@ -43633,7 +43633,7 @@
         <v>5.13</v>
       </c>
       <c r="O419" s="4" t="n">
-        <v>-13.71</v>
+        <v>-13.72</v>
       </c>
       <c r="P419" s="4" t="n">
         <v>-0.8100000000000001</v>
@@ -43711,7 +43711,7 @@
         </is>
       </c>
       <c r="I420" s="4" t="n">
-        <v>-3.05</v>
+        <v>-3.06</v>
       </c>
       <c r="J420" s="4" t="n">
         <v>26.3</v>
@@ -43819,7 +43819,7 @@
         </is>
       </c>
       <c r="I421" s="4" t="n">
-        <v>-11.64</v>
+        <v>-11.65</v>
       </c>
       <c r="J421" s="4" t="n">
         <v>1.2</v>
@@ -43833,13 +43833,13 @@
         </is>
       </c>
       <c r="M421" s="4" t="n">
-        <v>-12.3</v>
+        <v>-12.31</v>
       </c>
       <c r="N421" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O421" s="4" t="n">
-        <v>-11.64</v>
+        <v>-11.65</v>
       </c>
       <c r="P421" s="4" t="n">
         <v>0</v>
@@ -43935,7 +43935,7 @@
         </is>
       </c>
       <c r="M422" s="4" t="n">
-        <v>-18.53</v>
+        <v>-18.54</v>
       </c>
       <c r="N422" s="4" t="n">
         <v>5.13</v>
@@ -43972,10 +43972,10 @@
         <v>0</v>
       </c>
       <c r="AB422" s="4" t="n">
-        <v>42.71</v>
+        <v>42.7</v>
       </c>
       <c r="AC422" s="4" t="n">
-        <v>57.29</v>
+        <v>57.3</v>
       </c>
       <c r="AD422" s="4" t="n">
         <v>0</v>
@@ -44023,7 +44023,7 @@
         </is>
       </c>
       <c r="I423" s="4" t="n">
-        <v>-23.32</v>
+        <v>-23.33</v>
       </c>
       <c r="J423" s="4" t="n">
         <v>0.1</v>
@@ -44037,13 +44037,13 @@
         </is>
       </c>
       <c r="M423" s="4" t="n">
-        <v>-19.65</v>
+        <v>-19.66</v>
       </c>
       <c r="N423" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O423" s="4" t="n">
-        <v>-23.32</v>
+        <v>-23.33</v>
       </c>
       <c r="P423" s="4" t="n">
         <v>-3.11</v>
@@ -44125,7 +44125,7 @@
         </is>
       </c>
       <c r="I424" s="4" t="n">
-        <v>-14.59</v>
+        <v>-14.6</v>
       </c>
       <c r="J424" s="4" t="n">
         <v>0.7</v>
@@ -44145,7 +44145,7 @@
         <v>5.13</v>
       </c>
       <c r="O424" s="4" t="n">
-        <v>-14.59</v>
+        <v>-14.6</v>
       </c>
       <c r="P424" s="4" t="n">
         <v>-1.33</v>
@@ -44227,13 +44227,13 @@
         </is>
       </c>
       <c r="I425" s="4" t="n">
-        <v>10.99</v>
+        <v>11.13</v>
       </c>
       <c r="J425" s="4" t="n">
-        <v>98.09999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K425" s="4" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="L425" t="inlineStr">
         <is>
@@ -44284,10 +44284,10 @@
         <v>0</v>
       </c>
       <c r="AB425" s="4" t="n">
-        <v>55.5</v>
+        <v>55.56</v>
       </c>
       <c r="AC425" s="4" t="n">
-        <v>44.5</v>
+        <v>44.44</v>
       </c>
       <c r="AD425" s="4" t="n">
         <v>0</v>
@@ -44335,7 +44335,7 @@
         </is>
       </c>
       <c r="I426" s="4" t="n">
-        <v>53.35</v>
+        <v>53.34</v>
       </c>
       <c r="J426" s="4" t="n">
         <v>100</v>
@@ -44349,13 +44349,13 @@
         </is>
       </c>
       <c r="M426" s="4" t="n">
-        <v>38.61</v>
+        <v>38.6</v>
       </c>
       <c r="N426" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O426" s="4" t="n">
-        <v>53.35</v>
+        <v>53.34</v>
       </c>
       <c r="P426" s="4" t="n">
         <v>0</v>
@@ -44433,7 +44433,7 @@
         </is>
       </c>
       <c r="I427" s="4" t="n">
-        <v>60.97</v>
+        <v>60.96</v>
       </c>
       <c r="J427" s="4" t="n">
         <v>100</v>
@@ -44447,13 +44447,13 @@
         </is>
       </c>
       <c r="M427" s="4" t="n">
-        <v>54.32</v>
+        <v>54.31</v>
       </c>
       <c r="N427" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O427" s="4" t="n">
-        <v>60.97</v>
+        <v>60.96</v>
       </c>
       <c r="P427" s="4" t="n">
         <v>0.21</v>
@@ -44549,13 +44549,13 @@
         </is>
       </c>
       <c r="M428" s="4" t="n">
-        <v>-17.81</v>
+        <v>-17.82</v>
       </c>
       <c r="N428" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O428" s="4" t="n">
-        <v>-18.88</v>
+        <v>-18.89</v>
       </c>
       <c r="P428" s="4" t="n">
         <v>-1.61</v>
@@ -44633,7 +44633,7 @@
         </is>
       </c>
       <c r="I429" s="4" t="n">
-        <v>-9.19</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="J429" s="4" t="n">
         <v>6.2</v>
@@ -44653,7 +44653,7 @@
         <v>5.13</v>
       </c>
       <c r="O429" s="4" t="n">
-        <v>-9.19</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="P429" s="4" t="n">
         <v>-1.93</v>
@@ -44731,7 +44731,7 @@
         </is>
       </c>
       <c r="I430" s="4" t="n">
-        <v>45.44</v>
+        <v>45.43</v>
       </c>
       <c r="J430" s="4" t="n">
         <v>100</v>
@@ -44751,7 +44751,7 @@
         <v>5.13</v>
       </c>
       <c r="O430" s="4" t="n">
-        <v>45.44</v>
+        <v>45.43</v>
       </c>
       <c r="P430" s="4" t="n">
         <v>0</v>
@@ -44833,7 +44833,7 @@
         </is>
       </c>
       <c r="I431" s="4" t="n">
-        <v>7.64</v>
+        <v>7.66</v>
       </c>
       <c r="J431" s="4" t="n">
         <v>89.5</v>
@@ -44853,7 +44853,7 @@
         <v>5.13</v>
       </c>
       <c r="O431" s="4" t="n">
-        <v>10.53</v>
+        <v>10.52</v>
       </c>
       <c r="P431" s="4" t="n">
         <v>0.16</v>
@@ -44890,10 +44890,10 @@
         <v>0</v>
       </c>
       <c r="AB431" s="4" t="n">
-        <v>53.82</v>
+        <v>53.83</v>
       </c>
       <c r="AC431" s="4" t="n">
-        <v>46.18</v>
+        <v>46.17</v>
       </c>
       <c r="AD431" s="4" t="n">
         <v>0</v>
@@ -44940,10 +44940,10 @@
         <v>2.52</v>
       </c>
       <c r="J432" s="4" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="K432" s="4" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="L432" t="inlineStr">
         <is>
@@ -44951,7 +44951,7 @@
         </is>
       </c>
       <c r="M432" s="4" t="n">
-        <v>-4.57</v>
+        <v>-4.58</v>
       </c>
       <c r="N432" s="4" t="n">
         <v>5.13</v>
@@ -45090,10 +45090,10 @@
         <v>0</v>
       </c>
       <c r="AB433" s="4" t="n">
-        <v>41.68</v>
+        <v>41.67</v>
       </c>
       <c r="AC433" s="4" t="n">
-        <v>58.32</v>
+        <v>58.33</v>
       </c>
       <c r="AD433" s="4" t="n">
         <v>0</v>
@@ -45259,7 +45259,7 @@
         <v>5.13</v>
       </c>
       <c r="O435" s="4" t="n">
-        <v>-14.18</v>
+        <v>-14.19</v>
       </c>
       <c r="P435" s="4" t="n">
         <v>-2.01</v>
@@ -45290,10 +45290,10 @@
         <v>0</v>
       </c>
       <c r="AB435" s="4" t="n">
-        <v>41.71</v>
+        <v>41.7</v>
       </c>
       <c r="AC435" s="4" t="n">
-        <v>56.11</v>
+        <v>56.12</v>
       </c>
       <c r="AD435" s="4" t="n">
         <v>2.18</v>
@@ -45853,13 +45853,13 @@
         </is>
       </c>
       <c r="I441" s="4" t="n">
-        <v>1.53</v>
+        <v>1.61</v>
       </c>
       <c r="J441" s="4" t="n">
-        <v>67.8</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K441" s="4" t="n">
-        <v>32.2</v>
+        <v>31.9</v>
       </c>
       <c r="L441" t="inlineStr">
         <is>
@@ -45910,10 +45910,10 @@
         <v>0</v>
       </c>
       <c r="AB441" s="4" t="n">
-        <v>50.77</v>
+        <v>50.8</v>
       </c>
       <c r="AC441" s="4" t="n">
-        <v>49.23</v>
+        <v>49.2</v>
       </c>
       <c r="AD441" s="4" t="n">
         <v>0</v>
@@ -46879,7 +46879,7 @@
         </is>
       </c>
       <c r="I451" s="4" t="n">
-        <v>36.3</v>
+        <v>36.29</v>
       </c>
       <c r="J451" s="4" t="n">
         <v>100</v>
@@ -46893,13 +46893,13 @@
         </is>
       </c>
       <c r="M451" s="4" t="n">
-        <v>20.6</v>
+        <v>20.58</v>
       </c>
       <c r="N451" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O451" s="4" t="n">
-        <v>36.32</v>
+        <v>36.29</v>
       </c>
       <c r="P451" s="4" t="n">
         <v>1.82</v>
@@ -47191,13 +47191,13 @@
         </is>
       </c>
       <c r="I454" s="4" t="n">
-        <v>5.09</v>
+        <v>5.14</v>
       </c>
       <c r="J454" s="4" t="n">
-        <v>81.2</v>
+        <v>81.3</v>
       </c>
       <c r="K454" s="4" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L454" t="inlineStr">
         <is>
@@ -47248,10 +47248,10 @@
         <v>0</v>
       </c>
       <c r="AB454" s="4" t="n">
-        <v>52.54</v>
+        <v>52.57</v>
       </c>
       <c r="AC454" s="4" t="n">
-        <v>47.46</v>
+        <v>47.43</v>
       </c>
       <c r="AD454" s="4" t="n">
         <v>0</v>
@@ -47397,7 +47397,7 @@
         </is>
       </c>
       <c r="I456" s="4" t="n">
-        <v>-22.74</v>
+        <v>-22.8</v>
       </c>
       <c r="J456" s="4" t="n">
         <v>0.1</v>
@@ -47454,10 +47454,10 @@
         <v>0</v>
       </c>
       <c r="AB456" s="4" t="n">
-        <v>38.63</v>
+        <v>38.6</v>
       </c>
       <c r="AC456" s="4" t="n">
-        <v>61.37</v>
+        <v>61.4</v>
       </c>
       <c r="AD456" s="4" t="n">
         <v>0</v>
@@ -48137,7 +48137,7 @@
         </is>
       </c>
       <c r="M463" s="4" t="n">
-        <v>41.85</v>
+        <v>41.86</v>
       </c>
       <c r="N463" s="4" t="n">
         <v>5.13</v>
@@ -48225,13 +48225,13 @@
         </is>
       </c>
       <c r="I464" s="4" t="n">
-        <v>3.69</v>
+        <v>3.71</v>
       </c>
       <c r="J464" s="4" t="n">
-        <v>76.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="K464" s="4" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="L464" t="inlineStr">
         <is>
@@ -48282,10 +48282,10 @@
         <v>0</v>
       </c>
       <c r="AB464" s="4" t="n">
-        <v>51.85</v>
+        <v>51.86</v>
       </c>
       <c r="AC464" s="4" t="n">
-        <v>48.15</v>
+        <v>48.14</v>
       </c>
       <c r="AD464" s="4" t="n">
         <v>0</v>
@@ -48333,7 +48333,7 @@
         </is>
       </c>
       <c r="I465" s="4" t="n">
-        <v>62.34</v>
+        <v>62.35</v>
       </c>
       <c r="J465" s="4" t="n">
         <v>100</v>
@@ -48353,7 +48353,7 @@
         <v>5.13</v>
       </c>
       <c r="O465" s="4" t="n">
-        <v>62.34</v>
+        <v>62.35</v>
       </c>
       <c r="P465" s="4" t="n">
         <v>0</v>
@@ -48449,7 +48449,7 @@
         </is>
       </c>
       <c r="M466" s="4" t="n">
-        <v>-22.2</v>
+        <v>-22.19</v>
       </c>
       <c r="N466" s="4" t="n">
         <v>5.13</v>
@@ -48486,10 +48486,10 @@
         <v>0</v>
       </c>
       <c r="AB466" s="4" t="n">
-        <v>37.59</v>
+        <v>37.6</v>
       </c>
       <c r="AC466" s="4" t="n">
-        <v>62.41</v>
+        <v>62.4</v>
       </c>
       <c r="AD466" s="4" t="n">
         <v>0</v>
@@ -48537,7 +48537,7 @@
         </is>
       </c>
       <c r="I467" s="4" t="n">
-        <v>-18.94</v>
+        <v>-18.93</v>
       </c>
       <c r="J467" s="4" t="n">
         <v>0.3</v>
@@ -48551,13 +48551,13 @@
         </is>
       </c>
       <c r="M467" s="4" t="n">
-        <v>-15.81</v>
+        <v>-15.8</v>
       </c>
       <c r="N467" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O467" s="4" t="n">
-        <v>-18.03</v>
+        <v>-18.02</v>
       </c>
       <c r="P467" s="4" t="n">
         <v>-1.71</v>
@@ -48594,10 +48594,10 @@
         <v>0</v>
       </c>
       <c r="AB467" s="4" t="n">
-        <v>40.53</v>
+        <v>40.54</v>
       </c>
       <c r="AC467" s="4" t="n">
-        <v>59.47</v>
+        <v>59.46</v>
       </c>
       <c r="AD467" s="4" t="n">
         <v>0</v>
@@ -48641,7 +48641,7 @@
         </is>
       </c>
       <c r="I468" s="4" t="n">
-        <v>-18.83</v>
+        <v>-18.82</v>
       </c>
       <c r="J468" s="4" t="n">
         <v>0.3</v>
@@ -48655,13 +48655,13 @@
         </is>
       </c>
       <c r="M468" s="4" t="n">
-        <v>-21.43</v>
+        <v>-21.42</v>
       </c>
       <c r="N468" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O468" s="4" t="n">
-        <v>-18.83</v>
+        <v>-18.82</v>
       </c>
       <c r="P468" s="4" t="n">
         <v>-1.54</v>
@@ -48794,10 +48794,10 @@
         <v>0</v>
       </c>
       <c r="AB469" s="4" t="n">
-        <v>42.77</v>
+        <v>42.78</v>
       </c>
       <c r="AC469" s="4" t="n">
-        <v>57.23</v>
+        <v>57.22</v>
       </c>
       <c r="AD469" s="4" t="n">
         <v>0</v>
@@ -49147,13 +49147,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-1.2</v>
+        <v>-0.91</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>46.8</v>
+        <v>47.3</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>53.2</v>
+        <v>52.7</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49161,13 +49161,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.72</v>
+        <v>-10.54</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.17</v>
+        <v>-1.99</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.37</v>
@@ -49204,10 +49204,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.37</v>
+        <v>45.42</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.63</v>
+        <v>46.58</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -49722,10 +49722,10 @@
         <v>0</v>
       </c>
       <c r="AB478" s="4" t="n">
-        <v>47.2</v>
+        <v>47.21</v>
       </c>
       <c r="AC478" s="4" t="n">
-        <v>52.8</v>
+        <v>52.79</v>
       </c>
       <c r="AD478" s="4" t="n">
         <v>0</v>
@@ -49787,13 +49787,13 @@
         </is>
       </c>
       <c r="M479" s="4" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="N479" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O479" s="4" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="P479" s="4" t="n">
         <v>1.71</v>
@@ -49877,13 +49877,13 @@
         </is>
       </c>
       <c r="I480" s="4" t="n">
-        <v>-1.49</v>
+        <v>-1.5</v>
       </c>
       <c r="J480" s="4" t="n">
-        <v>32.4</v>
+        <v>32.3</v>
       </c>
       <c r="K480" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="L480" t="inlineStr">
         <is>
@@ -49985,7 +49985,7 @@
         </is>
       </c>
       <c r="I481" s="4" t="n">
-        <v>-39.35</v>
+        <v>-39.36</v>
       </c>
       <c r="J481" s="4" t="n">
         <v>0</v>
@@ -50505,7 +50505,7 @@
         </is>
       </c>
       <c r="I486" s="4" t="n">
-        <v>29.78</v>
+        <v>29.81</v>
       </c>
       <c r="J486" s="4" t="n">
         <v>100</v>
@@ -50525,7 +50525,7 @@
         <v>5.13</v>
       </c>
       <c r="O486" s="4" t="n">
-        <v>35.74</v>
+        <v>35.75</v>
       </c>
       <c r="P486" s="4" t="n">
         <v>0.66</v>
@@ -50562,10 +50562,10 @@
         <v>0</v>
       </c>
       <c r="AB486" s="4" t="n">
-        <v>64.89</v>
+        <v>64.91</v>
       </c>
       <c r="AC486" s="4" t="n">
-        <v>35.11</v>
+        <v>35.09</v>
       </c>
       <c r="AD486" s="4" t="n">
         <v>0</v>
@@ -50613,13 +50613,13 @@
         </is>
       </c>
       <c r="I487" s="4" t="n">
-        <v>2.12</v>
+        <v>2.09</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>70.09999999999999</v>
+        <v>70</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>29.9</v>
+        <v>30</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -50627,7 +50627,7 @@
         </is>
       </c>
       <c r="M487" s="4" t="n">
-        <v>8.74</v>
+        <v>8.73</v>
       </c>
       <c r="N487" s="4" t="n">
         <v>5.13</v>
@@ -50670,10 +50670,10 @@
         <v>0</v>
       </c>
       <c r="AB487" s="4" t="n">
-        <v>51.06</v>
+        <v>51.04</v>
       </c>
       <c r="AC487" s="4" t="n">
-        <v>48.94</v>
+        <v>48.96</v>
       </c>
       <c r="AD487" s="4" t="n">
         <v>0</v>
@@ -50717,7 +50717,7 @@
         </is>
       </c>
       <c r="I488" s="4" t="n">
-        <v>5.04</v>
+        <v>5.05</v>
       </c>
       <c r="J488" s="4" t="n">
         <v>81</v>
@@ -50774,10 +50774,10 @@
         <v>0</v>
       </c>
       <c r="AB488" s="4" t="n">
-        <v>52.52</v>
+        <v>52.53</v>
       </c>
       <c r="AC488" s="4" t="n">
-        <v>47.48</v>
+        <v>47.47</v>
       </c>
       <c r="AD488" s="4" t="n">
         <v>0</v>
@@ -50835,7 +50835,7 @@
         </is>
       </c>
       <c r="M489" s="4" t="n">
-        <v>6.87</v>
+        <v>6.86</v>
       </c>
       <c r="N489" s="4" t="n">
         <v>5.13</v>
@@ -51037,7 +51037,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-20.82</v>
+        <v>-21</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>4.9</v>
@@ -51092,16 +51092,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>9.710000000000001</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>32.91</v>
+        <v>32.73</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.72</v>
+        <v>53.74</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51253,13 +51253,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-6.51</v>
+        <v>-6.95</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>30.5</v>
+        <v>29.2</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>69.5</v>
+        <v>70.8</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51308,16 +51308,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>46.74</v>
+        <v>46.52</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>30.5</v>
+        <v>29.2</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>53.26</v>
+        <v>53.48</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>
@@ -51361,7 +51361,7 @@
         </is>
       </c>
       <c r="I494" s="4" t="n">
-        <v>7.1</v>
+        <v>7.11</v>
       </c>
       <c r="J494" s="4" t="n">
         <v>87.8</v>
@@ -51375,7 +51375,7 @@
         </is>
       </c>
       <c r="M494" s="4" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="N494" s="4" t="n">
         <v>5.13</v>
@@ -51571,7 +51571,7 @@
         </is>
       </c>
       <c r="I496" s="4" t="n">
-        <v>18.61</v>
+        <v>18.62</v>
       </c>
       <c r="J496" s="4" t="n">
         <v>99.7</v>
@@ -51585,13 +51585,13 @@
         </is>
       </c>
       <c r="M496" s="4" t="n">
-        <v>7.53</v>
+        <v>7.54</v>
       </c>
       <c r="N496" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O496" s="4" t="n">
-        <v>18.61</v>
+        <v>18.62</v>
       </c>
       <c r="P496" s="4" t="n">
         <v>3.16</v>
@@ -51693,7 +51693,7 @@
         <v>5.13</v>
       </c>
       <c r="O497" s="4" t="n">
-        <v>-1.95</v>
+        <v>-1.96</v>
       </c>
       <c r="P497" s="4" t="n">
         <v>0.6</v>
@@ -51893,7 +51893,7 @@
         </is>
       </c>
       <c r="M499" s="4" t="n">
-        <v>12.55</v>
+        <v>12.56</v>
       </c>
       <c r="N499" s="4" t="n">
         <v>5.13</v>
@@ -51981,7 +51981,7 @@
         </is>
       </c>
       <c r="I500" s="4" t="n">
-        <v>22.77</v>
+        <v>22.82</v>
       </c>
       <c r="J500" s="4" t="n">
         <v>99.90000000000001</v>
@@ -51995,7 +51995,7 @@
         </is>
       </c>
       <c r="M500" s="4" t="n">
-        <v>17.1</v>
+        <v>17.11</v>
       </c>
       <c r="N500" s="4" t="n">
         <v>5.13</v>
@@ -52038,10 +52038,10 @@
         <v>0</v>
       </c>
       <c r="AB500" s="4" t="n">
-        <v>61.39</v>
+        <v>61.41</v>
       </c>
       <c r="AC500" s="4" t="n">
-        <v>38.61</v>
+        <v>38.59</v>
       </c>
       <c r="AD500" s="4" t="n">
         <v>0</v>
@@ -52397,7 +52397,7 @@
         </is>
       </c>
       <c r="I504" s="4" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="J504" s="4" t="n">
         <v>63.2</v>
@@ -52933,7 +52933,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -53627,7 +53627,7 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>121.4</v>
+        <v>121.5</v>
       </c>
       <c r="K14" t="n">
         <v>125</v>
@@ -55089,7 +55089,7 @@
         <v>112</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>72.8</v>
+        <v>72.7</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -55547,13 +55547,13 @@
         <v>42</v>
       </c>
       <c r="L47" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M47" t="n">
         <v>53</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TX-32: correct Dem nominee to Dan Barrios
Alex Cornwallis (C-0925) was carried as the *projected* Dem nominee, but
Dan Barrios won the March 3 primary. Add C-1046 Dan Barrios and repoint
TX-32; dem_status projected -> confirmed. C-0925 is left in place as an
orphan, matching the 19 existing primary-loser rows.

Strength stays 0.0 (same as Cornwallis), so TX-32's forecast is unchanged
at D 18.2% / Likely R -- this is a name/id/status correction only.

Reran 2026-07-28 + 2026-07-29. Movement in the 12 AK/ME/MT/NE RCV and
three-way races is unseeded Monte-Carlo noise from the rerun, not signal.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>49.4</v>
+        <v>50.5</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.2</v>
+        <v>232.1</v>
       </c>
       <c r="C9" t="n">
-        <v>202.8</v>
+        <v>202.9</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>80.90000000000001</v>
+        <v>80.2</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>40.3</v>
+        <v>40.6</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-2.96</v>
+        <v>-3.29</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>39.8</v>
+        <v>40.9</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>60.2</v>
+        <v>59.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4695,13 +4695,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.95</v>
+        <v>-2.98</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>42</v>
+        <v>40.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>58</v>
+        <v>59.9</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4709,13 +4709,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.49</v>
+        <v>-2.54</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.15</v>
+        <v>-1.2</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.1</v>
@@ -4750,16 +4750,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.53</v>
+        <v>48.51</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>42</v>
+        <v>40.1</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.47</v>
+        <v>51.49</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -24673,7 +24673,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>31.04</v>
+        <v>30.56</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24771,13 +24771,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.14</v>
+        <v>-4.31</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>36.4</v>
+        <v>35.3</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>63.6</v>
+        <v>64.7</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28261,7 +28261,7 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.26</v>
+        <v>-6.24</v>
       </c>
       <c r="J269" s="4" t="n">
         <v>14.9</v>
@@ -28275,13 +28275,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-11.51</v>
+        <v>-11.49</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-7.47</v>
+        <v>-7.45</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28318,10 +28318,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.87</v>
+        <v>46.88</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.13</v>
+        <v>53.12</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28369,7 +28369,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.21</v>
+        <v>-33.18</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28383,13 +28383,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-30.48</v>
+        <v>-30.45</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.21</v>
+        <v>-33.18</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28420,10 +28420,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.4</v>
+        <v>33.41</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>66.59</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -30025,13 +30025,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.699999999999999</v>
+        <v>-9.67</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>95.09999999999999</v>
+        <v>95</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -30039,13 +30039,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.970000000000001</v>
+        <v>-8.93</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.29</v>
+        <v>-10.25</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30082,10 +30082,10 @@
         <v>0</v>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>45.15</v>
+        <v>45.17</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>54.85</v>
+        <v>54.83</v>
       </c>
       <c r="AD286" s="4" t="n">
         <v>0</v>
@@ -30129,7 +30129,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>12.46</v>
+        <v>12.49</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>98.90000000000001</v>
@@ -30143,13 +30143,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.890000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.13</v>
+        <v>14.17</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30186,10 +30186,10 @@
         <v>0</v>
       </c>
       <c r="AB287" s="4" t="n">
-        <v>56.23</v>
+        <v>56.25</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>43.77</v>
+        <v>43.75</v>
       </c>
       <c r="AD287" s="4" t="n">
         <v>0</v>
@@ -30237,7 +30237,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.84</v>
+        <v>-52.8</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30251,13 +30251,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.92</v>
+        <v>-49.88</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.84</v>
+        <v>-52.8</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30288,10 +30288,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.58</v>
+        <v>23.6</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.42</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -44624,7 +44624,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Alex Cornwallis</t>
+          <t>Dan Barrios</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
@@ -49153,13 +49153,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.72</v>
+        <v>-0.66</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>47.4</v>
+        <v>47.8</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>52.6</v>
+        <v>52.2</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49167,13 +49167,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.56</v>
+        <v>-10.65</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-1.97</v>
+        <v>-2.06</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.37</v>
@@ -49210,10 +49210,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.42</v>
+        <v>45.39</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.58</v>
+        <v>46.61</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -51043,13 +51043,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-22.79</v>
+        <v>-22.7</v>
       </c>
       <c r="J491" s="4" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>96.40000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51098,16 +51098,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>11.63</v>
+        <v>11.66</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>30.96</v>
+        <v>30.99</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.75</v>
+        <v>53.69</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51259,13 +51259,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-6.69</v>
+        <v>-6.48</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>30.1</v>
+        <v>31.6</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>69.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51314,16 +51314,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>46.65</v>
+        <v>46.76</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>30.1</v>
+        <v>31.6</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>53.35</v>
+        <v>53.24</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
OH-07 de-spoilered strength + LA-06 open (Fields out); rerun 2026-07-29
Max Miller's candidate strength -4.37 -> -0.5. The inherited value credited him
with a personal R+4.4 that was an artifact of 2024's three-way race (Kucinich,
a former Dem congressman, took 12.8% out of the Dem column). Netting the spoiler
out (2/3 D / 1/3 R) puts Miller at par with the district's R+11.1 pres lean;
2022's clean two-way puts him ~1 pt off par. OH-07: -7.6 -> -5.4, Likely R ->
Lean R.

Cleo Fields dropped from LA-06 (announced 2026-07-21 he won't seek reelection
after the post-Callais map redrew the seat R+32; running for state Senate D14).
Dem slot -> placeholder C-1047, incumbent_party cleared (seat_holder stays DEM),
C-0499 incumbent flag 0, LA-06 candidate_meta row removed. LA-06: -20.1 -> -28.1.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="C8" t="n">
-        <v>49.5</v>
+        <v>49.4</v>
       </c>
       <c r="D8" t="n">
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>50.5</v>
+        <v>50.9</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>80.2</v>
+        <v>80.8</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="C10" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="D10" t="n">
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>40.6</v>
+        <v>40.1</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.29</v>
+        <v>-3.35</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>40.9</v>
+        <v>39.9</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>59.1</v>
+        <v>60.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Toss-up</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4695,13 +4695,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.98</v>
+        <v>-3.04</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>40.1</v>
+        <v>40.6</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>59.9</v>
+        <v>59.4</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4709,13 +4709,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.54</v>
+        <v>-2.61</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.2</v>
+        <v>-1.27</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.1</v>
@@ -4750,16 +4750,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.51</v>
+        <v>48.48</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>40.1</v>
+        <v>40.6</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.49</v>
+        <v>51.52</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -22830,7 +22830,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Cleo Fields</t>
+          <t>Democratic candidate (LA-06)</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -22838,24 +22838,20 @@
           <t>Peter Williams</t>
         </is>
       </c>
-      <c r="G216" t="inlineStr">
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>DEM</t>
-        </is>
-      </c>
       <c r="I216" s="4" t="n">
-        <v>-20.11</v>
+        <v>-28.11</v>
       </c>
       <c r="J216" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K216" s="4" t="n">
-        <v>99.8</v>
+        <v>100</v>
       </c>
       <c r="L216" t="inlineStr">
         <is>
@@ -22869,13 +22865,13 @@
         <v>5.17</v>
       </c>
       <c r="O216" s="4" t="n">
-        <v>-20.11</v>
+        <v>-28.11</v>
       </c>
       <c r="P216" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q216" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R216" s="4" t="n">
         <v>-32.4</v>
@@ -22900,10 +22896,10 @@
         <v>0</v>
       </c>
       <c r="AB216" s="4" t="n">
-        <v>39.95</v>
+        <v>35.95</v>
       </c>
       <c r="AC216" s="4" t="n">
-        <v>60.05</v>
+        <v>64.05</v>
       </c>
       <c r="AD216" s="4" t="n">
         <v>0</v>
@@ -24673,7 +24669,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.56</v>
+        <v>30.48</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24771,13 +24767,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.31</v>
+        <v>-4.97</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>35.3</v>
+        <v>34.6</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>64.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28261,13 +28257,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.24</v>
+        <v>-6.29</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>85.09999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28275,13 +28271,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-11.49</v>
+        <v>-11.56</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-7.45</v>
+        <v>-7.52</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28318,10 +28314,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.88</v>
+        <v>46.86</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.12</v>
+        <v>53.14</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28369,7 +28365,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.18</v>
+        <v>-33.25</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28383,13 +28379,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-30.45</v>
+        <v>-30.52</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.18</v>
+        <v>-33.25</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28420,10 +28416,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.41</v>
+        <v>33.37</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.59</v>
+        <v>66.63</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -30025,7 +30021,7 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.67</v>
+        <v>-9.65</v>
       </c>
       <c r="J286" s="4" t="n">
         <v>5</v>
@@ -30035,17 +30031,17 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>Safe R</t>
+          <t>Likely R</t>
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.93</v>
+        <v>-8.91</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.25</v>
+        <v>-10.24</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30129,7 +30125,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>12.49</v>
+        <v>12.51</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>98.90000000000001</v>
@@ -30143,13 +30139,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.93</v>
+        <v>8.94</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.17</v>
+        <v>14.18</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30237,7 +30233,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.8</v>
+        <v>-52.78</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30251,13 +30247,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.88</v>
+        <v>-49.87</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.8</v>
+        <v>-52.78</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30288,10 +30284,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.6</v>
+        <v>23.61</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.40000000000001</v>
+        <v>76.39</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -35773,13 +35769,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>-6.66</v>
+        <v>-4.86</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>13.6</v>
+        <v>19.6</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>86.40000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35793,13 +35789,13 @@
         <v>5.17</v>
       </c>
       <c r="O342" s="4" t="n">
-        <v>-7.82</v>
+        <v>-5.24</v>
       </c>
       <c r="P342" s="4" t="n">
         <v>-0.51</v>
       </c>
       <c r="Q342" s="4" t="n">
-        <v>-4.58</v>
+        <v>-2</v>
       </c>
       <c r="R342" s="4" t="n">
         <v>-11.15</v>
@@ -35830,10 +35826,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>46.67</v>
+        <v>47.57</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>53.33</v>
+        <v>52.43</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -49153,13 +49149,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.66</v>
+        <v>-0.95</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>47.8</v>
+        <v>47.6</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49167,13 +49163,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.65</v>
+        <v>-10.66</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.06</v>
+        <v>-2.07</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.37</v>
@@ -51043,13 +51039,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-22.7</v>
+        <v>-22.98</v>
       </c>
       <c r="J491" s="4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>96.59999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51098,16 +51094,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>11.66</v>
+        <v>11.21</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>30.99</v>
+        <v>31.08</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.69</v>
+        <v>54.06</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51259,13 +51255,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-6.48</v>
+        <v>-6.41</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>31.6</v>
+        <v>30.8</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51314,16 +51310,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>46.76</v>
+        <v>46.79</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>31.6</v>
+        <v>30.8</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>53.24</v>
+        <v>53.21</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>
@@ -52939,7 +52935,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -55550,7 +55546,7 @@
         <v>41</v>
       </c>
       <c r="K47" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L47" t="n">
         <v>27</v>

</xml_diff>

<commit_message>
Forecast 2026-08-07: SD-GOV Rhoden, TN primary nominees
SD-GOV: Doeden led the June 2 primary but cleared no 35% threshold; Rhoden
won the July 28 runoff 70.8-29.2. Rep slot back to the incumbent governor
(C-0134), status confirmed.

TN (Aug 6 primaries), all slots confirmed:
- TN-05 Ogles LOST to Charlie Hatcher 53.2-46.8 -> open seat, Safe R to Likely R
- TN-06 Johnny Garrett (R) / Mike Croley (D) for the open Rose seat
- TN-03 Anna Golladay (D), TN-08 Heidi Kuhn (D)
- TN-GOV Blackburn/Green, TN-SEN Hagerty/Bradshaw and the rest confirmed as projected

Fundraising re-scraped before the run so the changed slots stopped carrying
the old candidates' money (TN-05 rep $613k Ogles -> $719k Hatcher; TN-06 rep
$1.55M Hilleary -> $2.38M Garrett).

Dropped candidate_meta's VA-04 "Robert Murray" row: it matched Robert Murray
Morris, a cavalry officer who died in 1896.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="C8" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="D8" t="n">
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>49</v>
+        <v>50.2</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.7</v>
+        <v>232.3</v>
       </c>
       <c r="C9" t="n">
-        <v>202.3</v>
+        <v>202.7</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>82.59999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>24</v>
       </c>
       <c r="E10" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.4</v>
+        <v>-3.18</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>39.1</v>
+        <v>40.5</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>60.9</v>
+        <v>59.5</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4067,23 +4067,27 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Toby Doeden</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>Larry Rhoden</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>REP</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>REP</t>
         </is>
       </c>
       <c r="I32" s="4" t="n">
-        <v>-25.16</v>
+        <v>-25.8</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -4097,13 +4101,13 @@
         <v>5.27</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-25.16</v>
+        <v>-25.8</v>
       </c>
       <c r="P32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q32" s="4" t="n">
-        <v>0</v>
+        <v>-0.64</v>
       </c>
       <c r="R32" s="4" t="n">
         <v>-29.98</v>
@@ -4128,10 +4132,10 @@
         <v>0</v>
       </c>
       <c r="AB32" s="4" t="n">
-        <v>37.42</v>
+        <v>37.1</v>
       </c>
       <c r="AC32" s="4" t="n">
-        <v>62.58</v>
+        <v>62.9</v>
       </c>
       <c r="AD32" s="4" t="n">
         <v>0</v>
@@ -4701,13 +4705,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.45</v>
+        <v>-2.38</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.6</v>
+        <v>28.9</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4715,13 +4719,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.6</v>
+        <v>-2.51</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.18</v>
+        <v>-1.09</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.13</v>
@@ -4756,16 +4760,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.77</v>
+        <v>48.81</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>28.6</v>
+        <v>28.9</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.23</v>
+        <v>51.19</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -24705,7 +24709,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.55</v>
+        <v>30.6</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24803,13 +24807,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-3.97</v>
+        <v>-3.85</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>37.4</v>
+        <v>37.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>62.6</v>
+        <v>62.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28293,7 +28297,7 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.79</v>
+        <v>-6.77</v>
       </c>
       <c r="J269" s="4" t="n">
         <v>13.2</v>
@@ -28307,13 +28311,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-12.21</v>
+        <v>-12.18</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-8.07</v>
+        <v>-8.029999999999999</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28350,10 +28354,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.6</v>
+        <v>46.62</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.4</v>
+        <v>53.38</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28401,7 +28405,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.8</v>
+        <v>-33.77</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28415,13 +28419,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-31.17</v>
+        <v>-31.14</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.8</v>
+        <v>-33.77</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28452,10 +28456,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.1</v>
+        <v>33.11</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.90000000000001</v>
+        <v>66.89</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -40521,7 +40525,7 @@
         </is>
       </c>
       <c r="I388" s="4" t="n">
-        <v>-23.56</v>
+        <v>-23.71</v>
       </c>
       <c r="J388" s="4" t="n">
         <v>0.1</v>
@@ -40535,13 +40539,13 @@
         </is>
       </c>
       <c r="M388" s="4" t="n">
-        <v>-26.61</v>
+        <v>-26.76</v>
       </c>
       <c r="N388" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O388" s="4" t="n">
-        <v>-23.56</v>
+        <v>-23.71</v>
       </c>
       <c r="P388" s="4" t="n">
         <v>-1.2</v>
@@ -40572,10 +40576,10 @@
         <v>0</v>
       </c>
       <c r="AB388" s="4" t="n">
-        <v>38.22</v>
+        <v>38.15</v>
       </c>
       <c r="AC388" s="4" t="n">
-        <v>61.78</v>
+        <v>61.85</v>
       </c>
       <c r="AD388" s="4" t="n">
         <v>0</v>
@@ -40808,7 +40812,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Joel Hawn</t>
+          <t>Anna Golladay</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
@@ -40827,7 +40831,7 @@
         </is>
       </c>
       <c r="I391" s="4" t="n">
-        <v>-35.61</v>
+        <v>-35.05</v>
       </c>
       <c r="J391" s="4" t="n">
         <v>0</v>
@@ -40847,10 +40851,10 @@
         <v>5.27</v>
       </c>
       <c r="O391" s="4" t="n">
-        <v>-35.61</v>
+        <v>-35.05</v>
       </c>
       <c r="P391" s="4" t="n">
-        <v>-2.9</v>
+        <v>-2.34</v>
       </c>
       <c r="Q391" s="4" t="n">
         <v>-3.43</v>
@@ -40865,7 +40869,7 @@
       </c>
       <c r="V391" s="4" t="n"/>
       <c r="W391" s="5" t="n">
-        <v>140</v>
+        <v>55555</v>
       </c>
       <c r="X391" s="5" t="n">
         <v>2330803</v>
@@ -40878,10 +40882,10 @@
         <v>0</v>
       </c>
       <c r="AB391" s="4" t="n">
-        <v>32.19</v>
+        <v>32.47</v>
       </c>
       <c r="AC391" s="4" t="n">
-        <v>67.81</v>
+        <v>67.53</v>
       </c>
       <c r="AD391" s="4" t="n">
         <v>0</v>
@@ -41017,27 +41021,23 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Andy Ogles</t>
-        </is>
-      </c>
-      <c r="G393" t="inlineStr">
+          <t>Charlie Hatcher</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr">
         <is>
           <t>REP</t>
         </is>
       </c>
-      <c r="H393" t="inlineStr">
-        <is>
-          <t>REP</t>
-        </is>
-      </c>
       <c r="I393" s="4" t="n">
-        <v>-13.76</v>
+        <v>-13.11</v>
       </c>
       <c r="J393" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="K393" s="4" t="n">
-        <v>99.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="L393" t="inlineStr">
         <is>
@@ -41051,34 +41051,28 @@
         <v>5.27</v>
       </c>
       <c r="O393" s="4" t="n">
-        <v>-14.72</v>
+        <v>-13.11</v>
       </c>
       <c r="P393" s="4" t="n">
-        <v>0.87</v>
+        <v>0.96</v>
       </c>
       <c r="Q393" s="4" t="n">
-        <v>-1.53</v>
+        <v>0</v>
       </c>
       <c r="R393" s="4" t="n">
         <v>-23.39</v>
       </c>
-      <c r="S393" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="T393" s="4" t="n">
-        <v>47</v>
-      </c>
+      <c r="S393" s="4" t="n"/>
+      <c r="T393" s="4" t="n"/>
       <c r="U393" t="n">
-        <v>1</v>
-      </c>
-      <c r="V393" s="4" t="n">
-        <v>-9</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V393" s="4" t="n"/>
       <c r="W393" s="5" t="n">
         <v>2599775</v>
       </c>
       <c r="X393" s="5" t="n">
-        <v>613135</v>
+        <v>719503</v>
       </c>
       <c r="Y393" t="inlineStr"/>
       <c r="Z393" s="4" t="n">
@@ -41088,10 +41082,10 @@
         <v>0</v>
       </c>
       <c r="AB393" s="4" t="n">
-        <v>43.12</v>
+        <v>43.45</v>
       </c>
       <c r="AC393" s="4" t="n">
-        <v>56.88</v>
+        <v>56.55</v>
       </c>
       <c r="AD393" s="4" t="n">
         <v>0</v>
@@ -41120,12 +41114,12 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Chaney Mosley</t>
+          <t>Mike Croley</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Van Hilleary</t>
+          <t>Johnny Garrett</t>
         </is>
       </c>
       <c r="G394" t="inlineStr"/>
@@ -41135,7 +41129,7 @@
         </is>
       </c>
       <c r="I394" s="4" t="n">
-        <v>-20.87</v>
+        <v>-21.31</v>
       </c>
       <c r="J394" s="4" t="n">
         <v>0.2</v>
@@ -41155,10 +41149,10 @@
         <v>5.27</v>
       </c>
       <c r="O394" s="4" t="n">
-        <v>-20.87</v>
+        <v>-21.31</v>
       </c>
       <c r="P394" s="4" t="n">
-        <v>-1.63</v>
+        <v>-2.07</v>
       </c>
       <c r="Q394" s="4" t="n">
         <v>0</v>
@@ -41173,10 +41167,10 @@
       </c>
       <c r="V394" s="4" t="n"/>
       <c r="W394" s="5" t="n">
-        <v>86869</v>
+        <v>35380</v>
       </c>
       <c r="X394" s="5" t="n">
-        <v>1552429</v>
+        <v>2380327</v>
       </c>
       <c r="Y394" t="inlineStr"/>
       <c r="Z394" s="4" t="n">
@@ -41186,10 +41180,10 @@
         <v>0</v>
       </c>
       <c r="AB394" s="4" t="n">
-        <v>39.57</v>
+        <v>39.35</v>
       </c>
       <c r="AC394" s="4" t="n">
-        <v>60.43</v>
+        <v>60.65</v>
       </c>
       <c r="AD394" s="4" t="n">
         <v>0</v>
@@ -41320,7 +41314,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>William Wicker</t>
+          <t>Heidi Kuhn</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
@@ -41339,13 +41333,13 @@
         </is>
       </c>
       <c r="I396" s="4" t="n">
-        <v>-18.63</v>
+        <v>-21.06</v>
       </c>
       <c r="J396" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K396" s="4" t="n">
-        <v>99.7</v>
+        <v>99.8</v>
       </c>
       <c r="L396" t="inlineStr">
         <is>
@@ -41359,10 +41353,10 @@
         <v>5.27</v>
       </c>
       <c r="O396" s="4" t="n">
-        <v>-18.63</v>
+        <v>-21.06</v>
       </c>
       <c r="P396" s="4" t="n">
-        <v>0</v>
+        <v>-2.43</v>
       </c>
       <c r="Q396" s="4" t="n">
         <v>-5.48</v>
@@ -41377,7 +41371,7 @@
       </c>
       <c r="V396" s="4" t="n"/>
       <c r="W396" s="5" t="n">
-        <v>0</v>
+        <v>39805</v>
       </c>
       <c r="X396" s="5" t="n">
         <v>2232874</v>
@@ -41390,10 +41384,10 @@
         <v>0</v>
       </c>
       <c r="AB396" s="4" t="n">
-        <v>40.68</v>
+        <v>39.47</v>
       </c>
       <c r="AC396" s="4" t="n">
-        <v>59.32</v>
+        <v>60.53</v>
       </c>
       <c r="AD396" s="4" t="n">
         <v>0</v>
@@ -49193,13 +49187,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.6</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>47.6</v>
+        <v>48.5</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>52.4</v>
+        <v>51.5</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49207,13 +49201,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.67</v>
+        <v>-10.62</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.01</v>
+        <v>-1.95</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.34</v>
@@ -49250,10 +49244,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.4</v>
+        <v>45.42</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.6</v>
+        <v>46.58</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -51089,7 +51083,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-25.58</v>
+        <v>-25.45</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0.1</v>
@@ -51144,16 +51138,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>14.05</v>
+        <v>14.07</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>28.36</v>
+        <v>28.41</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.93</v>
+        <v>53.86</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -52245,7 +52239,7 @@
         </is>
       </c>
       <c r="I502" s="4" t="n">
-        <v>-20.83</v>
+        <v>-20.93</v>
       </c>
       <c r="J502" s="4" t="n">
         <v>0.2</v>
@@ -52259,13 +52253,13 @@
         </is>
       </c>
       <c r="M502" s="4" t="n">
-        <v>-22.2</v>
+        <v>-22.36</v>
       </c>
       <c r="N502" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O502" s="4" t="n">
-        <v>-23.41</v>
+        <v>-23.57</v>
       </c>
       <c r="P502" s="4" t="n">
         <v>-1.06</v>
@@ -52300,7 +52294,7 @@
         </is>
       </c>
       <c r="Z502" s="4" t="n">
-        <v>39.59</v>
+        <v>39.53</v>
       </c>
       <c r="AA502" s="4" t="n">
         <v>0.2</v>
@@ -52309,7 +52303,7 @@
         <v>0</v>
       </c>
       <c r="AC502" s="4" t="n">
-        <v>60.41</v>
+        <v>60.47</v>
       </c>
       <c r="AD502" s="4" t="n">
         <v>0</v>
@@ -57049,7 +57043,7 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K72" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
Add Tavern Research OH-07 poll (Aug 4-5) and rerun 2026-08-10 forecast
Tavern Research toplines (635 LV online, Aug 4-5, MoE +/-4.8) put OH-07 at
Poindexter 54 / Miller 46 on the leaner-pushed named ballot. New pollster:
an explicitly Democratic shop with no public track record, so rated 1.3
with a D house lean.

OH-07 moves R+2.41 -> R+2.3 (Dem win 40.7% -> 41.1%); nowcast has it D+2.0.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>48.4</v>
+        <v>48.7</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>233</v>
+        <v>232.8</v>
       </c>
       <c r="C9" t="n">
-        <v>202</v>
+        <v>202.2</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>81.90000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.84</v>
+        <v>-3.03</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>38.1</v>
+        <v>41.9</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>61.9</v>
+        <v>58.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4705,13 +4705,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.53</v>
+        <v>-2.29</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.3</v>
+        <v>29.3</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.7</v>
+        <v>70.7</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4719,13 +4719,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.8</v>
+        <v>-2.5</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.3</v>
+        <v>-1</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.06</v>
@@ -4760,16 +4760,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.74</v>
+        <v>48.86</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>28.3</v>
+        <v>29.3</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.26</v>
+        <v>51.14</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -21487,7 +21487,7 @@
         </is>
       </c>
       <c r="M202" s="4" t="n">
-        <v>-17.12</v>
+        <v>-17.13</v>
       </c>
       <c r="N202" s="4" t="n">
         <v>5.29</v>
@@ -24715,7 +24715,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.05</v>
+        <v>30.23</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24729,13 +24729,13 @@
         </is>
       </c>
       <c r="M234" s="4" t="n">
-        <v>22.14</v>
+        <v>22.05</v>
       </c>
       <c r="N234" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O234" s="4" t="n">
-        <v>31.26</v>
+        <v>31.17</v>
       </c>
       <c r="P234" s="4" t="n">
         <v>1</v>
@@ -24766,10 +24766,10 @@
         <v>0</v>
       </c>
       <c r="AB234" s="4" t="n">
-        <v>62.35</v>
+        <v>62.3</v>
       </c>
       <c r="AC234" s="4" t="n">
-        <v>32.65</v>
+        <v>32.7</v>
       </c>
       <c r="AD234" s="4" t="n">
         <v>5</v>
@@ -24813,13 +24813,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.22</v>
+        <v>-3.99</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -24827,13 +24827,13 @@
         </is>
       </c>
       <c r="M235" s="4" t="n">
-        <v>-9.01</v>
+        <v>-9.1</v>
       </c>
       <c r="N235" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O235" s="4" t="n">
-        <v>-5.2</v>
+        <v>-5.28</v>
       </c>
       <c r="P235" s="4" t="n">
         <v>-0.48</v>
@@ -24870,10 +24870,10 @@
         <v>0</v>
       </c>
       <c r="AB235" s="4" t="n">
-        <v>45.42</v>
+        <v>45.39</v>
       </c>
       <c r="AC235" s="4" t="n">
-        <v>49.58</v>
+        <v>49.61</v>
       </c>
       <c r="AD235" s="4" t="n">
         <v>5</v>
@@ -28303,13 +28303,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.78</v>
+        <v>-6.87</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>86.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28317,13 +28317,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-12.17</v>
+        <v>-12.29</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-8.01</v>
+        <v>-8.130000000000001</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28360,10 +28360,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.61</v>
+        <v>46.57</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.39</v>
+        <v>53.43</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28411,7 +28411,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.74</v>
+        <v>-33.86</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28425,13 +28425,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-31.13</v>
+        <v>-31.25</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.74</v>
+        <v>-33.86</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28462,10 +28462,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.13</v>
+        <v>33.07</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.87</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -30057,13 +30057,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.140000000000001</v>
+        <v>-9.27</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>93.7</v>
+        <v>94</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -30071,13 +30071,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.34</v>
+        <v>-8.5</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-9.550000000000001</v>
+        <v>-9.710000000000001</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30114,10 +30114,10 @@
         <v>0</v>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>45.43</v>
+        <v>45.36</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>54.57</v>
+        <v>54.64</v>
       </c>
       <c r="AD286" s="4" t="n">
         <v>0</v>
@@ -30161,13 +30161,13 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>13.09</v>
+        <v>12.96</v>
       </c>
       <c r="J287" s="4" t="n">
-        <v>99.09999999999999</v>
+        <v>99</v>
       </c>
       <c r="K287" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -30175,13 +30175,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>9.51</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.87</v>
+        <v>14.72</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30218,10 +30218,10 @@
         <v>0</v>
       </c>
       <c r="AB287" s="4" t="n">
-        <v>56.55</v>
+        <v>56.48</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>43.45</v>
+        <v>43.52</v>
       </c>
       <c r="AD287" s="4" t="n">
         <v>0</v>
@@ -30269,7 +30269,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.09</v>
+        <v>-52.25</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30283,13 +30283,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.3</v>
+        <v>-49.45</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.09</v>
+        <v>-52.25</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30320,10 +30320,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.95</v>
+        <v>23.87</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.05</v>
+        <v>76.13</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -35805,13 +35805,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>1.76</v>
+        <v>2</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>68.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>31.3</v>
+        <v>30.4</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35837,16 +35837,16 @@
         <v>-11.15</v>
       </c>
       <c r="S342" s="4" t="n">
-        <v>44.77</v>
+        <v>48.25</v>
       </c>
       <c r="T342" s="4" t="n">
-        <v>38.42</v>
+        <v>41.28</v>
       </c>
       <c r="U342" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V342" s="4" t="n">
-        <v>7.44</v>
+        <v>6.52</v>
       </c>
       <c r="W342" s="5" t="n">
         <v>603156</v>
@@ -35862,10 +35862,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>50.88</v>
+        <v>51</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>49.12</v>
+        <v>49</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -47443,7 +47443,7 @@
         </is>
       </c>
       <c r="I456" s="4" t="n">
-        <v>-23.33</v>
+        <v>-23.89</v>
       </c>
       <c r="J456" s="4" t="n">
         <v>0.1</v>
@@ -47484,7 +47484,7 @@
         <v>1</v>
       </c>
       <c r="V456" s="4" t="n">
-        <v>-6</v>
+        <v>-9</v>
       </c>
       <c r="W456" s="5" t="n">
         <v>396217</v>
@@ -47500,10 +47500,10 @@
         <v>0</v>
       </c>
       <c r="AB456" s="4" t="n">
-        <v>38.33</v>
+        <v>38.06</v>
       </c>
       <c r="AC456" s="4" t="n">
-        <v>61.67</v>
+        <v>61.94</v>
       </c>
       <c r="AD456" s="4" t="n">
         <v>0</v>
@@ -48583,7 +48583,7 @@
         </is>
       </c>
       <c r="I467" s="4" t="n">
-        <v>-18.64</v>
+        <v>-19.21</v>
       </c>
       <c r="J467" s="4" t="n">
         <v>0.3</v>
@@ -48624,7 +48624,7 @@
         <v>1</v>
       </c>
       <c r="V467" s="4" t="n">
-        <v>-22</v>
+        <v>-25</v>
       </c>
       <c r="W467" s="5" t="n">
         <v>44015</v>
@@ -48640,10 +48640,10 @@
         <v>0</v>
       </c>
       <c r="AB467" s="4" t="n">
-        <v>40.68</v>
+        <v>40.39</v>
       </c>
       <c r="AC467" s="4" t="n">
-        <v>59.32</v>
+        <v>59.61</v>
       </c>
       <c r="AD467" s="4" t="n">
         <v>0</v>
@@ -49193,13 +49193,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-1.41</v>
+        <v>-0.7</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>45.5</v>
+        <v>48.4</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>54.5</v>
+        <v>51.6</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49207,13 +49207,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.78</v>
+        <v>-10.58</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.01</v>
+        <v>-1.8</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.43</v>
@@ -49250,10 +49250,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.4</v>
+        <v>45.45</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.6</v>
+        <v>46.55</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -50247,13 +50247,13 @@
         </is>
       </c>
       <c r="I483" s="4" t="n">
-        <v>-10.33</v>
+        <v>-10.34</v>
       </c>
       <c r="J483" s="4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="K483" s="4" t="n">
-        <v>96.59999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="L483" t="inlineStr">
         <is>
@@ -50279,16 +50279,16 @@
         <v>-16.41</v>
       </c>
       <c r="S483" s="4" t="n">
-        <v>43.26</v>
+        <v>43.1</v>
       </c>
       <c r="T483" s="4" t="n">
-        <v>47.6</v>
+        <v>47.22</v>
       </c>
       <c r="U483" t="n">
         <v>2</v>
       </c>
       <c r="V483" s="4" t="n">
-        <v>-7.09</v>
+        <v>-7.13</v>
       </c>
       <c r="W483" s="5" t="n">
         <v>4169078</v>
@@ -50665,13 +50665,13 @@
         </is>
       </c>
       <c r="I487" s="4" t="n">
-        <v>1.62</v>
+        <v>1.19</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>68.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>31.8</v>
+        <v>33.6</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -50697,7 +50697,7 @@
         <v>7.09</v>
       </c>
       <c r="S487" s="4" t="n">
-        <v>49.75</v>
+        <v>49.19</v>
       </c>
       <c r="T487" s="4" t="n">
         <v>44.91</v>
@@ -50706,7 +50706,7 @@
         <v>6</v>
       </c>
       <c r="V487" s="4" t="n">
-        <v>3.7</v>
+        <v>2.86</v>
       </c>
       <c r="W487" s="5" t="n">
         <v>0</v>
@@ -50722,10 +50722,10 @@
         <v>0</v>
       </c>
       <c r="AB487" s="4" t="n">
-        <v>50.81</v>
+        <v>50.6</v>
       </c>
       <c r="AC487" s="4" t="n">
-        <v>49.19</v>
+        <v>49.4</v>
       </c>
       <c r="AD487" s="4" t="n">
         <v>0</v>
@@ -51089,13 +51089,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-25.42</v>
+        <v>-25.9</v>
       </c>
       <c r="J491" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51121,16 +51121,16 @@
         <v>-20.58</v>
       </c>
       <c r="S491" s="4" t="n">
-        <v>31.11</v>
+        <v>30.8</v>
       </c>
       <c r="T491" s="4" t="n">
-        <v>43.81</v>
+        <v>43.51</v>
       </c>
       <c r="U491" t="n">
         <v>6</v>
       </c>
       <c r="V491" s="4" t="n">
-        <v>-12.97</v>
+        <v>-13.03</v>
       </c>
       <c r="W491" s="5" t="n">
         <v>58829</v>
@@ -51144,16 +51144,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>28.41</v>
+        <v>28.02</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.83</v>
+        <v>53.92</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51305,13 +51305,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-3.66</v>
+        <v>-4.45</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>24</v>
+        <v>21.1</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>76</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51340,13 +51340,13 @@
         <v>47</v>
       </c>
       <c r="T493" s="4" t="n">
-        <v>42.31</v>
+        <v>42.8</v>
       </c>
       <c r="U493" t="n">
         <v>3</v>
       </c>
       <c r="V493" s="4" t="n">
-        <v>4.54</v>
+        <v>1.2</v>
       </c>
       <c r="W493" s="5" t="n">
         <v>0</v>
@@ -51360,16 +51360,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>48.17</v>
+        <v>47.78</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>24</v>
+        <v>21.1</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>51.83</v>
+        <v>52.22</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>
@@ -52991,7 +52991,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -55135,7 +55135,7 @@
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>85</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="K39" t="n">
         <v>84</v>
@@ -55147,7 +55147,7 @@
         <v>112</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>72.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -55599,7 +55599,7 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>40.8</v>
+        <v>40.7</v>
       </c>
       <c r="K47" t="n">
         <v>41</v>
@@ -55611,7 +55611,7 @@
         <v>53</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Drop duplicate Tavern Research OH-07 poll; rerun 2026-08-15
The NYT feed picked up the Tavern Research OH-07 survey with end_date
2026-08-04, while the hand-entered copy in manual_race_polls.csv used
2026-08-05 (the PDF's own field dates are Aug 4-5). The merge dedupes on
race + pollster + end date, so the one-day gap let both survive and the
poll was counted twice.

Removed the manual row, so the feed's version is the only one and a future
scrape_race_polls won't reintroduce it. OH-07 drops from 6 polls to 5:
polling average D+1.18 -> D+0.67, margin R+3.27 -> R+3.49, dem_prob
37.5% -> 36.7%. Other race deltas are chamber-sim Monte Carlo noise.
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>51</v>
       </c>
       <c r="E8" t="n">
-        <v>56.8</v>
+        <v>56.2</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>229</v>
       </c>
       <c r="E9" t="n">
-        <v>81.2</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.5</v>
+        <v>24.4</v>
       </c>
       <c r="C10" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="D10" t="n">
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>40.4</v>
+        <v>39.3</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.1</v>
+        <v>-3.76</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>41</v>
+        <v>38.6</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>59</v>
+        <v>61.4</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Toss-up</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4711,13 +4711,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.18</v>
+        <v>-3.34</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>25.8</v>
+        <v>25.2</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>74.2</v>
+        <v>74.8</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4725,13 +4725,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.43</v>
+        <v>-2.7</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.32</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-0.88</v>
+        <v>-1.14</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.04</v>
@@ -4766,16 +4766,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.41</v>
+        <v>48.33</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>25.8</v>
+        <v>25.2</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.59</v>
+        <v>51.67</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -24717,7 +24717,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.36</v>
+        <v>30.38</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24815,13 +24815,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.36</v>
+        <v>-3.99</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>35.7</v>
+        <v>38.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>64.3</v>
+        <v>61.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28305,13 +28305,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-7.21</v>
+        <v>-7.2</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>88.2</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-12.71</v>
+        <v>-12.7</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.32</v>
@@ -28413,7 +28413,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-34.25</v>
+        <v>-34.24</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28427,13 +28427,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-31.67</v>
+        <v>-31.66</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.32</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-34.25</v>
+        <v>-34.24</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28464,10 +28464,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>32.87</v>
+        <v>32.88</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>67.13</v>
+        <v>67.12</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -35807,13 +35807,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>-0.7</v>
+        <v>-1.17</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>35.5</v>
+        <v>33.6</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>64.5</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35839,16 +35839,16 @@
         <v>-11.15</v>
       </c>
       <c r="S342" s="4" t="n">
-        <v>46.08</v>
+        <v>45.02</v>
       </c>
       <c r="T342" s="4" t="n">
-        <v>42.69</v>
+        <v>42.25</v>
       </c>
       <c r="U342" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V342" s="4" t="n">
-        <v>1.18</v>
+        <v>0.67</v>
       </c>
       <c r="W342" s="5" t="n">
         <v>603156</v>
@@ -35864,10 +35864,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>49.65</v>
+        <v>49.41</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>50.35</v>
+        <v>50.59</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -49195,13 +49195,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.31</v>
+        <v>-0.97</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>49.5</v>
+        <v>47.2</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>50.5</v>
+        <v>52.8</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49209,13 +49209,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.6</v>
+        <v>-10.76</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.32</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-1.82</v>
+        <v>-1.99</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.4</v>
@@ -49252,10 +49252,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.6</v>
+        <v>45.56</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.4</v>
+        <v>46.44</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -51091,7 +51091,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-27.57</v>
+        <v>-27.54</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -51146,13 +51146,13 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>14.27</v>
+        <v>14.24</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>27.25</v>
+        <v>27.28</v>
       </c>
       <c r="AC491" s="4" t="n">
         <v>54.82</v>
@@ -53044,7 +53044,7 @@
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="K3" t="n">
         <v>9</v>

</xml_diff>

<commit_message>
data: refresh 2026-09-04 with late-breaking FL-09 + FL-16 polls
Two SEA Polling internals landed in the NYT house feed after this
morning's scrape. Both are D-sponsored, so the average de-biases them.

FL-09 Soto 41 - Green 41 (de-biased R+3.0): D+0.25 -> R+0.68, Toss-up
FL-16 Kirschner 40 - Gruters 39 (de-biased R+2.0): R+5.13 -> R+4.16, Lean R

House D 237.7 (70.8%) - Senate D 50.4 (49.1%) - Gov D 25.5 (56.2%)

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0166PDfFpVfDzteyax1T6AK3
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>51</v>
       </c>
       <c r="E8" t="n">
-        <v>54.9</v>
+        <v>55.7</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.6</v>
+        <v>232.3</v>
       </c>
       <c r="C9" t="n">
-        <v>202.4</v>
+        <v>202.7</v>
       </c>
       <c r="D9" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>81.3</v>
+        <v>80.7</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>66.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4724,10 +4724,10 @@
         <v>-4.89</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>81.09999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
         <v>44.12</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>3.8</v>
@@ -14433,17 +14433,17 @@
         </is>
       </c>
       <c r="I133" s="4" t="n">
-        <v>0.36</v>
+        <v>-1.47</v>
       </c>
       <c r="J133" s="4" t="n">
-        <v>63.2</v>
+        <v>32.5</v>
       </c>
       <c r="K133" s="4" t="n">
-        <v>36.8</v>
+        <v>67.5</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Lean D</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M133" s="4" t="n">
@@ -14464,12 +14464,18 @@
       <c r="R133" s="4" t="n">
         <v>-17.93</v>
       </c>
-      <c r="S133" s="4" t="n"/>
-      <c r="T133" s="4" t="n"/>
+      <c r="S133" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="T133" s="4" t="n">
+        <v>41</v>
+      </c>
       <c r="U133" t="n">
-        <v>0</v>
-      </c>
-      <c r="V133" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V133" s="4" t="n">
+        <v>-3</v>
+      </c>
       <c r="W133" s="5" t="n">
         <v>2157834</v>
       </c>
@@ -14484,10 +14490,10 @@
         <v>0</v>
       </c>
       <c r="AB133" s="4" t="n">
-        <v>50.18</v>
+        <v>49.26</v>
       </c>
       <c r="AC133" s="4" t="n">
-        <v>49.82</v>
+        <v>50.74</v>
       </c>
       <c r="AD133" s="4" t="n">
         <v>0</v>
@@ -15157,13 +15163,13 @@
         </is>
       </c>
       <c r="I140" s="4" t="n">
-        <v>-5.02</v>
+        <v>-3.4</v>
       </c>
       <c r="J140" s="4" t="n">
-        <v>19.1</v>
+        <v>25</v>
       </c>
       <c r="K140" s="4" t="n">
-        <v>80.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -15188,12 +15194,18 @@
       <c r="R140" s="4" t="n">
         <v>-13.81</v>
       </c>
-      <c r="S140" s="4" t="n"/>
-      <c r="T140" s="4" t="n"/>
+      <c r="S140" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="T140" s="4" t="n">
+        <v>39</v>
+      </c>
       <c r="U140" t="n">
-        <v>0</v>
-      </c>
-      <c r="V140" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V140" s="4" t="n">
+        <v>-2</v>
+      </c>
       <c r="W140" s="5" t="n">
         <v>296507</v>
       </c>
@@ -15208,10 +15220,10 @@
         <v>0</v>
       </c>
       <c r="AB140" s="4" t="n">
-        <v>47.49</v>
+        <v>48.3</v>
       </c>
       <c r="AC140" s="4" t="n">
-        <v>52.51</v>
+        <v>51.7</v>
       </c>
       <c r="AD140" s="4" t="n">
         <v>0</v>
@@ -24842,10 +24854,10 @@
         <v>-4.59</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>20.4</v>
+        <v>20.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>79.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -49272,10 +49284,10 @@
         <v>-0.54</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>36.8</v>
+        <v>36.5</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>63.2</v>
+        <v>63.5</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -50744,10 +50756,10 @@
         <v>1.1</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.5</v>
+        <v>33.9</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -51165,13 +51177,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-27.84</v>
+        <v>-27.91</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51220,16 +51232,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>22.27</v>
+        <v>22.29</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>23.12</v>
+        <v>23.07</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>50.96</v>
+        <v>50.98</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
data: Missouri county/town segments follow the 2022 map
The 2026 Missouri lines revert to the 2022-enacted map. The district
baselines shipped in b61bf19a; this is the geography under them —
county_segments.csv (MO 122 -> 125 segments) and town_segments.csv
(1,414 -> 1,423), re-aggregated from 2020 census blocks against the
reverted CD map, with vote conservation exact for 2016/2020/2024.

Jackson County is back to 87/11/2 across MO-05/04/06 instead of the
mid-decade plan's three-way carve of Kansas City, and Boone splits
MO-03/MO-04 rather than MO-03/MO-05.

Reran run_all for 2026-09-08 so the county, town and CD projections sit
on the new segments; no backdate, so the timeline before today is
untouched. The RCV races (AK, ME, MT-SEN) move by their sim's RNG.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K9Aum4a7MYefpCMveEQ2i1
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50.6</v>
+        <v>50.7</v>
       </c>
       <c r="C8" t="n">
-        <v>49.4</v>
+        <v>49.3</v>
       </c>
       <c r="D8" t="n">
         <v>51</v>
       </c>
       <c r="E8" t="n">
-        <v>54.6</v>
+        <v>55</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>231</v>
       </c>
       <c r="E9" t="n">
-        <v>82.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>67.3</v>
+        <v>67</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4724,10 +4724,10 @@
         <v>-4.75</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>19.2</v>
+        <v>19.5</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>80.8</v>
+        <v>80.5</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
         <v>44.19</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>19.2</v>
+        <v>19.5</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>3.8</v>
@@ -24860,10 +24860,10 @@
         <v>-4.62</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>20.3</v>
+        <v>20.6</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>79.7</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -49290,10 +49290,10 @@
         <v>-0.59</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>37</v>
+        <v>38.1</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>63</v>
+        <v>61.9</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -50762,10 +50762,10 @@
         <v>1.02</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -51238,16 +51238,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>22.58</v>
+        <v>22.65</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>22.94</v>
+        <v>22.9</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>50.82</v>
+        <v>50.78</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Daily forecast update: 2026-09-17 (RCV polls read as first preferences)
Ranked polls now feed the margin from round 1 only, summed into blocs;
later rounds go to rcv_transfers.csv (Fabrizio AK-GOV ratios) and the new
rcv_keep.csv exhaustion level (2022 actuals blended with polls by volume).
AK-GOV D+20 -> D+15.1. Adds Rick Beard (LMN) to NE-GOV third parties.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>51.5</v>
+        <v>51.4</v>
       </c>
       <c r="C8" t="n">
-        <v>48.5</v>
+        <v>48.6</v>
       </c>
       <c r="D8" t="n">
         <v>52</v>
       </c>
       <c r="E8" t="n">
-        <v>65.7</v>
+        <v>63.1</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>236.6</v>
+        <v>235.9</v>
       </c>
       <c r="C9" t="n">
-        <v>198.4</v>
+        <v>199.1</v>
       </c>
       <c r="D9" t="n">
         <v>233</v>
       </c>
       <c r="E9" t="n">
-        <v>85.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.5</v>
+        <v>26.6</v>
       </c>
       <c r="C10" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="D10" t="n">
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>70.09999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -925,13 +925,13 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>24.49</v>
+        <v>16.8</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>99.7</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -957,16 +957,16 @@
         <v>-13.8</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>52.7</v>
+        <v>40.58</v>
       </c>
       <c r="T2" s="4" t="n">
-        <v>40.2</v>
+        <v>41.38</v>
       </c>
       <c r="U2" t="n">
         <v>2</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>13.07</v>
+        <v>-0.23</v>
       </c>
       <c r="W2" s="5" t="n">
         <v>0</v>
@@ -983,10 +983,10 @@
         <v>0</v>
       </c>
       <c r="AC2" s="4" t="n">
-        <v>52.61</v>
+        <v>48.39</v>
       </c>
       <c r="AD2" s="4" t="n">
-        <v>47.39</v>
+        <v>51.61</v>
       </c>
       <c r="AE2" s="4" t="n">
         <v>0</v>
@@ -4945,13 +4945,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.32</v>
+        <v>-4.87</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>24.7</v>
+        <v>18.9</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>75.3</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4959,13 +4959,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-0.42</v>
+        <v>-2.48</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.95</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>1.77</v>
+        <v>-0.28</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.03</v>
@@ -4977,16 +4977,16 @@
         <v>-13.8</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>39.82</v>
+        <v>33.66</v>
       </c>
       <c r="T38" s="4" t="n">
-        <v>52.73</v>
+        <v>47.35</v>
       </c>
       <c r="U38" t="n">
         <v>6</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-13.63</v>
+        <v>-14.42</v>
       </c>
       <c r="W38" s="5" t="n">
         <v>0</v>
@@ -5005,16 +5005,16 @@
         </is>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>44.9</v>
+        <v>44.2</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>24.7</v>
+        <v>18.9</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
       </c>
       <c r="AD38" s="4" t="n">
-        <v>50.1</v>
+        <v>50.8</v>
       </c>
       <c r="AE38" s="4" t="n">
         <v>1.2</v>
@@ -16912,13 +16912,13 @@
         </is>
       </c>
       <c r="I151" s="4" t="n">
-        <v>-4.47</v>
+        <v>-4.43</v>
       </c>
       <c r="J151" s="4" t="n">
-        <v>21</v>
+        <v>21.2</v>
       </c>
       <c r="K151" s="4" t="n">
-        <v>79</v>
+        <v>78.8</v>
       </c>
       <c r="L151" t="inlineStr">
         <is>
@@ -16944,16 +16944,16 @@
         <v>-14.7</v>
       </c>
       <c r="S151" s="4" t="n">
-        <v>44.92</v>
+        <v>45.53</v>
       </c>
       <c r="T151" s="4" t="n">
-        <v>45.04</v>
+        <v>46.16</v>
       </c>
       <c r="U151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V151" s="4" t="n">
-        <v>-3</v>
+        <v>-3.57</v>
       </c>
       <c r="W151" s="5" t="n">
         <v>661173</v>
@@ -16970,10 +16970,10 @@
         <v>0</v>
       </c>
       <c r="AC151" s="4" t="n">
-        <v>47.76</v>
+        <v>47.79</v>
       </c>
       <c r="AD151" s="4" t="n">
-        <v>52.24</v>
+        <v>52.21</v>
       </c>
       <c r="AE151" s="4" t="n">
         <v>0</v>
@@ -25769,10 +25769,10 @@
         <v>-3.94</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>22.8</v>
+        <v>22.6</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>77.2</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -51314,13 +51314,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>2.29</v>
+        <v>0.42</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>72.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>27.7</v>
+        <v>35.1</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -51328,13 +51328,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-8.52</v>
+        <v>-10.62</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.95</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>0.83</v>
+        <v>-1.28</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.34</v>
@@ -51346,16 +51346,16 @@
         <v>-13.8</v>
       </c>
       <c r="S473" s="4" t="n">
-        <v>50.13</v>
+        <v>47.77</v>
       </c>
       <c r="T473" s="4" t="n">
-        <v>47.75</v>
+        <v>47.35</v>
       </c>
       <c r="U473" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V473" s="4" t="n">
-        <v>2.18</v>
+        <v>0.4</v>
       </c>
       <c r="W473" s="5" t="n">
         <v>18545132</v>
@@ -51372,10 +51372,10 @@
         <v>0</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>49.47</v>
+        <v>48.54</v>
       </c>
       <c r="AD473" s="4" t="n">
-        <v>48.03</v>
+        <v>48.96</v>
       </c>
       <c r="AE473" s="4" t="n">
         <v>2.5</v>
@@ -52871,10 +52871,10 @@
         <v>1.76</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>68.5</v>
+        <v>68.8</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>31.5</v>
+        <v>31.2</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53316,7 +53316,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-24.44</v>
+        <v>-24.47</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53376,13 +53376,13 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>25.64</v>
+        <v>25.61</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>20.62</v>
+        <v>20.64</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>50.08</v>
@@ -55339,7 +55339,7 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
       <c r="K2" t="n">
         <v>17</v>
@@ -55351,7 +55351,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -55414,7 +55414,7 @@
         <v>10</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily forecast update: 2026-09-17 (ranked-race sim centred on the count)
Within-bloc noise in the IRV Monte Carlo is now multiplicative, so a 1%
candidate no longer inflates in the draws. AK-SEN R+0.2 now reads D 48.6%
instead of 52%.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>51.4</v>
+        <v>51.3</v>
       </c>
       <c r="C8" t="n">
-        <v>48.6</v>
+        <v>48.7</v>
       </c>
       <c r="D8" t="n">
         <v>52</v>
       </c>
       <c r="E8" t="n">
-        <v>63.1</v>
+        <v>62.2</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,10 +566,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>235.9</v>
+        <v>236.2</v>
       </c>
       <c r="C9" t="n">
-        <v>199.1</v>
+        <v>198.8</v>
       </c>
       <c r="D9" t="n">
         <v>233</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="C10" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="D10" t="n">
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>70.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4948,10 +4948,10 @@
         <v>-4.87</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>18.9</v>
+        <v>19.3</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>81.09999999999999</v>
+        <v>80.7</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>44.2</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>18.9</v>
+        <v>19.3</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25769,10 +25769,10 @@
         <v>-3.94</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>22.6</v>
+        <v>23.2</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>77.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -51317,10 +51317,10 @@
         <v>0.42</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>63.9</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>35.1</v>
+        <v>36.1</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52871,10 +52871,10 @@
         <v>1.76</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>68.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>31.2</v>
+        <v>30.6</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53316,7 +53316,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-24.47</v>
+        <v>-24.44</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53382,10 +53382,10 @@
         <v>0.1</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>20.64</v>
+        <v>20.68</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>50.08</v>
+        <v>50.05</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Re-run 2026-09-21: nowcast on the scaled confidence curve
The late-cycle confidence push is now scaled by how decided a race is, so on
the election-day clock a dead heat reads 50% (IA-SEN 61.9% -> 50.3%) and the
Toss-up rating band collapses to nothing — every nowcast race is rated Lean
or better. The published (November) forecast is unchanged at 43 days out:
the 500 two-way races are bit-identical; the six ranked/three-way races
carry their usual Monte-Carlo jitter (<= 0.5 pt), no rating moved.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>51.9</v>
+        <v>51.6</v>
       </c>
       <c r="C8" t="n">
-        <v>48.1</v>
+        <v>48.4</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>67.5</v>
+        <v>61.1</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>237.9</v>
+        <v>237.8</v>
       </c>
       <c r="C9" t="n">
-        <v>197.1</v>
+        <v>197.2</v>
       </c>
       <c r="D9" t="n">
         <v>235</v>
       </c>
       <c r="E9" t="n">
-        <v>87.5</v>
+        <v>86.8</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>72.40000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -1812,14 +1812,14 @@
         <v>3.42</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>75.09999999999999</v>
+        <v>73.8</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>24.9</v>
+        <v>26.2</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Likely D</t>
+          <t>Lean D</t>
         </is>
       </c>
       <c r="M10" s="4" t="n">
@@ -3380,10 +3380,10 @@
         <v>3.79</v>
       </c>
       <c r="J24" s="4" t="n">
-        <v>76.5</v>
+        <v>76.3</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>23.5</v>
+        <v>23.7</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -3602,10 +3602,10 @@
         <v>-1.77</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>31.3</v>
+        <v>37.5</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>68.7</v>
+        <v>62.5</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -3826,10 +3826,10 @@
         <v>3.33</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>74.7</v>
+        <v>73.2</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>25.3</v>
+        <v>26.8</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -4732,14 +4732,14 @@
         <v>3.47</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>75.3</v>
+        <v>74.2</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>24.7</v>
+        <v>25.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Likely D</t>
+          <t>Lean D</t>
         </is>
       </c>
       <c r="M36" s="4" t="n">
@@ -4948,10 +4948,10 @@
         <v>-4.33</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>21.1</v>
+        <v>20.7</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>78.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>44.47</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>21.1</v>
+        <v>20.7</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -5164,10 +5164,10 @@
         <v>-1.43</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>32.6</v>
+        <v>39.9</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>60.1</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -5899,10 +5899,10 @@
         <v>-3.74</v>
       </c>
       <c r="J47" s="4" t="n">
-        <v>23.7</v>
+        <v>24.1</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>76.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -6335,10 +6335,10 @@
         <v>0.7</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>64.5</v>
+        <v>55</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>35.5</v>
+        <v>45</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -12765,10 +12765,10 @@
         <v>-0.35</v>
       </c>
       <c r="J113" s="4" t="n">
-        <v>36.9</v>
+        <v>47.5</v>
       </c>
       <c r="K113" s="4" t="n">
-        <v>63.1</v>
+        <v>52.5</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -12882,14 +12882,14 @@
         <v>-3.54</v>
       </c>
       <c r="J114" s="4" t="n">
-        <v>24.5</v>
+        <v>25.4</v>
       </c>
       <c r="K114" s="4" t="n">
-        <v>75.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M114" s="4" t="n">
@@ -14723,10 +14723,10 @@
         <v>0.47</v>
       </c>
       <c r="J131" s="4" t="n">
-        <v>63.6</v>
+        <v>53.3</v>
       </c>
       <c r="K131" s="4" t="n">
-        <v>36.4</v>
+        <v>46.7</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -14943,10 +14943,10 @@
         <v>0.36</v>
       </c>
       <c r="J133" s="4" t="n">
-        <v>63.2</v>
+        <v>52.6</v>
       </c>
       <c r="K133" s="4" t="n">
-        <v>36.8</v>
+        <v>47.4</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -15712,10 +15712,10 @@
         <v>-2.59</v>
       </c>
       <c r="J140" s="4" t="n">
-        <v>28.1</v>
+        <v>31.8</v>
       </c>
       <c r="K140" s="4" t="n">
-        <v>71.90000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -16376,10 +16376,10 @@
         <v>1.35</v>
       </c>
       <c r="J146" s="4" t="n">
-        <v>67.09999999999999</v>
+        <v>59.6</v>
       </c>
       <c r="K146" s="4" t="n">
-        <v>32.9</v>
+        <v>40.4</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
@@ -18900,14 +18900,14 @@
         <v>3.5</v>
       </c>
       <c r="J170" s="4" t="n">
-        <v>75.40000000000001</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="K170" s="4" t="n">
-        <v>24.6</v>
+        <v>25.6</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>Likely D</t>
+          <t>Lean D</t>
         </is>
       </c>
       <c r="M170" s="4" t="n">
@@ -25769,10 +25769,10 @@
         <v>-3.71</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>23.7</v>
+        <v>23.2</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>76.3</v>
+        <v>76.8</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -26211,10 +26211,10 @@
         <v>-1.36</v>
       </c>
       <c r="J239" s="4" t="n">
-        <v>32.9</v>
+        <v>40.4</v>
       </c>
       <c r="K239" s="4" t="n">
-        <v>67.09999999999999</v>
+        <v>59.6</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -26550,10 +26550,10 @@
         <v>1.83</v>
       </c>
       <c r="J242" s="4" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="K242" s="4" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -26885,10 +26885,10 @@
         <v>1.98</v>
       </c>
       <c r="J245" s="4" t="n">
-        <v>69.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="K245" s="4" t="n">
-        <v>30.4</v>
+        <v>36</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -29491,10 +29491,10 @@
         <v>-3.15</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>-2.26</v>
       </c>
       <c r="J281" s="4" t="n">
-        <v>29.3</v>
+        <v>34.1</v>
       </c>
       <c r="K281" s="4" t="n">
-        <v>70.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="L281" t="inlineStr">
         <is>
@@ -33683,10 +33683,10 @@
         <v>-1.57</v>
       </c>
       <c r="J307" s="4" t="n">
-        <v>32</v>
+        <v>38.9</v>
       </c>
       <c r="K307" s="4" t="n">
-        <v>68</v>
+        <v>61.1</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -34022,10 +34022,10 @@
         <v>-3.1</v>
       </c>
       <c r="J310" s="4" t="n">
-        <v>26.1</v>
+        <v>28.3</v>
       </c>
       <c r="K310" s="4" t="n">
-        <v>73.90000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -35698,10 +35698,10 @@
         <v>3.8</v>
       </c>
       <c r="J326" s="4" t="n">
-        <v>76.5</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K326" s="4" t="n">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -37390,10 +37390,10 @@
         <v>1.01</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>65.7</v>
+        <v>57.2</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>34.3</v>
+        <v>42.8</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -38248,10 +38248,10 @@
         <v>-3.07</v>
       </c>
       <c r="J350" s="4" t="n">
-        <v>26.2</v>
+        <v>28.5</v>
       </c>
       <c r="K350" s="4" t="n">
-        <v>73.8</v>
+        <v>71.5</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -39534,10 +39534,10 @@
         <v>-2.13</v>
       </c>
       <c r="J362" s="4" t="n">
-        <v>29.9</v>
+        <v>35</v>
       </c>
       <c r="K362" s="4" t="n">
-        <v>70.09999999999999</v>
+        <v>65</v>
       </c>
       <c r="L362" t="inlineStr">
         <is>
@@ -40271,10 +40271,10 @@
         <v>1.59</v>
       </c>
       <c r="J369" s="4" t="n">
-        <v>68</v>
+        <v>61.2</v>
       </c>
       <c r="K369" s="4" t="n">
-        <v>32</v>
+        <v>38.8</v>
       </c>
       <c r="L369" t="inlineStr">
         <is>
@@ -41523,10 +41523,10 @@
         <v>-2.59</v>
       </c>
       <c r="J381" s="4" t="n">
-        <v>28.1</v>
+        <v>31.8</v>
       </c>
       <c r="K381" s="4" t="n">
-        <v>71.90000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="L381" t="inlineStr">
         <is>
@@ -44816,10 +44816,10 @@
         <v>1.7</v>
       </c>
       <c r="J412" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>62</v>
       </c>
       <c r="K412" s="4" t="n">
-        <v>31.6</v>
+        <v>38</v>
       </c>
       <c r="L412" t="inlineStr">
         <is>
@@ -45630,10 +45630,10 @@
         <v>-1.23</v>
       </c>
       <c r="J420" s="4" t="n">
-        <v>33.4</v>
+        <v>41.3</v>
       </c>
       <c r="K420" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>58.7</v>
       </c>
       <c r="L420" t="inlineStr">
         <is>
@@ -46908,10 +46908,10 @@
         <v>1.13</v>
       </c>
       <c r="J432" s="4" t="n">
-        <v>66.2</v>
+        <v>58</v>
       </c>
       <c r="K432" s="4" t="n">
-        <v>33.8</v>
+        <v>42</v>
       </c>
       <c r="L432" t="inlineStr">
         <is>
@@ -47770,10 +47770,10 @@
         <v>-2.36</v>
       </c>
       <c r="J440" s="4" t="n">
-        <v>29</v>
+        <v>33.4</v>
       </c>
       <c r="K440" s="4" t="n">
-        <v>71</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="L440" t="inlineStr">
         <is>
@@ -50140,14 +50140,14 @@
         <v>-3.42</v>
       </c>
       <c r="J462" s="4" t="n">
-        <v>24.9</v>
+        <v>26.2</v>
       </c>
       <c r="K462" s="4" t="n">
-        <v>75.09999999999999</v>
+        <v>73.8</v>
       </c>
       <c r="L462" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M462" s="4" t="n">
@@ -51323,10 +51323,10 @@
         <v>0.72</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>65.3</v>
+        <v>55.6</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>34.7</v>
+        <v>44.4</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52090,10 +52090,10 @@
         <v>0.04</v>
       </c>
       <c r="J480" s="4" t="n">
-        <v>61.9</v>
+        <v>50.3</v>
       </c>
       <c r="K480" s="4" t="n">
-        <v>38.1</v>
+        <v>49.7</v>
       </c>
       <c r="L480" t="inlineStr">
         <is>
@@ -52431,14 +52431,14 @@
         <v>-3.41</v>
       </c>
       <c r="J483" s="4" t="n">
-        <v>25</v>
+        <v>26.3</v>
       </c>
       <c r="K483" s="4" t="n">
-        <v>75</v>
+        <v>73.7</v>
       </c>
       <c r="L483" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M483" s="4" t="n">
@@ -52877,10 +52877,10 @@
         <v>2.1</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>69.90000000000001</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>30.1</v>
+        <v>35.4</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53322,7 +53322,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-23.94</v>
+        <v>-24.02</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53382,16 +53382,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>25.73</v>
+        <v>25.69</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>20.95</v>
+        <v>20.94</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.67</v>
+        <v>49.71</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -53555,10 +53555,10 @@
         <v>-1.74</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>31.2</v>
+        <v>37.5</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>68.8</v>
+        <v>62.5</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -53615,7 +53615,7 @@
         <v>48.04</v>
       </c>
       <c r="AB493" s="4" t="n">
-        <v>31.2</v>
+        <v>37.5</v>
       </c>
       <c r="AC493" s="4" t="n">
         <v>0</v>
@@ -53999,10 +53999,10 @@
         <v>2.45</v>
       </c>
       <c r="J497" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="K497" s="4" t="n">
-        <v>28.6</v>
+        <v>32.7</v>
       </c>
       <c r="L497" t="inlineStr">
         <is>
@@ -54804,10 +54804,10 @@
         <v>1.96</v>
       </c>
       <c r="J504" s="4" t="n">
-        <v>69.5</v>
+        <v>63.8</v>
       </c>
       <c r="K504" s="4" t="n">
-        <v>30.5</v>
+        <v>36.2</v>
       </c>
       <c r="L504" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-09-23 (re-run: Toss-up band holds to election day, no Tilt ratings)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>66.09999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>240.2</v>
+        <v>239.8</v>
       </c>
       <c r="C9" t="n">
-        <v>194.8</v>
+        <v>195.2</v>
       </c>
       <c r="D9" t="n">
         <v>236</v>
       </c>
       <c r="E9" t="n">
-        <v>88</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>69.5</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M10" s="4" t="n">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Tilt R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M26" s="4" t="n">
@@ -4948,10 +4948,10 @@
         <v>-3.73</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>77.09999999999999</v>
+        <v>77</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>44.76</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Tilt R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M40" s="4" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M51" s="4" t="n">
@@ -12772,7 +12772,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M113" s="4" t="n">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M131" s="4" t="n">
@@ -14956,7 +14956,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M133" s="4" t="n">
@@ -25775,10 +25775,10 @@
         <v>-3.17</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>28.9</v>
+        <v>28.4</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>71.09999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -26224,7 +26224,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>Tilt R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M239" s="4" t="n">
@@ -33696,7 +33696,7 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>Tilt R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M307" s="4" t="n">
@@ -45643,7 +45643,7 @@
       </c>
       <c r="L420" t="inlineStr">
         <is>
-          <t>Tilt R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M420" s="4" t="n">
@@ -51329,14 +51329,14 @@
         <v>1.17</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>58.7</v>
+        <v>58.3</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>41.3</v>
+        <v>41.7</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M473" s="4" t="n">
@@ -52103,7 +52103,7 @@
       </c>
       <c r="L480" t="inlineStr">
         <is>
-          <t>Tilt D</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M480" s="4" t="n">
@@ -52883,10 +52883,10 @@
         <v>2.54</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>67.7</v>
+        <v>67.2</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>32.3</v>
+        <v>32.8</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53328,7 +53328,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-23.73</v>
+        <v>-23.62</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53388,13 +53388,13 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>25.75</v>
+        <v>25.86</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>21.11</v>
+        <v>21</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>49.48</v>
@@ -53568,7 +53568,7 @@
       </c>
       <c r="L493" t="inlineStr">
         <is>
-          <t>Tilt R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M493" s="4" t="n">

</xml_diff>

<commit_message>
2026-09-29 forecast update; manual polls: ATR Idaho (ID-GOV, ID-SEN), Crosby internals (UT-02)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -479,7 +479,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Generic ballot D+6.7 · House popular vote D+9.3</t>
+          <t>Generic ballot D+6.7 · House popular vote D+9.4</t>
         </is>
       </c>
     </row>
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.1</v>
+        <v>52.3</v>
       </c>
       <c r="C8" t="n">
-        <v>47.9</v>
+        <v>47.7</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>68</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241.1</v>
+        <v>241.5</v>
       </c>
       <c r="C9" t="n">
-        <v>193.9</v>
+        <v>193.5</v>
       </c>
       <c r="D9" t="n">
         <v>236</v>
       </c>
       <c r="E9" t="n">
-        <v>88.40000000000001</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>71.8</v>
+        <v>71.3</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="I13" s="4" t="n">
-        <v>-38.51</v>
+        <v>-31.05</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0</v>
@@ -2158,16 +2158,16 @@
         <v>-37.52</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>29</v>
+        <v>27.82</v>
       </c>
       <c r="T13" s="4" t="n">
-        <v>50.5</v>
+        <v>41.81</v>
       </c>
       <c r="U13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-22.85</v>
+        <v>-14.14</v>
       </c>
       <c r="W13" s="5" t="n">
         <v>136953</v>
@@ -2186,16 +2186,16 @@
         </is>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>5</v>
+        <v>10.13</v>
       </c>
       <c r="AB13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>29.21</v>
+        <v>30.98</v>
       </c>
       <c r="AD13" s="4" t="n">
-        <v>65.79000000000001</v>
+        <v>58.89</v>
       </c>
       <c r="AE13" s="4" t="n">
         <v>0</v>
@@ -4053,7 +4053,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>23.07</v>
+        <v>22.4</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.90000000000001</v>
@@ -4085,16 +4085,16 @@
         <v>14.16</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>42.35</v>
+        <v>41.75</v>
       </c>
       <c r="T30" s="4" t="n">
-        <v>16.26</v>
+        <v>17.47</v>
       </c>
       <c r="U30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>26.83</v>
+        <v>24.76</v>
       </c>
       <c r="W30" s="5" t="n">
         <v>0</v>
@@ -4113,16 +4113,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>22.7</v>
+        <v>23.27</v>
       </c>
       <c r="AB30" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>47.57</v>
+        <v>46.96</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>29.73</v>
+        <v>29.77</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4948,10 +4948,10 @@
         <v>-3.17</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>26.5</v>
+        <v>27.7</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>73.5</v>
+        <v>72.3</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.04</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>26.5</v>
+        <v>27.7</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -19228,7 +19228,7 @@
         </is>
       </c>
       <c r="I173" s="4" t="n">
-        <v>-32.53</v>
+        <v>-31.17</v>
       </c>
       <c r="J173" s="4" t="n">
         <v>0</v>
@@ -19242,13 +19242,13 @@
         </is>
       </c>
       <c r="M173" s="4" t="n">
-        <v>-44.88</v>
+        <v>-43.02</v>
       </c>
       <c r="N173" s="4" t="n">
         <v>6.68</v>
       </c>
       <c r="O173" s="4" t="n">
-        <v>-40.9</v>
+        <v>-39.03</v>
       </c>
       <c r="P173" s="4" t="n">
         <v>-0.84</v>
@@ -19294,10 +19294,10 @@
         <v>0</v>
       </c>
       <c r="AC173" s="4" t="n">
-        <v>30.43</v>
+        <v>31.05</v>
       </c>
       <c r="AD173" s="4" t="n">
-        <v>59.78</v>
+        <v>59.16</v>
       </c>
       <c r="AE173" s="4" t="n">
         <v>3.81</v>
@@ -19345,13 +19345,13 @@
         </is>
       </c>
       <c r="I174" s="4" t="n">
-        <v>-26.78</v>
+        <v>-24.92</v>
       </c>
       <c r="J174" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K174" s="4" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -19359,13 +19359,13 @@
         </is>
       </c>
       <c r="M174" s="4" t="n">
-        <v>-27.07</v>
+        <v>-25.2</v>
       </c>
       <c r="N174" s="4" t="n">
         <v>6.68</v>
       </c>
       <c r="O174" s="4" t="n">
-        <v>-27.53</v>
+        <v>-25.67</v>
       </c>
       <c r="P174" s="4" t="n">
         <v>-1.51</v>
@@ -19405,10 +19405,10 @@
         <v>0</v>
       </c>
       <c r="AC174" s="4" t="n">
-        <v>32.95</v>
+        <v>33.79</v>
       </c>
       <c r="AD174" s="4" t="n">
-        <v>57.05</v>
+        <v>56.21</v>
       </c>
       <c r="AE174" s="4" t="n">
         <v>5</v>
@@ -25781,10 +25781,10 @@
         <v>-0.47</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>46.5</v>
+        <v>45.2</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>53.5</v>
+        <v>54.8</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -41346,7 +41346,7 @@
         </is>
       </c>
       <c r="I379" s="4" t="n">
-        <v>45.37</v>
+        <v>45.22</v>
       </c>
       <c r="J379" s="4" t="n">
         <v>100</v>
@@ -41360,13 +41360,13 @@
         </is>
       </c>
       <c r="M379" s="4" t="n">
-        <v>28.19</v>
+        <v>28.03</v>
       </c>
       <c r="N379" s="4" t="n">
         <v>6.68</v>
       </c>
       <c r="O379" s="4" t="n">
-        <v>45.53</v>
+        <v>45.37</v>
       </c>
       <c r="P379" s="4" t="n">
         <v>2.51</v>
@@ -41406,10 +41406,10 @@
         <v>0</v>
       </c>
       <c r="AC379" s="4" t="n">
-        <v>70.44</v>
+        <v>70.36</v>
       </c>
       <c r="AD379" s="4" t="n">
-        <v>26.47</v>
+        <v>26.55</v>
       </c>
       <c r="AE379" s="4" t="n">
         <v>0</v>
@@ -41457,7 +41457,7 @@
         </is>
       </c>
       <c r="I380" s="4" t="n">
-        <v>19.77</v>
+        <v>19.62</v>
       </c>
       <c r="J380" s="4" t="n">
         <v>99.8</v>
@@ -41471,13 +41471,13 @@
         </is>
       </c>
       <c r="M380" s="4" t="n">
-        <v>12.33</v>
+        <v>12.17</v>
       </c>
       <c r="N380" s="4" t="n">
         <v>6.68</v>
       </c>
       <c r="O380" s="4" t="n">
-        <v>19.77</v>
+        <v>19.62</v>
       </c>
       <c r="P380" s="4" t="n">
         <v>-0.57</v>
@@ -41509,10 +41509,10 @@
         <v>0</v>
       </c>
       <c r="AC380" s="4" t="n">
-        <v>59.89</v>
+        <v>59.81</v>
       </c>
       <c r="AD380" s="4" t="n">
-        <v>40.11</v>
+        <v>40.19</v>
       </c>
       <c r="AE380" s="4" t="n">
         <v>0</v>
@@ -47470,13 +47470,13 @@
         </is>
       </c>
       <c r="I437" s="4" t="n">
-        <v>-33.63</v>
+        <v>-15.58</v>
       </c>
       <c r="J437" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K437" s="4" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="L437" t="inlineStr">
         <is>
@@ -47501,12 +47501,18 @@
       <c r="R437" s="4" t="n">
         <v>-29.9</v>
       </c>
-      <c r="S437" s="4" t="n"/>
-      <c r="T437" s="4" t="n"/>
+      <c r="S437" s="4" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="T437" s="4" t="n">
+        <v>32.18</v>
+      </c>
       <c r="U437" t="n">
-        <v>0</v>
-      </c>
-      <c r="V437" s="4" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="V437" s="4" t="n">
+        <v>-1.64</v>
+      </c>
       <c r="W437" s="5" t="n">
         <v>60225</v>
       </c>
@@ -47530,10 +47536,10 @@
         <v>0</v>
       </c>
       <c r="AC437" s="4" t="n">
-        <v>28.87</v>
+        <v>36.72</v>
       </c>
       <c r="AD437" s="4" t="n">
-        <v>58.13</v>
+        <v>50.28</v>
       </c>
       <c r="AE437" s="4" t="n">
         <v>7</v>
@@ -51359,10 +51365,10 @@
         <v>1.41</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>61.3</v>
+        <v>61</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>38.7</v>
+        <v>39</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52240,13 +52246,13 @@
         </is>
       </c>
       <c r="I481" s="4" t="n">
-        <v>-19.31</v>
+        <v>-10.34</v>
       </c>
       <c r="J481" s="4" t="n">
-        <v>0.2</v>
+        <v>2.3</v>
       </c>
       <c r="K481" s="4" t="n">
-        <v>99.8</v>
+        <v>97.7</v>
       </c>
       <c r="L481" t="inlineStr">
         <is>
@@ -52254,13 +52260,13 @@
         </is>
       </c>
       <c r="M481" s="4" t="n">
-        <v>-30.52</v>
+        <v>-28.65</v>
       </c>
       <c r="N481" s="4" t="n">
         <v>6.68</v>
       </c>
       <c r="O481" s="4" t="n">
-        <v>-27.14</v>
+        <v>-25.27</v>
       </c>
       <c r="P481" s="4" t="n">
         <v>-1.14</v>
@@ -52272,16 +52278,16 @@
         <v>-37.52</v>
       </c>
       <c r="S481" s="4" t="n">
-        <v>29.96</v>
+        <v>44.02</v>
       </c>
       <c r="T481" s="4" t="n">
-        <v>39.02</v>
+        <v>38.97</v>
       </c>
       <c r="U481" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V481" s="4" t="n">
-        <v>-8.93</v>
+        <v>5.47</v>
       </c>
       <c r="W481" s="5" t="n">
         <v>0</v>
@@ -52300,16 +52306,16 @@
         </is>
       </c>
       <c r="AA481" s="4" t="n">
-        <v>38.15</v>
+        <v>42.63</v>
       </c>
       <c r="AB481" s="4" t="n">
-        <v>0.2</v>
+        <v>2.3</v>
       </c>
       <c r="AC481" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AD481" s="4" t="n">
-        <v>57.46</v>
+        <v>52.98</v>
       </c>
       <c r="AE481" s="4" t="n">
         <v>4.39</v>
@@ -52919,10 +52925,10 @@
         <v>1.98</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>64.7</v>
+        <v>63.1</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>35.3</v>
+        <v>36.9</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53364,7 +53370,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.59</v>
+        <v>-21.54</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53424,16 +53430,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.74</v>
+        <v>27.75</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.27</v>
+        <v>19.3</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.33</v>
+        <v>49.29</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -54379,7 +54385,7 @@
         </is>
       </c>
       <c r="I500" s="4" t="n">
-        <v>24.72</v>
+        <v>24.62</v>
       </c>
       <c r="J500" s="4" t="n">
         <v>99.90000000000001</v>
@@ -54393,13 +54399,13 @@
         </is>
       </c>
       <c r="M500" s="4" t="n">
-        <v>17.98</v>
+        <v>17.81</v>
       </c>
       <c r="N500" s="4" t="n">
         <v>6.68</v>
       </c>
       <c r="O500" s="4" t="n">
-        <v>28.15</v>
+        <v>27.98</v>
       </c>
       <c r="P500" s="4" t="n">
         <v>2.03</v>
@@ -54445,10 +54451,10 @@
         <v>0</v>
       </c>
       <c r="AC500" s="4" t="n">
-        <v>59.73</v>
+        <v>59.68</v>
       </c>
       <c r="AD500" s="4" t="n">
-        <v>36.05</v>
+        <v>36.1</v>
       </c>
       <c r="AE500" s="4" t="n">
         <v>0</v>
@@ -54846,10 +54852,10 @@
         <v>3.05</v>
       </c>
       <c r="J504" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="K504" s="4" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="L504" t="inlineStr">
         <is>
@@ -54875,16 +54881,16 @@
         <v>-13.88</v>
       </c>
       <c r="S504" s="4" t="n">
-        <v>47.78</v>
+        <v>47.74</v>
       </c>
       <c r="T504" s="4" t="n">
-        <v>44.61</v>
+        <v>44.67</v>
       </c>
       <c r="U504" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="V504" s="4" t="n">
-        <v>4.29</v>
+        <v>4.23</v>
       </c>
       <c r="W504" s="5" t="n">
         <v>68560930</v>
@@ -54903,7 +54909,7 @@
         </is>
       </c>
       <c r="AA504" s="4" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="AB504" s="4" t="n">
         <v>0</v>
@@ -54912,7 +54918,7 @@
         <v>51.02</v>
       </c>
       <c r="AD504" s="4" t="n">
-        <v>48</v>
+        <v>48.01</v>
       </c>
       <c r="AE504" s="4" t="n">
         <v>0</v>
@@ -56789,16 +56795,16 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="K26" t="n">
         <v>13</v>
-      </c>
-      <c r="K26" t="n">
-        <v>12</v>
       </c>
       <c r="L26" t="n">
         <v>8</v>
       </c>
       <c r="M26" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N26" s="4" t="n">
         <v>0.2</v>
@@ -56847,7 +56853,7 @@
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="K27" t="n">
         <v>7</v>
@@ -56859,7 +56865,7 @@
         <v>10</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-09-30 (rerun: new polls)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.3</v>
+        <v>52.2</v>
       </c>
       <c r="C8" t="n">
-        <v>47.7</v>
+        <v>47.8</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>68.8</v>
+        <v>68.3</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241.5</v>
+        <v>242</v>
       </c>
       <c r="C9" t="n">
-        <v>193.5</v>
+        <v>193</v>
       </c>
       <c r="D9" t="n">
         <v>236</v>
       </c>
       <c r="E9" t="n">
-        <v>89</v>
+        <v>89.5</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27</v>
+        <v>26.8</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>72</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -3823,17 +3823,17 @@
         </is>
       </c>
       <c r="I28" s="4" t="n">
-        <v>4.31</v>
+        <v>3.37</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>78.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>21.6</v>
+        <v>26.5</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Likely D</t>
+          <t>Lean D</t>
         </is>
       </c>
       <c r="M28" s="4" t="n">
@@ -3855,16 +3855,16 @@
         <v>14.89</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>43.16</v>
+        <v>44.92</v>
       </c>
       <c r="T28" s="4" t="n">
-        <v>45.29</v>
+        <v>46.35</v>
       </c>
       <c r="U28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.58</v>
+        <v>-0.83</v>
       </c>
       <c r="W28" s="5" t="n">
         <v>0</v>
@@ -3883,16 +3883,16 @@
         </is>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>3.46</v>
+        <v>3.17</v>
       </c>
       <c r="AB28" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC28" s="4" t="n">
-        <v>50.35</v>
+        <v>50.05</v>
       </c>
       <c r="AD28" s="4" t="n">
-        <v>46.19</v>
+        <v>46.78</v>
       </c>
       <c r="AE28" s="4" t="n">
         <v>0</v>
@@ -4729,17 +4729,17 @@
         </is>
       </c>
       <c r="I36" s="4" t="n">
-        <v>4.27</v>
+        <v>3.58</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>78.3</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>21.7</v>
+        <v>25.1</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Likely D</t>
+          <t>Lean D</t>
         </is>
       </c>
       <c r="M36" s="4" t="n">
@@ -4761,16 +4761,16 @@
         <v>-0.87</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>46.33</v>
+        <v>47.02</v>
       </c>
       <c r="T36" s="4" t="n">
-        <v>43.81</v>
+        <v>44.86</v>
       </c>
       <c r="U36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>4.37</v>
+        <v>2.96</v>
       </c>
       <c r="W36" s="5" t="n">
         <v>1426778</v>
@@ -4787,10 +4787,10 @@
         <v>0</v>
       </c>
       <c r="AC36" s="4" t="n">
-        <v>52.14</v>
+        <v>51.79</v>
       </c>
       <c r="AD36" s="4" t="n">
-        <v>47.86</v>
+        <v>48.21</v>
       </c>
       <c r="AE36" s="4" t="n">
         <v>0</v>
@@ -4948,10 +4948,10 @@
         <v>-3.04</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>27.7</v>
+        <v>28.4</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>72.3</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.1</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>27.7</v>
+        <v>28.4</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -18790,7 +18790,7 @@
         </is>
       </c>
       <c r="I169" s="4" t="n">
-        <v>14.13</v>
+        <v>14.15</v>
       </c>
       <c r="J169" s="4" t="n">
         <v>99.2</v>
@@ -18804,13 +18804,13 @@
         </is>
       </c>
       <c r="M169" s="4" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="N169" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O169" s="4" t="n">
-        <v>16.68</v>
+        <v>16.7</v>
       </c>
       <c r="P169" s="4" t="n">
         <v>0.08</v>
@@ -18903,13 +18903,13 @@
         </is>
       </c>
       <c r="I170" s="4" t="n">
-        <v>4.71</v>
+        <v>4.73</v>
       </c>
       <c r="J170" s="4" t="n">
-        <v>79.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="K170" s="4" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -18917,13 +18917,13 @@
         </is>
       </c>
       <c r="M170" s="4" t="n">
-        <v>-1.07</v>
+        <v>-1.05</v>
       </c>
       <c r="N170" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O170" s="4" t="n">
-        <v>5.02</v>
+        <v>5.04</v>
       </c>
       <c r="P170" s="4" t="n">
         <v>0.15</v>
@@ -18969,10 +18969,10 @@
         <v>0</v>
       </c>
       <c r="AC170" s="4" t="n">
-        <v>49.6</v>
+        <v>49.61</v>
       </c>
       <c r="AD170" s="4" t="n">
-        <v>45.14</v>
+        <v>45.13</v>
       </c>
       <c r="AE170" s="4" t="n">
         <v>2.63</v>
@@ -19020,7 +19020,7 @@
         </is>
       </c>
       <c r="I171" s="4" t="n">
-        <v>7.84</v>
+        <v>7.86</v>
       </c>
       <c r="J171" s="4" t="n">
         <v>90.09999999999999</v>
@@ -19034,13 +19034,13 @@
         </is>
       </c>
       <c r="M171" s="4" t="n">
-        <v>4.03</v>
+        <v>4.05</v>
       </c>
       <c r="N171" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O171" s="4" t="n">
-        <v>9.25</v>
+        <v>9.27</v>
       </c>
       <c r="P171" s="4" t="n">
         <v>0.12</v>
@@ -19078,10 +19078,10 @@
         <v>0</v>
       </c>
       <c r="AC171" s="4" t="n">
-        <v>53.92</v>
+        <v>53.93</v>
       </c>
       <c r="AD171" s="4" t="n">
-        <v>46.08</v>
+        <v>46.07</v>
       </c>
       <c r="AE171" s="4" t="n">
         <v>0</v>
@@ -19125,7 +19125,7 @@
         </is>
       </c>
       <c r="I172" s="4" t="n">
-        <v>-17.98</v>
+        <v>-17.96</v>
       </c>
       <c r="J172" s="4" t="n">
         <v>0.4</v>
@@ -19139,13 +19139,13 @@
         </is>
       </c>
       <c r="M172" s="4" t="n">
-        <v>-23.04</v>
+        <v>-23.02</v>
       </c>
       <c r="N172" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O172" s="4" t="n">
-        <v>-17.98</v>
+        <v>-17.96</v>
       </c>
       <c r="P172" s="4" t="n">
         <v>-1.08</v>
@@ -19177,10 +19177,10 @@
         <v>0</v>
       </c>
       <c r="AC172" s="4" t="n">
-        <v>41.01</v>
+        <v>41.02</v>
       </c>
       <c r="AD172" s="4" t="n">
-        <v>58.99</v>
+        <v>58.98</v>
       </c>
       <c r="AE172" s="4" t="n">
         <v>0</v>
@@ -25781,10 +25781,10 @@
         <v>-0.4</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.5</v>
+        <v>47.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.5</v>
+        <v>52.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29754,13 +29754,13 @@
         </is>
       </c>
       <c r="M271" s="4" t="n">
-        <v>-6.95</v>
+        <v>-6.94</v>
       </c>
       <c r="N271" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O271" s="4" t="n">
-        <v>6.05</v>
+        <v>6.06</v>
       </c>
       <c r="P271" s="4" t="n">
         <v>0.22</v>
@@ -29857,7 +29857,7 @@
         </is>
       </c>
       <c r="I272" s="4" t="n">
-        <v>48.3</v>
+        <v>48.31</v>
       </c>
       <c r="J272" s="4" t="n">
         <v>100</v>
@@ -29982,7 +29982,7 @@
         </is>
       </c>
       <c r="M273" s="4" t="n">
-        <v>-8.99</v>
+        <v>-8.98</v>
       </c>
       <c r="N273" s="4" t="n">
         <v>6.77</v>
@@ -30034,10 +30034,10 @@
         <v>0</v>
       </c>
       <c r="AC273" s="4" t="n">
-        <v>46.89</v>
+        <v>46.9</v>
       </c>
       <c r="AD273" s="4" t="n">
-        <v>51.61</v>
+        <v>51.6</v>
       </c>
       <c r="AE273" s="4" t="n">
         <v>0</v>
@@ -30085,7 +30085,7 @@
         </is>
       </c>
       <c r="I274" s="4" t="n">
-        <v>61.78</v>
+        <v>61.79</v>
       </c>
       <c r="J274" s="4" t="n">
         <v>100</v>
@@ -30099,7 +30099,7 @@
         </is>
       </c>
       <c r="M274" s="4" t="n">
-        <v>49.52</v>
+        <v>49.53</v>
       </c>
       <c r="N274" s="4" t="n">
         <v>6.77</v>
@@ -30196,7 +30196,7 @@
         </is>
       </c>
       <c r="I275" s="4" t="n">
-        <v>-7.9</v>
+        <v>-7.89</v>
       </c>
       <c r="J275" s="4" t="n">
         <v>9.800000000000001</v>
@@ -30210,13 +30210,13 @@
         </is>
       </c>
       <c r="M275" s="4" t="n">
-        <v>-13.85</v>
+        <v>-13.84</v>
       </c>
       <c r="N275" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O275" s="4" t="n">
-        <v>-8.23</v>
+        <v>-8.220000000000001</v>
       </c>
       <c r="P275" s="4" t="n">
         <v>-0.82</v>
@@ -30307,7 +30307,7 @@
         </is>
       </c>
       <c r="I276" s="4" t="n">
-        <v>-10.47</v>
+        <v>-10.46</v>
       </c>
       <c r="J276" s="4" t="n">
         <v>3.1</v>
@@ -30321,13 +30321,13 @@
         </is>
       </c>
       <c r="M276" s="4" t="n">
-        <v>-14.02</v>
+        <v>-14.01</v>
       </c>
       <c r="N276" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O276" s="4" t="n">
-        <v>-10.47</v>
+        <v>-10.46</v>
       </c>
       <c r="P276" s="4" t="n">
         <v>-1.22</v>
@@ -30424,13 +30424,13 @@
         </is>
       </c>
       <c r="M277" s="4" t="n">
-        <v>-10.04</v>
+        <v>-10.03</v>
       </c>
       <c r="N277" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O277" s="4" t="n">
-        <v>-8.5</v>
+        <v>-8.49</v>
       </c>
       <c r="P277" s="4" t="n">
         <v>-1.34</v>
@@ -30476,10 +30476,10 @@
         <v>0</v>
       </c>
       <c r="AC277" s="4" t="n">
-        <v>45.37</v>
+        <v>45.38</v>
       </c>
       <c r="AD277" s="4" t="n">
-        <v>53.13</v>
+        <v>53.12</v>
       </c>
       <c r="AE277" s="4" t="n">
         <v>0</v>
@@ -30527,7 +30527,7 @@
         </is>
       </c>
       <c r="I278" s="4" t="n">
-        <v>-15</v>
+        <v>-14.99</v>
       </c>
       <c r="J278" s="4" t="n">
         <v>0.7</v>
@@ -30541,13 +30541,13 @@
         </is>
       </c>
       <c r="M278" s="4" t="n">
-        <v>-16.07</v>
+        <v>-16.06</v>
       </c>
       <c r="N278" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O278" s="4" t="n">
-        <v>-14.56</v>
+        <v>-14.55</v>
       </c>
       <c r="P278" s="4" t="n">
         <v>-1.86</v>
@@ -30587,10 +30587,10 @@
         <v>0</v>
       </c>
       <c r="AC278" s="4" t="n">
-        <v>41.75</v>
+        <v>41.76</v>
       </c>
       <c r="AD278" s="4" t="n">
-        <v>56.49</v>
+        <v>56.48</v>
       </c>
       <c r="AE278" s="4" t="n">
         <v>0</v>
@@ -30638,7 +30638,7 @@
         </is>
       </c>
       <c r="I279" s="4" t="n">
-        <v>-7.73</v>
+        <v>-7.72</v>
       </c>
       <c r="J279" s="4" t="n">
         <v>10.3</v>
@@ -30652,13 +30652,13 @@
         </is>
       </c>
       <c r="M279" s="4" t="n">
-        <v>-12.37</v>
+        <v>-12.36</v>
       </c>
       <c r="N279" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O279" s="4" t="n">
-        <v>-9.050000000000001</v>
+        <v>-9.039999999999999</v>
       </c>
       <c r="P279" s="4" t="n">
         <v>-0.22</v>
@@ -30747,7 +30747,7 @@
         </is>
       </c>
       <c r="I280" s="4" t="n">
-        <v>-12.88</v>
+        <v>-12.87</v>
       </c>
       <c r="J280" s="4" t="n">
         <v>1</v>
@@ -30761,7 +30761,7 @@
         </is>
       </c>
       <c r="M280" s="4" t="n">
-        <v>-14.19</v>
+        <v>-14.18</v>
       </c>
       <c r="N280" s="4" t="n">
         <v>6.77</v>
@@ -30813,10 +30813,10 @@
         <v>0</v>
       </c>
       <c r="AC280" s="4" t="n">
-        <v>42.8</v>
+        <v>42.81</v>
       </c>
       <c r="AD280" s="4" t="n">
-        <v>55.46</v>
+        <v>55.45</v>
       </c>
       <c r="AE280" s="4" t="n">
         <v>0</v>
@@ -30874,13 +30874,13 @@
         </is>
       </c>
       <c r="M281" s="4" t="n">
-        <v>-7.01</v>
+        <v>-7</v>
       </c>
       <c r="N281" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O281" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.95</v>
       </c>
       <c r="P281" s="4" t="n">
         <v>0</v>
@@ -30977,7 +30977,7 @@
         </is>
       </c>
       <c r="I282" s="4" t="n">
-        <v>62.21</v>
+        <v>62.22</v>
       </c>
       <c r="J282" s="4" t="n">
         <v>100</v>
@@ -30991,13 +30991,13 @@
         </is>
       </c>
       <c r="M282" s="4" t="n">
-        <v>51.24</v>
+        <v>51.25</v>
       </c>
       <c r="N282" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O282" s="4" t="n">
-        <v>62.21</v>
+        <v>62.22</v>
       </c>
       <c r="P282" s="4" t="n">
         <v>1.26</v>
@@ -31080,7 +31080,7 @@
         </is>
       </c>
       <c r="I283" s="4" t="n">
-        <v>-10.24</v>
+        <v>-10.23</v>
       </c>
       <c r="J283" s="4" t="n">
         <v>3.6</v>
@@ -31100,7 +31100,7 @@
         <v>6.77</v>
       </c>
       <c r="O283" s="4" t="n">
-        <v>-10.61</v>
+        <v>-10.6</v>
       </c>
       <c r="P283" s="4" t="n">
         <v>-0.19</v>
@@ -31191,7 +31191,7 @@
         </is>
       </c>
       <c r="I284" s="4" t="n">
-        <v>-10.45</v>
+        <v>-10.44</v>
       </c>
       <c r="J284" s="4" t="n">
         <v>3.1</v>
@@ -31211,7 +31211,7 @@
         <v>6.77</v>
       </c>
       <c r="O284" s="4" t="n">
-        <v>-11.91</v>
+        <v>-11.9</v>
       </c>
       <c r="P284" s="4" t="n">
         <v>-2.3</v>
@@ -38933,7 +38933,7 @@
         </is>
       </c>
       <c r="I356" s="4" t="n">
-        <v>51.35</v>
+        <v>51.11</v>
       </c>
       <c r="J356" s="4" t="n">
         <v>100</v>
@@ -38947,13 +38947,13 @@
         </is>
       </c>
       <c r="M356" s="4" t="n">
-        <v>39.03</v>
+        <v>38.79</v>
       </c>
       <c r="N356" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O356" s="4" t="n">
-        <v>51.35</v>
+        <v>51.11</v>
       </c>
       <c r="P356" s="4" t="n">
         <v>2.08</v>
@@ -38985,10 +38985,10 @@
         <v>0</v>
       </c>
       <c r="AC356" s="4" t="n">
-        <v>75.67</v>
+        <v>75.56</v>
       </c>
       <c r="AD356" s="4" t="n">
-        <v>24.33</v>
+        <v>24.44</v>
       </c>
       <c r="AE356" s="4" t="n">
         <v>0</v>
@@ -39036,7 +39036,7 @@
         </is>
       </c>
       <c r="I357" s="4" t="n">
-        <v>-27.13</v>
+        <v>-27.36</v>
       </c>
       <c r="J357" s="4" t="n">
         <v>0</v>
@@ -39050,13 +39050,13 @@
         </is>
       </c>
       <c r="M357" s="4" t="n">
-        <v>-27.8</v>
+        <v>-28.03</v>
       </c>
       <c r="N357" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O357" s="4" t="n">
-        <v>-27.13</v>
+        <v>-27.36</v>
       </c>
       <c r="P357" s="4" t="n">
         <v>-1.49</v>
@@ -39088,10 +39088,10 @@
         <v>0</v>
       </c>
       <c r="AC357" s="4" t="n">
-        <v>36.44</v>
+        <v>36.32</v>
       </c>
       <c r="AD357" s="4" t="n">
-        <v>63.56</v>
+        <v>63.68</v>
       </c>
       <c r="AE357" s="4" t="n">
         <v>0</v>
@@ -39139,7 +39139,7 @@
         </is>
       </c>
       <c r="I358" s="4" t="n">
-        <v>57.05</v>
+        <v>56.82</v>
       </c>
       <c r="J358" s="4" t="n">
         <v>100</v>
@@ -39153,13 +39153,13 @@
         </is>
       </c>
       <c r="M358" s="4" t="n">
-        <v>47.6</v>
+        <v>47.37</v>
       </c>
       <c r="N358" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O358" s="4" t="n">
-        <v>57.05</v>
+        <v>56.82</v>
       </c>
       <c r="P358" s="4" t="n">
         <v>0</v>
@@ -39191,10 +39191,10 @@
         <v>0</v>
       </c>
       <c r="AC358" s="4" t="n">
-        <v>78.53</v>
+        <v>78.41</v>
       </c>
       <c r="AD358" s="4" t="n">
-        <v>21.47</v>
+        <v>21.59</v>
       </c>
       <c r="AE358" s="4" t="n">
         <v>0</v>
@@ -39242,7 +39242,7 @@
         </is>
       </c>
       <c r="I359" s="4" t="n">
-        <v>17.62</v>
+        <v>17.39</v>
       </c>
       <c r="J359" s="4" t="n">
         <v>99.59999999999999</v>
@@ -39256,13 +39256,13 @@
         </is>
       </c>
       <c r="M359" s="4" t="n">
-        <v>12.1</v>
+        <v>11.87</v>
       </c>
       <c r="N359" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O359" s="4" t="n">
-        <v>18.8</v>
+        <v>18.56</v>
       </c>
       <c r="P359" s="4" t="n">
         <v>0.38</v>
@@ -39302,10 +39302,10 @@
         <v>0</v>
       </c>
       <c r="AC359" s="4" t="n">
-        <v>56.05</v>
+        <v>55.94</v>
       </c>
       <c r="AD359" s="4" t="n">
-        <v>39.25</v>
+        <v>39.36</v>
       </c>
       <c r="AE359" s="4" t="n">
         <v>0</v>
@@ -39353,7 +39353,7 @@
         </is>
       </c>
       <c r="I360" s="4" t="n">
-        <v>17.34</v>
+        <v>17.1</v>
       </c>
       <c r="J360" s="4" t="n">
         <v>99.59999999999999</v>
@@ -39367,13 +39367,13 @@
         </is>
       </c>
       <c r="M360" s="4" t="n">
-        <v>8.33</v>
+        <v>8.1</v>
       </c>
       <c r="N360" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O360" s="4" t="n">
-        <v>18.51</v>
+        <v>18.28</v>
       </c>
       <c r="P360" s="4" t="n">
         <v>1.57</v>
@@ -39413,10 +39413,10 @@
         <v>0</v>
       </c>
       <c r="AC360" s="4" t="n">
-        <v>55.92</v>
+        <v>55.81</v>
       </c>
       <c r="AD360" s="4" t="n">
-        <v>39.39</v>
+        <v>39.5</v>
       </c>
       <c r="AE360" s="4" t="n">
         <v>0</v>
@@ -39464,7 +39464,7 @@
         </is>
       </c>
       <c r="I361" s="4" t="n">
-        <v>19.88</v>
+        <v>19.65</v>
       </c>
       <c r="J361" s="4" t="n">
         <v>99.8</v>
@@ -39478,13 +39478,13 @@
         </is>
       </c>
       <c r="M361" s="4" t="n">
-        <v>11.56</v>
+        <v>11.32</v>
       </c>
       <c r="N361" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O361" s="4" t="n">
-        <v>19.88</v>
+        <v>19.65</v>
       </c>
       <c r="P361" s="4" t="n">
         <v>2.46</v>
@@ -39516,10 +39516,10 @@
         <v>0</v>
       </c>
       <c r="AC361" s="4" t="n">
-        <v>59.94</v>
+        <v>59.82</v>
       </c>
       <c r="AD361" s="4" t="n">
-        <v>40.06</v>
+        <v>40.18</v>
       </c>
       <c r="AE361" s="4" t="n">
         <v>0</v>
@@ -44235,13 +44235,13 @@
         </is>
       </c>
       <c r="I406" s="4" t="n">
-        <v>-4.21</v>
+        <v>-6.29</v>
       </c>
       <c r="J406" s="4" t="n">
-        <v>22</v>
+        <v>14.8</v>
       </c>
       <c r="K406" s="4" t="n">
-        <v>78</v>
+        <v>85.2</v>
       </c>
       <c r="L406" t="inlineStr">
         <is>
@@ -44266,12 +44266,18 @@
       <c r="R406" s="4" t="n">
         <v>-20.07</v>
       </c>
-      <c r="S406" s="4" t="n"/>
-      <c r="T406" s="4" t="n"/>
+      <c r="S406" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="T406" s="4" t="n">
+        <v>45</v>
+      </c>
       <c r="U406" t="n">
-        <v>0</v>
-      </c>
-      <c r="V406" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V406" s="4" t="n">
+        <v>-8.470000000000001</v>
+      </c>
       <c r="W406" s="5" t="n">
         <v>55358</v>
       </c>
@@ -44287,10 +44293,10 @@
         <v>0</v>
       </c>
       <c r="AC406" s="4" t="n">
-        <v>47.9</v>
+        <v>46.86</v>
       </c>
       <c r="AD406" s="4" t="n">
-        <v>52.1</v>
+        <v>53.14</v>
       </c>
       <c r="AE406" s="4" t="n">
         <v>0</v>
@@ -50179,13 +50185,13 @@
         </is>
       </c>
       <c r="I462" s="4" t="n">
-        <v>-2.55</v>
+        <v>-2.66</v>
       </c>
       <c r="J462" s="4" t="n">
-        <v>32.1</v>
+        <v>31.3</v>
       </c>
       <c r="K462" s="4" t="n">
-        <v>67.90000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="L462" t="inlineStr">
         <is>
@@ -50193,13 +50199,13 @@
         </is>
       </c>
       <c r="M462" s="4" t="n">
-        <v>-2.54</v>
+        <v>-2.71</v>
       </c>
       <c r="N462" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O462" s="4" t="n">
-        <v>-2.52</v>
+        <v>-2.69</v>
       </c>
       <c r="P462" s="4" t="n">
         <v>-1.44</v>
@@ -50237,10 +50243,10 @@
         <v>0</v>
       </c>
       <c r="AC462" s="4" t="n">
-        <v>48.72</v>
+        <v>48.67</v>
       </c>
       <c r="AD462" s="4" t="n">
-        <v>51.28</v>
+        <v>51.33</v>
       </c>
       <c r="AE462" s="4" t="n">
         <v>0</v>
@@ -50288,7 +50294,7 @@
         </is>
       </c>
       <c r="I463" s="4" t="n">
-        <v>51.17</v>
+        <v>50.99</v>
       </c>
       <c r="J463" s="4" t="n">
         <v>100</v>
@@ -50302,13 +50308,13 @@
         </is>
       </c>
       <c r="M463" s="4" t="n">
-        <v>42.45</v>
+        <v>42.27</v>
       </c>
       <c r="N463" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O463" s="4" t="n">
-        <v>51.17</v>
+        <v>50.99</v>
       </c>
       <c r="P463" s="4" t="n">
         <v>0</v>
@@ -50340,10 +50346,10 @@
         <v>0</v>
       </c>
       <c r="AC463" s="4" t="n">
-        <v>75.58</v>
+        <v>75.5</v>
       </c>
       <c r="AD463" s="4" t="n">
-        <v>24.42</v>
+        <v>24.5</v>
       </c>
       <c r="AE463" s="4" t="n">
         <v>0</v>
@@ -50391,13 +50397,13 @@
         </is>
       </c>
       <c r="I464" s="4" t="n">
-        <v>6.24</v>
+        <v>6.12</v>
       </c>
       <c r="J464" s="4" t="n">
-        <v>85.09999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="K464" s="4" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="L464" t="inlineStr">
         <is>
@@ -50405,13 +50411,13 @@
         </is>
       </c>
       <c r="M464" s="4" t="n">
-        <v>-5.37</v>
+        <v>-5.54</v>
       </c>
       <c r="N464" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O464" s="4" t="n">
-        <v>7.94</v>
+        <v>7.76</v>
       </c>
       <c r="P464" s="4" t="n">
         <v>0.17</v>
@@ -50457,10 +50463,10 @@
         <v>0</v>
       </c>
       <c r="AC464" s="4" t="n">
-        <v>51.77</v>
+        <v>51.71</v>
       </c>
       <c r="AD464" s="4" t="n">
-        <v>45.69</v>
+        <v>45.75</v>
       </c>
       <c r="AE464" s="4" t="n">
         <v>0</v>
@@ -50508,7 +50514,7 @@
         </is>
       </c>
       <c r="I465" s="4" t="n">
-        <v>64.45</v>
+        <v>64.28</v>
       </c>
       <c r="J465" s="4" t="n">
         <v>100</v>
@@ -50522,13 +50528,13 @@
         </is>
       </c>
       <c r="M465" s="4" t="n">
-        <v>54.17</v>
+        <v>54</v>
       </c>
       <c r="N465" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O465" s="4" t="n">
-        <v>64.58</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="P465" s="4" t="n">
         <v>0</v>
@@ -50568,10 +50574,10 @@
         <v>0</v>
       </c>
       <c r="AC465" s="4" t="n">
-        <v>80.16</v>
+        <v>80.08</v>
       </c>
       <c r="AD465" s="4" t="n">
-        <v>17.33</v>
+        <v>17.41</v>
       </c>
       <c r="AE465" s="4" t="n">
         <v>0</v>
@@ -50619,7 +50625,7 @@
         </is>
       </c>
       <c r="I466" s="4" t="n">
-        <v>-22.59</v>
+        <v>-22.76</v>
       </c>
       <c r="J466" s="4" t="n">
         <v>0.1</v>
@@ -50633,13 +50639,13 @@
         </is>
       </c>
       <c r="M466" s="4" t="n">
-        <v>-21.6</v>
+        <v>-21.78</v>
       </c>
       <c r="N466" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O466" s="4" t="n">
-        <v>-22.59</v>
+        <v>-22.76</v>
       </c>
       <c r="P466" s="4" t="n">
         <v>-2.32</v>
@@ -50671,10 +50677,10 @@
         <v>0</v>
       </c>
       <c r="AC466" s="4" t="n">
-        <v>38.71</v>
+        <v>38.62</v>
       </c>
       <c r="AD466" s="4" t="n">
-        <v>61.29</v>
+        <v>61.38</v>
       </c>
       <c r="AE466" s="4" t="n">
         <v>0</v>
@@ -50722,7 +50728,7 @@
         </is>
       </c>
       <c r="I467" s="4" t="n">
-        <v>-17.15</v>
+        <v>-17.3</v>
       </c>
       <c r="J467" s="4" t="n">
         <v>0.4</v>
@@ -50736,13 +50742,13 @@
         </is>
       </c>
       <c r="M467" s="4" t="n">
-        <v>-15.21</v>
+        <v>-15.39</v>
       </c>
       <c r="N467" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O467" s="4" t="n">
-        <v>-15.22</v>
+        <v>-15.39</v>
       </c>
       <c r="P467" s="4" t="n">
         <v>-1.13</v>
@@ -50788,10 +50794,10 @@
         <v>0</v>
       </c>
       <c r="AC467" s="4" t="n">
-        <v>39.43</v>
+        <v>39.36</v>
       </c>
       <c r="AD467" s="4" t="n">
-        <v>55.75</v>
+        <v>55.82</v>
       </c>
       <c r="AE467" s="4" t="n">
         <v>2.41</v>
@@ -50835,7 +50841,7 @@
         </is>
       </c>
       <c r="I468" s="4" t="n">
-        <v>-16.2</v>
+        <v>-16.38</v>
       </c>
       <c r="J468" s="4" t="n">
         <v>0.5</v>
@@ -50849,13 +50855,13 @@
         </is>
       </c>
       <c r="M468" s="4" t="n">
-        <v>-20.83</v>
+        <v>-21.01</v>
       </c>
       <c r="N468" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O468" s="4" t="n">
-        <v>-16.2</v>
+        <v>-16.38</v>
       </c>
       <c r="P468" s="4" t="n">
         <v>-1.15</v>
@@ -50887,10 +50893,10 @@
         <v>0</v>
       </c>
       <c r="AC468" s="4" t="n">
-        <v>41.9</v>
+        <v>41.81</v>
       </c>
       <c r="AD468" s="4" t="n">
-        <v>58.1</v>
+        <v>58.19</v>
       </c>
       <c r="AE468" s="4" t="n">
         <v>0</v>
@@ -50938,7 +50944,7 @@
         </is>
       </c>
       <c r="I469" s="4" t="n">
-        <v>-12.56</v>
+        <v>-12.74</v>
       </c>
       <c r="J469" s="4" t="n">
         <v>1</v>
@@ -50952,13 +50958,13 @@
         </is>
       </c>
       <c r="M469" s="4" t="n">
-        <v>-15.01</v>
+        <v>-15.18</v>
       </c>
       <c r="N469" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O469" s="4" t="n">
-        <v>-12.56</v>
+        <v>-12.74</v>
       </c>
       <c r="P469" s="4" t="n">
         <v>-1.69</v>
@@ -50990,10 +50996,10 @@
         <v>0</v>
       </c>
       <c r="AC469" s="4" t="n">
-        <v>43.72</v>
+        <v>43.63</v>
       </c>
       <c r="AD469" s="4" t="n">
-        <v>56.28</v>
+        <v>56.37</v>
       </c>
       <c r="AE469" s="4" t="n">
         <v>0</v>
@@ -51365,10 +51371,10 @@
         <v>1.49</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>61.8</v>
+        <v>60.6</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>38.2</v>
+        <v>39.4</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52129,13 +52135,13 @@
         </is>
       </c>
       <c r="I480" s="4" t="n">
-        <v>1.65</v>
+        <v>1.75</v>
       </c>
       <c r="J480" s="4" t="n">
-        <v>61.7</v>
+        <v>62.4</v>
       </c>
       <c r="K480" s="4" t="n">
-        <v>38.3</v>
+        <v>37.6</v>
       </c>
       <c r="L480" t="inlineStr">
         <is>
@@ -52161,16 +52167,16 @@
         <v>-13.45</v>
       </c>
       <c r="S480" s="4" t="n">
-        <v>46.22</v>
+        <v>46.25</v>
       </c>
       <c r="T480" s="4" t="n">
-        <v>43.93</v>
+        <v>44.05</v>
       </c>
       <c r="U480" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="V480" s="4" t="n">
-        <v>3.56</v>
+        <v>3.5</v>
       </c>
       <c r="W480" s="5" t="n">
         <v>6276527</v>
@@ -52195,10 +52201,10 @@
         <v>0</v>
       </c>
       <c r="AC480" s="4" t="n">
-        <v>50.57</v>
+        <v>50.62</v>
       </c>
       <c r="AD480" s="4" t="n">
-        <v>48.93</v>
+        <v>48.88</v>
       </c>
       <c r="AE480" s="4" t="n">
         <v>0</v>
@@ -52925,10 +52931,10 @@
         <v>2.05</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>64.09999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>35.9</v>
+        <v>35.5</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53370,7 +53376,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.38</v>
+        <v>-21.41</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53430,16 +53436,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.82</v>
+        <v>27.8</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.32</v>
+        <v>19.33</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.2</v>
+        <v>49.21</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -53483,13 +53489,13 @@
         </is>
       </c>
       <c r="I492" s="4" t="n">
-        <v>9.66</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J492" s="4" t="n">
-        <v>95</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="K492" s="4" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="L492" t="inlineStr">
         <is>
@@ -53515,16 +53521,16 @@
         <v>-3.27</v>
       </c>
       <c r="S492" s="4" t="n">
-        <v>50.93</v>
+        <v>50.73</v>
       </c>
       <c r="T492" s="4" t="n">
-        <v>40.02</v>
+        <v>39.82</v>
       </c>
       <c r="U492" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V492" s="4" t="n">
-        <v>11.86</v>
+        <v>11.84</v>
       </c>
       <c r="W492" s="5" t="n">
         <v>34975789</v>
@@ -53543,13 +53549,13 @@
         </is>
       </c>
       <c r="AA492" s="4" t="n">
-        <v>0.55</v>
+        <v>0.51</v>
       </c>
       <c r="AB492" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC492" s="4" t="n">
-        <v>53.5</v>
+        <v>53.54</v>
       </c>
       <c r="AD492" s="4" t="n">
         <v>44.08</v>
@@ -54274,7 +54280,7 @@
         </is>
       </c>
       <c r="I499" s="4" t="n">
-        <v>23.68</v>
+        <v>23.45</v>
       </c>
       <c r="J499" s="4" t="n">
         <v>99.90000000000001</v>
@@ -54288,13 +54294,13 @@
         </is>
       </c>
       <c r="M499" s="4" t="n">
-        <v>12.53</v>
+        <v>12.3</v>
       </c>
       <c r="N499" s="4" t="n">
         <v>6.77</v>
       </c>
       <c r="O499" s="4" t="n">
-        <v>22.98</v>
+        <v>22.75</v>
       </c>
       <c r="P499" s="4" t="n">
         <v>2.47</v>
@@ -54334,10 +54340,10 @@
         <v>0</v>
       </c>
       <c r="AC499" s="4" t="n">
-        <v>56.05</v>
+        <v>55.95</v>
       </c>
       <c r="AD499" s="4" t="n">
-        <v>34.59</v>
+        <v>34.69</v>
       </c>
       <c r="AE499" s="4" t="n">
         <v>4.68</v>
@@ -54619,13 +54625,13 @@
         </is>
       </c>
       <c r="I502" s="4" t="n">
-        <v>-15.24</v>
+        <v>-14.66</v>
       </c>
       <c r="J502" s="4" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K502" s="4" t="n">
-        <v>99.40000000000001</v>
+        <v>99.3</v>
       </c>
       <c r="L502" t="inlineStr">
         <is>
@@ -54651,16 +54657,16 @@
         <v>-29.98</v>
       </c>
       <c r="S502" s="4" t="n">
-        <v>41.27</v>
+        <v>42.84</v>
       </c>
       <c r="T502" s="4" t="n">
-        <v>46.07</v>
+        <v>47.96</v>
       </c>
       <c r="U502" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V502" s="4" t="n">
-        <v>-5.67</v>
+        <v>-6.58</v>
       </c>
       <c r="W502" s="5" t="n">
         <v>0</v>
@@ -54679,16 +54685,16 @@
         </is>
       </c>
       <c r="AA502" s="4" t="n">
-        <v>42.38</v>
+        <v>42.67</v>
       </c>
       <c r="AB502" s="4" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="AC502" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AD502" s="4" t="n">
-        <v>57.62</v>
+        <v>57.33</v>
       </c>
       <c r="AE502" s="4" t="n">
         <v>0</v>
@@ -59069,7 +59075,7 @@
         <v>47</v>
       </c>
       <c r="N65" s="4" t="n">
-        <v>97.2</v>
+        <v>97</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -59115,7 +59121,7 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="K66" t="n">
         <v>20</v>
@@ -59127,7 +59133,7 @@
         <v>22</v>
       </c>
       <c r="N66" s="4" t="n">
-        <v>97.90000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -59463,7 +59469,7 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="K72" t="n">
         <v>9</v>
@@ -60159,7 +60165,7 @@
         </is>
       </c>
       <c r="J84" s="4" t="n">
-        <v>51.5</v>
+        <v>51.4</v>
       </c>
       <c r="K84" t="n">
         <v>51</v>
@@ -60171,7 +60177,7 @@
         <v>67</v>
       </c>
       <c r="N84" s="4" t="n">
-        <v>57</v>
+        <v>56.5</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -60217,7 +60223,7 @@
         </is>
       </c>
       <c r="J85" s="4" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="K85" t="n">
         <v>18</v>
@@ -60226,10 +60232,10 @@
         <v>14</v>
       </c>
       <c r="M85" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N85" s="4" t="n">
-        <v>70.90000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-10-02 (rerun: new polls)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>68.7</v>
+        <v>68.5</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241.3</v>
+        <v>241.7</v>
       </c>
       <c r="C9" t="n">
-        <v>193.7</v>
+        <v>193.3</v>
       </c>
       <c r="D9" t="n">
         <v>237</v>
       </c>
       <c r="E9" t="n">
-        <v>88.40000000000001</v>
+        <v>88.5</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>69.3</v>
+        <v>69.2</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -3038,13 +3038,13 @@
         </is>
       </c>
       <c r="I21" s="4" t="n">
-        <v>-11.43</v>
+        <v>-10.47</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1.3</v>
+        <v>3</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>98.7</v>
+        <v>97</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -3070,16 +3070,16 @@
         <v>-20.84</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>35.5</v>
+        <v>35.68</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>43.36</v>
+        <v>43.26</v>
       </c>
       <c r="U21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>-7.72</v>
+        <v>-7.23</v>
       </c>
       <c r="W21" s="5" t="n">
         <v>0</v>
@@ -3098,16 +3098,16 @@
         </is>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>3.33</v>
+        <v>3.52</v>
       </c>
       <c r="AB21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>42.81</v>
+        <v>43.19</v>
       </c>
       <c r="AD21" s="4" t="n">
-        <v>53.86</v>
+        <v>53.29</v>
       </c>
       <c r="AE21" s="4" t="n">
         <v>0</v>
@@ -4948,10 +4948,10 @@
         <v>-2.4</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>32.7</v>
+        <v>33.3</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>67.3</v>
+        <v>66.7</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.42</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>32.7</v>
+        <v>33.3</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -23133,17 +23133,17 @@
         </is>
       </c>
       <c r="I210" s="4" t="n">
-        <v>-4.06</v>
+        <v>-2.42</v>
       </c>
       <c r="J210" s="4" t="n">
-        <v>22.5</v>
+        <v>33</v>
       </c>
       <c r="K210" s="4" t="n">
-        <v>77.5</v>
+        <v>67</v>
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M210" s="4" t="n">
@@ -23165,16 +23165,16 @@
         <v>-15.31</v>
       </c>
       <c r="S210" s="4" t="n">
-        <v>44.91</v>
+        <v>42.78</v>
       </c>
       <c r="T210" s="4" t="n">
-        <v>44.86</v>
+        <v>39.1</v>
       </c>
       <c r="U210" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V210" s="4" t="n">
-        <v>-1.2</v>
+        <v>1.15</v>
       </c>
       <c r="W210" s="5" t="n">
         <v>1463855</v>
@@ -23199,10 +23199,10 @@
         <v>0</v>
       </c>
       <c r="AC210" s="4" t="n">
-        <v>46.74</v>
+        <v>47.54</v>
       </c>
       <c r="AD210" s="4" t="n">
-        <v>50.7</v>
+        <v>49.9</v>
       </c>
       <c r="AE210" s="4" t="n">
         <v>0</v>
@@ -25781,10 +25781,10 @@
         <v>-0.34</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.2</v>
+        <v>47.4</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.8</v>
+        <v>52.6</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -31411,13 +31411,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-6.35</v>
+        <v>-6.2</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>14.6</v>
+        <v>15.1</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>85.40000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -31425,13 +31425,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-10.85</v>
+        <v>-10.61</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.6</v>
+        <v>-10.36</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -31477,10 +31477,10 @@
         <v>0</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>44.57</v>
+        <v>44.64</v>
       </c>
       <c r="AD286" s="4" t="n">
-        <v>50.61</v>
+        <v>50.54</v>
       </c>
       <c r="AE286" s="4" t="n">
         <v>2.41</v>
@@ -31524,13 +31524,13 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>10.52</v>
+        <v>10.66</v>
       </c>
       <c r="J287" s="4" t="n">
-        <v>97.09999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="K287" s="4" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -31538,13 +31538,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>7.01</v>
+        <v>7.25</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>13.92</v>
+        <v>14.16</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.53</v>
@@ -31590,10 +31590,10 @@
         <v>0</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>54.07</v>
+        <v>54.13</v>
       </c>
       <c r="AD287" s="4" t="n">
-        <v>43.77</v>
+        <v>43.71</v>
       </c>
       <c r="AE287" s="4" t="n">
         <v>0</v>
@@ -31641,7 +31641,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-53.34</v>
+        <v>-53.1</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -31655,13 +31655,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-51.8</v>
+        <v>-51.56</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-53.15</v>
+        <v>-52.91</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -31701,10 +31701,10 @@
         <v>0</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>22.4</v>
+        <v>22.52</v>
       </c>
       <c r="AD288" s="4" t="n">
-        <v>73.64</v>
+        <v>73.52</v>
       </c>
       <c r="AE288" s="4" t="n">
         <v>1.98</v>
@@ -41556,13 +41556,13 @@
         </is>
       </c>
       <c r="I381" s="4" t="n">
-        <v>-1.5</v>
+        <v>-1.56</v>
       </c>
       <c r="J381" s="4" t="n">
-        <v>39.4</v>
+        <v>38.9</v>
       </c>
       <c r="K381" s="4" t="n">
-        <v>60.6</v>
+        <v>61.1</v>
       </c>
       <c r="L381" t="inlineStr">
         <is>
@@ -41588,16 +41588,16 @@
         <v>-13.29</v>
       </c>
       <c r="S381" s="4" t="n">
-        <v>40.06</v>
+        <v>40.04</v>
       </c>
       <c r="T381" s="4" t="n">
-        <v>41.08</v>
+        <v>42.96</v>
       </c>
       <c r="U381" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V381" s="4" t="n">
-        <v>-3.03</v>
+        <v>-3.02</v>
       </c>
       <c r="W381" s="5" t="n">
         <v>2279585</v>
@@ -41616,16 +41616,16 @@
         </is>
       </c>
       <c r="AA381" s="4" t="n">
-        <v>0.5</v>
+        <v>1.55</v>
       </c>
       <c r="AB381" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC381" s="4" t="n">
-        <v>49</v>
+        <v>48.46</v>
       </c>
       <c r="AD381" s="4" t="n">
-        <v>50.5</v>
+        <v>49.99</v>
       </c>
       <c r="AE381" s="4" t="n">
         <v>0</v>
@@ -51401,10 +51401,10 @@
         <v>1.45</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>60.4</v>
+        <v>60.8</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>39.6</v>
+        <v>39.2</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52961,10 +52961,10 @@
         <v>2.12</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>63.3</v>
+        <v>64.3</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>36.7</v>
+        <v>35.7</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53406,7 +53406,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.54</v>
+        <v>-21.56</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53466,16 +53466,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.78</v>
+        <v>27.75</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.24</v>
+        <v>19.28</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.32</v>
+        <v>49.31</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -53636,13 +53636,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-1.07</v>
+        <v>-0.72</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>42.2</v>
+        <v>44.8</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>57.8</v>
+        <v>55.2</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -53650,13 +53650,13 @@
         </is>
       </c>
       <c r="M493" s="4" t="n">
-        <v>-18.56</v>
+        <v>-18.32</v>
       </c>
       <c r="N493" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O493" s="4" t="n">
-        <v>-4.01</v>
+        <v>-3.77</v>
       </c>
       <c r="P493" s="4" t="n">
         <v>-0.35</v>
@@ -53668,16 +53668,16 @@
         <v>-20.84</v>
       </c>
       <c r="S493" s="4" t="n">
-        <v>46.59</v>
+        <v>45.97</v>
       </c>
       <c r="T493" s="4" t="n">
-        <v>44.84</v>
+        <v>44.93</v>
       </c>
       <c r="U493" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V493" s="4" t="n">
-        <v>2.01</v>
+        <v>1.67</v>
       </c>
       <c r="W493" s="5" t="n">
         <v>0</v>
@@ -53696,16 +53696,16 @@
         </is>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>48.38</v>
+        <v>48.55</v>
       </c>
       <c r="AB493" s="4" t="n">
-        <v>42.2</v>
+        <v>44.8</v>
       </c>
       <c r="AC493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AD493" s="4" t="n">
-        <v>49.44</v>
+        <v>49.27</v>
       </c>
       <c r="AE493" s="4" t="n">
         <v>2.18</v>
@@ -58400,7 +58400,7 @@
         <v>18.6</v>
       </c>
       <c r="K53" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L53" t="n">
         <v>15</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-02 (rerun: race polls match the nominee, not a namesake — NH-SEN, SC-SEN, NM-SEN)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>68.5</v>
+        <v>68.2</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>237</v>
       </c>
       <c r="E9" t="n">
-        <v>88.5</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.9</v>
+        <v>26.8</v>
       </c>
       <c r="C10" t="n">
-        <v>23.1</v>
+        <v>23.2</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>69.2</v>
+        <v>69</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4948,10 +4948,10 @@
         <v>-2.4</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>33.3</v>
+        <v>32.7</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>66.7</v>
+        <v>67.3</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.42</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>33.3</v>
+        <v>32.7</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25781,10 +25781,10 @@
         <v>-0.34</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.4</v>
+        <v>48.2</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.6</v>
+        <v>51.8</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -31748,13 +31748,13 @@
         </is>
       </c>
       <c r="I289" s="4" t="n">
-        <v>5.76</v>
+        <v>5.75</v>
       </c>
       <c r="J289" s="4" t="n">
-        <v>83.5</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="K289" s="4" t="n">
-        <v>16.5</v>
+        <v>16.6</v>
       </c>
       <c r="L289" t="inlineStr">
         <is>
@@ -31762,7 +31762,7 @@
         </is>
       </c>
       <c r="M289" s="4" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="N289" s="4" t="n">
         <v>6.74</v>
@@ -31857,7 +31857,7 @@
         </is>
       </c>
       <c r="I290" s="4" t="n">
-        <v>17.98</v>
+        <v>17.97</v>
       </c>
       <c r="J290" s="4" t="n">
         <v>99.59999999999999</v>
@@ -31871,13 +31871,13 @@
         </is>
       </c>
       <c r="M290" s="4" t="n">
-        <v>3.1</v>
+        <v>3.09</v>
       </c>
       <c r="N290" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O290" s="4" t="n">
-        <v>16.83</v>
+        <v>16.82</v>
       </c>
       <c r="P290" s="4" t="n">
         <v>0.92</v>
@@ -33282,7 +33282,7 @@
         </is>
       </c>
       <c r="I303" s="4" t="n">
-        <v>28.9</v>
+        <v>28.58</v>
       </c>
       <c r="J303" s="4" t="n">
         <v>100</v>
@@ -33296,13 +33296,13 @@
         </is>
       </c>
       <c r="M303" s="4" t="n">
-        <v>17.28</v>
+        <v>16.96</v>
       </c>
       <c r="N303" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O303" s="4" t="n">
-        <v>28.9</v>
+        <v>28.58</v>
       </c>
       <c r="P303" s="4" t="n">
         <v>1.68</v>
@@ -33334,10 +33334,10 @@
         <v>0</v>
       </c>
       <c r="AC303" s="4" t="n">
-        <v>64.45</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="AD303" s="4" t="n">
-        <v>35.55</v>
+        <v>35.71</v>
       </c>
       <c r="AE303" s="4" t="n">
         <v>0</v>
@@ -33385,7 +33385,7 @@
         </is>
       </c>
       <c r="I304" s="4" t="n">
-        <v>14.85</v>
+        <v>14.62</v>
       </c>
       <c r="J304" s="4" t="n">
         <v>99.3</v>
@@ -33399,13 +33399,13 @@
         </is>
       </c>
       <c r="M304" s="4" t="n">
-        <v>4.43</v>
+        <v>4.11</v>
       </c>
       <c r="N304" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O304" s="4" t="n">
-        <v>19.25</v>
+        <v>18.93</v>
       </c>
       <c r="P304" s="4" t="n">
         <v>0.62</v>
@@ -33443,10 +33443,10 @@
         <v>0</v>
       </c>
       <c r="AC304" s="4" t="n">
-        <v>57.42</v>
+        <v>57.31</v>
       </c>
       <c r="AD304" s="4" t="n">
-        <v>42.58</v>
+        <v>42.69</v>
       </c>
       <c r="AE304" s="4" t="n">
         <v>0</v>
@@ -33494,13 +33494,13 @@
         </is>
       </c>
       <c r="I305" s="4" t="n">
-        <v>25.91</v>
+        <v>25.59</v>
       </c>
       <c r="J305" s="4" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="K305" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L305" t="inlineStr">
         <is>
@@ -33508,13 +33508,13 @@
         </is>
       </c>
       <c r="M305" s="4" t="n">
-        <v>11.03</v>
+        <v>10.71</v>
       </c>
       <c r="N305" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O305" s="4" t="n">
-        <v>25.91</v>
+        <v>25.59</v>
       </c>
       <c r="P305" s="4" t="n">
         <v>0.73</v>
@@ -33546,10 +33546,10 @@
         <v>0</v>
       </c>
       <c r="AC305" s="4" t="n">
-        <v>62.96</v>
+        <v>62.8</v>
       </c>
       <c r="AD305" s="4" t="n">
-        <v>37.04</v>
+        <v>37.2</v>
       </c>
       <c r="AE305" s="4" t="n">
         <v>0</v>
@@ -41556,13 +41556,13 @@
         </is>
       </c>
       <c r="I381" s="4" t="n">
-        <v>-1.56</v>
+        <v>-1.54</v>
       </c>
       <c r="J381" s="4" t="n">
-        <v>38.9</v>
+        <v>39.1</v>
       </c>
       <c r="K381" s="4" t="n">
-        <v>61.1</v>
+        <v>60.9</v>
       </c>
       <c r="L381" t="inlineStr">
         <is>
@@ -41570,13 +41570,13 @@
         </is>
       </c>
       <c r="M381" s="4" t="n">
-        <v>-7.66</v>
+        <v>-7.61</v>
       </c>
       <c r="N381" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O381" s="4" t="n">
-        <v>-0.9</v>
+        <v>-0.85</v>
       </c>
       <c r="P381" s="4" t="n">
         <v>0.47</v>
@@ -41622,10 +41622,10 @@
         <v>0</v>
       </c>
       <c r="AC381" s="4" t="n">
-        <v>48.46</v>
+        <v>48.47</v>
       </c>
       <c r="AD381" s="4" t="n">
-        <v>49.99</v>
+        <v>49.98</v>
       </c>
       <c r="AE381" s="4" t="n">
         <v>0</v>
@@ -41673,13 +41673,13 @@
         </is>
       </c>
       <c r="I382" s="4" t="n">
-        <v>-8.93</v>
+        <v>-8.880000000000001</v>
       </c>
       <c r="J382" s="4" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="K382" s="4" t="n">
-        <v>93.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L382" t="inlineStr">
         <is>
@@ -41687,13 +41687,13 @@
         </is>
       </c>
       <c r="M382" s="4" t="n">
-        <v>-8.84</v>
+        <v>-8.789999999999999</v>
       </c>
       <c r="N382" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O382" s="4" t="n">
-        <v>-8.82</v>
+        <v>-8.77</v>
       </c>
       <c r="P382" s="4" t="n">
         <v>-1.93</v>
@@ -41733,10 +41733,10 @@
         <v>0</v>
       </c>
       <c r="AC382" s="4" t="n">
-        <v>44.61</v>
+        <v>44.63</v>
       </c>
       <c r="AD382" s="4" t="n">
-        <v>53.35</v>
+        <v>53.33</v>
       </c>
       <c r="AE382" s="4" t="n">
         <v>0</v>
@@ -41784,7 +41784,7 @@
         </is>
       </c>
       <c r="I383" s="4" t="n">
-        <v>-38.56</v>
+        <v>-38.51</v>
       </c>
       <c r="J383" s="4" t="n">
         <v>0</v>
@@ -41798,13 +41798,13 @@
         </is>
       </c>
       <c r="M383" s="4" t="n">
-        <v>-37.3</v>
+        <v>-37.25</v>
       </c>
       <c r="N383" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O383" s="4" t="n">
-        <v>-38.9</v>
+        <v>-38.85</v>
       </c>
       <c r="P383" s="4" t="n">
         <v>-1.36</v>
@@ -41844,10 +41844,10 @@
         <v>0</v>
       </c>
       <c r="AC383" s="4" t="n">
-        <v>30.19</v>
+        <v>30.22</v>
       </c>
       <c r="AD383" s="4" t="n">
-        <v>68.09999999999999</v>
+        <v>68.06999999999999</v>
       </c>
       <c r="AE383" s="4" t="n">
         <v>0</v>
@@ -41895,7 +41895,7 @@
         </is>
       </c>
       <c r="I384" s="4" t="n">
-        <v>-14.9</v>
+        <v>-14.85</v>
       </c>
       <c r="J384" s="4" t="n">
         <v>0.7</v>
@@ -41909,13 +41909,13 @@
         </is>
       </c>
       <c r="M384" s="4" t="n">
-        <v>-18.15</v>
+        <v>-18.1</v>
       </c>
       <c r="N384" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O384" s="4" t="n">
-        <v>-15.35</v>
+        <v>-15.3</v>
       </c>
       <c r="P384" s="4" t="n">
         <v>-2.31</v>
@@ -41955,10 +41955,10 @@
         <v>0</v>
       </c>
       <c r="AC384" s="4" t="n">
-        <v>41.6</v>
+        <v>41.62</v>
       </c>
       <c r="AD384" s="4" t="n">
-        <v>56.16</v>
+        <v>56.14</v>
       </c>
       <c r="AE384" s="4" t="n">
         <v>0</v>
@@ -42002,7 +42002,7 @@
         </is>
       </c>
       <c r="I385" s="4" t="n">
-        <v>-12.05</v>
+        <v>-12</v>
       </c>
       <c r="J385" s="4" t="n">
         <v>1.1</v>
@@ -42016,13 +42016,13 @@
         </is>
       </c>
       <c r="M385" s="4" t="n">
-        <v>-17.12</v>
+        <v>-17.07</v>
       </c>
       <c r="N385" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O385" s="4" t="n">
-        <v>-12.05</v>
+        <v>-12</v>
       </c>
       <c r="P385" s="4" t="n">
         <v>-1.2</v>
@@ -42054,10 +42054,10 @@
         <v>0</v>
       </c>
       <c r="AC385" s="4" t="n">
-        <v>43.98</v>
+        <v>44</v>
       </c>
       <c r="AD385" s="4" t="n">
-        <v>56.02</v>
+        <v>56</v>
       </c>
       <c r="AE385" s="4" t="n">
         <v>0</v>
@@ -42105,7 +42105,7 @@
         </is>
       </c>
       <c r="I386" s="4" t="n">
-        <v>38.86</v>
+        <v>38.91</v>
       </c>
       <c r="J386" s="4" t="n">
         <v>100</v>
@@ -42119,13 +42119,13 @@
         </is>
       </c>
       <c r="M386" s="4" t="n">
-        <v>30.61</v>
+        <v>30.66</v>
       </c>
       <c r="N386" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O386" s="4" t="n">
-        <v>38.86</v>
+        <v>38.91</v>
       </c>
       <c r="P386" s="4" t="n">
         <v>0</v>
@@ -42157,10 +42157,10 @@
         <v>0</v>
       </c>
       <c r="AC386" s="4" t="n">
-        <v>69.43000000000001</v>
+        <v>69.45</v>
       </c>
       <c r="AD386" s="4" t="n">
-        <v>30.57</v>
+        <v>30.55</v>
       </c>
       <c r="AE386" s="4" t="n">
         <v>0</v>
@@ -42208,7 +42208,7 @@
         </is>
       </c>
       <c r="I387" s="4" t="n">
-        <v>-16.08</v>
+        <v>-16.04</v>
       </c>
       <c r="J387" s="4" t="n">
         <v>0.5</v>
@@ -42222,13 +42222,13 @@
         </is>
       </c>
       <c r="M387" s="4" t="n">
-        <v>-19.72</v>
+        <v>-19.67</v>
       </c>
       <c r="N387" s="4" t="n">
         <v>6.74</v>
       </c>
       <c r="O387" s="4" t="n">
-        <v>-18.8</v>
+        <v>-18.75</v>
       </c>
       <c r="P387" s="4" t="n">
         <v>-1.22</v>
@@ -42266,10 +42266,10 @@
         <v>0</v>
       </c>
       <c r="AC387" s="4" t="n">
-        <v>41.96</v>
+        <v>41.98</v>
       </c>
       <c r="AD387" s="4" t="n">
-        <v>58.04</v>
+        <v>58.02</v>
       </c>
       <c r="AE387" s="4" t="n">
         <v>0</v>
@@ -51401,10 +51401,10 @@
         <v>1.45</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>60.8</v>
+        <v>61.3</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>39.2</v>
+        <v>38.7</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52961,10 +52961,10 @@
         <v>2.12</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>64.3</v>
+        <v>64.7</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>35.7</v>
+        <v>35.3</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53406,7 +53406,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.56</v>
+        <v>-21.55</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53466,13 +53466,13 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.75</v>
+        <v>27.76</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.28</v>
+        <v>19.26</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>49.31</v>
@@ -53749,13 +53749,13 @@
         </is>
       </c>
       <c r="I494" s="4" t="n">
-        <v>8.220000000000001</v>
+        <v>8.18</v>
       </c>
       <c r="J494" s="4" t="n">
-        <v>91.09999999999999</v>
+        <v>91</v>
       </c>
       <c r="K494" s="4" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="L494" t="inlineStr">
         <is>
@@ -53781,13 +53781,13 @@
         <v>2.82</v>
       </c>
       <c r="S494" s="4" t="n">
-        <v>48.4</v>
+        <v>48.41</v>
       </c>
       <c r="T494" s="4" t="n">
         <v>43.57</v>
       </c>
       <c r="U494" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="V494" s="4" t="n">
         <v>5.74</v>
@@ -53815,10 +53815,10 @@
         <v>0</v>
       </c>
       <c r="AC494" s="4" t="n">
-        <v>53.84</v>
+        <v>53.82</v>
       </c>
       <c r="AD494" s="4" t="n">
-        <v>45.66</v>
+        <v>45.68</v>
       </c>
       <c r="AE494" s="4" t="n">
         <v>0</v>
@@ -53977,7 +53977,7 @@
         </is>
       </c>
       <c r="I496" s="4" t="n">
-        <v>21.39</v>
+        <v>19.79</v>
       </c>
       <c r="J496" s="4" t="n">
         <v>99.8</v>
@@ -54008,12 +54008,18 @@
       <c r="R496" s="4" t="n">
         <v>6.14</v>
       </c>
-      <c r="S496" s="4" t="n"/>
-      <c r="T496" s="4" t="n"/>
+      <c r="S496" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="T496" s="4" t="n">
+        <v>38</v>
+      </c>
       <c r="U496" t="n">
-        <v>0</v>
-      </c>
-      <c r="V496" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V496" s="4" t="n">
+        <v>16.45</v>
+      </c>
       <c r="W496" s="5" t="n">
         <v>5626629</v>
       </c>
@@ -54029,10 +54035,10 @@
         <v>0</v>
       </c>
       <c r="AC496" s="4" t="n">
-        <v>60.69</v>
+        <v>59.9</v>
       </c>
       <c r="AD496" s="4" t="n">
-        <v>39.31</v>
+        <v>40.1</v>
       </c>
       <c r="AE496" s="4" t="n">
         <v>0</v>
@@ -54538,13 +54544,13 @@
         </is>
       </c>
       <c r="I501" s="4" t="n">
-        <v>-2.92</v>
+        <v>-2.66</v>
       </c>
       <c r="J501" s="4" t="n">
-        <v>29.6</v>
+        <v>31.3</v>
       </c>
       <c r="K501" s="4" t="n">
-        <v>70.40000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="L501" t="inlineStr">
         <is>
@@ -54570,16 +54576,16 @@
         <v>-18.12</v>
       </c>
       <c r="S501" s="4" t="n">
-        <v>40.14</v>
+        <v>39.96</v>
       </c>
       <c r="T501" s="4" t="n">
-        <v>42.99</v>
+        <v>42.79</v>
       </c>
       <c r="U501" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V501" s="4" t="n">
-        <v>-1.18</v>
+        <v>-1.05</v>
       </c>
       <c r="W501" s="5" t="n">
         <v>10804040</v>
@@ -54598,16 +54604,16 @@
         </is>
       </c>
       <c r="AA501" s="4" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AB501" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC501" s="4" t="n">
-        <v>47.04</v>
+        <v>47.14</v>
       </c>
       <c r="AD501" s="4" t="n">
-        <v>49.87</v>
+        <v>49.72</v>
       </c>
       <c r="AE501" s="4" t="n">
         <v>1.87</v>
@@ -58455,10 +58461,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>223.5</v>
+        <v>223.4</v>
       </c>
       <c r="K54" t="n">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="L54" t="n">
         <v>143</v>
@@ -58571,7 +58577,7 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
       <c r="K56" t="n">
         <v>47</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-03 (rerun: NYT/Siena governor polls — TX, AK, OH, IA, KS)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
       <c r="C8" t="n">
-        <v>47.6</v>
+        <v>47.7</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>69.8</v>
+        <v>69.7</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241.3</v>
+        <v>241.4</v>
       </c>
       <c r="C9" t="n">
-        <v>193.7</v>
+        <v>193.6</v>
       </c>
       <c r="D9" t="n">
         <v>237</v>
       </c>
       <c r="E9" t="n">
-        <v>88.5</v>
+        <v>88.2</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -925,13 +925,13 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>15.81</v>
+        <v>17.98</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>99.59999999999999</v>
+        <v>99.8</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -957,16 +957,16 @@
         <v>-13.8</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>40.58</v>
+        <v>50.22</v>
       </c>
       <c r="T2" s="4" t="n">
-        <v>41.38</v>
+        <v>46.97</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.61</v>
+        <v>3.47</v>
       </c>
       <c r="W2" s="5" t="n">
         <v>0</v>
@@ -983,10 +983,10 @@
         <v>0</v>
       </c>
       <c r="AC2" s="4" t="n">
-        <v>48.21</v>
+        <v>49.46</v>
       </c>
       <c r="AD2" s="4" t="n">
-        <v>51.79</v>
+        <v>50.54</v>
       </c>
       <c r="AE2" s="4" t="n">
         <v>0</v>
@@ -2017,13 +2017,13 @@
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>8.859999999999999</v>
+        <v>9.02</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2049,16 +2049,16 @@
         <v>-13.45</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>51.58</v>
+        <v>51.65</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>42.26</v>
+        <v>42.07</v>
       </c>
       <c r="U12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>10.15</v>
+        <v>10.28</v>
       </c>
       <c r="W12" s="5" t="n">
         <v>19860206</v>
@@ -2075,10 +2075,10 @@
         <v>0</v>
       </c>
       <c r="AC12" s="4" t="n">
-        <v>54.43</v>
+        <v>54.51</v>
       </c>
       <c r="AD12" s="4" t="n">
-        <v>45.57</v>
+        <v>45.49</v>
       </c>
       <c r="AE12" s="4" t="n">
         <v>0</v>
@@ -2356,13 +2356,13 @@
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>-7.09</v>
+        <v>-6.85</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>12.2</v>
+        <v>13</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>87.8</v>
+        <v>87</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -2388,16 +2388,16 @@
         <v>-16.41</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>45.06</v>
+        <v>44.5</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>50.2</v>
+        <v>49.56</v>
       </c>
       <c r="U15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>-4.96</v>
+        <v>-4.98</v>
       </c>
       <c r="W15" s="5" t="n">
         <v>0</v>
@@ -2414,10 +2414,10 @@
         <v>0</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>46.45</v>
+        <v>46.57</v>
       </c>
       <c r="AD15" s="4" t="n">
-        <v>53.55</v>
+        <v>53.43</v>
       </c>
       <c r="AE15" s="4" t="n">
         <v>0</v>
@@ -3599,13 +3599,13 @@
         </is>
       </c>
       <c r="I26" s="4" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>50.9</v>
+        <v>51.1</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>49.1</v>
+        <v>48.9</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -3631,16 +3631,16 @@
         <v>-11.31</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>49.05</v>
+        <v>49.03</v>
       </c>
       <c r="T26" s="4" t="n">
-        <v>45.08</v>
+        <v>45.06</v>
       </c>
       <c r="U26" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>4.56</v>
+        <v>4.39</v>
       </c>
       <c r="W26" s="5" t="n">
         <v>15928993</v>
@@ -3659,16 +3659,16 @@
         </is>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>1.06</v>
+        <v>0.73</v>
       </c>
       <c r="AB26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC26" s="4" t="n">
-        <v>49.53</v>
+        <v>49.71</v>
       </c>
       <c r="AD26" s="4" t="n">
-        <v>49.41</v>
+        <v>49.56</v>
       </c>
       <c r="AE26" s="4" t="n">
         <v>0</v>
@@ -4499,13 +4499,13 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>-4.38</v>
+        <v>-3.93</v>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21.3</v>
+        <v>23</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>78.7</v>
+        <v>77</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -4531,16 +4531,16 @@
         <v>-13.88</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>46.44</v>
+        <v>46.8</v>
       </c>
       <c r="T34" s="4" t="n">
-        <v>48.78</v>
+        <v>48.39</v>
       </c>
       <c r="U34" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="V34" s="4" t="n">
-        <v>-1.57</v>
+        <v>-0.93</v>
       </c>
       <c r="W34" s="5" t="n">
         <v>8433631</v>
@@ -4559,16 +4559,16 @@
         </is>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="AB34" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC34" s="4" t="n">
-        <v>47.54</v>
+        <v>47.8</v>
       </c>
       <c r="AD34" s="4" t="n">
-        <v>51.9</v>
+        <v>51.7</v>
       </c>
       <c r="AE34" s="4" t="n">
         <v>0</v>
@@ -4945,13 +4945,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.29</v>
+        <v>-3.03</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>26.4</v>
+        <v>27.9</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>73.59999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4959,13 +4959,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.04</v>
+        <v>-1.49</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>1.27</v>
+        <v>1.82</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-0.72</v>
@@ -5005,16 +5005,16 @@
         </is>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>45.05</v>
+        <v>45.18</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>26.4</v>
+        <v>27.9</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
       </c>
       <c r="AD38" s="4" t="n">
-        <v>49.95</v>
+        <v>49.82</v>
       </c>
       <c r="AE38" s="4" t="n">
         <v>1.2</v>
@@ -18790,7 +18790,7 @@
         </is>
       </c>
       <c r="I169" s="4" t="n">
-        <v>14.07</v>
+        <v>14.09</v>
       </c>
       <c r="J169" s="4" t="n">
         <v>99.2</v>
@@ -18804,13 +18804,13 @@
         </is>
       </c>
       <c r="M169" s="4" t="n">
-        <v>0.39</v>
+        <v>0.42</v>
       </c>
       <c r="N169" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O169" s="4" t="n">
-        <v>16.58</v>
+        <v>16.62</v>
       </c>
       <c r="P169" s="4" t="n">
         <v>0.09</v>
@@ -18856,10 +18856,10 @@
         <v>0</v>
       </c>
       <c r="AC169" s="4" t="n">
-        <v>50.76</v>
+        <v>50.77</v>
       </c>
       <c r="AD169" s="4" t="n">
-        <v>38.24</v>
+        <v>38.23</v>
       </c>
       <c r="AE169" s="4" t="n">
         <v>0</v>
@@ -18903,13 +18903,13 @@
         </is>
       </c>
       <c r="I170" s="4" t="n">
-        <v>4.6</v>
+        <v>4.62</v>
       </c>
       <c r="J170" s="4" t="n">
-        <v>79.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="K170" s="4" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -18917,13 +18917,13 @@
         </is>
       </c>
       <c r="M170" s="4" t="n">
-        <v>-1.15</v>
+        <v>-1.12</v>
       </c>
       <c r="N170" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O170" s="4" t="n">
-        <v>4.88</v>
+        <v>4.91</v>
       </c>
       <c r="P170" s="4" t="n">
         <v>0.11</v>
@@ -18969,10 +18969,10 @@
         <v>0</v>
       </c>
       <c r="AC170" s="4" t="n">
-        <v>49.55</v>
+        <v>49.56</v>
       </c>
       <c r="AD170" s="4" t="n">
-        <v>45.19</v>
+        <v>45.18</v>
       </c>
       <c r="AE170" s="4" t="n">
         <v>2.63</v>
@@ -19020,13 +19020,13 @@
         </is>
       </c>
       <c r="I171" s="4" t="n">
-        <v>7.75</v>
+        <v>7.78</v>
       </c>
       <c r="J171" s="4" t="n">
-        <v>89.8</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="K171" s="4" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="L171" t="inlineStr">
         <is>
@@ -19034,13 +19034,13 @@
         </is>
       </c>
       <c r="M171" s="4" t="n">
-        <v>3.94</v>
+        <v>3.97</v>
       </c>
       <c r="N171" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O171" s="4" t="n">
-        <v>9.16</v>
+        <v>9.19</v>
       </c>
       <c r="P171" s="4" t="n">
         <v>0.14</v>
@@ -19078,10 +19078,10 @@
         <v>0</v>
       </c>
       <c r="AC171" s="4" t="n">
-        <v>53.88</v>
+        <v>53.89</v>
       </c>
       <c r="AD171" s="4" t="n">
-        <v>46.12</v>
+        <v>46.11</v>
       </c>
       <c r="AE171" s="4" t="n">
         <v>0</v>
@@ -19125,7 +19125,7 @@
         </is>
       </c>
       <c r="I172" s="4" t="n">
-        <v>-18.09</v>
+        <v>-18.05</v>
       </c>
       <c r="J172" s="4" t="n">
         <v>0.4</v>
@@ -19139,13 +19139,13 @@
         </is>
       </c>
       <c r="M172" s="4" t="n">
-        <v>-23.13</v>
+        <v>-23.1</v>
       </c>
       <c r="N172" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O172" s="4" t="n">
-        <v>-18.09</v>
+        <v>-18.05</v>
       </c>
       <c r="P172" s="4" t="n">
         <v>-1.08</v>
@@ -19177,10 +19177,10 @@
         <v>0</v>
       </c>
       <c r="AC172" s="4" t="n">
-        <v>40.96</v>
+        <v>40.97</v>
       </c>
       <c r="AD172" s="4" t="n">
-        <v>59.04</v>
+        <v>59.03</v>
       </c>
       <c r="AE172" s="4" t="n">
         <v>0</v>
@@ -22158,7 +22158,7 @@
         </is>
       </c>
       <c r="I201" s="4" t="n">
-        <v>-27.54</v>
+        <v>-27.49</v>
       </c>
       <c r="J201" s="4" t="n">
         <v>0</v>
@@ -22172,13 +22172,13 @@
         </is>
       </c>
       <c r="M201" s="4" t="n">
-        <v>-27.02</v>
+        <v>-26.96</v>
       </c>
       <c r="N201" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O201" s="4" t="n">
-        <v>-28.08</v>
+        <v>-28.03</v>
       </c>
       <c r="P201" s="4" t="n">
         <v>-2.06</v>
@@ -22218,10 +22218,10 @@
         <v>0</v>
       </c>
       <c r="AC201" s="4" t="n">
-        <v>35.26</v>
+        <v>35.28</v>
       </c>
       <c r="AD201" s="4" t="n">
-        <v>62.06</v>
+        <v>62.04</v>
       </c>
       <c r="AE201" s="4" t="n">
         <v>0</v>
@@ -22269,7 +22269,7 @@
         </is>
       </c>
       <c r="I202" s="4" t="n">
-        <v>-13.33</v>
+        <v>-13.28</v>
       </c>
       <c r="J202" s="4" t="n">
         <v>0.9</v>
@@ -22283,13 +22283,13 @@
         </is>
       </c>
       <c r="M202" s="4" t="n">
-        <v>-14.59</v>
+        <v>-14.54</v>
       </c>
       <c r="N202" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O202" s="4" t="n">
-        <v>-13.9</v>
+        <v>-13.84</v>
       </c>
       <c r="P202" s="4" t="n">
         <v>-0.47</v>
@@ -22329,10 +22329,10 @@
         <v>0</v>
       </c>
       <c r="AC202" s="4" t="n">
-        <v>42.11</v>
+        <v>42.13</v>
       </c>
       <c r="AD202" s="4" t="n">
-        <v>55.05</v>
+        <v>55.03</v>
       </c>
       <c r="AE202" s="4" t="n">
         <v>0</v>
@@ -22380,7 +22380,7 @@
         </is>
       </c>
       <c r="I203" s="4" t="n">
-        <v>25.46</v>
+        <v>25.51</v>
       </c>
       <c r="J203" s="4" t="n">
         <v>99.90000000000001</v>
@@ -22394,13 +22394,13 @@
         </is>
       </c>
       <c r="M203" s="4" t="n">
-        <v>8.380000000000001</v>
+        <v>8.44</v>
       </c>
       <c r="N203" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O203" s="4" t="n">
-        <v>24.87</v>
+        <v>24.92</v>
       </c>
       <c r="P203" s="4" t="n">
         <v>3</v>
@@ -22440,10 +22440,10 @@
         <v>0</v>
       </c>
       <c r="AC203" s="4" t="n">
-        <v>60.89</v>
+        <v>60.91</v>
       </c>
       <c r="AD203" s="4" t="n">
-        <v>36.17</v>
+        <v>36.15</v>
       </c>
       <c r="AE203" s="4" t="n">
         <v>0</v>
@@ -22491,7 +22491,7 @@
         </is>
       </c>
       <c r="I204" s="4" t="n">
-        <v>-18.78</v>
+        <v>-18.73</v>
       </c>
       <c r="J204" s="4" t="n">
         <v>0.3</v>
@@ -22505,13 +22505,13 @@
         </is>
       </c>
       <c r="M204" s="4" t="n">
-        <v>-18.97</v>
+        <v>-18.92</v>
       </c>
       <c r="N204" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O204" s="4" t="n">
-        <v>-19.36</v>
+        <v>-19.3</v>
       </c>
       <c r="P204" s="4" t="n">
         <v>-1.43</v>
@@ -22551,10 +22551,10 @@
         <v>0</v>
       </c>
       <c r="AC204" s="4" t="n">
-        <v>39.44</v>
+        <v>39.47</v>
       </c>
       <c r="AD204" s="4" t="n">
-        <v>57.68</v>
+        <v>57.65</v>
       </c>
       <c r="AE204" s="4" t="n">
         <v>0</v>
@@ -25781,10 +25781,10 @@
         <v>-0.4</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.1</v>
+        <v>48.3</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.9</v>
+        <v>51.7</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -36789,7 +36789,7 @@
         <v>6.75</v>
       </c>
       <c r="O336" s="4" t="n">
-        <v>14.67</v>
+        <v>14.68</v>
       </c>
       <c r="P336" s="4" t="n">
         <v>0.72</v>
@@ -36886,7 +36886,7 @@
         </is>
       </c>
       <c r="I337" s="4" t="n">
-        <v>-33.23</v>
+        <v>-33.22</v>
       </c>
       <c r="J337" s="4" t="n">
         <v>0</v>
@@ -36900,13 +36900,13 @@
         </is>
       </c>
       <c r="M337" s="4" t="n">
-        <v>-36.38</v>
+        <v>-36.37</v>
       </c>
       <c r="N337" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O337" s="4" t="n">
-        <v>-33.23</v>
+        <v>-33.22</v>
       </c>
       <c r="P337" s="4" t="n">
         <v>0</v>
@@ -37003,7 +37003,7 @@
         </is>
       </c>
       <c r="M338" s="4" t="n">
-        <v>46.7</v>
+        <v>46.71</v>
       </c>
       <c r="N338" s="4" t="n">
         <v>6.75</v>
@@ -37041,10 +37041,10 @@
         <v>0</v>
       </c>
       <c r="AC338" s="4" t="n">
-        <v>77.83</v>
+        <v>77.84</v>
       </c>
       <c r="AD338" s="4" t="n">
-        <v>22.17</v>
+        <v>22.16</v>
       </c>
       <c r="AE338" s="4" t="n">
         <v>0</v>
@@ -37092,7 +37092,7 @@
         </is>
       </c>
       <c r="I339" s="4" t="n">
-        <v>-35.81</v>
+        <v>-35.8</v>
       </c>
       <c r="J339" s="4" t="n">
         <v>0</v>
@@ -37106,13 +37106,13 @@
         </is>
       </c>
       <c r="M339" s="4" t="n">
-        <v>-37.14</v>
+        <v>-37.13</v>
       </c>
       <c r="N339" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O339" s="4" t="n">
-        <v>-35.73</v>
+        <v>-35.72</v>
       </c>
       <c r="P339" s="4" t="n">
         <v>-3.26</v>
@@ -37203,7 +37203,7 @@
         </is>
       </c>
       <c r="I340" s="4" t="n">
-        <v>-19.02</v>
+        <v>-19.01</v>
       </c>
       <c r="J340" s="4" t="n">
         <v>0.3</v>
@@ -37314,7 +37314,7 @@
         </is>
       </c>
       <c r="I341" s="4" t="n">
-        <v>-25.71</v>
+        <v>-25.7</v>
       </c>
       <c r="J341" s="4" t="n">
         <v>0.1</v>
@@ -37328,13 +37328,13 @@
         </is>
       </c>
       <c r="M341" s="4" t="n">
-        <v>-28.05</v>
+        <v>-28.04</v>
       </c>
       <c r="N341" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O341" s="4" t="n">
-        <v>-25.71</v>
+        <v>-25.7</v>
       </c>
       <c r="P341" s="4" t="n">
         <v>-2.34</v>
@@ -37431,7 +37431,7 @@
         </is>
       </c>
       <c r="M342" s="4" t="n">
-        <v>-5.58</v>
+        <v>-5.57</v>
       </c>
       <c r="N342" s="4" t="n">
         <v>6.75</v>
@@ -37526,13 +37526,13 @@
         </is>
       </c>
       <c r="I343" s="4" t="n">
-        <v>-5.73</v>
+        <v>-5.72</v>
       </c>
       <c r="J343" s="4" t="n">
-        <v>16.6</v>
+        <v>16.7</v>
       </c>
       <c r="K343" s="4" t="n">
-        <v>83.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="L343" t="inlineStr">
         <is>
@@ -37540,13 +37540,13 @@
         </is>
       </c>
       <c r="M343" s="4" t="n">
-        <v>-10.58</v>
+        <v>-10.57</v>
       </c>
       <c r="N343" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O343" s="4" t="n">
-        <v>-5.73</v>
+        <v>-5.72</v>
       </c>
       <c r="P343" s="4" t="n">
         <v>0</v>
@@ -37629,7 +37629,7 @@
         </is>
       </c>
       <c r="I344" s="4" t="n">
-        <v>7.85</v>
+        <v>7.86</v>
       </c>
       <c r="J344" s="4" t="n">
         <v>90.09999999999999</v>
@@ -37649,7 +37649,7 @@
         <v>6.75</v>
       </c>
       <c r="O344" s="4" t="n">
-        <v>14.09</v>
+        <v>14.1</v>
       </c>
       <c r="P344" s="4" t="n">
         <v>0.74</v>
@@ -37738,7 +37738,7 @@
         </is>
       </c>
       <c r="I345" s="4" t="n">
-        <v>-6.08</v>
+        <v>-6.07</v>
       </c>
       <c r="J345" s="4" t="n">
         <v>15.5</v>
@@ -37752,13 +37752,13 @@
         </is>
       </c>
       <c r="M345" s="4" t="n">
-        <v>-2.18</v>
+        <v>-2.17</v>
       </c>
       <c r="N345" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O345" s="4" t="n">
-        <v>-6.19</v>
+        <v>-6.18</v>
       </c>
       <c r="P345" s="4" t="n">
         <v>-0.12</v>
@@ -37907,10 +37907,10 @@
         <v>0</v>
       </c>
       <c r="AC346" s="4" t="n">
-        <v>86.78</v>
+        <v>86.79000000000001</v>
       </c>
       <c r="AD346" s="4" t="n">
-        <v>13.22</v>
+        <v>13.21</v>
       </c>
       <c r="AE346" s="4" t="n">
         <v>0</v>
@@ -38061,7 +38061,7 @@
         </is>
       </c>
       <c r="I348" s="4" t="n">
-        <v>21.59</v>
+        <v>21.6</v>
       </c>
       <c r="J348" s="4" t="n">
         <v>99.8</v>
@@ -38081,7 +38081,7 @@
         <v>6.75</v>
       </c>
       <c r="O348" s="4" t="n">
-        <v>21.67</v>
+        <v>21.68</v>
       </c>
       <c r="P348" s="4" t="n">
         <v>2.15</v>
@@ -38121,10 +38121,10 @@
         <v>0</v>
       </c>
       <c r="AC348" s="4" t="n">
-        <v>59.84</v>
+        <v>59.85</v>
       </c>
       <c r="AD348" s="4" t="n">
-        <v>38.59</v>
+        <v>38.58</v>
       </c>
       <c r="AE348" s="4" t="n">
         <v>0</v>
@@ -38172,7 +38172,7 @@
         </is>
       </c>
       <c r="I349" s="4" t="n">
-        <v>-16.94</v>
+        <v>-16.93</v>
       </c>
       <c r="J349" s="4" t="n">
         <v>0.5</v>
@@ -38192,7 +38192,7 @@
         <v>6.75</v>
       </c>
       <c r="O349" s="4" t="n">
-        <v>-16.94</v>
+        <v>-16.93</v>
       </c>
       <c r="P349" s="4" t="n">
         <v>-1.93</v>
@@ -38275,7 +38275,7 @@
         </is>
       </c>
       <c r="I350" s="4" t="n">
-        <v>-2.18</v>
+        <v>-2.17</v>
       </c>
       <c r="J350" s="4" t="n">
         <v>34.7</v>
@@ -38289,13 +38289,13 @@
         </is>
       </c>
       <c r="M350" s="4" t="n">
-        <v>-4.3</v>
+        <v>-4.29</v>
       </c>
       <c r="N350" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O350" s="4" t="n">
-        <v>-2.45</v>
+        <v>-2.44</v>
       </c>
       <c r="P350" s="4" t="n">
         <v>-0.9</v>
@@ -43421,7 +43421,7 @@
         </is>
       </c>
       <c r="I398" s="4" t="n">
-        <v>-40.83</v>
+        <v>-40.73</v>
       </c>
       <c r="J398" s="4" t="n">
         <v>0</v>
@@ -43435,13 +43435,13 @@
         </is>
       </c>
       <c r="M398" s="4" t="n">
-        <v>-43.29</v>
+        <v>-43.19</v>
       </c>
       <c r="N398" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O398" s="4" t="n">
-        <v>-40.83</v>
+        <v>-40.73</v>
       </c>
       <c r="P398" s="4" t="n">
         <v>-2.58</v>
@@ -43473,10 +43473,10 @@
         <v>0</v>
       </c>
       <c r="AC398" s="4" t="n">
-        <v>29.59</v>
+        <v>29.64</v>
       </c>
       <c r="AD398" s="4" t="n">
-        <v>70.41</v>
+        <v>70.36</v>
       </c>
       <c r="AE398" s="4" t="n">
         <v>0</v>
@@ -43520,13 +43520,13 @@
         </is>
       </c>
       <c r="I399" s="4" t="n">
-        <v>-9.99</v>
+        <v>-9.890000000000001</v>
       </c>
       <c r="J399" s="4" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="K399" s="4" t="n">
-        <v>95.8</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="L399" t="inlineStr">
         <is>
@@ -43534,13 +43534,13 @@
         </is>
       </c>
       <c r="M399" s="4" t="n">
-        <v>-18.09</v>
+        <v>-17.99</v>
       </c>
       <c r="N399" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O399" s="4" t="n">
-        <v>-9.99</v>
+        <v>-9.890000000000001</v>
       </c>
       <c r="P399" s="4" t="n">
         <v>0.88</v>
@@ -43572,10 +43572,10 @@
         <v>0</v>
       </c>
       <c r="AC399" s="4" t="n">
-        <v>45</v>
+        <v>45.05</v>
       </c>
       <c r="AD399" s="4" t="n">
-        <v>55</v>
+        <v>54.95</v>
       </c>
       <c r="AE399" s="4" t="n">
         <v>0</v>
@@ -43623,7 +43623,7 @@
         </is>
       </c>
       <c r="I400" s="4" t="n">
-        <v>-13.07</v>
+        <v>-12.97</v>
       </c>
       <c r="J400" s="4" t="n">
         <v>1</v>
@@ -43637,13 +43637,13 @@
         </is>
       </c>
       <c r="M400" s="4" t="n">
-        <v>-17.89</v>
+        <v>-17.79</v>
       </c>
       <c r="N400" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O400" s="4" t="n">
-        <v>-13.07</v>
+        <v>-12.97</v>
       </c>
       <c r="P400" s="4" t="n">
         <v>-0.25</v>
@@ -43675,10 +43675,10 @@
         <v>0</v>
       </c>
       <c r="AC400" s="4" t="n">
-        <v>43.46</v>
+        <v>43.51</v>
       </c>
       <c r="AD400" s="4" t="n">
-        <v>56.54</v>
+        <v>56.49</v>
       </c>
       <c r="AE400" s="4" t="n">
         <v>0</v>
@@ -43726,7 +43726,7 @@
         </is>
       </c>
       <c r="I401" s="4" t="n">
-        <v>-18.51</v>
+        <v>-18.41</v>
       </c>
       <c r="J401" s="4" t="n">
         <v>0.3</v>
@@ -43740,13 +43740,13 @@
         </is>
       </c>
       <c r="M401" s="4" t="n">
-        <v>-18.74</v>
+        <v>-18.64</v>
       </c>
       <c r="N401" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O401" s="4" t="n">
-        <v>-18.51</v>
+        <v>-18.41</v>
       </c>
       <c r="P401" s="4" t="n">
         <v>-1.91</v>
@@ -43778,10 +43778,10 @@
         <v>0</v>
       </c>
       <c r="AC401" s="4" t="n">
-        <v>40.75</v>
+        <v>40.8</v>
       </c>
       <c r="AD401" s="4" t="n">
-        <v>59.25</v>
+        <v>59.2</v>
       </c>
       <c r="AE401" s="4" t="n">
         <v>0</v>
@@ -43829,7 +43829,7 @@
         </is>
       </c>
       <c r="I402" s="4" t="n">
-        <v>-12.76</v>
+        <v>-12.66</v>
       </c>
       <c r="J402" s="4" t="n">
         <v>1</v>
@@ -43843,13 +43843,13 @@
         </is>
       </c>
       <c r="M402" s="4" t="n">
-        <v>-15.58</v>
+        <v>-15.48</v>
       </c>
       <c r="N402" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O402" s="4" t="n">
-        <v>-12.76</v>
+        <v>-12.66</v>
       </c>
       <c r="P402" s="4" t="n">
         <v>-2.33</v>
@@ -43881,10 +43881,10 @@
         <v>0</v>
       </c>
       <c r="AC402" s="4" t="n">
-        <v>43.62</v>
+        <v>43.67</v>
       </c>
       <c r="AD402" s="4" t="n">
-        <v>56.38</v>
+        <v>56.33</v>
       </c>
       <c r="AE402" s="4" t="n">
         <v>0</v>
@@ -43932,7 +43932,7 @@
         </is>
       </c>
       <c r="I403" s="4" t="n">
-        <v>-16.41</v>
+        <v>-16.31</v>
       </c>
       <c r="J403" s="4" t="n">
         <v>0.5</v>
@@ -43946,13 +43946,13 @@
         </is>
       </c>
       <c r="M403" s="4" t="n">
-        <v>-17.66</v>
+        <v>-17.56</v>
       </c>
       <c r="N403" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O403" s="4" t="n">
-        <v>-16.41</v>
+        <v>-16.31</v>
       </c>
       <c r="P403" s="4" t="n">
         <v>-2.94</v>
@@ -43984,10 +43984,10 @@
         <v>0</v>
       </c>
       <c r="AC403" s="4" t="n">
-        <v>41.79</v>
+        <v>41.84</v>
       </c>
       <c r="AD403" s="4" t="n">
-        <v>58.21</v>
+        <v>58.16</v>
       </c>
       <c r="AE403" s="4" t="n">
         <v>0</v>
@@ -44035,7 +44035,7 @@
         </is>
       </c>
       <c r="I404" s="4" t="n">
-        <v>42.63</v>
+        <v>42.73</v>
       </c>
       <c r="J404" s="4" t="n">
         <v>100</v>
@@ -44049,13 +44049,13 @@
         </is>
       </c>
       <c r="M404" s="4" t="n">
-        <v>31.67</v>
+        <v>31.77</v>
       </c>
       <c r="N404" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O404" s="4" t="n">
-        <v>43.35</v>
+        <v>43.45</v>
       </c>
       <c r="P404" s="4" t="n">
         <v>1.84</v>
@@ -44095,10 +44095,10 @@
         <v>0</v>
       </c>
       <c r="AC404" s="4" t="n">
-        <v>69.25</v>
+        <v>69.3</v>
       </c>
       <c r="AD404" s="4" t="n">
-        <v>27.86</v>
+        <v>27.81</v>
       </c>
       <c r="AE404" s="4" t="n">
         <v>0</v>
@@ -44142,7 +44142,7 @@
         </is>
       </c>
       <c r="I405" s="4" t="n">
-        <v>-15.5</v>
+        <v>-15.4</v>
       </c>
       <c r="J405" s="4" t="n">
         <v>0.6</v>
@@ -44156,13 +44156,13 @@
         </is>
       </c>
       <c r="M405" s="4" t="n">
-        <v>-20.37</v>
+        <v>-20.27</v>
       </c>
       <c r="N405" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O405" s="4" t="n">
-        <v>-15.5</v>
+        <v>-15.4</v>
       </c>
       <c r="P405" s="4" t="n">
         <v>-2.72</v>
@@ -44194,10 +44194,10 @@
         <v>0</v>
       </c>
       <c r="AC405" s="4" t="n">
-        <v>42.25</v>
+        <v>42.3</v>
       </c>
       <c r="AD405" s="4" t="n">
-        <v>57.75</v>
+        <v>57.7</v>
       </c>
       <c r="AE405" s="4" t="n">
         <v>0</v>
@@ -44241,13 +44241,13 @@
         </is>
       </c>
       <c r="I406" s="4" t="n">
-        <v>-6.22</v>
+        <v>-6.17</v>
       </c>
       <c r="J406" s="4" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="K406" s="4" t="n">
-        <v>85</v>
+        <v>84.8</v>
       </c>
       <c r="L406" t="inlineStr">
         <is>
@@ -44255,13 +44255,13 @@
         </is>
       </c>
       <c r="M406" s="4" t="n">
-        <v>-11.34</v>
+        <v>-11.24</v>
       </c>
       <c r="N406" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O406" s="4" t="n">
-        <v>-4.29</v>
+        <v>-4.19</v>
       </c>
       <c r="P406" s="4" t="n">
         <v>-1.88</v>
@@ -44299,10 +44299,10 @@
         <v>0</v>
       </c>
       <c r="AC406" s="4" t="n">
-        <v>46.89</v>
+        <v>46.92</v>
       </c>
       <c r="AD406" s="4" t="n">
-        <v>53.11</v>
+        <v>53.08</v>
       </c>
       <c r="AE406" s="4" t="n">
         <v>0</v>
@@ -44346,13 +44346,13 @@
         </is>
       </c>
       <c r="I407" s="4" t="n">
-        <v>-10.28</v>
+        <v>-10.23</v>
       </c>
       <c r="J407" s="4" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K407" s="4" t="n">
-        <v>96.5</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="L407" t="inlineStr">
         <is>
@@ -44360,13 +44360,13 @@
         </is>
       </c>
       <c r="M407" s="4" t="n">
-        <v>-16.02</v>
+        <v>-15.92</v>
       </c>
       <c r="N407" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O407" s="4" t="n">
-        <v>-10.72</v>
+        <v>-10.62</v>
       </c>
       <c r="P407" s="4" t="n">
         <v>-1.52</v>
@@ -44404,10 +44404,10 @@
         <v>0</v>
       </c>
       <c r="AC407" s="4" t="n">
-        <v>44.86</v>
+        <v>44.89</v>
       </c>
       <c r="AD407" s="4" t="n">
-        <v>55.14</v>
+        <v>55.11</v>
       </c>
       <c r="AE407" s="4" t="n">
         <v>0</v>
@@ -44455,7 +44455,7 @@
         </is>
       </c>
       <c r="I408" s="4" t="n">
-        <v>-25.08</v>
+        <v>-24.98</v>
       </c>
       <c r="J408" s="4" t="n">
         <v>0.1</v>
@@ -44469,13 +44469,13 @@
         </is>
       </c>
       <c r="M408" s="4" t="n">
-        <v>-28.71</v>
+        <v>-28.61</v>
       </c>
       <c r="N408" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O408" s="4" t="n">
-        <v>-25.08</v>
+        <v>-24.98</v>
       </c>
       <c r="P408" s="4" t="n">
         <v>-2.36</v>
@@ -44507,10 +44507,10 @@
         <v>0</v>
       </c>
       <c r="AC408" s="4" t="n">
-        <v>37.46</v>
+        <v>37.51</v>
       </c>
       <c r="AD408" s="4" t="n">
-        <v>62.54</v>
+        <v>62.49</v>
       </c>
       <c r="AE408" s="4" t="n">
         <v>0</v>
@@ -44558,7 +44558,7 @@
         </is>
       </c>
       <c r="I409" s="4" t="n">
-        <v>-16.44</v>
+        <v>-16.34</v>
       </c>
       <c r="J409" s="4" t="n">
         <v>0.5</v>
@@ -44572,13 +44572,13 @@
         </is>
       </c>
       <c r="M409" s="4" t="n">
-        <v>-17.66</v>
+        <v>-17.56</v>
       </c>
       <c r="N409" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O409" s="4" t="n">
-        <v>-16.44</v>
+        <v>-16.34</v>
       </c>
       <c r="P409" s="4" t="n">
         <v>0</v>
@@ -44610,10 +44610,10 @@
         <v>0</v>
       </c>
       <c r="AC409" s="4" t="n">
-        <v>41.78</v>
+        <v>41.83</v>
       </c>
       <c r="AD409" s="4" t="n">
-        <v>58.22</v>
+        <v>58.17</v>
       </c>
       <c r="AE409" s="4" t="n">
         <v>0</v>
@@ -44661,7 +44661,7 @@
         </is>
       </c>
       <c r="I410" s="4" t="n">
-        <v>-38.37</v>
+        <v>-38.27</v>
       </c>
       <c r="J410" s="4" t="n">
         <v>0</v>
@@ -44675,13 +44675,13 @@
         </is>
       </c>
       <c r="M410" s="4" t="n">
-        <v>-41.31</v>
+        <v>-41.21</v>
       </c>
       <c r="N410" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O410" s="4" t="n">
-        <v>-38.37</v>
+        <v>-38.27</v>
       </c>
       <c r="P410" s="4" t="n">
         <v>-2.47</v>
@@ -44713,10 +44713,10 @@
         <v>0</v>
       </c>
       <c r="AC410" s="4" t="n">
-        <v>30.82</v>
+        <v>30.87</v>
       </c>
       <c r="AD410" s="4" t="n">
-        <v>69.18000000000001</v>
+        <v>69.13</v>
       </c>
       <c r="AE410" s="4" t="n">
         <v>0</v>
@@ -44764,7 +44764,7 @@
         </is>
       </c>
       <c r="I411" s="4" t="n">
-        <v>-17.36</v>
+        <v>-17.26</v>
       </c>
       <c r="J411" s="4" t="n">
         <v>0.4</v>
@@ -44778,13 +44778,13 @@
         </is>
       </c>
       <c r="M411" s="4" t="n">
-        <v>-18.72</v>
+        <v>-18.62</v>
       </c>
       <c r="N411" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O411" s="4" t="n">
-        <v>-17.36</v>
+        <v>-17.26</v>
       </c>
       <c r="P411" s="4" t="n">
         <v>-1.94</v>
@@ -44816,10 +44816,10 @@
         <v>0</v>
       </c>
       <c r="AC411" s="4" t="n">
-        <v>41.32</v>
+        <v>41.37</v>
       </c>
       <c r="AD411" s="4" t="n">
-        <v>58.68</v>
+        <v>58.63</v>
       </c>
       <c r="AE411" s="4" t="n">
         <v>0</v>
@@ -44867,13 +44867,13 @@
         </is>
       </c>
       <c r="I412" s="4" t="n">
-        <v>3.78</v>
+        <v>3.84</v>
       </c>
       <c r="J412" s="4" t="n">
-        <v>76.2</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="K412" s="4" t="n">
-        <v>23.8</v>
+        <v>23.4</v>
       </c>
       <c r="L412" t="inlineStr">
         <is>
@@ -44881,13 +44881,13 @@
         </is>
       </c>
       <c r="M412" s="4" t="n">
-        <v>-7.41</v>
+        <v>-7.31</v>
       </c>
       <c r="N412" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O412" s="4" t="n">
-        <v>0.87</v>
+        <v>0.97</v>
       </c>
       <c r="P412" s="4" t="n">
         <v>-0.22</v>
@@ -44925,10 +44925,10 @@
         <v>0</v>
       </c>
       <c r="AC412" s="4" t="n">
-        <v>51.89</v>
+        <v>51.92</v>
       </c>
       <c r="AD412" s="4" t="n">
-        <v>48.11</v>
+        <v>48.08</v>
       </c>
       <c r="AE412" s="4" t="n">
         <v>0</v>
@@ -44976,7 +44976,7 @@
         </is>
       </c>
       <c r="I413" s="4" t="n">
-        <v>38.89</v>
+        <v>38.99</v>
       </c>
       <c r="J413" s="4" t="n">
         <v>100</v>
@@ -44990,13 +44990,13 @@
         </is>
       </c>
       <c r="M413" s="4" t="n">
-        <v>27.64</v>
+        <v>27.74</v>
       </c>
       <c r="N413" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O413" s="4" t="n">
-        <v>38.89</v>
+        <v>38.99</v>
       </c>
       <c r="P413" s="4" t="n">
         <v>0</v>
@@ -45028,10 +45028,10 @@
         <v>0</v>
       </c>
       <c r="AC413" s="4" t="n">
-        <v>69.45</v>
+        <v>69.5</v>
       </c>
       <c r="AD413" s="4" t="n">
-        <v>30.55</v>
+        <v>30.5</v>
       </c>
       <c r="AE413" s="4" t="n">
         <v>0</v>
@@ -45079,7 +45079,7 @@
         </is>
       </c>
       <c r="I414" s="4" t="n">
-        <v>-14.7</v>
+        <v>-14.6</v>
       </c>
       <c r="J414" s="4" t="n">
         <v>0.7</v>
@@ -45093,13 +45093,13 @@
         </is>
       </c>
       <c r="M414" s="4" t="n">
-        <v>-15.49</v>
+        <v>-15.39</v>
       </c>
       <c r="N414" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O414" s="4" t="n">
-        <v>-14.7</v>
+        <v>-14.6</v>
       </c>
       <c r="P414" s="4" t="n">
         <v>-2.2</v>
@@ -45131,10 +45131,10 @@
         <v>0</v>
       </c>
       <c r="AC414" s="4" t="n">
-        <v>42.65</v>
+        <v>42.7</v>
       </c>
       <c r="AD414" s="4" t="n">
-        <v>57.35</v>
+        <v>57.3</v>
       </c>
       <c r="AE414" s="4" t="n">
         <v>0</v>
@@ -45182,7 +45182,7 @@
         </is>
       </c>
       <c r="I415" s="4" t="n">
-        <v>73.43000000000001</v>
+        <v>73.53</v>
       </c>
       <c r="J415" s="4" t="n">
         <v>100</v>
@@ -45196,13 +45196,13 @@
         </is>
       </c>
       <c r="M415" s="4" t="n">
-        <v>63.73</v>
+        <v>63.83</v>
       </c>
       <c r="N415" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O415" s="4" t="n">
-        <v>73.43000000000001</v>
+        <v>73.53</v>
       </c>
       <c r="P415" s="4" t="n">
         <v>0</v>
@@ -45234,10 +45234,10 @@
         <v>0</v>
       </c>
       <c r="AC415" s="4" t="n">
-        <v>86.70999999999999</v>
+        <v>86.76000000000001</v>
       </c>
       <c r="AD415" s="4" t="n">
-        <v>13.29</v>
+        <v>13.24</v>
       </c>
       <c r="AE415" s="4" t="n">
         <v>0</v>
@@ -45281,7 +45281,7 @@
         </is>
       </c>
       <c r="I416" s="4" t="n">
-        <v>-40.43</v>
+        <v>-40.33</v>
       </c>
       <c r="J416" s="4" t="n">
         <v>0</v>
@@ -45295,13 +45295,13 @@
         </is>
       </c>
       <c r="M416" s="4" t="n">
-        <v>-45.67</v>
+        <v>-45.57</v>
       </c>
       <c r="N416" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O416" s="4" t="n">
-        <v>-40.43</v>
+        <v>-40.33</v>
       </c>
       <c r="P416" s="4" t="n">
         <v>-2.39</v>
@@ -45333,10 +45333,10 @@
         <v>0</v>
       </c>
       <c r="AC416" s="4" t="n">
-        <v>29.79</v>
+        <v>29.84</v>
       </c>
       <c r="AD416" s="4" t="n">
-        <v>70.20999999999999</v>
+        <v>70.16</v>
       </c>
       <c r="AE416" s="4" t="n">
         <v>0</v>
@@ -45384,7 +45384,7 @@
         </is>
       </c>
       <c r="I417" s="4" t="n">
-        <v>51.57</v>
+        <v>51.67</v>
       </c>
       <c r="J417" s="4" t="n">
         <v>100</v>
@@ -45398,13 +45398,13 @@
         </is>
       </c>
       <c r="M417" s="4" t="n">
-        <v>37.48</v>
+        <v>37.58</v>
       </c>
       <c r="N417" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O417" s="4" t="n">
-        <v>51.57</v>
+        <v>51.67</v>
       </c>
       <c r="P417" s="4" t="n">
         <v>1.31</v>
@@ -45436,10 +45436,10 @@
         <v>0</v>
       </c>
       <c r="AC417" s="4" t="n">
-        <v>75.78</v>
+        <v>75.83</v>
       </c>
       <c r="AD417" s="4" t="n">
-        <v>24.22</v>
+        <v>24.17</v>
       </c>
       <c r="AE417" s="4" t="n">
         <v>0</v>
@@ -45483,13 +45483,13 @@
         </is>
       </c>
       <c r="I418" s="4" t="n">
-        <v>-9.949999999999999</v>
+        <v>-9.85</v>
       </c>
       <c r="J418" s="4" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="K418" s="4" t="n">
-        <v>95.7</v>
+        <v>95.5</v>
       </c>
       <c r="L418" t="inlineStr">
         <is>
@@ -45497,13 +45497,13 @@
         </is>
       </c>
       <c r="M418" s="4" t="n">
-        <v>-16</v>
+        <v>-15.9</v>
       </c>
       <c r="N418" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O418" s="4" t="n">
-        <v>-9.949999999999999</v>
+        <v>-9.85</v>
       </c>
       <c r="P418" s="4" t="n">
         <v>-2.02</v>
@@ -45535,10 +45535,10 @@
         <v>0</v>
       </c>
       <c r="AC418" s="4" t="n">
-        <v>45.03</v>
+        <v>45.08</v>
       </c>
       <c r="AD418" s="4" t="n">
-        <v>54.97</v>
+        <v>54.92</v>
       </c>
       <c r="AE418" s="4" t="n">
         <v>0</v>
@@ -45582,13 +45582,13 @@
         </is>
       </c>
       <c r="I419" s="4" t="n">
-        <v>-10.7</v>
+        <v>-10.6</v>
       </c>
       <c r="J419" s="4" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="K419" s="4" t="n">
-        <v>97.5</v>
+        <v>97.3</v>
       </c>
       <c r="L419" t="inlineStr">
         <is>
@@ -45596,13 +45596,13 @@
         </is>
       </c>
       <c r="M419" s="4" t="n">
-        <v>-16.58</v>
+        <v>-16.48</v>
       </c>
       <c r="N419" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O419" s="4" t="n">
-        <v>-10.7</v>
+        <v>-10.6</v>
       </c>
       <c r="P419" s="4" t="n">
         <v>-0.8100000000000001</v>
@@ -45634,10 +45634,10 @@
         <v>0</v>
       </c>
       <c r="AC419" s="4" t="n">
-        <v>44.65</v>
+        <v>44.7</v>
       </c>
       <c r="AD419" s="4" t="n">
-        <v>55.35</v>
+        <v>55.3</v>
       </c>
       <c r="AE419" s="4" t="n">
         <v>0</v>
@@ -45681,13 +45681,13 @@
         </is>
       </c>
       <c r="I420" s="4" t="n">
-        <v>-0.11</v>
+        <v>-0.03</v>
       </c>
       <c r="J420" s="4" t="n">
-        <v>49.2</v>
+        <v>49.8</v>
       </c>
       <c r="K420" s="4" t="n">
-        <v>50.8</v>
+        <v>50.2</v>
       </c>
       <c r="L420" t="inlineStr">
         <is>
@@ -45695,13 +45695,13 @@
         </is>
       </c>
       <c r="M420" s="4" t="n">
-        <v>-7.58</v>
+        <v>-7.48</v>
       </c>
       <c r="N420" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O420" s="4" t="n">
-        <v>0.37</v>
+        <v>0.47</v>
       </c>
       <c r="P420" s="4" t="n">
         <v>-0.84</v>
@@ -45747,10 +45747,10 @@
         <v>0</v>
       </c>
       <c r="AC420" s="4" t="n">
-        <v>49.01</v>
+        <v>49.06</v>
       </c>
       <c r="AD420" s="4" t="n">
-        <v>49.13</v>
+        <v>49.08</v>
       </c>
       <c r="AE420" s="4" t="n">
         <v>0</v>
@@ -45798,13 +45798,13 @@
         </is>
       </c>
       <c r="I421" s="4" t="n">
-        <v>-10.36</v>
+        <v>-10.26</v>
       </c>
       <c r="J421" s="4" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="K421" s="4" t="n">
-        <v>96.7</v>
+        <v>96.5</v>
       </c>
       <c r="L421" t="inlineStr">
         <is>
@@ -45812,13 +45812,13 @@
         </is>
       </c>
       <c r="M421" s="4" t="n">
-        <v>-10.91</v>
+        <v>-10.81</v>
       </c>
       <c r="N421" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O421" s="4" t="n">
-        <v>-10.36</v>
+        <v>-10.26</v>
       </c>
       <c r="P421" s="4" t="n">
         <v>-1.72</v>
@@ -45850,10 +45850,10 @@
         <v>0</v>
       </c>
       <c r="AC421" s="4" t="n">
-        <v>44.82</v>
+        <v>44.87</v>
       </c>
       <c r="AD421" s="4" t="n">
-        <v>55.18</v>
+        <v>55.13</v>
       </c>
       <c r="AE421" s="4" t="n">
         <v>0</v>
@@ -45901,13 +45901,13 @@
         </is>
       </c>
       <c r="I422" s="4" t="n">
-        <v>-11.58</v>
+        <v>-11.48</v>
       </c>
       <c r="J422" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K422" s="4" t="n">
-        <v>98.8</v>
+        <v>98.7</v>
       </c>
       <c r="L422" t="inlineStr">
         <is>
@@ -45915,13 +45915,13 @@
         </is>
       </c>
       <c r="M422" s="4" t="n">
-        <v>-17.14</v>
+        <v>-17.04</v>
       </c>
       <c r="N422" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O422" s="4" t="n">
-        <v>-11.58</v>
+        <v>-11.48</v>
       </c>
       <c r="P422" s="4" t="n">
         <v>0</v>
@@ -45953,10 +45953,10 @@
         <v>0</v>
       </c>
       <c r="AC422" s="4" t="n">
-        <v>44.21</v>
+        <v>44.26</v>
       </c>
       <c r="AD422" s="4" t="n">
-        <v>55.79</v>
+        <v>55.74</v>
       </c>
       <c r="AE422" s="4" t="n">
         <v>0</v>
@@ -46004,7 +46004,7 @@
         </is>
       </c>
       <c r="I423" s="4" t="n">
-        <v>-19.92</v>
+        <v>-19.82</v>
       </c>
       <c r="J423" s="4" t="n">
         <v>0.2</v>
@@ -46018,13 +46018,13 @@
         </is>
       </c>
       <c r="M423" s="4" t="n">
-        <v>-18.26</v>
+        <v>-18.16</v>
       </c>
       <c r="N423" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O423" s="4" t="n">
-        <v>-20.31</v>
+        <v>-20.21</v>
       </c>
       <c r="P423" s="4" t="n">
         <v>-3.11</v>
@@ -46064,10 +46064,10 @@
         <v>0</v>
       </c>
       <c r="AC423" s="4" t="n">
-        <v>39.25</v>
+        <v>39.3</v>
       </c>
       <c r="AD423" s="4" t="n">
-        <v>58.77</v>
+        <v>58.72</v>
       </c>
       <c r="AE423" s="4" t="n">
         <v>0</v>
@@ -46115,13 +46115,13 @@
         </is>
       </c>
       <c r="I424" s="4" t="n">
-        <v>-11.58</v>
+        <v>-11.48</v>
       </c>
       <c r="J424" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K424" s="4" t="n">
-        <v>98.8</v>
+        <v>98.7</v>
       </c>
       <c r="L424" t="inlineStr">
         <is>
@@ -46129,13 +46129,13 @@
         </is>
       </c>
       <c r="M424" s="4" t="n">
-        <v>-15.5</v>
+        <v>-15.4</v>
       </c>
       <c r="N424" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O424" s="4" t="n">
-        <v>-11.58</v>
+        <v>-11.48</v>
       </c>
       <c r="P424" s="4" t="n">
         <v>-1.33</v>
@@ -46167,10 +46167,10 @@
         <v>0</v>
       </c>
       <c r="AC424" s="4" t="n">
-        <v>44.21</v>
+        <v>44.26</v>
       </c>
       <c r="AD424" s="4" t="n">
-        <v>55.79</v>
+        <v>55.74</v>
       </c>
       <c r="AE424" s="4" t="n">
         <v>0</v>
@@ -46218,13 +46218,13 @@
         </is>
       </c>
       <c r="I425" s="4" t="n">
-        <v>18.1</v>
+        <v>18.17</v>
       </c>
       <c r="J425" s="4" t="n">
-        <v>99.59999999999999</v>
+        <v>99.7</v>
       </c>
       <c r="K425" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L425" t="inlineStr">
         <is>
@@ -46232,13 +46232,13 @@
         </is>
       </c>
       <c r="M425" s="4" t="n">
-        <v>2.16</v>
+        <v>2.26</v>
       </c>
       <c r="N425" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O425" s="4" t="n">
-        <v>22.56</v>
+        <v>22.66</v>
       </c>
       <c r="P425" s="4" t="n">
         <v>0.45</v>
@@ -46284,10 +46284,10 @@
         <v>0</v>
       </c>
       <c r="AC425" s="4" t="n">
-        <v>55.95</v>
+        <v>55.98</v>
       </c>
       <c r="AD425" s="4" t="n">
-        <v>38.8</v>
+        <v>38.77</v>
       </c>
       <c r="AE425" s="4" t="n">
         <v>0</v>
@@ -46335,7 +46335,7 @@
         </is>
       </c>
       <c r="I426" s="4" t="n">
-        <v>56.36</v>
+        <v>56.46</v>
       </c>
       <c r="J426" s="4" t="n">
         <v>100</v>
@@ -46349,13 +46349,13 @@
         </is>
       </c>
       <c r="M426" s="4" t="n">
-        <v>40</v>
+        <v>40.1</v>
       </c>
       <c r="N426" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O426" s="4" t="n">
-        <v>56.36</v>
+        <v>56.46</v>
       </c>
       <c r="P426" s="4" t="n">
         <v>0</v>
@@ -46387,10 +46387,10 @@
         <v>0</v>
       </c>
       <c r="AC426" s="4" t="n">
-        <v>78.18000000000001</v>
+        <v>78.23</v>
       </c>
       <c r="AD426" s="4" t="n">
-        <v>21.82</v>
+        <v>21.77</v>
       </c>
       <c r="AE426" s="4" t="n">
         <v>0</v>
@@ -46434,7 +46434,7 @@
         </is>
       </c>
       <c r="I427" s="4" t="n">
-        <v>65.33</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="J427" s="4" t="n">
         <v>100</v>
@@ -46448,13 +46448,13 @@
         </is>
       </c>
       <c r="M427" s="4" t="n">
-        <v>55.71</v>
+        <v>55.81</v>
       </c>
       <c r="N427" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O427" s="4" t="n">
-        <v>65.33</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="P427" s="4" t="n">
         <v>1.56</v>
@@ -46486,10 +46486,10 @@
         <v>0</v>
       </c>
       <c r="AC427" s="4" t="n">
-        <v>82.66</v>
+        <v>82.70999999999999</v>
       </c>
       <c r="AD427" s="4" t="n">
-        <v>17.34</v>
+        <v>17.29</v>
       </c>
       <c r="AE427" s="4" t="n">
         <v>0</v>
@@ -46537,7 +46537,7 @@
         </is>
       </c>
       <c r="I428" s="4" t="n">
-        <v>-16.46</v>
+        <v>-16.36</v>
       </c>
       <c r="J428" s="4" t="n">
         <v>0.5</v>
@@ -46551,13 +46551,13 @@
         </is>
       </c>
       <c r="M428" s="4" t="n">
-        <v>-16.42</v>
+        <v>-16.32</v>
       </c>
       <c r="N428" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O428" s="4" t="n">
-        <v>-15.87</v>
+        <v>-15.77</v>
       </c>
       <c r="P428" s="4" t="n">
         <v>-1.61</v>
@@ -46597,10 +46597,10 @@
         <v>0</v>
       </c>
       <c r="AC428" s="4" t="n">
-        <v>40.79</v>
+        <v>40.84</v>
       </c>
       <c r="AD428" s="4" t="n">
-        <v>56.87</v>
+        <v>56.82</v>
       </c>
       <c r="AE428" s="4" t="n">
         <v>0</v>
@@ -46644,13 +46644,13 @@
         </is>
       </c>
       <c r="I429" s="4" t="n">
-        <v>-5.96</v>
+        <v>-5.86</v>
       </c>
       <c r="J429" s="4" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="K429" s="4" t="n">
-        <v>84.2</v>
+        <v>83.8</v>
       </c>
       <c r="L429" t="inlineStr">
         <is>
@@ -46658,13 +46658,13 @@
         </is>
       </c>
       <c r="M429" s="4" t="n">
-        <v>-11.27</v>
+        <v>-11.17</v>
       </c>
       <c r="N429" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O429" s="4" t="n">
-        <v>-5.96</v>
+        <v>-5.86</v>
       </c>
       <c r="P429" s="4" t="n">
         <v>-1.71</v>
@@ -46696,10 +46696,10 @@
         <v>0</v>
       </c>
       <c r="AC429" s="4" t="n">
-        <v>47.02</v>
+        <v>47.07</v>
       </c>
       <c r="AD429" s="4" t="n">
-        <v>52.98</v>
+        <v>52.93</v>
       </c>
       <c r="AE429" s="4" t="n">
         <v>0</v>
@@ -46743,7 +46743,7 @@
         </is>
       </c>
       <c r="I430" s="4" t="n">
-        <v>48.45</v>
+        <v>48.55</v>
       </c>
       <c r="J430" s="4" t="n">
         <v>100</v>
@@ -46757,13 +46757,13 @@
         </is>
       </c>
       <c r="M430" s="4" t="n">
-        <v>41.87</v>
+        <v>41.97</v>
       </c>
       <c r="N430" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O430" s="4" t="n">
-        <v>48.45</v>
+        <v>48.55</v>
       </c>
       <c r="P430" s="4" t="n">
         <v>0</v>
@@ -46795,10 +46795,10 @@
         <v>0</v>
       </c>
       <c r="AC430" s="4" t="n">
-        <v>74.22</v>
+        <v>74.27</v>
       </c>
       <c r="AD430" s="4" t="n">
-        <v>25.78</v>
+        <v>25.73</v>
       </c>
       <c r="AE430" s="4" t="n">
         <v>0</v>
@@ -46846,13 +46846,13 @@
         </is>
       </c>
       <c r="I431" s="4" t="n">
-        <v>11.16</v>
+        <v>11.23</v>
       </c>
       <c r="J431" s="4" t="n">
-        <v>98.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="K431" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L431" t="inlineStr">
         <is>
@@ -46860,13 +46860,13 @@
         </is>
       </c>
       <c r="M431" s="4" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.59</v>
       </c>
       <c r="N431" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O431" s="4" t="n">
-        <v>13.74</v>
+        <v>13.84</v>
       </c>
       <c r="P431" s="4" t="n">
         <v>0.36</v>
@@ -46912,10 +46912,10 @@
         <v>0</v>
       </c>
       <c r="AC431" s="4" t="n">
-        <v>53.17</v>
+        <v>53.21</v>
       </c>
       <c r="AD431" s="4" t="n">
-        <v>42.5</v>
+        <v>42.46</v>
       </c>
       <c r="AE431" s="4" t="n">
         <v>1.53</v>
@@ -46959,13 +46959,13 @@
         </is>
       </c>
       <c r="I432" s="4" t="n">
-        <v>2.67</v>
+        <v>2.74</v>
       </c>
       <c r="J432" s="4" t="n">
-        <v>68.7</v>
+        <v>69.2</v>
       </c>
       <c r="K432" s="4" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="L432" t="inlineStr">
         <is>
@@ -46973,13 +46973,13 @@
         </is>
       </c>
       <c r="M432" s="4" t="n">
-        <v>-3.18</v>
+        <v>-3.08</v>
       </c>
       <c r="N432" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O432" s="4" t="n">
-        <v>5.23</v>
+        <v>5.33</v>
       </c>
       <c r="P432" s="4" t="n">
         <v>-0.22</v>
@@ -47017,10 +47017,10 @@
         <v>0</v>
       </c>
       <c r="AC432" s="4" t="n">
-        <v>51.33</v>
+        <v>51.37</v>
       </c>
       <c r="AD432" s="4" t="n">
-        <v>48.67</v>
+        <v>48.63</v>
       </c>
       <c r="AE432" s="4" t="n">
         <v>0</v>
@@ -47068,7 +47068,7 @@
         </is>
       </c>
       <c r="I433" s="4" t="n">
-        <v>-13.64</v>
+        <v>-13.54</v>
       </c>
       <c r="J433" s="4" t="n">
         <v>0.9</v>
@@ -47082,13 +47082,13 @@
         </is>
       </c>
       <c r="M433" s="4" t="n">
-        <v>-18.3</v>
+        <v>-18.2</v>
       </c>
       <c r="N433" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O433" s="4" t="n">
-        <v>-13.64</v>
+        <v>-13.54</v>
       </c>
       <c r="P433" s="4" t="n">
         <v>0</v>
@@ -47120,10 +47120,10 @@
         <v>0</v>
       </c>
       <c r="AC433" s="4" t="n">
-        <v>43.18</v>
+        <v>43.23</v>
       </c>
       <c r="AD433" s="4" t="n">
-        <v>56.82</v>
+        <v>56.77</v>
       </c>
       <c r="AE433" s="4" t="n">
         <v>0</v>
@@ -47171,7 +47171,7 @@
         </is>
       </c>
       <c r="I434" s="4" t="n">
-        <v>73.51000000000001</v>
+        <v>73.61</v>
       </c>
       <c r="J434" s="4" t="n">
         <v>100</v>
@@ -47185,13 +47185,13 @@
         </is>
       </c>
       <c r="M434" s="4" t="n">
-        <v>64.48999999999999</v>
+        <v>64.59</v>
       </c>
       <c r="N434" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O434" s="4" t="n">
-        <v>73.51000000000001</v>
+        <v>73.61</v>
       </c>
       <c r="P434" s="4" t="n">
         <v>1.49</v>
@@ -47223,10 +47223,10 @@
         <v>0</v>
       </c>
       <c r="AC434" s="4" t="n">
-        <v>86.76000000000001</v>
+        <v>86.81</v>
       </c>
       <c r="AD434" s="4" t="n">
-        <v>13.24</v>
+        <v>13.19</v>
       </c>
       <c r="AE434" s="4" t="n">
         <v>0</v>
@@ -47270,7 +47270,7 @@
         </is>
       </c>
       <c r="I435" s="4" t="n">
-        <v>-11.72</v>
+        <v>-11.62</v>
       </c>
       <c r="J435" s="4" t="n">
         <v>1.2</v>
@@ -47284,13 +47284,13 @@
         </is>
       </c>
       <c r="M435" s="4" t="n">
-        <v>-15.74</v>
+        <v>-15.64</v>
       </c>
       <c r="N435" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O435" s="4" t="n">
-        <v>-11.17</v>
+        <v>-11.07</v>
       </c>
       <c r="P435" s="4" t="n">
         <v>-2.01</v>
@@ -47330,10 +47330,10 @@
         <v>0</v>
       </c>
       <c r="AC435" s="4" t="n">
-        <v>43.18</v>
+        <v>43.23</v>
       </c>
       <c r="AD435" s="4" t="n">
-        <v>54.64</v>
+        <v>54.59</v>
       </c>
       <c r="AE435" s="4" t="n">
         <v>0</v>
@@ -51404,27 +51404,27 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>3.01</v>
+        <v>3.28</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>72.3</v>
+        <v>75</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>27.7</v>
+        <v>25</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
-          <t>Lean D</t>
+          <t>Likely D</t>
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.71</v>
+        <v>-10.09</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-0.66</v>
+        <v>-0.03</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.26</v>
@@ -51462,10 +51462,10 @@
         <v>0</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>49.83</v>
+        <v>49.96</v>
       </c>
       <c r="AD473" s="4" t="n">
-        <v>47.67</v>
+        <v>47.54</v>
       </c>
       <c r="AE473" s="4" t="n">
         <v>2.5</v>
@@ -52171,13 +52171,13 @@
         </is>
       </c>
       <c r="I480" s="4" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="J480" s="4" t="n">
-        <v>59.5</v>
+        <v>59.6</v>
       </c>
       <c r="K480" s="4" t="n">
-        <v>40.5</v>
+        <v>40.4</v>
       </c>
       <c r="L480" t="inlineStr">
         <is>
@@ -52185,13 +52185,13 @@
         </is>
       </c>
       <c r="M480" s="4" t="n">
-        <v>-6.56</v>
+        <v>-6.52</v>
       </c>
       <c r="N480" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O480" s="4" t="n">
-        <v>-1.67</v>
+        <v>-1.63</v>
       </c>
       <c r="P480" s="4" t="n">
         <v>-0.22</v>
@@ -52512,13 +52512,13 @@
         </is>
       </c>
       <c r="I483" s="4" t="n">
-        <v>-2.13</v>
+        <v>-2.11</v>
       </c>
       <c r="J483" s="4" t="n">
-        <v>35</v>
+        <v>35.1</v>
       </c>
       <c r="K483" s="4" t="n">
-        <v>65</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="L483" t="inlineStr">
         <is>
@@ -52526,13 +52526,13 @@
         </is>
       </c>
       <c r="M483" s="4" t="n">
-        <v>-14.09</v>
+        <v>-14.03</v>
       </c>
       <c r="N483" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O483" s="4" t="n">
-        <v>-8.539999999999999</v>
+        <v>-8.48</v>
       </c>
       <c r="P483" s="4" t="n">
         <v>0.32</v>
@@ -52578,10 +52578,10 @@
         <v>0</v>
       </c>
       <c r="AC483" s="4" t="n">
-        <v>47.63</v>
+        <v>47.64</v>
       </c>
       <c r="AD483" s="4" t="n">
-        <v>49.7</v>
+        <v>49.69</v>
       </c>
       <c r="AE483" s="4" t="n">
         <v>0</v>
@@ -52967,10 +52967,10 @@
         <v>1.84</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>63.3</v>
+        <v>63.2</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>36.7</v>
+        <v>36.8</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53412,7 +53412,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.55</v>
+        <v>-21.59</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53472,16 +53472,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.78</v>
+        <v>27.73</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.23</v>
+        <v>19.28</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.33</v>
+        <v>49.32</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -54095,10 +54095,10 @@
         <v>3.47</v>
       </c>
       <c r="J497" s="4" t="n">
-        <v>74.09999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="K497" s="4" t="n">
-        <v>25.9</v>
+        <v>25.8</v>
       </c>
       <c r="L497" t="inlineStr">
         <is>
@@ -54106,7 +54106,7 @@
         </is>
       </c>
       <c r="M497" s="4" t="n">
-        <v>-7.52</v>
+        <v>-7.51</v>
       </c>
       <c r="N497" s="4" t="n">
         <v>6.75</v>
@@ -54897,13 +54897,13 @@
         </is>
       </c>
       <c r="I504" s="4" t="n">
-        <v>3.12</v>
+        <v>3.16</v>
       </c>
       <c r="J504" s="4" t="n">
-        <v>71.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="K504" s="4" t="n">
-        <v>28.2</v>
+        <v>27.9</v>
       </c>
       <c r="L504" t="inlineStr">
         <is>
@@ -54911,13 +54911,13 @@
         </is>
       </c>
       <c r="M504" s="4" t="n">
-        <v>-9.56</v>
+        <v>-9.44</v>
       </c>
       <c r="N504" s="4" t="n">
         <v>6.75</v>
       </c>
       <c r="O504" s="4" t="n">
-        <v>0.39</v>
+        <v>0.5</v>
       </c>
       <c r="P504" s="4" t="n">
         <v>0.11</v>
@@ -54963,10 +54963,10 @@
         <v>0</v>
       </c>
       <c r="AC504" s="4" t="n">
-        <v>51.24</v>
+        <v>51.27</v>
       </c>
       <c r="AD504" s="4" t="n">
-        <v>48.15</v>
+        <v>48.12</v>
       </c>
       <c r="AE504" s="4" t="n">
         <v>0</v>
@@ -55441,7 +55441,7 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="K2" t="n">
         <v>17</v>
@@ -55453,7 +55453,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -55516,7 +55516,7 @@
         <v>10</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -57191,7 +57191,7 @@
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>50</v>
+        <v>50.1</v>
       </c>
       <c r="K32" t="n">
         <v>49</v>
@@ -57203,7 +57203,7 @@
         <v>70</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -59743,7 +59743,7 @@
         </is>
       </c>
       <c r="J76" s="4" t="n">
-        <v>72.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="K76" t="n">
         <v>70</v>
@@ -59755,7 +59755,7 @@
         <v>96</v>
       </c>
       <c r="N76" s="4" t="n">
-        <v>34.1</v>
+        <v>34.3</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -59813,7 +59813,7 @@
         <v>16</v>
       </c>
       <c r="N77" s="4" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-10-04 (adds Larsen for Congress UT-04 internal)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.3</v>
+        <v>52.4</v>
       </c>
       <c r="C8" t="n">
-        <v>47.7</v>
+        <v>47.6</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>68.90000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>242</v>
+        <v>241.9</v>
       </c>
       <c r="C9" t="n">
-        <v>193</v>
+        <v>193.1</v>
       </c>
       <c r="D9" t="n">
         <v>238</v>
       </c>
       <c r="E9" t="n">
-        <v>89.3</v>
+        <v>89</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.8</v>
+        <v>26.9</v>
       </c>
       <c r="C10" t="n">
-        <v>23.2</v>
+        <v>23.1</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>69.09999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -928,10 +928,10 @@
         <v>9.15</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>95.3</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4948,14 +4948,14 @@
         <v>-3.45</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>75</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M38" s="4" t="n">
@@ -5008,7 +5008,7 @@
         <v>44.97</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25781,10 +25781,10 @@
         <v>-0.37</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.5</v>
+        <v>45.6</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.5</v>
+        <v>54.4</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -47728,13 +47728,13 @@
         </is>
       </c>
       <c r="I439" s="4" t="n">
-        <v>-25.54</v>
+        <v>-19.1</v>
       </c>
       <c r="J439" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="K439" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>99.7</v>
       </c>
       <c r="L439" t="inlineStr">
         <is>
@@ -47760,16 +47760,16 @@
         <v>-33.43</v>
       </c>
       <c r="S439" s="4" t="n">
-        <v>32.9</v>
+        <v>37.85</v>
       </c>
       <c r="T439" s="4" t="n">
-        <v>41.7</v>
+        <v>36.12</v>
       </c>
       <c r="U439" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V439" s="4" t="n">
-        <v>-8.220000000000001</v>
+        <v>1.41</v>
       </c>
       <c r="W439" s="5" t="n">
         <v>53579</v>
@@ -47788,16 +47788,16 @@
         </is>
       </c>
       <c r="AA439" s="4" t="n">
-        <v>5.7</v>
+        <v>5.03</v>
       </c>
       <c r="AB439" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC439" s="4" t="n">
-        <v>32.5</v>
+        <v>35.58</v>
       </c>
       <c r="AD439" s="4" t="n">
-        <v>54.8</v>
+        <v>52.39</v>
       </c>
       <c r="AE439" s="4" t="n">
         <v>7</v>
@@ -52967,10 +52967,10 @@
         <v>1.88</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>62.9</v>
+        <v>63.2</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>37.1</v>
+        <v>36.8</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53412,7 +53412,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.57</v>
+        <v>-21.48</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53472,16 +53472,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.75</v>
+        <v>27.78</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.28</v>
+        <v>19.29</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.32</v>
+        <v>49.27</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-06 (rerun)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>69.7</v>
+        <v>70</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241.9</v>
+        <v>242.1</v>
       </c>
       <c r="C9" t="n">
-        <v>193.1</v>
+        <v>192.9</v>
       </c>
       <c r="D9" t="n">
         <v>238</v>
       </c>
       <c r="E9" t="n">
-        <v>88.40000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>68.40000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -928,10 +928,10 @@
         <v>9.130000000000001</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>95.5</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4948,10 +4948,10 @@
         <v>-3.32</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>26.2</v>
+        <v>25</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>73.8</v>
+        <v>75</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.03</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>26.2</v>
+        <v>25</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25781,10 +25781,10 @@
         <v>-0.38</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>48.3</v>
+        <v>47.1</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>51.7</v>
+        <v>52.9</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -51407,10 +51407,10 @@
         <v>2.75</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>70</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>30</v>
+        <v>29.6</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52973,10 +52973,10 @@
         <v>2.19</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>65.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53418,7 +53418,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.59</v>
+        <v>-21.56</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53478,16 +53478,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.72</v>
+        <v>27.77</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.3</v>
+        <v>19.24</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.31</v>
+        <v>49.33</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-11 (rerun: +3 race polls, refreshed fundraising)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>70.40000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>242.6</v>
+        <v>242.9</v>
       </c>
       <c r="C9" t="n">
-        <v>192.4</v>
+        <v>192.1</v>
       </c>
       <c r="D9" t="n">
         <v>239</v>
       </c>
       <c r="E9" t="n">
-        <v>89.40000000000001</v>
+        <v>89.8</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.9</v>
+        <v>27</v>
       </c>
       <c r="C10" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>68.7</v>
+        <v>69.7</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4945,13 +4945,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.3</v>
+        <v>-3.29</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>25.7</v>
+        <v>26.4</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>74.3</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4959,13 +4959,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.58</v>
+        <v>-2.56</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-0.6</v>
@@ -5005,16 +5005,16 @@
         </is>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>45.04</v>
+        <v>45.05</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>25.7</v>
+        <v>26.4</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
       </c>
       <c r="AD38" s="4" t="n">
-        <v>49.96</v>
+        <v>49.95</v>
       </c>
       <c r="AE38" s="4" t="n">
         <v>1.2</v>
@@ -22164,7 +22164,7 @@
         </is>
       </c>
       <c r="I201" s="4" t="n">
-        <v>-26.96</v>
+        <v>-26.92</v>
       </c>
       <c r="J201" s="4" t="n">
         <v>0</v>
@@ -22178,13 +22178,13 @@
         </is>
       </c>
       <c r="M201" s="4" t="n">
-        <v>-26.69</v>
+        <v>-26.65</v>
       </c>
       <c r="N201" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O201" s="4" t="n">
-        <v>-27.49</v>
+        <v>-27.45</v>
       </c>
       <c r="P201" s="4" t="n">
         <v>-2.06</v>
@@ -22224,10 +22224,10 @@
         <v>0</v>
       </c>
       <c r="AC201" s="4" t="n">
-        <v>35.54</v>
+        <v>35.56</v>
       </c>
       <c r="AD201" s="4" t="n">
-        <v>61.78</v>
+        <v>61.76</v>
       </c>
       <c r="AE201" s="4" t="n">
         <v>0</v>
@@ -22275,7 +22275,7 @@
         </is>
       </c>
       <c r="I202" s="4" t="n">
-        <v>-12.74</v>
+        <v>-12.7</v>
       </c>
       <c r="J202" s="4" t="n">
         <v>1</v>
@@ -22289,13 +22289,13 @@
         </is>
       </c>
       <c r="M202" s="4" t="n">
-        <v>-14.27</v>
+        <v>-14.22</v>
       </c>
       <c r="N202" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O202" s="4" t="n">
-        <v>-13.31</v>
+        <v>-13.27</v>
       </c>
       <c r="P202" s="4" t="n">
         <v>-0.47</v>
@@ -22335,10 +22335,10 @@
         <v>0</v>
       </c>
       <c r="AC202" s="4" t="n">
-        <v>42.39</v>
+        <v>42.41</v>
       </c>
       <c r="AD202" s="4" t="n">
-        <v>54.77</v>
+        <v>54.75</v>
       </c>
       <c r="AE202" s="4" t="n">
         <v>0</v>
@@ -22386,7 +22386,7 @@
         </is>
       </c>
       <c r="I203" s="4" t="n">
-        <v>26.04</v>
+        <v>26.09</v>
       </c>
       <c r="J203" s="4" t="n">
         <v>100</v>
@@ -22400,13 +22400,13 @@
         </is>
       </c>
       <c r="M203" s="4" t="n">
-        <v>8.710000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="N203" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O203" s="4" t="n">
-        <v>25.46</v>
+        <v>25.5</v>
       </c>
       <c r="P203" s="4" t="n">
         <v>3</v>
@@ -22446,10 +22446,10 @@
         <v>0</v>
       </c>
       <c r="AC203" s="4" t="n">
-        <v>61.17</v>
+        <v>61.19</v>
       </c>
       <c r="AD203" s="4" t="n">
-        <v>35.89</v>
+        <v>35.87</v>
       </c>
       <c r="AE203" s="4" t="n">
         <v>0</v>
@@ -22497,7 +22497,7 @@
         </is>
       </c>
       <c r="I204" s="4" t="n">
-        <v>-18.2</v>
+        <v>-18.15</v>
       </c>
       <c r="J204" s="4" t="n">
         <v>0.3</v>
@@ -22511,13 +22511,13 @@
         </is>
       </c>
       <c r="M204" s="4" t="n">
-        <v>-18.65</v>
+        <v>-18.61</v>
       </c>
       <c r="N204" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O204" s="4" t="n">
-        <v>-18.77</v>
+        <v>-18.73</v>
       </c>
       <c r="P204" s="4" t="n">
         <v>-1.43</v>
@@ -22557,10 +22557,10 @@
         <v>0</v>
       </c>
       <c r="AC204" s="4" t="n">
-        <v>39.72</v>
+        <v>39.74</v>
       </c>
       <c r="AD204" s="4" t="n">
-        <v>57.4</v>
+        <v>57.38</v>
       </c>
       <c r="AE204" s="4" t="n">
         <v>0</v>
@@ -25787,10 +25787,10 @@
         <v>-0.26</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.6</v>
+        <v>46.9</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.4</v>
+        <v>53.1</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -25913,7 +25913,7 @@
         <v>7.01</v>
       </c>
       <c r="O236" s="4" t="n">
-        <v>-10.84</v>
+        <v>-10.85</v>
       </c>
       <c r="P236" s="4" t="n">
         <v>-0.55</v>
@@ -26129,7 +26129,7 @@
         </is>
       </c>
       <c r="M238" s="4" t="n">
-        <v>11.73</v>
+        <v>11.72</v>
       </c>
       <c r="N238" s="4" t="n">
         <v>7.01</v>
@@ -26226,7 +26226,7 @@
         </is>
       </c>
       <c r="I239" s="4" t="n">
-        <v>-0.93</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="J239" s="4" t="n">
         <v>43.4</v>
@@ -26240,13 +26240,13 @@
         </is>
       </c>
       <c r="M239" s="4" t="n">
-        <v>-1.43</v>
+        <v>-1.44</v>
       </c>
       <c r="N239" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O239" s="4" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.08</v>
       </c>
       <c r="P239" s="4" t="n">
         <v>-0.2</v>
@@ -26363,7 +26363,7 @@
         <v>7.01</v>
       </c>
       <c r="O240" s="4" t="n">
-        <v>-23.62</v>
+        <v>-23.63</v>
       </c>
       <c r="P240" s="4" t="n">
         <v>-2.12</v>
@@ -26403,10 +26403,10 @@
         <v>0</v>
       </c>
       <c r="AC240" s="4" t="n">
-        <v>36.53</v>
+        <v>36.52</v>
       </c>
       <c r="AD240" s="4" t="n">
-        <v>59.25</v>
+        <v>59.26</v>
       </c>
       <c r="AE240" s="4" t="n">
         <v>2.11</v>
@@ -26454,7 +26454,7 @@
         </is>
       </c>
       <c r="I241" s="4" t="n">
-        <v>40.41</v>
+        <v>40.4</v>
       </c>
       <c r="J241" s="4" t="n">
         <v>100</v>
@@ -26474,7 +26474,7 @@
         <v>7.01</v>
       </c>
       <c r="O241" s="4" t="n">
-        <v>40.54</v>
+        <v>40.53</v>
       </c>
       <c r="P241" s="4" t="n">
         <v>0</v>
@@ -26579,7 +26579,7 @@
         </is>
       </c>
       <c r="M242" s="4" t="n">
-        <v>3.11</v>
+        <v>3.1</v>
       </c>
       <c r="N242" s="4" t="n">
         <v>7.01</v>
@@ -26631,10 +26631,10 @@
         <v>0</v>
       </c>
       <c r="AC242" s="4" t="n">
-        <v>50.6</v>
+        <v>50.59</v>
       </c>
       <c r="AD242" s="4" t="n">
-        <v>47.13</v>
+        <v>47.14</v>
       </c>
       <c r="AE242" s="4" t="n">
         <v>0</v>
@@ -26793,7 +26793,7 @@
         </is>
       </c>
       <c r="I244" s="4" t="n">
-        <v>-30.73</v>
+        <v>-30.74</v>
       </c>
       <c r="J244" s="4" t="n">
         <v>0</v>
@@ -27027,7 +27027,7 @@
         </is>
       </c>
       <c r="M246" s="4" t="n">
-        <v>21.17</v>
+        <v>21.16</v>
       </c>
       <c r="N246" s="4" t="n">
         <v>7.01</v>
@@ -27124,7 +27124,7 @@
         </is>
       </c>
       <c r="I247" s="4" t="n">
-        <v>60.04</v>
+        <v>60.03</v>
       </c>
       <c r="J247" s="4" t="n">
         <v>100</v>
@@ -27231,7 +27231,7 @@
         </is>
       </c>
       <c r="I248" s="4" t="n">
-        <v>55.17</v>
+        <v>55.16</v>
       </c>
       <c r="J248" s="4" t="n">
         <v>100</v>
@@ -27245,13 +27245,13 @@
         </is>
       </c>
       <c r="M248" s="4" t="n">
-        <v>48.71</v>
+        <v>48.7</v>
       </c>
       <c r="N248" s="4" t="n">
         <v>7.01</v>
       </c>
       <c r="O248" s="4" t="n">
-        <v>55.8</v>
+        <v>55.79</v>
       </c>
       <c r="P248" s="4" t="n">
         <v>0</v>
@@ -51416,13 +51416,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>2.46</v>
+        <v>2.57</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>68.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>31.8</v>
+        <v>30.9</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -51448,16 +51448,16 @@
         <v>-13.8</v>
       </c>
       <c r="S473" s="4" t="n">
-        <v>48.64</v>
+        <v>48.69</v>
       </c>
       <c r="T473" s="4" t="n">
-        <v>45.63</v>
+        <v>45.71</v>
       </c>
       <c r="U473" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="V473" s="4" t="n">
-        <v>3.78</v>
+        <v>3.82</v>
       </c>
       <c r="W473" s="5" t="n">
         <v>18545132</v>
@@ -51474,10 +51474,10 @@
         <v>0</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>49.55</v>
+        <v>49.61</v>
       </c>
       <c r="AD473" s="4" t="n">
-        <v>47.95</v>
+        <v>47.89</v>
       </c>
       <c r="AE473" s="4" t="n">
         <v>2.5</v>
@@ -52530,17 +52530,17 @@
         </is>
       </c>
       <c r="I483" s="4" t="n">
-        <v>-1.49</v>
+        <v>-1.28</v>
       </c>
       <c r="J483" s="4" t="n">
-        <v>39.4</v>
+        <v>40.9</v>
       </c>
       <c r="K483" s="4" t="n">
-        <v>60.6</v>
+        <v>59.1</v>
       </c>
       <c r="L483" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M483" s="4" t="n">
@@ -52562,16 +52562,16 @@
         <v>-16.41</v>
       </c>
       <c r="S483" s="4" t="n">
-        <v>46.47</v>
+        <v>46.49</v>
       </c>
       <c r="T483" s="4" t="n">
-        <v>45.07</v>
+        <v>45.1</v>
       </c>
       <c r="U483" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V483" s="4" t="n">
-        <v>1.39</v>
+        <v>1.43</v>
       </c>
       <c r="W483" s="5" t="n">
         <v>4169078</v>
@@ -52590,16 +52590,16 @@
         </is>
       </c>
       <c r="AA483" s="4" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="AB483" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC483" s="4" t="n">
-        <v>48.27</v>
+        <v>48.39</v>
       </c>
       <c r="AD483" s="4" t="n">
-        <v>49.74</v>
+        <v>49.65</v>
       </c>
       <c r="AE483" s="4" t="n">
         <v>0</v>
@@ -52985,10 +52985,10 @@
         <v>2.33</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.5</v>
+        <v>66.7</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.5</v>
+        <v>33.3</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53087,13 +53087,13 @@
         </is>
       </c>
       <c r="I488" s="4" t="n">
-        <v>5.91</v>
+        <v>5.88</v>
       </c>
       <c r="J488" s="4" t="n">
-        <v>84</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="K488" s="4" t="n">
-        <v>16</v>
+        <v>16.1</v>
       </c>
       <c r="L488" t="inlineStr">
         <is>
@@ -53119,16 +53119,16 @@
         <v>-1.44</v>
       </c>
       <c r="S488" s="4" t="n">
-        <v>48.78</v>
+        <v>48.77</v>
       </c>
       <c r="T488" s="4" t="n">
         <v>45.75</v>
       </c>
       <c r="U488" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="V488" s="4" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="W488" s="5" t="n">
         <v>14514336</v>
@@ -53153,10 +53153,10 @@
         <v>0</v>
       </c>
       <c r="AC488" s="4" t="n">
-        <v>51.46</v>
+        <v>51.45</v>
       </c>
       <c r="AD488" s="4" t="n">
-        <v>45.73</v>
+        <v>45.74</v>
       </c>
       <c r="AE488" s="4" t="n">
         <v>2.31</v>
@@ -53430,7 +53430,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.58</v>
+        <v>-21.67</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53490,16 +53490,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.73</v>
+        <v>27.69</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.3</v>
+        <v>19.28</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.31</v>
+        <v>49.37</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -58091,7 +58091,7 @@
         <v>55</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
2026-10-13: AK-01 borough/HD projections follow partisan lean (Hill no longer spread flat)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.3</v>
+        <v>52.4</v>
       </c>
       <c r="C8" t="n">
-        <v>47.7</v>
+        <v>47.6</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>68.8</v>
+        <v>69.8</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>243</v>
+        <v>242.9</v>
       </c>
       <c r="C9" t="n">
-        <v>192</v>
+        <v>192.1</v>
       </c>
       <c r="D9" t="n">
         <v>239</v>
       </c>
       <c r="E9" t="n">
-        <v>90.2</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>69.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4948,10 +4948,10 @@
         <v>-3.21</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>73.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.09</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25793,10 +25793,10 @@
         <v>-0.3</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.7</v>
+        <v>47.4</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.3</v>
+        <v>52.6</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -51425,10 +51425,10 @@
         <v>2.56</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>31.6</v>
+        <v>31.1</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52991,10 +52991,10 @@
         <v>2.3</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.09999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.9</v>
+        <v>33.7</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53436,7 +53436,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.77</v>
+        <v>-21.62</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53496,16 +53496,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.68</v>
+        <v>27.75</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.21</v>
+        <v>19.22</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.45</v>
+        <v>49.37</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -58097,7 +58097,7 @@
         <v>55</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-10-14 (VA-02 CNU poll)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>69.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>243.1</v>
+        <v>242.5</v>
       </c>
       <c r="C9" t="n">
-        <v>191.9</v>
+        <v>192.5</v>
       </c>
       <c r="D9" t="n">
         <v>239</v>
       </c>
       <c r="E9" t="n">
-        <v>90.8</v>
+        <v>90.3</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>69.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4948,10 +4948,10 @@
         <v>-3.11</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.5</v>
+        <v>27.8</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.5</v>
+        <v>72.2</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.13</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>28.5</v>
+        <v>27.8</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25793,10 +25793,10 @@
         <v>-0.3</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>48.2</v>
+        <v>47.5</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>51.8</v>
+        <v>52.5</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -47978,13 +47978,13 @@
         </is>
       </c>
       <c r="I441" s="4" t="n">
-        <v>6.71</v>
+        <v>5.84</v>
       </c>
       <c r="J441" s="4" t="n">
-        <v>86.59999999999999</v>
+        <v>83.7</v>
       </c>
       <c r="K441" s="4" t="n">
-        <v>13.4</v>
+        <v>16.3</v>
       </c>
       <c r="L441" t="inlineStr">
         <is>
@@ -48010,16 +48010,16 @@
         <v>-0.27</v>
       </c>
       <c r="S441" s="4" t="n">
-        <v>47</v>
+        <v>46.04</v>
       </c>
       <c r="T441" s="4" t="n">
-        <v>47</v>
+        <v>43.17</v>
       </c>
       <c r="U441" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V441" s="4" t="n">
-        <v>-0.68</v>
+        <v>2.85</v>
       </c>
       <c r="W441" s="5" t="n">
         <v>4659795</v>
@@ -48044,10 +48044,10 @@
         <v>0</v>
       </c>
       <c r="AC441" s="4" t="n">
-        <v>52.09</v>
+        <v>51.67</v>
       </c>
       <c r="AD441" s="4" t="n">
-        <v>45.55</v>
+        <v>45.97</v>
       </c>
       <c r="AE441" s="4" t="n">
         <v>0</v>
@@ -51431,10 +51431,10 @@
         <v>2.59</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>68.7</v>
+        <v>68</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>31.3</v>
+        <v>32</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52997,10 +52997,10 @@
         <v>2.33</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>34.6</v>
+        <v>33.6</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53442,7 +53442,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.69</v>
+        <v>-21.65</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53508,10 +53508,10 @@
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.24</v>
+        <v>19.28</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.39</v>
+        <v>49.36</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -58103,7 +58103,7 @@
         <v>55</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-10-14 (RI-GOV three-way: Block splits the anti-D vote)
RI-GOV now runs as a three-way plurality race (races.csv threeway=True).
Ken Block (IND) shares the anti-Democratic vote with a weak Republican, so
the model mirrors the MT-SEN three-way: Dem vs the R+IND coalition, split
by Block's polled share of it. Once polled three ways the split comes from
the polls (decided-normalised), not the D-vs-R fundamentals blend.
Today: Foulkes 49.8 / Block 35.5 / Guckian 14.7, D+14.2 over Block,
Block 3.7%. RI-GOV's timeline rebuilt from 2026-04-02 (Block's entry).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>69.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>242.5</v>
+        <v>242.9</v>
       </c>
       <c r="C9" t="n">
-        <v>192.5</v>
+        <v>192.1</v>
       </c>
       <c r="D9" t="n">
         <v>239</v>
       </c>
       <c r="E9" t="n">
-        <v>90.3</v>
+        <v>89.7</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>69.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -718,7 +718,7 @@
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="11" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
@@ -4053,10 +4053,10 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>26.34</v>
+        <v>14.25</v>
       </c>
       <c r="J30" s="4" t="n">
-        <v>100</v>
+        <v>99.2</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>0</v>
@@ -4094,7 +4094,7 @@
         <v>5</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>32.53</v>
+        <v>-0.8699999999999974</v>
       </c>
       <c r="W30" s="5" t="n">
         <v>0</v>
@@ -4113,16 +4113,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>30</v>
+        <v>35.48</v>
       </c>
       <c r="AB30" s="4" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>44.22</v>
+        <v>49.73</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>25.78</v>
+        <v>14.79</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4948,10 +4948,10 @@
         <v>-3.11</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>27.8</v>
+        <v>27.4</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>72.2</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>45.13</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>27.8</v>
+        <v>27.4</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25793,10 +25793,10 @@
         <v>-0.3</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>47.5</v>
+        <v>47.2</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>52.5</v>
+        <v>52.8</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -41358,7 +41358,7 @@
         </is>
       </c>
       <c r="I379" s="4" t="n">
-        <v>47.44</v>
+        <v>45.39</v>
       </c>
       <c r="J379" s="4" t="n">
         <v>100</v>
@@ -41372,13 +41372,13 @@
         </is>
       </c>
       <c r="M379" s="4" t="n">
-        <v>29.87</v>
+        <v>27.81</v>
       </c>
       <c r="N379" s="4" t="n">
         <v>7.07</v>
       </c>
       <c r="O379" s="4" t="n">
-        <v>47.6</v>
+        <v>45.54</v>
       </c>
       <c r="P379" s="4" t="n">
         <v>2.51</v>
@@ -41418,10 +41418,10 @@
         <v>0</v>
       </c>
       <c r="AC379" s="4" t="n">
-        <v>71.44</v>
+        <v>70.45</v>
       </c>
       <c r="AD379" s="4" t="n">
-        <v>25.47</v>
+        <v>26.46</v>
       </c>
       <c r="AE379" s="4" t="n">
         <v>0</v>
@@ -41469,13 +41469,13 @@
         </is>
       </c>
       <c r="I380" s="4" t="n">
-        <v>18.61</v>
+        <v>17.72</v>
       </c>
       <c r="J380" s="4" t="n">
-        <v>99.7</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="K380" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L380" t="inlineStr">
         <is>
@@ -41483,13 +41483,13 @@
         </is>
       </c>
       <c r="M380" s="4" t="n">
-        <v>14.01</v>
+        <v>11.96</v>
       </c>
       <c r="N380" s="4" t="n">
         <v>7.07</v>
       </c>
       <c r="O380" s="4" t="n">
-        <v>21.85</v>
+        <v>19.8</v>
       </c>
       <c r="P380" s="4" t="n">
         <v>-0.57</v>
@@ -41527,10 +41527,10 @@
         <v>0</v>
       </c>
       <c r="AC380" s="4" t="n">
-        <v>59.3</v>
+        <v>58.86</v>
       </c>
       <c r="AD380" s="4" t="n">
-        <v>40.7</v>
+        <v>41.14</v>
       </c>
       <c r="AE380" s="4" t="n">
         <v>0</v>
@@ -51431,10 +51431,10 @@
         <v>2.59</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>68</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>32</v>
+        <v>31.4</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52997,10 +52997,10 @@
         <v>2.33</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.40000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.6</v>
+        <v>33.5</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53442,7 +53442,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.65</v>
+        <v>-21.7</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53502,16 +53502,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.7</v>
+        <v>27.69</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.28</v>
+        <v>19.26</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.36</v>
+        <v>49.39</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -54463,7 +54463,7 @@
         </is>
       </c>
       <c r="I500" s="4" t="n">
-        <v>29.86</v>
+        <v>28.25</v>
       </c>
       <c r="J500" s="4" t="n">
         <v>100</v>
@@ -54477,13 +54477,13 @@
         </is>
       </c>
       <c r="M500" s="4" t="n">
-        <v>18.8</v>
+        <v>15.75</v>
       </c>
       <c r="N500" s="4" t="n">
         <v>7.07</v>
       </c>
       <c r="O500" s="4" t="n">
-        <v>29.36</v>
+        <v>26.31</v>
       </c>
       <c r="P500" s="4" t="n">
         <v>2.03</v>
@@ -54529,10 +54529,10 @@
         <v>0</v>
       </c>
       <c r="AC500" s="4" t="n">
-        <v>60.8</v>
+        <v>60.05</v>
       </c>
       <c r="AD500" s="4" t="n">
-        <v>32.84</v>
+        <v>33.59</v>
       </c>
       <c r="AE500" s="4" t="n">
         <v>0</v>
@@ -58103,7 +58103,7 @@
         <v>55</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -59367,19 +59367,19 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K69" t="n">
         <v>66</v>
       </c>
       <c r="L69" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="M69" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N69" s="4" t="n">
-        <v>99.5</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -59425,7 +59425,7 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>34.4</v>
+        <v>34.2</v>
       </c>
       <c r="K70" t="n">
         <v>35</v>
@@ -59437,7 +59437,7 @@
         <v>36</v>
       </c>
       <c r="N70" s="4" t="n">
-        <v>99.5</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
2026-10-15: add Cross Timbers OK-GOV poll (Oct 7-12, LV Mazzei 39 / Munson 36), rerun forecast
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.5</v>
+        <v>52.4</v>
       </c>
       <c r="C8" t="n">
-        <v>47.5</v>
+        <v>47.6</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>70.5</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>243.2</v>
+        <v>243.3</v>
       </c>
       <c r="C9" t="n">
-        <v>191.8</v>
+        <v>191.7</v>
       </c>
       <c r="D9" t="n">
         <v>239</v>
       </c>
       <c r="E9" t="n">
-        <v>90.09999999999999</v>
+        <v>90</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>70</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -3712,13 +3712,13 @@
         </is>
       </c>
       <c r="I27" s="4" t="n">
-        <v>-28.56</v>
+        <v>-14.37</v>
       </c>
       <c r="J27" s="4" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>100</v>
+        <v>99.2</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -3743,12 +3743,18 @@
       <c r="R27" s="4" t="n">
         <v>-34.95</v>
       </c>
-      <c r="S27" s="4" t="n"/>
-      <c r="T27" s="4" t="n"/>
+      <c r="S27" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="T27" s="4" t="n">
+        <v>39</v>
+      </c>
       <c r="U27" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V27" s="4" t="n">
+        <v>-3</v>
+      </c>
       <c r="W27" s="5" t="n">
         <v>0</v>
       </c>
@@ -3766,16 +3772,16 @@
         </is>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>2.62</v>
+        <v>7</v>
       </c>
       <c r="AB27" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>34.78</v>
+        <v>39.82</v>
       </c>
       <c r="AD27" s="4" t="n">
-        <v>62.6</v>
+        <v>53.18</v>
       </c>
       <c r="AE27" s="4" t="n">
         <v>0</v>
@@ -4053,7 +4059,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.26</v>
+        <v>14.3</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.2</v>
@@ -4119,10 +4125,10 @@
         <v>0.8</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.75</v>
+        <v>49.8</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>14.75</v>
+        <v>14.7</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4948,10 +4954,10 @@
         <v>-3.01</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28</v>
+        <v>28.7</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>72</v>
+        <v>71.3</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5008,7 +5014,7 @@
         <v>45.19</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>28</v>
+        <v>28.7</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25793,10 +25799,10 @@
         <v>-0.25</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>49</v>
+        <v>48.7</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>51</v>
+        <v>51.3</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -38412,13 +38418,13 @@
         </is>
       </c>
       <c r="I351" s="4" t="n">
-        <v>-15.3</v>
+        <v>-11.9</v>
       </c>
       <c r="J351" s="4" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="K351" s="4" t="n">
-        <v>99.40000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -38426,13 +38432,13 @@
         </is>
       </c>
       <c r="M351" s="4" t="n">
-        <v>-20.17</v>
+        <v>-16.77</v>
       </c>
       <c r="N351" s="4" t="n">
         <v>7.13</v>
       </c>
       <c r="O351" s="4" t="n">
-        <v>-15.3</v>
+        <v>-11.9</v>
       </c>
       <c r="P351" s="4" t="n">
         <v>-1.7</v>
@@ -38464,10 +38470,10 @@
         <v>0</v>
       </c>
       <c r="AC351" s="4" t="n">
-        <v>42.35</v>
+        <v>44.05</v>
       </c>
       <c r="AD351" s="4" t="n">
-        <v>57.65</v>
+        <v>55.95</v>
       </c>
       <c r="AE351" s="4" t="n">
         <v>0</v>
@@ -38515,7 +38521,7 @@
         </is>
       </c>
       <c r="I352" s="4" t="n">
-        <v>-49.2</v>
+        <v>-45.8</v>
       </c>
       <c r="J352" s="4" t="n">
         <v>0</v>
@@ -38529,13 +38535,13 @@
         </is>
       </c>
       <c r="M352" s="4" t="n">
-        <v>-53.44</v>
+        <v>-50.03</v>
       </c>
       <c r="N352" s="4" t="n">
         <v>7.13</v>
       </c>
       <c r="O352" s="4" t="n">
-        <v>-49.1</v>
+        <v>-45.69</v>
       </c>
       <c r="P352" s="4" t="n">
         <v>-1.2</v>
@@ -38575,10 +38581,10 @@
         <v>0</v>
       </c>
       <c r="AC352" s="4" t="n">
-        <v>24.87</v>
+        <v>26.54</v>
       </c>
       <c r="AD352" s="4" t="n">
-        <v>73.06</v>
+        <v>71.39</v>
       </c>
       <c r="AE352" s="4" t="n">
         <v>0</v>
@@ -38626,7 +38632,7 @@
         </is>
       </c>
       <c r="I353" s="4" t="n">
-        <v>-40.73</v>
+        <v>-37.33</v>
       </c>
       <c r="J353" s="4" t="n">
         <v>0</v>
@@ -38640,13 +38646,13 @@
         </is>
       </c>
       <c r="M353" s="4" t="n">
-        <v>-43.14</v>
+        <v>-39.74</v>
       </c>
       <c r="N353" s="4" t="n">
         <v>7.13</v>
       </c>
       <c r="O353" s="4" t="n">
-        <v>-40.73</v>
+        <v>-37.33</v>
       </c>
       <c r="P353" s="4" t="n">
         <v>0</v>
@@ -38678,10 +38684,10 @@
         <v>0</v>
       </c>
       <c r="AC353" s="4" t="n">
-        <v>29.64</v>
+        <v>31.34</v>
       </c>
       <c r="AD353" s="4" t="n">
-        <v>70.36</v>
+        <v>68.66</v>
       </c>
       <c r="AE353" s="4" t="n">
         <v>0</v>
@@ -38729,7 +38735,7 @@
         </is>
       </c>
       <c r="I354" s="4" t="n">
-        <v>-32.14</v>
+        <v>-28.73</v>
       </c>
       <c r="J354" s="4" t="n">
         <v>0</v>
@@ -38743,13 +38749,13 @@
         </is>
       </c>
       <c r="M354" s="4" t="n">
-        <v>-31.17</v>
+        <v>-27.76</v>
       </c>
       <c r="N354" s="4" t="n">
         <v>7.13</v>
       </c>
       <c r="O354" s="4" t="n">
-        <v>-32.01</v>
+        <v>-28.6</v>
       </c>
       <c r="P354" s="4" t="n">
         <v>-2.38</v>
@@ -38789,10 +38795,10 @@
         <v>0</v>
       </c>
       <c r="AC354" s="4" t="n">
-        <v>33.03</v>
+        <v>34.69</v>
       </c>
       <c r="AD354" s="4" t="n">
-        <v>64.31999999999999</v>
+        <v>62.66</v>
       </c>
       <c r="AE354" s="4" t="n">
         <v>0</v>
@@ -38840,27 +38846,27 @@
         </is>
       </c>
       <c r="I355" s="4" t="n">
-        <v>-11.57</v>
+        <v>-9.460000000000001</v>
       </c>
       <c r="J355" s="4" t="n">
-        <v>1.2</v>
+        <v>5.5</v>
       </c>
       <c r="K355" s="4" t="n">
-        <v>98.8</v>
+        <v>94.5</v>
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>Safe R</t>
+          <t>Likely R</t>
         </is>
       </c>
       <c r="M355" s="4" t="n">
-        <v>-16.93</v>
+        <v>-13.52</v>
       </c>
       <c r="N355" s="4" t="n">
         <v>7.13</v>
       </c>
       <c r="O355" s="4" t="n">
-        <v>-13.98</v>
+        <v>-10.57</v>
       </c>
       <c r="P355" s="4" t="n">
         <v>-0.7</v>
@@ -38906,10 +38912,10 @@
         <v>0</v>
       </c>
       <c r="AC355" s="4" t="n">
-        <v>42.87</v>
+        <v>43.9</v>
       </c>
       <c r="AD355" s="4" t="n">
-        <v>54.09</v>
+        <v>53.06</v>
       </c>
       <c r="AE355" s="4" t="n">
         <v>0</v>
@@ -51443,10 +51449,10 @@
         <v>2.64</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>67.8</v>
+        <v>69</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>32.2</v>
+        <v>31</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -53009,10 +53015,10 @@
         <v>2.39</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.5</v>
+        <v>67.8</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.5</v>
+        <v>32.2</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53454,7 +53460,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-21.72</v>
+        <v>-21.62</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53514,16 +53520,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>27.71</v>
+        <v>27.74</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>19.21</v>
+        <v>19.24</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>49.43</v>
+        <v>49.36</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -54247,7 +54253,7 @@
         </is>
       </c>
       <c r="I498" s="4" t="n">
-        <v>-30.33</v>
+        <v>-27.5</v>
       </c>
       <c r="J498" s="4" t="n">
         <v>0</v>
@@ -54261,13 +54267,13 @@
         </is>
       </c>
       <c r="M498" s="4" t="n">
-        <v>-33.26</v>
+        <v>-29.72</v>
       </c>
       <c r="N498" s="4" t="n">
         <v>7.13</v>
       </c>
       <c r="O498" s="4" t="n">
-        <v>-32.79</v>
+        <v>-29.25</v>
       </c>
       <c r="P498" s="4" t="n">
         <v>-3.18</v>
@@ -54313,10 +54319,10 @@
         <v>0</v>
       </c>
       <c r="AC498" s="4" t="n">
-        <v>32.53</v>
+        <v>33.85</v>
       </c>
       <c r="AD498" s="4" t="n">
-        <v>60.85</v>
+        <v>59.53</v>
       </c>
       <c r="AE498" s="4" t="n">
         <v>2.62</v>
@@ -58103,7 +58109,7 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>42.4</v>
+        <v>42.5</v>
       </c>
       <c r="K47" t="n">
         <v>43</v>
@@ -59031,19 +59037,19 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>22.9</v>
+        <v>23.5</v>
       </c>
       <c r="K63" t="n">
         <v>22</v>
       </c>
       <c r="L63" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M63" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N63" s="4" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -59089,7 +59095,7 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>8.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="K64" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
2026-10-16: MT-SEN feeds Montana's swing via (D+I)-R; repolarize MT-SEN local breakdown; rebuild MT-01/MT-02 timelines
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>70</v>
+        <v>69.8</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -572,10 +572,10 @@
         <v>190.8</v>
       </c>
       <c r="D9" t="n">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E9" t="n">
-        <v>90.7</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27.1</v>
+        <v>27</v>
       </c>
       <c r="C10" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>70.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>41.1</v>
+        <v>41.2</v>
       </c>
     </row>
     <row r="18">
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.37</v>
+        <v>14.3</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.2</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>35.45</v>
+        <v>35.52</v>
       </c>
       <c r="AB30" s="4" t="n">
         <v>0.8</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.82</v>
+        <v>49.81</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>14.73</v>
+        <v>14.67</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-2.9</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.9</v>
+        <v>28.4</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.09999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.24</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>28.9</v>
+        <v>28.4</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25805,10 +25805,10 @@
         <v>-0.13</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>48.5</v>
+        <v>49.1</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>51.5</v>
+        <v>50.9</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29530,27 +29530,27 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-1.88</v>
+        <v>0.7</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>36.7</v>
+        <v>55</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>63.3</v>
+        <v>45</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-10.96</v>
+        <v>-6.03</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>7.15</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-5.2</v>
+        <v>-0.27</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.41</v>
@@ -29596,10 +29596,10 @@
         <v>0</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>47.75</v>
+        <v>49.01</v>
       </c>
       <c r="AD269" s="4" t="n">
-        <v>49.59</v>
+        <v>48.33</v>
       </c>
       <c r="AE269" s="4" t="n">
         <v>0</v>
@@ -29647,13 +29647,13 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-27.33</v>
+        <v>-23.89</v>
       </c>
       <c r="J270" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K270" s="4" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L270" t="inlineStr">
         <is>
@@ -29661,13 +29661,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-29.92</v>
+        <v>-24.99</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>7.15</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-30.74</v>
+        <v>-25.8</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.65</v>
@@ -29713,10 +29713,10 @@
         <v>0</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>31.74</v>
+        <v>33.25</v>
       </c>
       <c r="AD270" s="4" t="n">
-        <v>55.62</v>
+        <v>54.11</v>
       </c>
       <c r="AE270" s="4" t="n">
         <v>3.64</v>
@@ -51455,10 +51455,10 @@
         <v>2.74</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>69.90000000000001</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>30.1</v>
+        <v>30.9</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -53021,10 +53021,10 @@
         <v>2.37</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.7</v>
+        <v>66.3</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.3</v>
+        <v>33.7</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53466,7 +53466,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-18.61</v>
+        <v>-18.57</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53526,16 +53526,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>29.96</v>
+        <v>30.02</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.3</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>17.81</v>
+        <v>17.73</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>48.57</v>
+        <v>48.59</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -58115,19 +58115,19 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>42.9</v>
+        <v>44.6</v>
       </c>
       <c r="K47" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L47" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="M47" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>12.8</v>
+        <v>18.4</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -58173,10 +58173,10 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>19.9</v>
+        <v>20.4</v>
       </c>
       <c r="K48" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L48" t="n">
         <v>16</v>
@@ -58185,7 +58185,7 @@
         <v>24</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Forecast update 2026-10-16 (rerun)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>53</v>
       </c>
       <c r="E8" t="n">
-        <v>69.8</v>
+        <v>70.5</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>244.2</v>
+        <v>243.9</v>
       </c>
       <c r="C9" t="n">
-        <v>190.8</v>
+        <v>191.1</v>
       </c>
       <c r="D9" t="n">
         <v>240</v>
       </c>
       <c r="E9" t="n">
-        <v>90.40000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>70.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.3</v>
+        <v>14.29</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.2</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>35.52</v>
+        <v>35.5</v>
       </c>
       <c r="AB30" s="4" t="n">
         <v>0.8</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.81</v>
+        <v>49.79</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>14.67</v>
+        <v>14.71</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-2.9</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.4</v>
+        <v>29.3</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.24</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>28.4</v>
+        <v>29.3</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25805,10 +25805,10 @@
         <v>-0.13</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>49.1</v>
+        <v>49.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>50.9</v>
+        <v>50.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29530,13 +29530,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>55</v>
+        <v>54.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -29544,13 +29544,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-6.03</v>
+        <v>-6.05</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>7.15</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-0.27</v>
+        <v>-0.29</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.41</v>
@@ -29596,10 +29596,10 @@
         <v>0</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>49.01</v>
+        <v>49</v>
       </c>
       <c r="AD269" s="4" t="n">
-        <v>48.33</v>
+        <v>48.34</v>
       </c>
       <c r="AE269" s="4" t="n">
         <v>0</v>
@@ -29647,7 +29647,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-23.89</v>
+        <v>-23.91</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0.1</v>
@@ -29661,13 +29661,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-24.99</v>
+        <v>-25.02</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>7.15</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-25.8</v>
+        <v>-25.83</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.65</v>
@@ -29713,10 +29713,10 @@
         <v>0</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>33.25</v>
+        <v>33.24</v>
       </c>
       <c r="AD270" s="4" t="n">
-        <v>54.11</v>
+        <v>54.12</v>
       </c>
       <c r="AE270" s="4" t="n">
         <v>3.64</v>
@@ -51455,10 +51455,10 @@
         <v>2.74</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>69.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>30.9</v>
+        <v>30.1</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -53021,10 +53021,10 @@
         <v>2.37</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.3</v>
+        <v>65.5</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.7</v>
+        <v>34.5</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53466,7 +53466,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-18.57</v>
+        <v>-18.71</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53526,16 +53526,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>30.02</v>
+        <v>29.93</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.3</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>17.73</v>
+        <v>17.76</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>48.59</v>
+        <v>48.64</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-20 (rerun)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,10 +541,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.7</v>
+        <v>52.6</v>
       </c>
       <c r="C8" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="D8" t="n">
         <v>53</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>244.7</v>
+        <v>245.2</v>
       </c>
       <c r="C9" t="n">
-        <v>190.3</v>
+        <v>189.8</v>
       </c>
       <c r="D9" t="n">
         <v>243</v>
       </c>
       <c r="E9" t="n">
-        <v>91</v>
+        <v>91.5</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>72.7</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.41</v>
+        <v>14.38</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.2</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>35.11</v>
+        <v>35.09</v>
       </c>
       <c r="AB30" s="4" t="n">
         <v>0.8</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.52</v>
+        <v>49.48</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>15.37</v>
+        <v>15.43</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-2.5</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>32.4</v>
+        <v>31.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.43</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>32.4</v>
+        <v>31.1</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -51455,10 +51455,10 @@
         <v>2.84</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>70</v>
+        <v>70.2</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>30</v>
+        <v>29.8</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -53021,10 +53021,10 @@
         <v>2.49</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>32.6</v>
+        <v>32.3</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53466,7 +53466,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-20.86</v>
+        <v>-20.87</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-21: refresh governor fundraising (TUSA)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -575,7 +575,7 @@
         <v>244</v>
       </c>
       <c r="E9" t="n">
-        <v>92.3</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27.2</v>
+        <v>27.3</v>
       </c>
       <c r="C10" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>72.7</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>20.52</v>
+        <v>20.45</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>99.8</v>
@@ -1494,10 +1494,10 @@
         <v>7.57</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>19.67</v>
+        <v>19.6</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.64</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q7" s="4" t="n">
         <v>0</v>
@@ -1518,10 +1518,10 @@
         <v>17.5</v>
       </c>
       <c r="W7" s="5" t="n">
-        <v>6951032</v>
+        <v>8740361</v>
       </c>
       <c r="X7" s="5" t="n">
-        <v>2935521</v>
+        <v>4115917</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -1540,10 +1540,10 @@
         <v>0</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>58.09</v>
+        <v>58.06</v>
       </c>
       <c r="AD7" s="4" t="n">
-        <v>38.31</v>
+        <v>38.34</v>
       </c>
       <c r="AE7" s="4" t="n">
         <v>0</v>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="I14" s="4" t="n">
-        <v>20.52</v>
+        <v>21.09</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>99.8</v>
@@ -2263,10 +2263,10 @@
         <v>7.57</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>22.3</v>
+        <v>23.15</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1.84</v>
+        <v>2.69</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>-0.02</v>
@@ -2287,10 +2287,10 @@
         <v>17.74</v>
       </c>
       <c r="W14" s="5" t="n">
-        <v>25619035</v>
+        <v>91778931</v>
       </c>
       <c r="X14" s="5" t="n">
-        <v>2166962</v>
+        <v>2501525</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
@@ -2309,10 +2309,10 @@
         <v>0</v>
       </c>
       <c r="AC14" s="4" t="n">
-        <v>56.65</v>
+        <v>56.92</v>
       </c>
       <c r="AD14" s="4" t="n">
-        <v>37.36</v>
+        <v>37.09</v>
       </c>
       <c r="AE14" s="4" t="n">
         <v>0</v>
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.67</v>
+        <v>14.63</v>
       </c>
       <c r="J30" s="4" t="n">
-        <v>99.2</v>
+        <v>99.3</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>0</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>34.99</v>
+        <v>34.96</v>
       </c>
       <c r="AB30" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.66</v>
+        <v>49.6</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>15.36</v>
+        <v>15.44</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-2.51</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>32.5</v>
+        <v>30.9</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>67.5</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.46</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>32.5</v>
+        <v>30.9</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -12552,7 +12552,7 @@
         </is>
       </c>
       <c r="I111" s="4" t="n">
-        <v>73.7</v>
+        <v>73.69</v>
       </c>
       <c r="J111" s="4" t="n">
         <v>100</v>
@@ -12566,13 +12566,13 @@
         </is>
       </c>
       <c r="M111" s="4" t="n">
-        <v>64.01000000000001</v>
+        <v>64</v>
       </c>
       <c r="N111" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O111" s="4" t="n">
-        <v>73.2</v>
+        <v>73.18000000000001</v>
       </c>
       <c r="P111" s="4" t="n">
         <v>1.28</v>
@@ -12612,10 +12612,10 @@
         <v>0</v>
       </c>
       <c r="AC111" s="4" t="n">
-        <v>81.02</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="AD111" s="4" t="n">
-        <v>12.26</v>
+        <v>12.27</v>
       </c>
       <c r="AE111" s="4" t="n">
         <v>3.36</v>
@@ -12663,7 +12663,7 @@
         </is>
       </c>
       <c r="I112" s="4" t="n">
-        <v>56.34</v>
+        <v>56.32</v>
       </c>
       <c r="J112" s="4" t="n">
         <v>100</v>
@@ -12677,13 +12677,13 @@
         </is>
       </c>
       <c r="M112" s="4" t="n">
-        <v>45.75</v>
+        <v>45.73</v>
       </c>
       <c r="N112" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O112" s="4" t="n">
-        <v>55.61</v>
+        <v>55.59</v>
       </c>
       <c r="P112" s="4" t="n">
         <v>0</v>
@@ -12723,10 +12723,10 @@
         <v>0</v>
       </c>
       <c r="AC112" s="4" t="n">
-        <v>75.31999999999999</v>
+        <v>75.31</v>
       </c>
       <c r="AD112" s="4" t="n">
-        <v>21.03</v>
+        <v>21.04</v>
       </c>
       <c r="AE112" s="4" t="n">
         <v>0</v>
@@ -12774,13 +12774,13 @@
         </is>
       </c>
       <c r="I113" s="4" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="J113" s="4" t="n">
-        <v>66.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="K113" s="4" t="n">
-        <v>33.9</v>
+        <v>34</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -12788,13 +12788,13 @@
         </is>
       </c>
       <c r="M113" s="4" t="n">
-        <v>-4.71</v>
+        <v>-4.73</v>
       </c>
       <c r="N113" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O113" s="4" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="P113" s="4" t="n">
         <v>-0.83</v>
@@ -12840,10 +12840,10 @@
         <v>0</v>
       </c>
       <c r="AC113" s="4" t="n">
-        <v>49.47</v>
+        <v>49.46</v>
       </c>
       <c r="AD113" s="4" t="n">
-        <v>47.25</v>
+        <v>47.26</v>
       </c>
       <c r="AE113" s="4" t="n">
         <v>0</v>
@@ -12891,13 +12891,13 @@
         </is>
       </c>
       <c r="I114" s="4" t="n">
-        <v>-2.03</v>
+        <v>-2.04</v>
       </c>
       <c r="J114" s="4" t="n">
-        <v>35.7</v>
+        <v>35.6</v>
       </c>
       <c r="K114" s="4" t="n">
-        <v>64.3</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -12905,13 +12905,13 @@
         </is>
       </c>
       <c r="M114" s="4" t="n">
-        <v>-14.21</v>
+        <v>-14.23</v>
       </c>
       <c r="N114" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O114" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.93</v>
       </c>
       <c r="P114" s="4" t="n">
         <v>1.67</v>
@@ -12957,10 +12957,10 @@
         <v>0</v>
       </c>
       <c r="AC114" s="4" t="n">
-        <v>44.58</v>
+        <v>44.57</v>
       </c>
       <c r="AD114" s="4" t="n">
-        <v>46.42</v>
+        <v>46.43</v>
       </c>
       <c r="AE114" s="4" t="n">
         <v>0</v>
@@ -13008,13 +13008,13 @@
         </is>
       </c>
       <c r="I115" s="4" t="n">
-        <v>-3.44</v>
+        <v>-3.45</v>
       </c>
       <c r="J115" s="4" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="K115" s="4" t="n">
-        <v>74</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -13022,13 +13022,13 @@
         </is>
       </c>
       <c r="M115" s="4" t="n">
-        <v>-5.26</v>
+        <v>-5.27</v>
       </c>
       <c r="N115" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O115" s="4" t="n">
-        <v>-3.78</v>
+        <v>-3.8</v>
       </c>
       <c r="P115" s="4" t="n">
         <v>0.25</v>
@@ -13074,10 +13074,10 @@
         <v>0</v>
       </c>
       <c r="AC115" s="4" t="n">
-        <v>46.07</v>
+        <v>46.06</v>
       </c>
       <c r="AD115" s="4" t="n">
-        <v>49.35</v>
+        <v>49.36</v>
       </c>
       <c r="AE115" s="4" t="n">
         <v>4.08</v>
@@ -13125,7 +13125,7 @@
         </is>
       </c>
       <c r="I116" s="4" t="n">
-        <v>37.01</v>
+        <v>36.99</v>
       </c>
       <c r="J116" s="4" t="n">
         <v>100</v>
@@ -13139,13 +13139,13 @@
         </is>
       </c>
       <c r="M116" s="4" t="n">
-        <v>26.03</v>
+        <v>26.01</v>
       </c>
       <c r="N116" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O116" s="4" t="n">
-        <v>36.46</v>
+        <v>36.44</v>
       </c>
       <c r="P116" s="4" t="n">
         <v>0</v>
@@ -13185,10 +13185,10 @@
         <v>0</v>
       </c>
       <c r="AC116" s="4" t="n">
-        <v>63.44</v>
+        <v>63.43</v>
       </c>
       <c r="AD116" s="4" t="n">
-        <v>29.16</v>
+        <v>29.17</v>
       </c>
       <c r="AE116" s="4" t="n">
         <v>3.7</v>
@@ -13236,7 +13236,7 @@
         </is>
       </c>
       <c r="I117" s="4" t="n">
-        <v>32.58</v>
+        <v>32.57</v>
       </c>
       <c r="J117" s="4" t="n">
         <v>100</v>
@@ -13250,13 +13250,13 @@
         </is>
       </c>
       <c r="M117" s="4" t="n">
-        <v>19.75</v>
+        <v>19.74</v>
       </c>
       <c r="N117" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O117" s="4" t="n">
-        <v>32.02</v>
+        <v>32.01</v>
       </c>
       <c r="P117" s="4" t="n">
         <v>2.03</v>
@@ -13347,7 +13347,7 @@
         </is>
       </c>
       <c r="I118" s="4" t="n">
-        <v>9.42</v>
+        <v>9.41</v>
       </c>
       <c r="J118" s="4" t="n">
         <v>94.40000000000001</v>
@@ -13361,13 +13361,13 @@
         </is>
       </c>
       <c r="M118" s="4" t="n">
-        <v>4.66</v>
+        <v>4.65</v>
       </c>
       <c r="N118" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O118" s="4" t="n">
-        <v>11.66</v>
+        <v>11.64</v>
       </c>
       <c r="P118" s="4" t="n">
         <v>0.33</v>
@@ -13413,10 +13413,10 @@
         <v>0</v>
       </c>
       <c r="AC118" s="4" t="n">
-        <v>52.68</v>
+        <v>52.67</v>
       </c>
       <c r="AD118" s="4" t="n">
-        <v>43.6</v>
+        <v>43.61</v>
       </c>
       <c r="AE118" s="4" t="n">
         <v>0</v>
@@ -19492,7 +19492,7 @@
         </is>
       </c>
       <c r="I175" s="4" t="n">
-        <v>48.57</v>
+        <v>48.7</v>
       </c>
       <c r="J175" s="4" t="n">
         <v>100</v>
@@ -19506,13 +19506,13 @@
         </is>
       </c>
       <c r="M175" s="4" t="n">
-        <v>38.92</v>
+        <v>39.05</v>
       </c>
       <c r="N175" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O175" s="4" t="n">
-        <v>48.57</v>
+        <v>48.7</v>
       </c>
       <c r="P175" s="4" t="n">
         <v>1.09</v>
@@ -19544,10 +19544,10 @@
         <v>0</v>
       </c>
       <c r="AC175" s="4" t="n">
-        <v>74.29000000000001</v>
+        <v>74.34999999999999</v>
       </c>
       <c r="AD175" s="4" t="n">
-        <v>25.71</v>
+        <v>25.65</v>
       </c>
       <c r="AE175" s="4" t="n">
         <v>0</v>
@@ -19591,7 +19591,7 @@
         </is>
       </c>
       <c r="I176" s="4" t="n">
-        <v>46.99</v>
+        <v>47.12</v>
       </c>
       <c r="J176" s="4" t="n">
         <v>100</v>
@@ -19605,13 +19605,13 @@
         </is>
       </c>
       <c r="M176" s="4" t="n">
-        <v>39.06</v>
+        <v>39.19</v>
       </c>
       <c r="N176" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O176" s="4" t="n">
-        <v>46.99</v>
+        <v>47.12</v>
       </c>
       <c r="P176" s="4" t="n">
         <v>0</v>
@@ -19643,10 +19643,10 @@
         <v>0</v>
       </c>
       <c r="AC176" s="4" t="n">
-        <v>73.48999999999999</v>
+        <v>73.56</v>
       </c>
       <c r="AD176" s="4" t="n">
-        <v>26.51</v>
+        <v>26.44</v>
       </c>
       <c r="AE176" s="4" t="n">
         <v>0</v>
@@ -19694,7 +19694,7 @@
         </is>
       </c>
       <c r="I177" s="4" t="n">
-        <v>52.52</v>
+        <v>52.65</v>
       </c>
       <c r="J177" s="4" t="n">
         <v>100</v>
@@ -19708,13 +19708,13 @@
         </is>
       </c>
       <c r="M177" s="4" t="n">
-        <v>38.26</v>
+        <v>38.39</v>
       </c>
       <c r="N177" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O177" s="4" t="n">
-        <v>52.52</v>
+        <v>52.65</v>
       </c>
       <c r="P177" s="4" t="n">
         <v>2.48</v>
@@ -19746,10 +19746,10 @@
         <v>0</v>
       </c>
       <c r="AC177" s="4" t="n">
-        <v>76.26000000000001</v>
+        <v>76.33</v>
       </c>
       <c r="AD177" s="4" t="n">
-        <v>23.74</v>
+        <v>23.67</v>
       </c>
       <c r="AE177" s="4" t="n">
         <v>0</v>
@@ -19793,7 +19793,7 @@
         </is>
       </c>
       <c r="I178" s="4" t="n">
-        <v>41.91</v>
+        <v>42.02</v>
       </c>
       <c r="J178" s="4" t="n">
         <v>100</v>
@@ -19807,13 +19807,13 @@
         </is>
       </c>
       <c r="M178" s="4" t="n">
-        <v>37.35</v>
+        <v>37.48</v>
       </c>
       <c r="N178" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O178" s="4" t="n">
-        <v>47.15</v>
+        <v>47.28</v>
       </c>
       <c r="P178" s="4" t="n">
         <v>0</v>
@@ -19859,10 +19859,10 @@
         <v>0</v>
       </c>
       <c r="AC178" s="4" t="n">
-        <v>62.55</v>
+        <v>62.59</v>
       </c>
       <c r="AD178" s="4" t="n">
-        <v>25.6</v>
+        <v>25.56</v>
       </c>
       <c r="AE178" s="4" t="n">
         <v>2.85</v>
@@ -19910,7 +19910,7 @@
         </is>
       </c>
       <c r="I179" s="4" t="n">
-        <v>50.78</v>
+        <v>50.91</v>
       </c>
       <c r="J179" s="4" t="n">
         <v>100</v>
@@ -19924,13 +19924,13 @@
         </is>
       </c>
       <c r="M179" s="4" t="n">
-        <v>41.78</v>
+        <v>41.91</v>
       </c>
       <c r="N179" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O179" s="4" t="n">
-        <v>50.78</v>
+        <v>50.91</v>
       </c>
       <c r="P179" s="4" t="n">
         <v>0</v>
@@ -19962,10 +19962,10 @@
         <v>0</v>
       </c>
       <c r="AC179" s="4" t="n">
-        <v>75.39</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="AD179" s="4" t="n">
-        <v>24.61</v>
+        <v>24.54</v>
       </c>
       <c r="AE179" s="4" t="n">
         <v>0</v>
@@ -20013,7 +20013,7 @@
         </is>
       </c>
       <c r="I180" s="4" t="n">
-        <v>22.23</v>
+        <v>22.36</v>
       </c>
       <c r="J180" s="4" t="n">
         <v>99.90000000000001</v>
@@ -20027,13 +20027,13 @@
         </is>
       </c>
       <c r="M180" s="4" t="n">
-        <v>10.3</v>
+        <v>10.43</v>
       </c>
       <c r="N180" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O180" s="4" t="n">
-        <v>22.23</v>
+        <v>22.36</v>
       </c>
       <c r="P180" s="4" t="n">
         <v>1.39</v>
@@ -20065,10 +20065,10 @@
         <v>0</v>
       </c>
       <c r="AC180" s="4" t="n">
-        <v>61.12</v>
+        <v>61.18</v>
       </c>
       <c r="AD180" s="4" t="n">
-        <v>38.88</v>
+        <v>38.82</v>
       </c>
       <c r="AE180" s="4" t="n">
         <v>0</v>
@@ -20112,7 +20112,7 @@
         </is>
       </c>
       <c r="I181" s="4" t="n">
-        <v>77.81</v>
+        <v>77.94</v>
       </c>
       <c r="J181" s="4" t="n">
         <v>100</v>
@@ -20126,13 +20126,13 @@
         </is>
       </c>
       <c r="M181" s="4" t="n">
-        <v>71.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="N181" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O181" s="4" t="n">
-        <v>77.81</v>
+        <v>77.94</v>
       </c>
       <c r="P181" s="4" t="n">
         <v>-0.07000000000000001</v>
@@ -20164,10 +20164,10 @@
         <v>0</v>
       </c>
       <c r="AC181" s="4" t="n">
-        <v>88.91</v>
+        <v>88.97</v>
       </c>
       <c r="AD181" s="4" t="n">
-        <v>11.09</v>
+        <v>11.03</v>
       </c>
       <c r="AE181" s="4" t="n">
         <v>0</v>
@@ -20211,7 +20211,7 @@
         </is>
       </c>
       <c r="I182" s="4" t="n">
-        <v>21.11</v>
+        <v>21.24</v>
       </c>
       <c r="J182" s="4" t="n">
         <v>99.8</v>
@@ -20225,13 +20225,13 @@
         </is>
       </c>
       <c r="M182" s="4" t="n">
-        <v>12.71</v>
+        <v>12.84</v>
       </c>
       <c r="N182" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O182" s="4" t="n">
-        <v>21.11</v>
+        <v>21.24</v>
       </c>
       <c r="P182" s="4" t="n">
         <v>0.75</v>
@@ -20263,10 +20263,10 @@
         <v>0</v>
       </c>
       <c r="AC182" s="4" t="n">
-        <v>60.56</v>
+        <v>60.62</v>
       </c>
       <c r="AD182" s="4" t="n">
-        <v>39.44</v>
+        <v>39.38</v>
       </c>
       <c r="AE182" s="4" t="n">
         <v>0</v>
@@ -20310,7 +20310,7 @@
         </is>
       </c>
       <c r="I183" s="4" t="n">
-        <v>49.22</v>
+        <v>49.35</v>
       </c>
       <c r="J183" s="4" t="n">
         <v>100</v>
@@ -20324,13 +20324,13 @@
         </is>
       </c>
       <c r="M183" s="4" t="n">
-        <v>41.97</v>
+        <v>42.1</v>
       </c>
       <c r="N183" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O183" s="4" t="n">
-        <v>49.22</v>
+        <v>49.35</v>
       </c>
       <c r="P183" s="4" t="n">
         <v>0</v>
@@ -20362,10 +20362,10 @@
         <v>0</v>
       </c>
       <c r="AC183" s="4" t="n">
-        <v>74.61</v>
+        <v>74.67</v>
       </c>
       <c r="AD183" s="4" t="n">
-        <v>25.39</v>
+        <v>25.33</v>
       </c>
       <c r="AE183" s="4" t="n">
         <v>0</v>
@@ -20413,7 +20413,7 @@
         </is>
       </c>
       <c r="I184" s="4" t="n">
-        <v>35.39</v>
+        <v>35.52</v>
       </c>
       <c r="J184" s="4" t="n">
         <v>100</v>
@@ -20427,13 +20427,13 @@
         </is>
       </c>
       <c r="M184" s="4" t="n">
-        <v>26.65</v>
+        <v>26.78</v>
       </c>
       <c r="N184" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O184" s="4" t="n">
-        <v>35.39</v>
+        <v>35.52</v>
       </c>
       <c r="P184" s="4" t="n">
         <v>0</v>
@@ -20465,10 +20465,10 @@
         <v>0</v>
       </c>
       <c r="AC184" s="4" t="n">
-        <v>67.69</v>
+        <v>67.76000000000001</v>
       </c>
       <c r="AD184" s="4" t="n">
-        <v>32.31</v>
+        <v>32.24</v>
       </c>
       <c r="AE184" s="4" t="n">
         <v>0</v>
@@ -20516,7 +20516,7 @@
         </is>
       </c>
       <c r="I185" s="4" t="n">
-        <v>26.79</v>
+        <v>26.92</v>
       </c>
       <c r="J185" s="4" t="n">
         <v>100</v>
@@ -20530,13 +20530,13 @@
         </is>
       </c>
       <c r="M185" s="4" t="n">
-        <v>15.74</v>
+        <v>15.87</v>
       </c>
       <c r="N185" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O185" s="4" t="n">
-        <v>26.79</v>
+        <v>26.92</v>
       </c>
       <c r="P185" s="4" t="n">
         <v>1.28</v>
@@ -20568,10 +20568,10 @@
         <v>0</v>
       </c>
       <c r="AC185" s="4" t="n">
-        <v>63.4</v>
+        <v>63.46</v>
       </c>
       <c r="AD185" s="4" t="n">
-        <v>36.6</v>
+        <v>36.54</v>
       </c>
       <c r="AE185" s="4" t="n">
         <v>0</v>
@@ -20619,7 +20619,7 @@
         </is>
       </c>
       <c r="I186" s="4" t="n">
-        <v>-39.55</v>
+        <v>-39.42</v>
       </c>
       <c r="J186" s="4" t="n">
         <v>0</v>
@@ -20633,13 +20633,13 @@
         </is>
       </c>
       <c r="M186" s="4" t="n">
-        <v>-40.65</v>
+        <v>-40.52</v>
       </c>
       <c r="N186" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O186" s="4" t="n">
-        <v>-39.55</v>
+        <v>-39.42</v>
       </c>
       <c r="P186" s="4" t="n">
         <v>-1.55</v>
@@ -20671,10 +20671,10 @@
         <v>0</v>
       </c>
       <c r="AC186" s="4" t="n">
-        <v>30.22</v>
+        <v>30.29</v>
       </c>
       <c r="AD186" s="4" t="n">
-        <v>69.78</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="AE186" s="4" t="n">
         <v>0</v>
@@ -20722,7 +20722,7 @@
         </is>
       </c>
       <c r="I187" s="4" t="n">
-        <v>28.79</v>
+        <v>28.92</v>
       </c>
       <c r="J187" s="4" t="n">
         <v>100</v>
@@ -20736,13 +20736,13 @@
         </is>
       </c>
       <c r="M187" s="4" t="n">
-        <v>14.1</v>
+        <v>14.23</v>
       </c>
       <c r="N187" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O187" s="4" t="n">
-        <v>28.79</v>
+        <v>28.92</v>
       </c>
       <c r="P187" s="4" t="n">
         <v>1.42</v>
@@ -20774,10 +20774,10 @@
         <v>0</v>
       </c>
       <c r="AC187" s="4" t="n">
-        <v>64.39</v>
+        <v>64.45999999999999</v>
       </c>
       <c r="AD187" s="4" t="n">
-        <v>35.61</v>
+        <v>35.54</v>
       </c>
       <c r="AE187" s="4" t="n">
         <v>0</v>
@@ -20825,7 +20825,7 @@
         </is>
       </c>
       <c r="I188" s="4" t="n">
-        <v>25.43</v>
+        <v>25.56</v>
       </c>
       <c r="J188" s="4" t="n">
         <v>99.90000000000001</v>
@@ -20839,13 +20839,13 @@
         </is>
       </c>
       <c r="M188" s="4" t="n">
-        <v>10.13</v>
+        <v>10.26</v>
       </c>
       <c r="N188" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O188" s="4" t="n">
-        <v>25.43</v>
+        <v>25.56</v>
       </c>
       <c r="P188" s="4" t="n">
         <v>1.83</v>
@@ -20877,10 +20877,10 @@
         <v>0</v>
       </c>
       <c r="AC188" s="4" t="n">
-        <v>62.72</v>
+        <v>62.78</v>
       </c>
       <c r="AD188" s="4" t="n">
-        <v>37.28</v>
+        <v>37.22</v>
       </c>
       <c r="AE188" s="4" t="n">
         <v>0</v>
@@ -20928,7 +20928,7 @@
         </is>
       </c>
       <c r="I189" s="4" t="n">
-        <v>-33.42</v>
+        <v>-33.29</v>
       </c>
       <c r="J189" s="4" t="n">
         <v>0</v>
@@ -20942,13 +20942,13 @@
         </is>
       </c>
       <c r="M189" s="4" t="n">
-        <v>-36.93</v>
+        <v>-36.8</v>
       </c>
       <c r="N189" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O189" s="4" t="n">
-        <v>-33.42</v>
+        <v>-33.29</v>
       </c>
       <c r="P189" s="4" t="n">
         <v>-1.49</v>
@@ -20980,10 +20980,10 @@
         <v>0</v>
       </c>
       <c r="AC189" s="4" t="n">
-        <v>33.29</v>
+        <v>33.36</v>
       </c>
       <c r="AD189" s="4" t="n">
-        <v>66.70999999999999</v>
+        <v>66.64</v>
       </c>
       <c r="AE189" s="4" t="n">
         <v>0</v>
@@ -21031,7 +21031,7 @@
         </is>
       </c>
       <c r="I190" s="4" t="n">
-        <v>-15.89</v>
+        <v>-15.76</v>
       </c>
       <c r="J190" s="4" t="n">
         <v>0.6</v>
@@ -21045,13 +21045,13 @@
         </is>
       </c>
       <c r="M190" s="4" t="n">
-        <v>-19.64</v>
+        <v>-19.51</v>
       </c>
       <c r="N190" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O190" s="4" t="n">
-        <v>-15.89</v>
+        <v>-15.76</v>
       </c>
       <c r="P190" s="4" t="n">
         <v>-1.4</v>
@@ -21083,10 +21083,10 @@
         <v>0</v>
       </c>
       <c r="AC190" s="4" t="n">
-        <v>42.06</v>
+        <v>42.12</v>
       </c>
       <c r="AD190" s="4" t="n">
-        <v>57.94</v>
+        <v>57.88</v>
       </c>
       <c r="AE190" s="4" t="n">
         <v>0</v>
@@ -21134,7 +21134,7 @@
         </is>
       </c>
       <c r="I191" s="4" t="n">
-        <v>22.39</v>
+        <v>22.52</v>
       </c>
       <c r="J191" s="4" t="n">
         <v>99.90000000000001</v>
@@ -21148,13 +21148,13 @@
         </is>
       </c>
       <c r="M191" s="4" t="n">
-        <v>8.99</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="N191" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O191" s="4" t="n">
-        <v>22.39</v>
+        <v>22.52</v>
       </c>
       <c r="P191" s="4" t="n">
         <v>1.34</v>
@@ -21186,10 +21186,10 @@
         <v>0</v>
       </c>
       <c r="AC191" s="4" t="n">
-        <v>61.19</v>
+        <v>61.26</v>
       </c>
       <c r="AD191" s="4" t="n">
-        <v>38.81</v>
+        <v>38.74</v>
       </c>
       <c r="AE191" s="4" t="n">
         <v>0</v>
@@ -25817,10 +25817,10 @@
         <v>0.35</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>52.3</v>
+        <v>52.5</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>47.7</v>
+        <v>47.5</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29542,7 +29542,7 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>1.31</v>
+        <v>1.32</v>
       </c>
       <c r="J269" s="4" t="n">
         <v>59.3</v>
@@ -29556,13 +29556,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-6.07</v>
+        <v>-6.06</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>0.02</v>
@@ -29659,7 +29659,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-23.64</v>
+        <v>-23.63</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0.1</v>
@@ -29673,13 +29673,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-25.03</v>
+        <v>-25.02</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-25.43</v>
+        <v>-25.42</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.65</v>
@@ -51467,10 +51467,10 @@
         <v>2.93</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>71</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>29</v>
+        <v>29.6</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -51795,7 +51795,7 @@
         </is>
       </c>
       <c r="I476" s="4" t="n">
-        <v>28.18</v>
+        <v>28.16</v>
       </c>
       <c r="J476" s="4" t="n">
         <v>100</v>
@@ -51809,13 +51809,13 @@
         </is>
       </c>
       <c r="M476" s="4" t="n">
-        <v>13.78</v>
+        <v>13.77</v>
       </c>
       <c r="N476" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O476" s="4" t="n">
-        <v>27.84</v>
+        <v>27.82</v>
       </c>
       <c r="P476" s="4" t="n">
         <v>2.94</v>
@@ -51855,10 +51855,10 @@
         <v>0</v>
       </c>
       <c r="AC476" s="4" t="n">
-        <v>56.91</v>
+        <v>56.9</v>
       </c>
       <c r="AD476" s="4" t="n">
-        <v>31.89</v>
+        <v>31.9</v>
       </c>
       <c r="AE476" s="4" t="n">
         <v>3.6</v>
@@ -52461,7 +52461,7 @@
         </is>
       </c>
       <c r="I482" s="4" t="n">
-        <v>18.12</v>
+        <v>18.18</v>
       </c>
       <c r="J482" s="4" t="n">
         <v>99.7</v>
@@ -52475,13 +52475,13 @@
         </is>
       </c>
       <c r="M482" s="4" t="n">
-        <v>15.25</v>
+        <v>15.4</v>
       </c>
       <c r="N482" s="4" t="n">
         <v>7.57</v>
       </c>
       <c r="O482" s="4" t="n">
-        <v>23.05</v>
+        <v>23.19</v>
       </c>
       <c r="P482" s="4" t="n">
         <v>0.22</v>
@@ -52527,10 +52527,10 @@
         <v>0</v>
       </c>
       <c r="AC482" s="4" t="n">
-        <v>57.36</v>
+        <v>57.39</v>
       </c>
       <c r="AD482" s="4" t="n">
-        <v>39.76</v>
+        <v>39.73</v>
       </c>
       <c r="AE482" s="4" t="n">
         <v>0</v>
@@ -53033,10 +53033,10 @@
         <v>2.76</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>69.3</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>30.7</v>
+        <v>30.4</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53538,16 +53538,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>29.27</v>
+        <v>29.25</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.3</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>18.4</v>
+        <v>18.43</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>48.67</v>
+        <v>48.66</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-22: add GSG CO-05 poll (Oct 14-18)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.9</v>
+        <v>52.8</v>
       </c>
       <c r="C8" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
       <c r="D8" t="n">
         <v>54</v>
       </c>
       <c r="E8" t="n">
-        <v>73.59999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>247.2</v>
+        <v>247</v>
       </c>
       <c r="C9" t="n">
-        <v>187.8</v>
+        <v>188</v>
       </c>
       <c r="D9" t="n">
         <v>244</v>
       </c>
       <c r="E9" t="n">
-        <v>92.3</v>
+        <v>92.2</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>74.3</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.73</v>
+        <v>14.69</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.3</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>34.94</v>
+        <v>34.95</v>
       </c>
       <c r="AB30" s="4" t="n">
         <v>0.7</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.67</v>
+        <v>49.64</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>15.39</v>
+        <v>15.42</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-2.45</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>31.3</v>
+        <v>32.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>68.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.49</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>31.3</v>
+        <v>32.1</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -13008,13 +13008,13 @@
         </is>
       </c>
       <c r="I115" s="4" t="n">
-        <v>-3.51</v>
+        <v>-1.7</v>
       </c>
       <c r="J115" s="4" t="n">
-        <v>25.6</v>
+        <v>38</v>
       </c>
       <c r="K115" s="4" t="n">
-        <v>74.40000000000001</v>
+        <v>62</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -13040,16 +13040,16 @@
         <v>-9.34</v>
       </c>
       <c r="S115" s="4" t="n">
-        <v>43.99</v>
+        <v>44.47</v>
       </c>
       <c r="T115" s="4" t="n">
-        <v>45</v>
+        <v>41.23</v>
       </c>
       <c r="U115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V115" s="4" t="n">
-        <v>-1.52</v>
+        <v>0.71</v>
       </c>
       <c r="W115" s="5" t="n">
         <v>4968409</v>
@@ -13068,16 +13068,16 @@
         </is>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>0.5</v>
+        <v>1.41</v>
       </c>
       <c r="AB115" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC115" s="4" t="n">
-        <v>46.04</v>
+        <v>46.45</v>
       </c>
       <c r="AD115" s="4" t="n">
-        <v>49.38</v>
+        <v>48.06</v>
       </c>
       <c r="AE115" s="4" t="n">
         <v>4.08</v>
@@ -25817,10 +25817,10 @@
         <v>0.37</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>52.3</v>
+        <v>53.1</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>47.7</v>
+        <v>46.9</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29542,13 +29542,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>2.32</v>
+        <v>2.3</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>66.40000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>33.6</v>
+        <v>33.8</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -29556,13 +29556,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-6.06</v>
+        <v>-6.11</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>7.56</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>0.15</v>
@@ -29608,10 +29608,10 @@
         <v>0</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>50.75</v>
+        <v>50.74</v>
       </c>
       <c r="AD269" s="4" t="n">
-        <v>48.45</v>
+        <v>48.46</v>
       </c>
       <c r="AE269" s="4" t="n">
         <v>0</v>
@@ -29659,7 +29659,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-23.66</v>
+        <v>-23.7</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0.1</v>
@@ -29673,13 +29673,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-25.02</v>
+        <v>-25.07</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>7.56</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-25.43</v>
+        <v>-25.48</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.65</v>
@@ -29725,10 +29725,10 @@
         <v>0</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>33.35</v>
+        <v>33.33</v>
       </c>
       <c r="AD270" s="4" t="n">
-        <v>54.01</v>
+        <v>54.03</v>
       </c>
       <c r="AE270" s="4" t="n">
         <v>3.64</v>
@@ -51467,10 +51467,10 @@
         <v>2.91</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>28.6</v>
+        <v>29.3</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -53033,10 +53033,10 @@
         <v>2.75</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>69.09999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>30.9</v>
+        <v>31.5</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53478,7 +53478,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-19.37</v>
+        <v>-19.55</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53538,16 +53538,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>29.29</v>
+        <v>29.2</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.3</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>18.4</v>
+        <v>18.38</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>48.66</v>
+        <v>48.76</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Forecast update 2026-10-30 (poll refresh)
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -547,10 +547,10 @@
         <v>47</v>
       </c>
       <c r="D8" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E8" t="n">
-        <v>74.7</v>
+        <v>74.8</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>244</v>
       </c>
       <c r="E9" t="n">
-        <v>91.7</v>
+        <v>91.8</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>73.90000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -2356,13 +2356,13 @@
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>-5.37</v>
+        <v>-5.46</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>17.8</v>
+        <v>17.5</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>82.2</v>
+        <v>82.5</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -2388,16 +2388,16 @@
         <v>-16.41</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>45.1</v>
+        <v>45.65</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>48.47</v>
+        <v>49.39</v>
       </c>
       <c r="U15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>-3.01</v>
+        <v>-3.45</v>
       </c>
       <c r="W15" s="5" t="n">
         <v>0</v>
@@ -2414,10 +2414,10 @@
         <v>0</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>47.31</v>
+        <v>47.27</v>
       </c>
       <c r="AD15" s="4" t="n">
-        <v>52.69</v>
+        <v>52.73</v>
       </c>
       <c r="AE15" s="4" t="n">
         <v>0</v>
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.76</v>
+        <v>14.8</v>
       </c>
       <c r="J30" s="4" t="n">
-        <v>99.2</v>
+        <v>99.3</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>0</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>34.95</v>
+        <v>34.92</v>
       </c>
       <c r="AB30" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.71</v>
+        <v>49.73</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>15.34</v>
+        <v>15.35</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-1.91</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>35.1</v>
+        <v>36.5</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.76</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>35.1</v>
+        <v>36.5</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -22200,7 +22200,7 @@
         </is>
       </c>
       <c r="I201" s="4" t="n">
-        <v>-25.55</v>
+        <v>-25.54</v>
       </c>
       <c r="J201" s="4" t="n">
         <v>0.1</v>
@@ -22214,13 +22214,13 @@
         </is>
       </c>
       <c r="M201" s="4" t="n">
-        <v>-26.27</v>
+        <v>-26.26</v>
       </c>
       <c r="N201" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O201" s="4" t="n">
-        <v>-26.09</v>
+        <v>-26.08</v>
       </c>
       <c r="P201" s="4" t="n">
         <v>-1.72</v>
@@ -22311,7 +22311,7 @@
         </is>
       </c>
       <c r="I202" s="4" t="n">
-        <v>-8.4</v>
+        <v>-8.390000000000001</v>
       </c>
       <c r="J202" s="4" t="n">
         <v>8.4</v>
@@ -22325,13 +22325,13 @@
         </is>
       </c>
       <c r="M202" s="4" t="n">
-        <v>-13.84</v>
+        <v>-13.83</v>
       </c>
       <c r="N202" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O202" s="4" t="n">
-        <v>-11.97</v>
+        <v>-11.96</v>
       </c>
       <c r="P202" s="4" t="n">
         <v>-0.19</v>
@@ -22428,7 +22428,7 @@
         </is>
       </c>
       <c r="I203" s="4" t="n">
-        <v>26.99</v>
+        <v>27</v>
       </c>
       <c r="J203" s="4" t="n">
         <v>100</v>
@@ -22442,13 +22442,13 @@
         </is>
       </c>
       <c r="M203" s="4" t="n">
-        <v>9.130000000000001</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="N203" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O203" s="4" t="n">
-        <v>26.4</v>
+        <v>26.41</v>
       </c>
       <c r="P203" s="4" t="n">
         <v>2.88</v>
@@ -22539,7 +22539,7 @@
         </is>
       </c>
       <c r="I204" s="4" t="n">
-        <v>-16.65</v>
+        <v>-16.64</v>
       </c>
       <c r="J204" s="4" t="n">
         <v>0.5</v>
@@ -22553,13 +22553,13 @@
         </is>
       </c>
       <c r="M204" s="4" t="n">
-        <v>-18.23</v>
+        <v>-18.22</v>
       </c>
       <c r="N204" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O204" s="4" t="n">
-        <v>-17.23</v>
+        <v>-17.22</v>
       </c>
       <c r="P204" s="4" t="n">
         <v>-0.95</v>
@@ -22599,10 +22599,10 @@
         <v>0</v>
       </c>
       <c r="AC204" s="4" t="n">
-        <v>40.47</v>
+        <v>40.48</v>
       </c>
       <c r="AD204" s="4" t="n">
-        <v>56.65</v>
+        <v>56.64</v>
       </c>
       <c r="AE204" s="4" t="n">
         <v>0</v>
@@ -25829,10 +25829,10 @@
         <v>0.13</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>50.6</v>
+        <v>51.1</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>49.4</v>
+        <v>48.9</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29560,13 +29560,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>4.01</v>
+        <v>4</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>77.3</v>
+        <v>77.2</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -29574,13 +29574,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-5.57</v>
+        <v>-5.59</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>0.11</v>
@@ -29677,7 +29677,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-18.77</v>
+        <v>-18.78</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0.3</v>
@@ -29691,13 +29691,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-24.53</v>
+        <v>-24.55</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-24.86</v>
+        <v>-24.88</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.67</v>
@@ -29743,10 +29743,10 @@
         <v>0</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>33.09</v>
+        <v>33.08</v>
       </c>
       <c r="AD270" s="4" t="n">
-        <v>48.38</v>
+        <v>48.39</v>
       </c>
       <c r="AE270" s="4" t="n">
         <v>3.64</v>
@@ -51485,10 +51485,10 @@
         <v>2.99</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>71.3</v>
+        <v>72.5</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>28.7</v>
+        <v>27.5</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -52596,13 +52596,13 @@
         </is>
       </c>
       <c r="I483" s="4" t="n">
-        <v>-0.11</v>
+        <v>0.01</v>
       </c>
       <c r="J483" s="4" t="n">
-        <v>49.2</v>
+        <v>50.1</v>
       </c>
       <c r="K483" s="4" t="n">
-        <v>50.8</v>
+        <v>49.9</v>
       </c>
       <c r="L483" t="inlineStr">
         <is>
@@ -52610,13 +52610,13 @@
         </is>
       </c>
       <c r="M483" s="4" t="n">
-        <v>-13.66</v>
+        <v>-13.69</v>
       </c>
       <c r="N483" s="4" t="n">
         <v>7.65</v>
       </c>
       <c r="O483" s="4" t="n">
-        <v>-6.9</v>
+        <v>-6.93</v>
       </c>
       <c r="P483" s="4" t="n">
         <v>0.63</v>
@@ -52628,16 +52628,16 @@
         <v>-16.41</v>
       </c>
       <c r="S483" s="4" t="n">
-        <v>47.73</v>
+        <v>48.05</v>
       </c>
       <c r="T483" s="4" t="n">
-        <v>44.86</v>
+        <v>45.26</v>
       </c>
       <c r="U483" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V483" s="4" t="n">
-        <v>3.35</v>
+        <v>3.18</v>
       </c>
       <c r="W483" s="5" t="n">
         <v>19175044</v>
@@ -52656,16 +52656,16 @@
         </is>
       </c>
       <c r="AA483" s="4" t="n">
-        <v>1.56</v>
+        <v>1.89</v>
       </c>
       <c r="AB483" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC483" s="4" t="n">
-        <v>49.17</v>
+        <v>49.06</v>
       </c>
       <c r="AD483" s="4" t="n">
-        <v>49.27</v>
+        <v>49.05</v>
       </c>
       <c r="AE483" s="4" t="n">
         <v>0</v>
@@ -53051,10 +53051,10 @@
         <v>2.95</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>71.2</v>
+        <v>71.3</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>28.8</v>
+        <v>28.7</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53496,7 +53496,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-17.91</v>
+        <v>-17.9</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53556,16 +53556,16 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>29.77</v>
+        <v>29.81</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.4</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>18.89</v>
+        <v>18.82</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>47.68</v>
+        <v>47.71</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>

</xml_diff>

<commit_message>
Poll refresh + forecast update 2026-10-31 (rerun)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="D8" t="n">
         <v>53</v>
       </c>
-      <c r="C8" t="n">
-        <v>47</v>
-      </c>
-      <c r="D8" t="n">
-        <v>54</v>
-      </c>
       <c r="E8" t="n">
-        <v>74.5</v>
+        <v>73.8</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,10 +566,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>246.9</v>
+        <v>247.3</v>
       </c>
       <c r="C9" t="n">
-        <v>188.1</v>
+        <v>187.7</v>
       </c>
       <c r="D9" t="n">
         <v>244</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="C10" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="D10" t="n">
         <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>73.59999999999999</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -3038,17 +3038,17 @@
         </is>
       </c>
       <c r="I21" s="4" t="n">
-        <v>-6.83</v>
+        <v>-10.2</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>13</v>
+        <v>3.7</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>87</v>
+        <v>96.3</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Safe R</t>
         </is>
       </c>
       <c r="M21" s="4" t="n">
@@ -3070,16 +3070,16 @@
         <v>-20.84</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>40.83</v>
+        <v>40.27</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>43.54</v>
+        <v>47.86</v>
       </c>
       <c r="U21" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>-2.3</v>
+        <v>-7.36</v>
       </c>
       <c r="W21" s="5" t="n">
         <v>0</v>
@@ -3098,16 +3098,16 @@
         </is>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>2.32</v>
+        <v>1.28</v>
       </c>
       <c r="AB21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>45.5</v>
+        <v>44.33</v>
       </c>
       <c r="AD21" s="4" t="n">
-        <v>52.18</v>
+        <v>54.39</v>
       </c>
       <c r="AE21" s="4" t="n">
         <v>0</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>14.72</v>
+        <v>14.67</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.3</v>
@@ -4119,16 +4119,16 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>34.96</v>
+        <v>34.99</v>
       </c>
       <c r="AB30" s="4" t="n">
         <v>0.7</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>49.68</v>
+        <v>49.66</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>15.36</v>
+        <v>15.35</v>
       </c>
       <c r="AE30" s="4" t="n">
         <v>0</v>
@@ -4511,13 +4511,13 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>-3.27</v>
+        <v>-3.24</v>
       </c>
       <c r="J34" s="4" t="n">
-        <v>27.2</v>
+        <v>27.4</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>72.8</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -4549,10 +4549,10 @@
         <v>48.89</v>
       </c>
       <c r="U34" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="V34" s="4" t="n">
-        <v>-1.31</v>
+        <v>-1.32</v>
       </c>
       <c r="W34" s="5" t="n">
         <v>21687161</v>
@@ -4571,7 +4571,7 @@
         </is>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="AB34" s="4" t="n">
         <v>0</v>
@@ -4580,7 +4580,7 @@
         <v>48.12</v>
       </c>
       <c r="AD34" s="4" t="n">
-        <v>51.36</v>
+        <v>51.35</v>
       </c>
       <c r="AE34" s="4" t="n">
         <v>0</v>
@@ -4960,10 +4960,10 @@
         <v>-1.93</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>35.6</v>
+        <v>34.7</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>64.40000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>45.75</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>35.6</v>
+        <v>34.7</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>3.8</v>
@@ -25835,10 +25835,10 @@
         <v>0.1</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>50.9</v>
+        <v>50.6</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>49.1</v>
+        <v>49.4</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -29566,7 +29566,7 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>3.96</v>
+        <v>3.97</v>
       </c>
       <c r="J269" s="4" t="n">
         <v>77.09999999999999</v>
@@ -29580,13 +29580,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-5.61</v>
+        <v>-5.58</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>1.16</v>
+        <v>1.19</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>0.11</v>
@@ -29683,7 +29683,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-18.89</v>
+        <v>-18.87</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0.3</v>
@@ -29697,13 +29697,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-24.57</v>
+        <v>-24.54</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-24.91</v>
+        <v>-24.88</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.67</v>
@@ -29749,10 +29749,10 @@
         <v>0</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>33.04</v>
+        <v>33.05</v>
       </c>
       <c r="AD270" s="4" t="n">
-        <v>48.43</v>
+        <v>48.42</v>
       </c>
       <c r="AE270" s="4" t="n">
         <v>3.64</v>
@@ -31471,13 +31471,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-4.05</v>
+        <v>-4.57</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>22.6</v>
+        <v>20.7</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>77.40000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -31485,13 +31485,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-9.699999999999999</v>
+        <v>-10.54</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-7.87</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.32</v>
@@ -31537,10 +31537,10 @@
         <v>0</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>45.66</v>
+        <v>45.41</v>
       </c>
       <c r="AD286" s="4" t="n">
-        <v>49.52</v>
+        <v>49.77</v>
       </c>
       <c r="AE286" s="4" t="n">
         <v>2.41</v>
@@ -31584,7 +31584,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>13.05</v>
+        <v>12.53</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>99</v>
@@ -31598,13 +31598,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.16</v>
+        <v>7.32</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>16.09</v>
+        <v>15.25</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.64</v>
@@ -31650,10 +31650,10 @@
         <v>0</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>55.86</v>
+        <v>55.6</v>
       </c>
       <c r="AD287" s="4" t="n">
-        <v>42.96</v>
+        <v>43.22</v>
       </c>
       <c r="AE287" s="4" t="n">
         <v>0</v>
@@ -31701,7 +31701,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-51.2</v>
+        <v>-52.04</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -31715,13 +31715,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-50.65</v>
+        <v>-51.49</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-51.01</v>
+        <v>-51.85</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.09</v>
@@ -31761,10 +31761,10 @@
         <v>0</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>23.43</v>
+        <v>23.03</v>
       </c>
       <c r="AD288" s="4" t="n">
-        <v>72.61</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="AE288" s="4" t="n">
         <v>1.98</v>
@@ -43551,10 +43551,10 @@
         <v>0</v>
       </c>
       <c r="AC398" s="4" t="n">
-        <v>30.2</v>
+        <v>30.21</v>
       </c>
       <c r="AD398" s="4" t="n">
-        <v>69.8</v>
+        <v>69.79000000000001</v>
       </c>
       <c r="AE398" s="4" t="n">
         <v>0</v>
@@ -43612,7 +43612,7 @@
         </is>
       </c>
       <c r="M399" s="4" t="n">
-        <v>-17.77</v>
+        <v>-17.76</v>
       </c>
       <c r="N399" s="4" t="n">
         <v>7.64</v>
@@ -43656,10 +43656,10 @@
         <v>0</v>
       </c>
       <c r="AC399" s="4" t="n">
-        <v>45.12</v>
+        <v>45.13</v>
       </c>
       <c r="AD399" s="4" t="n">
-        <v>54.88</v>
+        <v>54.87</v>
       </c>
       <c r="AE399" s="4" t="n">
         <v>0</v>
@@ -43759,10 +43759,10 @@
         <v>0</v>
       </c>
       <c r="AC400" s="4" t="n">
-        <v>44.11</v>
+        <v>44.12</v>
       </c>
       <c r="AD400" s="4" t="n">
-        <v>55.89</v>
+        <v>55.88</v>
       </c>
       <c r="AE400" s="4" t="n">
         <v>0</v>
@@ -43824,7 +43824,7 @@
         </is>
       </c>
       <c r="M401" s="4" t="n">
-        <v>-18.42</v>
+        <v>-18.41</v>
       </c>
       <c r="N401" s="4" t="n">
         <v>7.64</v>
@@ -43913,7 +43913,7 @@
         </is>
       </c>
       <c r="I402" s="4" t="n">
-        <v>-11.25</v>
+        <v>-11.24</v>
       </c>
       <c r="J402" s="4" t="n">
         <v>1.3</v>
@@ -43927,13 +43927,13 @@
         </is>
       </c>
       <c r="M402" s="4" t="n">
-        <v>-15.26</v>
+        <v>-15.25</v>
       </c>
       <c r="N402" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O402" s="4" t="n">
-        <v>-11.25</v>
+        <v>-11.24</v>
       </c>
       <c r="P402" s="4" t="n">
         <v>-2.02</v>
@@ -44030,7 +44030,7 @@
         </is>
       </c>
       <c r="M403" s="4" t="n">
-        <v>-17.34</v>
+        <v>-17.33</v>
       </c>
       <c r="N403" s="4" t="n">
         <v>7.64</v>
@@ -44068,10 +44068,10 @@
         <v>0</v>
       </c>
       <c r="AC403" s="4" t="n">
-        <v>42.61</v>
+        <v>42.62</v>
       </c>
       <c r="AD403" s="4" t="n">
-        <v>57.39</v>
+        <v>57.38</v>
       </c>
       <c r="AE403" s="4" t="n">
         <v>0</v>
@@ -44119,7 +44119,7 @@
         </is>
       </c>
       <c r="I404" s="4" t="n">
-        <v>43.82</v>
+        <v>43.83</v>
       </c>
       <c r="J404" s="4" t="n">
         <v>100</v>
@@ -44133,13 +44133,13 @@
         </is>
       </c>
       <c r="M404" s="4" t="n">
-        <v>31.99</v>
+        <v>32</v>
       </c>
       <c r="N404" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O404" s="4" t="n">
-        <v>44.54</v>
+        <v>44.55</v>
       </c>
       <c r="P404" s="4" t="n">
         <v>1.83</v>
@@ -44179,10 +44179,10 @@
         <v>0</v>
       </c>
       <c r="AC404" s="4" t="n">
-        <v>69.83</v>
+        <v>69.84</v>
       </c>
       <c r="AD404" s="4" t="n">
-        <v>27.28</v>
+        <v>27.27</v>
       </c>
       <c r="AE404" s="4" t="n">
         <v>0</v>
@@ -44226,7 +44226,7 @@
         </is>
       </c>
       <c r="I405" s="4" t="n">
-        <v>-14.31</v>
+        <v>-14.3</v>
       </c>
       <c r="J405" s="4" t="n">
         <v>0.8</v>
@@ -44240,13 +44240,13 @@
         </is>
       </c>
       <c r="M405" s="4" t="n">
-        <v>-20.05</v>
+        <v>-20.04</v>
       </c>
       <c r="N405" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O405" s="4" t="n">
-        <v>-14.31</v>
+        <v>-14.3</v>
       </c>
       <c r="P405" s="4" t="n">
         <v>-2.73</v>
@@ -44339,13 +44339,13 @@
         </is>
       </c>
       <c r="M406" s="4" t="n">
-        <v>-11.02</v>
+        <v>-11.01</v>
       </c>
       <c r="N406" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O406" s="4" t="n">
-        <v>-2.92</v>
+        <v>-2.91</v>
       </c>
       <c r="P406" s="4" t="n">
         <v>-1.72</v>
@@ -44430,13 +44430,13 @@
         </is>
       </c>
       <c r="I407" s="4" t="n">
-        <v>-9.25</v>
+        <v>-9.24</v>
       </c>
       <c r="J407" s="4" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="K407" s="4" t="n">
-        <v>94</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="L407" t="inlineStr">
         <is>
@@ -44539,7 +44539,7 @@
         </is>
       </c>
       <c r="I408" s="4" t="n">
-        <v>-23.79</v>
+        <v>-23.78</v>
       </c>
       <c r="J408" s="4" t="n">
         <v>0.1</v>
@@ -44559,7 +44559,7 @@
         <v>7.64</v>
       </c>
       <c r="O408" s="4" t="n">
-        <v>-23.79</v>
+        <v>-23.78</v>
       </c>
       <c r="P408" s="4" t="n">
         <v>-2.28</v>
@@ -44642,7 +44642,7 @@
         </is>
       </c>
       <c r="I409" s="4" t="n">
-        <v>-15.23</v>
+        <v>-15.22</v>
       </c>
       <c r="J409" s="4" t="n">
         <v>0.6</v>
@@ -44662,7 +44662,7 @@
         <v>7.64</v>
       </c>
       <c r="O409" s="4" t="n">
-        <v>-15.23</v>
+        <v>-15.22</v>
       </c>
       <c r="P409" s="4" t="n">
         <v>0</v>
@@ -44745,7 +44745,7 @@
         </is>
       </c>
       <c r="I410" s="4" t="n">
-        <v>-37.13</v>
+        <v>-37.12</v>
       </c>
       <c r="J410" s="4" t="n">
         <v>0</v>
@@ -44759,13 +44759,13 @@
         </is>
       </c>
       <c r="M410" s="4" t="n">
-        <v>-40.99</v>
+        <v>-40.98</v>
       </c>
       <c r="N410" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O410" s="4" t="n">
-        <v>-37.13</v>
+        <v>-37.12</v>
       </c>
       <c r="P410" s="4" t="n">
         <v>-2.44</v>
@@ -44848,7 +44848,7 @@
         </is>
       </c>
       <c r="I411" s="4" t="n">
-        <v>-16.15</v>
+        <v>-16.14</v>
       </c>
       <c r="J411" s="4" t="n">
         <v>0.5</v>
@@ -44862,13 +44862,13 @@
         </is>
       </c>
       <c r="M411" s="4" t="n">
-        <v>-18.4</v>
+        <v>-18.39</v>
       </c>
       <c r="N411" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O411" s="4" t="n">
-        <v>-16.15</v>
+        <v>-16.14</v>
       </c>
       <c r="P411" s="4" t="n">
         <v>-1.94</v>
@@ -44951,7 +44951,7 @@
         </is>
       </c>
       <c r="I412" s="4" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="J412" s="4" t="n">
         <v>80.8</v>
@@ -44965,13 +44965,13 @@
         </is>
       </c>
       <c r="M412" s="4" t="n">
-        <v>-7.09</v>
+        <v>-7.08</v>
       </c>
       <c r="N412" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O412" s="4" t="n">
-        <v>2.45</v>
+        <v>2.46</v>
       </c>
       <c r="P412" s="4" t="n">
         <v>0.15</v>
@@ -45112,10 +45112,10 @@
         <v>0</v>
       </c>
       <c r="AC413" s="4" t="n">
-        <v>71.19</v>
+        <v>71.2</v>
       </c>
       <c r="AD413" s="4" t="n">
-        <v>28.81</v>
+        <v>28.8</v>
       </c>
       <c r="AE413" s="4" t="n">
         <v>0</v>
@@ -45163,7 +45163,7 @@
         </is>
       </c>
       <c r="I414" s="4" t="n">
-        <v>-12.99</v>
+        <v>-12.98</v>
       </c>
       <c r="J414" s="4" t="n">
         <v>1</v>
@@ -45183,7 +45183,7 @@
         <v>7.64</v>
       </c>
       <c r="O414" s="4" t="n">
-        <v>-12.99</v>
+        <v>-12.98</v>
       </c>
       <c r="P414" s="4" t="n">
         <v>-1.7</v>
@@ -45266,7 +45266,7 @@
         </is>
       </c>
       <c r="I415" s="4" t="n">
-        <v>74.64</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="J415" s="4" t="n">
         <v>100</v>
@@ -45280,13 +45280,13 @@
         </is>
       </c>
       <c r="M415" s="4" t="n">
-        <v>64.05</v>
+        <v>64.06</v>
       </c>
       <c r="N415" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O415" s="4" t="n">
-        <v>74.64</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="P415" s="4" t="n">
         <v>0</v>
@@ -45468,7 +45468,7 @@
         </is>
       </c>
       <c r="I417" s="4" t="n">
-        <v>52.73</v>
+        <v>52.74</v>
       </c>
       <c r="J417" s="4" t="n">
         <v>100</v>
@@ -45488,7 +45488,7 @@
         <v>7.64</v>
       </c>
       <c r="O417" s="4" t="n">
-        <v>52.73</v>
+        <v>52.74</v>
       </c>
       <c r="P417" s="4" t="n">
         <v>1.26</v>
@@ -45581,7 +45581,7 @@
         </is>
       </c>
       <c r="M418" s="4" t="n">
-        <v>-15.68</v>
+        <v>-15.67</v>
       </c>
       <c r="N418" s="4" t="n">
         <v>7.64</v>
@@ -45619,10 +45619,10 @@
         <v>0</v>
       </c>
       <c r="AC418" s="4" t="n">
-        <v>45.74</v>
+        <v>45.75</v>
       </c>
       <c r="AD418" s="4" t="n">
-        <v>54.26</v>
+        <v>54.25</v>
       </c>
       <c r="AE418" s="4" t="n">
         <v>0</v>
@@ -45666,7 +45666,7 @@
         </is>
       </c>
       <c r="I419" s="4" t="n">
-        <v>-9.65</v>
+        <v>-9.640000000000001</v>
       </c>
       <c r="J419" s="4" t="n">
         <v>5</v>
@@ -45680,13 +45680,13 @@
         </is>
       </c>
       <c r="M419" s="4" t="n">
-        <v>-16.26</v>
+        <v>-16.25</v>
       </c>
       <c r="N419" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O419" s="4" t="n">
-        <v>-9.65</v>
+        <v>-9.640000000000001</v>
       </c>
       <c r="P419" s="4" t="n">
         <v>-0.96</v>
@@ -45718,10 +45718,10 @@
         <v>0</v>
       </c>
       <c r="AC419" s="4" t="n">
-        <v>45.17</v>
+        <v>45.18</v>
       </c>
       <c r="AD419" s="4" t="n">
-        <v>54.83</v>
+        <v>54.82</v>
       </c>
       <c r="AE419" s="4" t="n">
         <v>0</v>
@@ -45779,7 +45779,7 @@
         </is>
       </c>
       <c r="M420" s="4" t="n">
-        <v>-7.26</v>
+        <v>-7.25</v>
       </c>
       <c r="N420" s="4" t="n">
         <v>7.64</v>
@@ -45934,10 +45934,10 @@
         <v>0</v>
       </c>
       <c r="AC421" s="4" t="n">
-        <v>45.5</v>
+        <v>45.51</v>
       </c>
       <c r="AD421" s="4" t="n">
-        <v>54.5</v>
+        <v>54.49</v>
       </c>
       <c r="AE421" s="4" t="n">
         <v>0</v>
@@ -46108,7 +46108,7 @@
         <v>7.64</v>
       </c>
       <c r="O423" s="4" t="n">
-        <v>-19.39</v>
+        <v>-19.38</v>
       </c>
       <c r="P423" s="4" t="n">
         <v>-3.4</v>
@@ -46199,7 +46199,7 @@
         </is>
       </c>
       <c r="I424" s="4" t="n">
-        <v>-10.08</v>
+        <v>-10.07</v>
       </c>
       <c r="J424" s="4" t="n">
         <v>4</v>
@@ -46213,13 +46213,13 @@
         </is>
       </c>
       <c r="M424" s="4" t="n">
-        <v>-15.18</v>
+        <v>-15.17</v>
       </c>
       <c r="N424" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O424" s="4" t="n">
-        <v>-10.08</v>
+        <v>-10.07</v>
       </c>
       <c r="P424" s="4" t="n">
         <v>-1.03</v>
@@ -46302,7 +46302,7 @@
         </is>
       </c>
       <c r="I425" s="4" t="n">
-        <v>20.14</v>
+        <v>20.15</v>
       </c>
       <c r="J425" s="4" t="n">
         <v>99.8</v>
@@ -46316,13 +46316,13 @@
         </is>
       </c>
       <c r="M425" s="4" t="n">
-        <v>2.48</v>
+        <v>2.49</v>
       </c>
       <c r="N425" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O425" s="4" t="n">
-        <v>24.05</v>
+        <v>24.06</v>
       </c>
       <c r="P425" s="4" t="n">
         <v>0.73</v>
@@ -46518,7 +46518,7 @@
         </is>
       </c>
       <c r="I427" s="4" t="n">
-        <v>66.76000000000001</v>
+        <v>66.77</v>
       </c>
       <c r="J427" s="4" t="n">
         <v>100</v>
@@ -46538,7 +46538,7 @@
         <v>7.64</v>
       </c>
       <c r="O427" s="4" t="n">
-        <v>66.76000000000001</v>
+        <v>66.77</v>
       </c>
       <c r="P427" s="4" t="n">
         <v>1.78</v>
@@ -46641,7 +46641,7 @@
         <v>7.64</v>
       </c>
       <c r="O428" s="4" t="n">
-        <v>-14.21</v>
+        <v>-14.2</v>
       </c>
       <c r="P428" s="4" t="n">
         <v>-1.15</v>
@@ -46728,13 +46728,13 @@
         </is>
       </c>
       <c r="I429" s="4" t="n">
-        <v>-4.78</v>
+        <v>-4.77</v>
       </c>
       <c r="J429" s="4" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="K429" s="4" t="n">
-        <v>80.09999999999999</v>
+        <v>80</v>
       </c>
       <c r="L429" t="inlineStr">
         <is>
@@ -46742,13 +46742,13 @@
         </is>
       </c>
       <c r="M429" s="4" t="n">
-        <v>-10.95</v>
+        <v>-10.94</v>
       </c>
       <c r="N429" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O429" s="4" t="n">
-        <v>-4.78</v>
+        <v>-4.77</v>
       </c>
       <c r="P429" s="4" t="n">
         <v>-1.73</v>
@@ -46841,7 +46841,7 @@
         </is>
       </c>
       <c r="M430" s="4" t="n">
-        <v>42.19</v>
+        <v>42.2</v>
       </c>
       <c r="N430" s="4" t="n">
         <v>7.64</v>
@@ -46944,13 +46944,13 @@
         </is>
       </c>
       <c r="M431" s="4" t="n">
-        <v>-0.37</v>
+        <v>-0.36</v>
       </c>
       <c r="N431" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O431" s="4" t="n">
-        <v>14.9</v>
+        <v>14.91</v>
       </c>
       <c r="P431" s="4" t="n">
         <v>0.31</v>
@@ -47046,10 +47046,10 @@
         <v>3.89</v>
       </c>
       <c r="J432" s="4" t="n">
-        <v>76.8</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="K432" s="4" t="n">
-        <v>23.2</v>
+        <v>23.1</v>
       </c>
       <c r="L432" t="inlineStr">
         <is>
@@ -47063,7 +47063,7 @@
         <v>7.64</v>
       </c>
       <c r="O432" s="4" t="n">
-        <v>6.67</v>
+        <v>6.68</v>
       </c>
       <c r="P432" s="4" t="n">
         <v>0.02</v>
@@ -47152,7 +47152,7 @@
         </is>
       </c>
       <c r="I433" s="4" t="n">
-        <v>-14.55</v>
+        <v>-14.54</v>
       </c>
       <c r="J433" s="4" t="n">
         <v>0.7</v>
@@ -47166,13 +47166,13 @@
         </is>
       </c>
       <c r="M433" s="4" t="n">
-        <v>-17.98</v>
+        <v>-17.97</v>
       </c>
       <c r="N433" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O433" s="4" t="n">
-        <v>-14.55</v>
+        <v>-14.54</v>
       </c>
       <c r="P433" s="4" t="n">
         <v>-2.12</v>
@@ -47255,7 +47255,7 @@
         </is>
       </c>
       <c r="I434" s="4" t="n">
-        <v>74.78</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="J434" s="4" t="n">
         <v>100</v>
@@ -47269,13 +47269,13 @@
         </is>
       </c>
       <c r="M434" s="4" t="n">
-        <v>64.81</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="N434" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O434" s="4" t="n">
-        <v>74.78</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="P434" s="4" t="n">
         <v>1.55</v>
@@ -47354,13 +47354,13 @@
         </is>
       </c>
       <c r="I435" s="4" t="n">
-        <v>-10.43</v>
+        <v>-10.42</v>
       </c>
       <c r="J435" s="4" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="K435" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>96.8</v>
       </c>
       <c r="L435" t="inlineStr">
         <is>
@@ -47368,7 +47368,7 @@
         </is>
       </c>
       <c r="M435" s="4" t="n">
-        <v>-15.42</v>
+        <v>-15.41</v>
       </c>
       <c r="N435" s="4" t="n">
         <v>7.64</v>
@@ -51491,10 +51491,10 @@
         <v>2.51</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>32.4</v>
+        <v>31.4</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -53057,10 +53057,10 @@
         <v>2.93</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>70.8</v>
+        <v>72</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>29.2</v>
+        <v>28</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -53502,7 +53502,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-18.03</v>
+        <v>-17.91</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -53562,7 +53562,7 @@
         </is>
       </c>
       <c r="AA491" s="4" t="n">
-        <v>29.73</v>
+        <v>29.79</v>
       </c>
       <c r="AB491" s="4" t="n">
         <v>0.4</v>
@@ -53571,7 +53571,7 @@
         <v>18.86</v>
       </c>
       <c r="AD491" s="4" t="n">
-        <v>47.75</v>
+        <v>47.69</v>
       </c>
       <c r="AE491" s="4" t="n">
         <v>3.66</v>
@@ -53732,27 +53732,27 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>0.02</v>
+        <v>-2.01</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>50.1</v>
+        <v>35.5</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>49.9</v>
+        <v>64.5</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
-          <t>Toss-up</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M493" s="4" t="n">
-        <v>-17.41</v>
+        <v>-18.25</v>
       </c>
       <c r="N493" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O493" s="4" t="n">
-        <v>-1.48</v>
+        <v>-2.32</v>
       </c>
       <c r="P493" s="4" t="n">
         <v>0.14</v>
@@ -53764,16 +53764,16 @@
         <v>-20.84</v>
       </c>
       <c r="S493" s="4" t="n">
-        <v>46.74</v>
+        <v>45.14</v>
       </c>
       <c r="T493" s="4" t="n">
-        <v>46.37</v>
+        <v>47.36</v>
       </c>
       <c r="U493" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="V493" s="4" t="n">
-        <v>0.92</v>
+        <v>-1.91</v>
       </c>
       <c r="W493" s="5" t="n">
         <v>0</v>
@@ -53792,16 +53792,16 @@
         </is>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>48.92</v>
+        <v>47.9</v>
       </c>
       <c r="AB493" s="4" t="n">
-        <v>50.1</v>
+        <v>35.5</v>
       </c>
       <c r="AC493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AD493" s="4" t="n">
-        <v>48.9</v>
+        <v>49.92</v>
       </c>
       <c r="AE493" s="4" t="n">
         <v>2.18</v>
@@ -55001,13 +55001,13 @@
         </is>
       </c>
       <c r="M504" s="4" t="n">
-        <v>-9.279999999999999</v>
+        <v>-9.27</v>
       </c>
       <c r="N504" s="4" t="n">
         <v>7.64</v>
       </c>
       <c r="O504" s="4" t="n">
-        <v>1.75</v>
+        <v>1.76</v>
       </c>
       <c r="P504" s="4" t="n">
         <v>0.3</v>
@@ -55019,16 +55019,16 @@
         <v>-13.88</v>
       </c>
       <c r="S504" s="4" t="n">
-        <v>49.33</v>
+        <v>49.3</v>
       </c>
       <c r="T504" s="4" t="n">
-        <v>45.66</v>
+        <v>45.65</v>
       </c>
       <c r="U504" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="V504" s="4" t="n">
-        <v>4.29</v>
+        <v>4.27</v>
       </c>
       <c r="W504" s="5" t="n">
         <v>146349912</v>
@@ -55047,7 +55047,7 @@
         </is>
       </c>
       <c r="AA504" s="4" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="AB504" s="4" t="n">
         <v>0</v>
@@ -55056,7 +55056,7 @@
         <v>51.47</v>
       </c>
       <c r="AD504" s="4" t="n">
-        <v>47.88</v>
+        <v>47.89</v>
       </c>
       <c r="AE504" s="4" t="n">
         <v>0</v>
@@ -58499,7 +58499,7 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="K53" t="n">
         <v>19</v>

</xml_diff>